<commit_message>
Escala de notas de 1 a 5 em cada subcritério do checklist
Acrescenta como medir, tipo de nota (faixa fixa, classe ou quintil), as
cinco faixas e a origem de cada faixa. A planilha passa a ser gerada por
scripts/gerar_checklist_subcriterios.py.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018419ScLbL3ubanHMYyaBnW
</commit_message>
<xml_diff>
--- a/dados/Recife_Resiliente_Checklist_Subcriterios.xlsx
+++ b/dados/Recife_Resiliente_Checklist_Subcriterios.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Checklist subcritérios" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Checklist subcritérios'!$A$4:$I$19</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Checklist subcritérios'!$A$4:$Q$19</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -71,7 +71,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="12">
     <fill>
       <patternFill/>
     </fill>
@@ -90,12 +90,32 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
+        <fgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E2EFDA"/>
+        <fgColor rgb="00F4F9EE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF9E5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FDE9D9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F8CBAD"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
     <fill>
@@ -135,7 +155,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -153,28 +173,43 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -579,31 +614,39 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I26"/>
+  <dimension ref="A1:Q26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="15" customWidth="1" min="1" max="1"/>
-    <col width="8" customWidth="1" min="2" max="2"/>
-    <col width="34" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
-    <col width="42" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
-    <col width="13" customWidth="1" min="7" max="7"/>
-    <col width="42" customWidth="1" min="8" max="8"/>
-    <col width="34" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="7" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="15" customWidth="1" min="9" max="9"/>
+    <col width="17" customWidth="1" min="10" max="10"/>
+    <col width="22" customWidth="1" min="11" max="11"/>
+    <col width="24" customWidth="1" min="12" max="12"/>
+    <col width="34" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+    <col width="12" customWidth="1" min="15" max="15"/>
+    <col width="34" customWidth="1" min="16" max="16"/>
+    <col width="30" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Recife Resiliente — Subcritérios, fontes e checklist de confirmação dos dados (RPA 6)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="42" customHeight="1">
+          <t>Recife Resiliente — Subcritérios, notas, fontes e checklist dos dados (RPA 6)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="44" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Proposta de 02/10/2026 (Pedro + Claude), ainda não validada pelo grupo. Preencha as colunas amarelas (F, G e H): Sim / Não / Parcial / Pendente. 'Fonte confirmada' = a base existe e é acessível. 'Dado existe na fonte' = a variável está lá, na escala necessária (círculo de 300 m) e cobre os 21 pontos.</t>
+          <t>Proposta de 02/10/2026 (Pedro + Claude), não validada pelo grupo. Nota 5 = mais crítico. Faixa fixa = valor absoluto (provisória: calibrar com os dados reais). Quintil = nota relativa entre os 21 pontos (Quintil 1 = 20% com menor valor). Preencha as colunas amarelas (N, O e P): Sim / Não / Parcial / Pendente. 'Fonte confirmada' = a base existe e é acessível; 'Dado existe na fonte' = a variável está lá, na escala do círculo de 300 m, e cobre os 21 pontos.</t>
         </is>
       </c>
     </row>
@@ -625,30 +668,70 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
+          <t>Como medir</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Tipo de nota</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Nota 1</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>Nota 2</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>Nota 3</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>Nota 4</t>
+        </is>
+      </c>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>Nota 5</t>
+        </is>
+      </c>
+      <c r="K4" s="3" t="inlineStr">
+        <is>
+          <t>Origem da faixa</t>
+        </is>
+      </c>
+      <c r="L4" s="3" t="inlineStr">
+        <is>
           <t>Recomendação</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="M4" s="3" t="inlineStr">
         <is>
           <t>Fonte</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="N4" s="3" t="inlineStr">
         <is>
           <t>Fonte confirmada?</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="O4" s="3" t="inlineStr">
         <is>
           <t>Dado existe na fonte?</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr">
+      <c r="P4" s="3" t="inlineStr">
         <is>
           <t>Observação</t>
         </is>
       </c>
-      <c r="I4" s="3" t="inlineStr">
+      <c r="Q4" s="3" t="inlineStr">
         <is>
           <t>Busca prévia (Claude)</t>
         </is>
@@ -667,35 +750,75 @@
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>Frequência de alagamento (eventos/ano)</t>
+          <t>Frequência de alagamento</t>
         </is>
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
+          <t>Média de eventos por ano nas 3 últimas estações chuvosas</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>Faixa fixa</t>
+        </is>
+      </c>
+      <c r="F5" s="8" t="inlineStr">
+        <is>
+          <t>&lt; 1</t>
+        </is>
+      </c>
+      <c r="G5" s="9" t="inlineStr">
+        <is>
+          <t>1–2</t>
+        </is>
+      </c>
+      <c r="H5" s="10" t="inlineStr">
+        <is>
+          <t>3–4</t>
+        </is>
+      </c>
+      <c r="I5" s="11" t="inlineStr">
+        <is>
+          <t>5–6</t>
+        </is>
+      </c>
+      <c r="J5" s="12" t="inlineStr">
+        <is>
+          <t>≥ 7</t>
+        </is>
+      </c>
+      <c r="K5" s="6" t="inlineStr">
+        <is>
+          <t>Planilha original (provisória)</t>
+        </is>
+      </c>
+      <c r="L5" s="6" t="inlineStr">
+        <is>
           <t>Manter — peso alto</t>
         </is>
       </c>
-      <c r="E5" s="6" t="inlineStr">
-        <is>
-          <t>Ficha preenchida com a EMLURB (agora); registros de ocorrências do COP e da Defesa Civil (confirmação)</t>
-        </is>
-      </c>
-      <c r="F5" s="7" t="inlineStr">
-        <is>
-          <t>Pendente</t>
-        </is>
-      </c>
-      <c r="G5" s="7" t="inlineStr">
-        <is>
-          <t>Pendente</t>
-        </is>
-      </c>
-      <c r="H5" s="8" t="inlineStr">
-        <is>
-          <t>Pedido ao COP via tutora/CGM. Chamados do 156 servem só para conferir, não como subcritério.</t>
-        </is>
-      </c>
-      <c r="I5" s="6" t="inlineStr">
+      <c r="M5" s="6" t="inlineStr">
+        <is>
+          <t>Ficha preenchida com a EMLURB (agora); ocorrências do COP e da Defesa Civil (confirmação)</t>
+        </is>
+      </c>
+      <c r="N5" s="13" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+      <c r="O5" s="13" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+      <c r="P5" s="14" t="inlineStr">
+        <is>
+          <t>Pedido ao COP via tutora/CGM. 156 só para conferir. Calibrar faixas com a distribuição real.</t>
+        </is>
+      </c>
+      <c r="Q5" s="6" t="inlineStr">
         <is>
           <t>Não verificado: depende de pedido aos órgãos.</t>
         </is>
@@ -714,35 +837,75 @@
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>Severidade (altura da água + tempo para baixar + extensão)</t>
+          <t>Severidade</t>
         </is>
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
+          <t>Altura máxima da água e tempo para baixar; nota = média das duas notas, arredondada para cima</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>Faixa fixa</t>
+        </is>
+      </c>
+      <c r="F6" s="8" t="inlineStr">
+        <is>
+          <t>Altura &lt; 10 cm / baixa em &lt; 1 h</t>
+        </is>
+      </c>
+      <c r="G6" s="9" t="inlineStr">
+        <is>
+          <t>10–30 cm (tornozelo) / 1–3 h</t>
+        </is>
+      </c>
+      <c r="H6" s="10" t="inlineStr">
+        <is>
+          <t>30–50 cm (joelho) / 3–6 h</t>
+        </is>
+      </c>
+      <c r="I6" s="11" t="inlineStr">
+        <is>
+          <t>50–100 cm (cintura) / 6–12 h</t>
+        </is>
+      </c>
+      <c r="J6" s="12" t="inlineStr">
+        <is>
+          <t>&gt; 100 cm / &gt; 12 h</t>
+        </is>
+      </c>
+      <c r="K6" s="6" t="inlineStr">
+        <is>
+          <t>Planilha original (provisória); regra da média: proposta Claude</t>
+        </is>
+      </c>
+      <c r="L6" s="6" t="inlineStr">
+        <is>
           <t>Manter — peso alto</t>
         </is>
       </c>
-      <c r="E6" s="6" t="inlineStr">
+      <c r="M6" s="6" t="inlineStr">
         <is>
           <t>Ficha EMLURB; escuta com Defesa Civil e moradores</t>
         </is>
       </c>
-      <c r="F6" s="7" t="inlineStr">
-        <is>
-          <t>Pendente</t>
-        </is>
-      </c>
-      <c r="G6" s="7" t="inlineStr">
-        <is>
-          <t>Pendente</t>
-        </is>
-      </c>
-      <c r="H6" s="8" t="inlineStr">
-        <is>
-          <t>Registrar em faixas (tornozelo, joelho, cintura; &lt;1 h a &gt;6 h).</t>
-        </is>
-      </c>
-      <c r="I6" s="6" t="inlineStr">
+      <c r="N6" s="13" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+      <c r="O6" s="13" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+      <c r="P6" s="14" t="inlineStr">
+        <is>
+          <t>Extensão da mancha fica registrada como informação, sem nota própria.</t>
+        </is>
+      </c>
+      <c r="Q6" s="6" t="inlineStr">
         <is>
           <t>Não verificado: dado de campo.</t>
         </is>
@@ -766,30 +929,70 @@
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
+          <t>O escoamento trava com a maré alta?</t>
+        </is>
+      </c>
+      <c r="E7" s="7" t="inlineStr">
+        <is>
+          <t>Classe</t>
+        </is>
+      </c>
+      <c r="F7" s="8" t="inlineStr">
+        <is>
+          <t>Não influencia</t>
+        </is>
+      </c>
+      <c r="G7" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H7" s="10" t="inlineStr">
+        <is>
+          <t>Agrava ocasionalmente</t>
+        </is>
+      </c>
+      <c r="I7" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J7" s="12" t="inlineStr">
+        <is>
+          <t>Alaga dependendo da maré / escoamento bloqueado</t>
+        </is>
+      </c>
+      <c r="K7" s="6" t="inlineStr">
+        <is>
+          <t>Planilha original</t>
+        </is>
+      </c>
+      <c r="L7" s="6" t="inlineStr">
+        <is>
           <t>Manter</t>
         </is>
       </c>
-      <c r="E7" s="6" t="inlineStr">
-        <is>
-          <t>Ficha EMLURB; APAC; tábua de marés (Marinha / Porto do Recife)</t>
-        </is>
-      </c>
-      <c r="F7" s="7" t="inlineStr">
-        <is>
-          <t>Pendente</t>
-        </is>
-      </c>
-      <c r="G7" s="7" t="inlineStr">
-        <is>
-          <t>Pendente</t>
-        </is>
-      </c>
-      <c r="H7" s="8" t="inlineStr">
-        <is>
-          <t>Relevante nas baixadas e trechos que descem 'até a maré'.</t>
-        </is>
-      </c>
-      <c r="I7" s="6" t="inlineStr">
+      <c r="M7" s="6" t="inlineStr">
+        <is>
+          <t>Ficha EMLURB; APAC; tábua de marés</t>
+        </is>
+      </c>
+      <c r="N7" s="13" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+      <c r="O7" s="13" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+      <c r="P7" s="14" t="inlineStr">
+        <is>
+          <t>Notas 2 e 4 ficam para casos intermediários, se a EMLURB indicar.</t>
+        </is>
+      </c>
+      <c r="Q7" s="6" t="inlineStr">
         <is>
           <t>APAC confirmada na busca; tábua de marés não verificada.</t>
         </is>
@@ -813,30 +1016,70 @@
       </c>
       <c r="D8" s="6" t="inlineStr">
         <is>
+          <t>Distância do ponto ao curso d'água mais próximo (m); quanto mais perto, maior a nota</t>
+        </is>
+      </c>
+      <c r="E8" s="7" t="inlineStr">
+        <is>
+          <t>Quintil (invertido)</t>
+        </is>
+      </c>
+      <c r="F8" s="8" t="inlineStr">
+        <is>
+          <t>Quintil mais distante</t>
+        </is>
+      </c>
+      <c r="G8" s="9" t="inlineStr">
+        <is>
+          <t>Quintil 2</t>
+        </is>
+      </c>
+      <c r="H8" s="10" t="inlineStr">
+        <is>
+          <t>Quintil 3</t>
+        </is>
+      </c>
+      <c r="I8" s="11" t="inlineStr">
+        <is>
+          <t>Quintil 4</t>
+        </is>
+      </c>
+      <c r="J8" s="12" t="inlineStr">
+        <is>
+          <t>Quintil mais próximo</t>
+        </is>
+      </c>
+      <c r="K8" s="6" t="inlineStr">
+        <is>
+          <t>Regra de quintis da planilha original</t>
+        </is>
+      </c>
+      <c r="L8" s="6" t="inlineStr">
+        <is>
           <t>Manter — peso menor (suscetibilidade)</t>
         </is>
       </c>
-      <c r="E8" s="6" t="inlineStr">
-        <is>
-          <t>Shapefile próprio da rede hidrográfica (15 feições); ESIG – recursos hídricos</t>
-        </is>
-      </c>
-      <c r="F8" s="7" t="inlineStr">
-        <is>
-          <t>Pendente</t>
-        </is>
-      </c>
-      <c r="G8" s="7" t="inlineStr">
-        <is>
-          <t>Pendente</t>
-        </is>
-      </c>
-      <c r="H8" s="8" t="inlineStr">
-        <is>
-          <t>Reprojetar de WGS 84 para EPSG:31985. Conferir se os canais estão no arquivo, não só rios.</t>
-        </is>
-      </c>
-      <c r="I8" s="6" t="inlineStr">
+      <c r="M8" s="6" t="inlineStr">
+        <is>
+          <t>Shapefile próprio da rede hidrográfica; ESIG – recursos hídricos</t>
+        </is>
+      </c>
+      <c r="N8" s="13" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+      <c r="O8" s="13" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+      <c r="P8" s="14" t="inlineStr">
+        <is>
+          <t>Reprojetar para EPSG:31985. Conferir se os canais estão no arquivo.</t>
+        </is>
+      </c>
+      <c r="Q8" s="6" t="inlineStr">
         <is>
           <t>ESIG com recursos hídricos confirmado na busca (não aberto).</t>
         </is>
@@ -855,35 +1098,75 @@
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>Impermeabilização do entorno (% construída no círculo)</t>
+          <t>Impermeabilização</t>
         </is>
       </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
+          <t>% do círculo de 300 m com vegetação ou solo permeável; quanto menos verde, maior a nota</t>
+        </is>
+      </c>
+      <c r="E9" s="7" t="inlineStr">
+        <is>
+          <t>Faixa fixa</t>
+        </is>
+      </c>
+      <c r="F9" s="8" t="inlineStr">
+        <is>
+          <t>&gt; 40%</t>
+        </is>
+      </c>
+      <c r="G9" s="9" t="inlineStr">
+        <is>
+          <t>30–40%</t>
+        </is>
+      </c>
+      <c r="H9" s="10" t="inlineStr">
+        <is>
+          <t>20–30%</t>
+        </is>
+      </c>
+      <c r="I9" s="11" t="inlineStr">
+        <is>
+          <t>10–20%</t>
+        </is>
+      </c>
+      <c r="J9" s="12" t="inlineStr">
+        <is>
+          <t>&lt; 10%</t>
+        </is>
+      </c>
+      <c r="K9" s="6" t="inlineStr">
+        <is>
+          <t>Planilha original (provisória)</t>
+        </is>
+      </c>
+      <c r="L9" s="6" t="inlineStr">
+        <is>
           <t>Manter — peso menor (suscetibilidade)</t>
         </is>
       </c>
-      <c r="E9" s="6" t="inlineStr">
-        <is>
-          <t>MapBiomas (cobertura do solo, 30 m); alternativa: edificações do ESIG</t>
-        </is>
-      </c>
-      <c r="F9" s="7" t="inlineStr">
-        <is>
-          <t>Pendente</t>
-        </is>
-      </c>
-      <c r="G9" s="7" t="inlineStr">
-        <is>
-          <t>Pendente</t>
-        </is>
-      </c>
-      <c r="H9" s="8" t="inlineStr">
-        <is>
-          <t>Círculo de 300 m ≈ 300 pixels do MapBiomas.</t>
-        </is>
-      </c>
-      <c r="I9" s="6" t="inlineStr">
+      <c r="M9" s="6" t="inlineStr">
+        <is>
+          <t>MapBiomas (30 m); alternativa: edificações do ESIG</t>
+        </is>
+      </c>
+      <c r="N9" s="13" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+      <c r="O9" s="13" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+      <c r="P9" s="14" t="inlineStr">
+        <is>
+          <t>Se quase todos os pontos ficarem em &lt; 10%, trocar por quintis.</t>
+        </is>
+      </c>
+      <c r="Q9" s="6" t="inlineStr">
         <is>
           <t>Não verificado.</t>
         </is>
@@ -902,557 +1185,953 @@
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>Baixio (cota do ponto em relação ao entorno)</t>
+          <t>Baixio</t>
         </is>
       </c>
       <c r="D10" s="6" t="inlineStr">
         <is>
-          <t>Condicional — só entra se houver curvas de nível ou modelo de terreno</t>
-        </is>
-      </c>
-      <c r="E10" s="6" t="inlineStr">
-        <is>
-          <t>ESIG (curvas de nível, a verificar); levantamento topográfico da Prefeitura</t>
-        </is>
-      </c>
-      <c r="F10" s="7" t="inlineStr">
-        <is>
-          <t>Pendente</t>
-        </is>
-      </c>
-      <c r="G10" s="7" t="inlineStr">
-        <is>
-          <t>Pendente</t>
-        </is>
-      </c>
-      <c r="H10" s="8" t="inlineStr">
+          <t>Cota do ponto menos a cota média do círculo (m); quanto mais baixo, maior a nota</t>
+        </is>
+      </c>
+      <c r="E10" s="7" t="inlineStr">
+        <is>
+          <t>Quintil (invertido)</t>
+        </is>
+      </c>
+      <c r="F10" s="8" t="inlineStr">
+        <is>
+          <t>Quintil mais alto</t>
+        </is>
+      </c>
+      <c r="G10" s="9" t="inlineStr">
+        <is>
+          <t>Quintil 2</t>
+        </is>
+      </c>
+      <c r="H10" s="10" t="inlineStr">
+        <is>
+          <t>Quintil 3</t>
+        </is>
+      </c>
+      <c r="I10" s="11" t="inlineStr">
+        <is>
+          <t>Quintil 4</t>
+        </is>
+      </c>
+      <c r="J10" s="12" t="inlineStr">
+        <is>
+          <t>Quintil mais baixo</t>
+        </is>
+      </c>
+      <c r="K10" s="6" t="inlineStr">
+        <is>
+          <t>Proposta Claude (quintis)</t>
+        </is>
+      </c>
+      <c r="L10" s="6" t="inlineStr">
+        <is>
+          <t>Condicional — só com curvas de nível ou modelo de terreno</t>
+        </is>
+      </c>
+      <c r="M10" s="6" t="inlineStr">
+        <is>
+          <t>ESIG (curvas de nível, a verificar); topografia da Prefeitura</t>
+        </is>
+      </c>
+      <c r="N10" s="13" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+      <c r="O10" s="13" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+      <c r="P10" s="14" t="inlineStr">
         <is>
           <t>Medida mais objetiva de acúmulo de água.</t>
         </is>
       </c>
-      <c r="I10" s="6" t="inlineStr">
+      <c r="Q10" s="6" t="inlineStr">
         <is>
           <t>Não encontrado modelo de terreno público na busca.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="9" t="inlineStr">
+      <c r="A11" s="15" t="inlineStr">
         <is>
           <t>Exposição</t>
         </is>
       </c>
-      <c r="B11" s="10" t="inlineStr">
+      <c r="B11" s="8" t="inlineStr">
         <is>
           <t>E1</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>População no círculo de 300 m</t>
+          <t>População</t>
         </is>
       </c>
       <c r="D11" s="6" t="inlineStr">
         <is>
+          <t>Moradores no círculo de 300 m (soma de população × fração da célula dentro do círculo)</t>
+        </is>
+      </c>
+      <c r="E11" s="7" t="inlineStr">
+        <is>
+          <t>Quintil</t>
+        </is>
+      </c>
+      <c r="F11" s="8" t="inlineStr">
+        <is>
+          <t>Quintil 1 (20% menores)</t>
+        </is>
+      </c>
+      <c r="G11" s="9" t="inlineStr">
+        <is>
+          <t>Quintil 2</t>
+        </is>
+      </c>
+      <c r="H11" s="10" t="inlineStr">
+        <is>
+          <t>Quintil 3</t>
+        </is>
+      </c>
+      <c r="I11" s="11" t="inlineStr">
+        <is>
+          <t>Quintil 4</t>
+        </is>
+      </c>
+      <c r="J11" s="12" t="inlineStr">
+        <is>
+          <t>Quintil 5 (20% maiores)</t>
+        </is>
+      </c>
+      <c r="K11" s="6" t="inlineStr">
+        <is>
+          <t>Planilha original</t>
+        </is>
+      </c>
+      <c r="L11" s="6" t="inlineStr">
+        <is>
           <t>Manter</t>
         </is>
       </c>
-      <c r="E11" s="6" t="inlineStr">
+      <c r="M11" s="6" t="inlineStr">
         <is>
           <t>IBGE — Grade Estatística 2022 (células de 200 × 200 m)</t>
         </is>
       </c>
-      <c r="F11" s="7" t="inlineStr">
-        <is>
-          <t>Pendente</t>
-        </is>
-      </c>
-      <c r="G11" s="7" t="inlineStr">
-        <is>
-          <t>Pendente</t>
-        </is>
-      </c>
-      <c r="H11" s="8" t="inlineStr">
-        <is>
-          <t>Somar população × fração da célula dentro do círculo.</t>
-        </is>
-      </c>
-      <c r="I11" s="6" t="inlineStr">
+      <c r="N11" s="13" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+      <c r="O11" s="13" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+      <c r="P11" s="14" t="inlineStr">
+        <is>
+          <t>No painel, mostrar também o valor em 1 km.</t>
+        </is>
+      </c>
+      <c r="Q11" s="6" t="inlineStr">
         <is>
           <t>Confirmado na busca (não baixado).</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="9" t="inlineStr">
+      <c r="A12" s="15" t="inlineStr">
         <is>
           <t>Exposição</t>
         </is>
       </c>
-      <c r="B12" s="10" t="inlineStr">
+      <c r="B12" s="8" t="inlineStr">
         <is>
           <t>E2</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>Equipamentos sensíveis (escolas, creches, unidades de saúde)</t>
+          <t>Equipamentos sensíveis</t>
         </is>
       </c>
       <c r="D12" s="6" t="inlineStr">
         <is>
+          <t>Nº de escolas, creches e unidades de saúde no círculo</t>
+        </is>
+      </c>
+      <c r="E12" s="7" t="inlineStr">
+        <is>
+          <t>Faixa fixa</t>
+        </is>
+      </c>
+      <c r="F12" s="8" t="inlineStr">
+        <is>
+          <t>Nenhum</t>
+        </is>
+      </c>
+      <c r="G12" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="H12" s="10" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I12" s="11" t="inlineStr">
+        <is>
+          <t>3–4</t>
+        </is>
+      </c>
+      <c r="J12" s="12" t="inlineStr">
+        <is>
+          <t>≥ 5 ou hospital/UPA no círculo</t>
+        </is>
+      </c>
+      <c r="K12" s="6" t="inlineStr">
+        <is>
+          <t>Proposta Claude (provisória)</t>
+        </is>
+      </c>
+      <c r="L12" s="6" t="inlineStr">
+        <is>
           <t>Manter</t>
         </is>
       </c>
-      <c r="E12" s="6" t="inlineStr">
-        <is>
-          <t>IBGE — CNEFE 2022 (endereços de ensino e saúde); CNES/DATASUS</t>
-        </is>
-      </c>
-      <c r="F12" s="7" t="inlineStr">
-        <is>
-          <t>Pendente</t>
-        </is>
-      </c>
-      <c r="G12" s="7" t="inlineStr">
-        <is>
-          <t>Pendente</t>
-        </is>
-      </c>
-      <c r="H12" s="8" t="inlineStr">
-        <is>
-          <t>Conferir se creches aparecem como 'ensino' no CNEFE.</t>
-        </is>
-      </c>
-      <c r="I12" s="6" t="inlineStr">
-        <is>
-          <t>CNEFE com coordenadas e espécie confirmado na busca (não baixado).</t>
+      <c r="M12" s="6" t="inlineStr">
+        <is>
+          <t>IBGE — CNEFE 2022 (ensino e saúde); CNES/DATASUS</t>
+        </is>
+      </c>
+      <c r="N12" s="13" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+      <c r="O12" s="13" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+      <c r="P12" s="14" t="inlineStr">
+        <is>
+          <t>Calibrar com as contagens reais. Conferir se creches aparecem como 'ensino'.</t>
+        </is>
+      </c>
+      <c r="Q12" s="6" t="inlineStr">
+        <is>
+          <t>CNEFE confirmado na busca (não baixado).</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="9" t="inlineStr">
+      <c r="A13" s="15" t="inlineStr">
         <is>
           <t>Exposição</t>
         </is>
       </c>
-      <c r="B13" s="10" t="inlineStr">
+      <c r="B13" s="8" t="inlineStr">
         <is>
           <t>E3</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>Atividade econômica (comércios e serviços)</t>
+          <t>Atividade econômica</t>
         </is>
       </c>
       <c r="D13" s="6" t="inlineStr">
         <is>
+          <t>Nº de comércios e serviços no círculo</t>
+        </is>
+      </c>
+      <c r="E13" s="7" t="inlineStr">
+        <is>
+          <t>Quintil</t>
+        </is>
+      </c>
+      <c r="F13" s="8" t="inlineStr">
+        <is>
+          <t>Quintil 1 (20% menores)</t>
+        </is>
+      </c>
+      <c r="G13" s="9" t="inlineStr">
+        <is>
+          <t>Quintil 2</t>
+        </is>
+      </c>
+      <c r="H13" s="10" t="inlineStr">
+        <is>
+          <t>Quintil 3</t>
+        </is>
+      </c>
+      <c r="I13" s="11" t="inlineStr">
+        <is>
+          <t>Quintil 4</t>
+        </is>
+      </c>
+      <c r="J13" s="12" t="inlineStr">
+        <is>
+          <t>Quintil 5 (20% maiores)</t>
+        </is>
+      </c>
+      <c r="K13" s="6" t="inlineStr">
+        <is>
+          <t>Planilha original</t>
+        </is>
+      </c>
+      <c r="L13" s="6" t="inlineStr">
+        <is>
           <t>Manter</t>
         </is>
       </c>
-      <c r="E13" s="6" t="inlineStr">
-        <is>
-          <t>IBGE — CNEFE 2022 (endereços de outras finalidades)</t>
-        </is>
-      </c>
-      <c r="F13" s="7" t="inlineStr">
-        <is>
-          <t>Pendente</t>
-        </is>
-      </c>
-      <c r="G13" s="7" t="inlineStr">
-        <is>
-          <t>Pendente</t>
-        </is>
-      </c>
-      <c r="H13" s="8" t="inlineStr">
-        <is>
-          <t>'Outras finalidades' pode incluir templos e órgãos públicos; verificar se dá para separar comércio.</t>
-        </is>
-      </c>
-      <c r="I13" s="6" t="inlineStr">
+      <c r="M13" s="6" t="inlineStr">
+        <is>
+          <t>IBGE — CNEFE 2022 (outras finalidades)</t>
+        </is>
+      </c>
+      <c r="N13" s="13" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+      <c r="O13" s="13" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+      <c r="P13" s="14" t="inlineStr">
+        <is>
+          <t>'Outras finalidades' pode incluir templos e órgãos públicos.</t>
+        </is>
+      </c>
+      <c r="Q13" s="6" t="inlineStr">
         <is>
           <t>CNEFE confirmado na busca (não baixado).</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="11" t="inlineStr">
+      <c r="A14" s="16" t="inlineStr">
         <is>
           <t>Vulnerabilidade</t>
         </is>
       </c>
-      <c r="B14" s="12" t="inlineStr">
+      <c r="B14" s="17" t="inlineStr">
         <is>
           <t>V2</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>Grupos sensíveis (% de idosos 60+ e crianças 0–4)</t>
+          <t>Grupos sensíveis</t>
         </is>
       </c>
       <c r="D14" s="6" t="inlineStr">
         <is>
+          <t>% de moradores com 60+ anos ou 0–4 anos nos setores do círculo (ponderado pela área)</t>
+        </is>
+      </c>
+      <c r="E14" s="7" t="inlineStr">
+        <is>
+          <t>Quintil</t>
+        </is>
+      </c>
+      <c r="F14" s="8" t="inlineStr">
+        <is>
+          <t>Quintil 1 (20% menores)</t>
+        </is>
+      </c>
+      <c r="G14" s="9" t="inlineStr">
+        <is>
+          <t>Quintil 2</t>
+        </is>
+      </c>
+      <c r="H14" s="10" t="inlineStr">
+        <is>
+          <t>Quintil 3</t>
+        </is>
+      </c>
+      <c r="I14" s="11" t="inlineStr">
+        <is>
+          <t>Quintil 4</t>
+        </is>
+      </c>
+      <c r="J14" s="12" t="inlineStr">
+        <is>
+          <t>Quintil 5 (20% maiores)</t>
+        </is>
+      </c>
+      <c r="K14" s="6" t="inlineStr">
+        <is>
+          <t>Planilha original</t>
+        </is>
+      </c>
+      <c r="L14" s="6" t="inlineStr">
+        <is>
           <t>Manter</t>
         </is>
       </c>
-      <c r="E14" s="6" t="inlineStr">
-        <is>
-          <t>IBGE — Agregados por setor censitário 2022 (idade)</t>
-        </is>
-      </c>
-      <c r="F14" s="7" t="inlineStr">
-        <is>
-          <t>Pendente</t>
-        </is>
-      </c>
-      <c r="G14" s="7" t="inlineStr">
-        <is>
-          <t>Pendente</t>
-        </is>
-      </c>
-      <c r="H14" s="8" t="inlineStr">
-        <is>
-          <t>Ponderar setores pela fração de área dentro do círculo.</t>
-        </is>
-      </c>
-      <c r="I14" s="6" t="inlineStr">
+      <c r="M14" s="6" t="inlineStr">
+        <is>
+          <t>IBGE — Agregados por setor 2022 (idade)</t>
+        </is>
+      </c>
+      <c r="N14" s="13" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+      <c r="O14" s="13" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+      <c r="P14" s="14" t="inlineStr"/>
+      <c r="Q14" s="6" t="inlineStr">
         <is>
           <t>Idade por setor confirmada na busca (não baixado).</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="11" t="inlineStr">
+      <c r="A15" s="16" t="inlineStr">
         <is>
           <t>Vulnerabilidade</t>
         </is>
       </c>
-      <c r="B15" s="12" t="inlineStr">
+      <c r="B15" s="17" t="inlineStr">
         <is>
           <t>V3</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>Favelas e comunidades urbanas (% do círculo)</t>
+          <t>Favelas e comunidades urbanas</t>
         </is>
       </c>
       <c r="D15" s="6" t="inlineStr">
         <is>
+          <t>% da área do círculo em favelas e comunidades urbanas</t>
+        </is>
+      </c>
+      <c r="E15" s="7" t="inlineStr">
+        <is>
+          <t>Faixa fixa</t>
+        </is>
+      </c>
+      <c r="F15" s="8" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="G15" s="9" t="inlineStr">
+        <is>
+          <t>&lt; 10%</t>
+        </is>
+      </c>
+      <c r="H15" s="10" t="inlineStr">
+        <is>
+          <t>10–25%</t>
+        </is>
+      </c>
+      <c r="I15" s="11" t="inlineStr">
+        <is>
+          <t>25–50%</t>
+        </is>
+      </c>
+      <c r="J15" s="12" t="inlineStr">
+        <is>
+          <t>&gt; 50%</t>
+        </is>
+      </c>
+      <c r="K15" s="6" t="inlineStr">
+        <is>
+          <t>Proposta Claude (provisória)</t>
+        </is>
+      </c>
+      <c r="L15" s="6" t="inlineStr">
+        <is>
           <t>Manter — substitui o V1 se a malha 2022 existir</t>
         </is>
       </c>
-      <c r="E15" s="6" t="inlineStr">
+      <c r="M15" s="6" t="inlineStr">
         <is>
           <t>IBGE — Favelas e Comunidades Urbanas 2022 (malha)</t>
         </is>
       </c>
-      <c r="F15" s="7" t="inlineStr">
-        <is>
-          <t>Pendente</t>
-        </is>
-      </c>
-      <c r="G15" s="7" t="inlineStr">
-        <is>
-          <t>Pendente</t>
-        </is>
-      </c>
-      <c r="H15" s="8" t="inlineStr">
+      <c r="N15" s="13" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+      <c r="O15" s="13" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+      <c r="P15" s="14" t="inlineStr">
         <is>
           <t>Mais atual que o IVS (2010).</t>
         </is>
       </c>
-      <c r="I15" s="6" t="inlineStr">
+      <c r="Q15" s="6" t="inlineStr">
         <is>
           <t>Não verificado.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="11" t="inlineStr">
+      <c r="A16" s="16" t="inlineStr">
         <is>
           <t>Vulnerabilidade</t>
         </is>
       </c>
-      <c r="B16" s="12" t="inlineStr">
+      <c r="B16" s="17" t="inlineStr">
         <is>
           <t>V4</t>
         </is>
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t>Tipo de moradia (% de domicílios tipo casa)</t>
+          <t>Tipo de moradia</t>
         </is>
       </c>
       <c r="D16" s="6" t="inlineStr">
         <is>
+          <t>% de domicílios do tipo casa nos setores do círculo</t>
+        </is>
+      </c>
+      <c r="E16" s="7" t="inlineStr">
+        <is>
+          <t>Quintil</t>
+        </is>
+      </c>
+      <c r="F16" s="8" t="inlineStr">
+        <is>
+          <t>Quintil 1 (20% menores)</t>
+        </is>
+      </c>
+      <c r="G16" s="9" t="inlineStr">
+        <is>
+          <t>Quintil 2</t>
+        </is>
+      </c>
+      <c r="H16" s="10" t="inlineStr">
+        <is>
+          <t>Quintil 3</t>
+        </is>
+      </c>
+      <c r="I16" s="11" t="inlineStr">
+        <is>
+          <t>Quintil 4</t>
+        </is>
+      </c>
+      <c r="J16" s="12" t="inlineStr">
+        <is>
+          <t>Quintil 5 (20% maiores)</t>
+        </is>
+      </c>
+      <c r="K16" s="6" t="inlineStr">
+        <is>
+          <t>Proposta Claude (quintis)</t>
+        </is>
+      </c>
+      <c r="L16" s="6" t="inlineStr">
+        <is>
           <t>Manter</t>
         </is>
       </c>
-      <c r="E16" s="6" t="inlineStr">
-        <is>
-          <t>IBGE — Agregados por setor censitário 2022 (tipo de domicílio)</t>
-        </is>
-      </c>
-      <c r="F16" s="7" t="inlineStr">
-        <is>
-          <t>Pendente</t>
-        </is>
-      </c>
-      <c r="G16" s="7" t="inlineStr">
-        <is>
-          <t>Pendente</t>
-        </is>
-      </c>
-      <c r="H16" s="8" t="inlineStr">
+      <c r="M16" s="6" t="inlineStr">
+        <is>
+          <t>IBGE — Agregados por setor 2022 (tipo de domicílio)</t>
+        </is>
+      </c>
+      <c r="N16" s="13" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+      <c r="O16" s="13" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+      <c r="P16" s="14" t="inlineStr">
         <is>
           <t>Casa térrea é mais atingida que apartamento.</t>
         </is>
       </c>
-      <c r="I16" s="6" t="inlineStr">
+      <c r="Q16" s="6" t="inlineStr">
         <is>
           <t>Não verificado se a variável está no arquivo por setor.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="11" t="inlineStr">
+      <c r="A17" s="16" t="inlineStr">
         <is>
           <t>Vulnerabilidade</t>
         </is>
       </c>
-      <c r="B17" s="12" t="inlineStr">
+      <c r="B17" s="17" t="inlineStr">
         <is>
           <t>V1</t>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>Vulnerabilidade social (IVS por UDH)</t>
+          <t>Vulnerabilidade social (IVS)</t>
         </is>
       </c>
       <c r="D17" s="6" t="inlineStr">
         <is>
+          <t>Maior IVS entre as UDHs que tocam o círculo</t>
+        </is>
+      </c>
+      <c r="E17" s="7" t="inlineStr">
+        <is>
+          <t>Faixa fixa</t>
+        </is>
+      </c>
+      <c r="F17" s="8" t="inlineStr">
+        <is>
+          <t>Muito baixa (0–0,200)</t>
+        </is>
+      </c>
+      <c r="G17" s="9" t="inlineStr">
+        <is>
+          <t>Baixa (0,201–0,300)</t>
+        </is>
+      </c>
+      <c r="H17" s="10" t="inlineStr">
+        <is>
+          <t>Média (0,301–0,400)</t>
+        </is>
+      </c>
+      <c r="I17" s="11" t="inlineStr">
+        <is>
+          <t>Alta (0,401–0,500)</t>
+        </is>
+      </c>
+      <c r="J17" s="12" t="inlineStr">
+        <is>
+          <t>Muito alta (&gt; 0,500)</t>
+        </is>
+      </c>
+      <c r="K17" s="6" t="inlineStr">
+        <is>
+          <t>Faixas do Ipea (conferir no Atlas)</t>
+        </is>
+      </c>
+      <c r="L17" s="6" t="inlineStr">
+        <is>
           <t>Plano B — só se o V3 não estiver disponível</t>
         </is>
       </c>
-      <c r="E17" s="6" t="inlineStr">
+      <c r="M17" s="6" t="inlineStr">
         <is>
           <t>Ipea — Atlas da Vulnerabilidade Social (UDH)</t>
         </is>
       </c>
-      <c r="F17" s="7" t="inlineStr">
-        <is>
-          <t>Pendente</t>
-        </is>
-      </c>
-      <c r="G17" s="7" t="inlineStr">
-        <is>
-          <t>Pendente</t>
-        </is>
-      </c>
-      <c r="H17" s="8" t="inlineStr">
-        <is>
-          <t>Base do Censo 2010; UDH maior que o círculo.</t>
-        </is>
-      </c>
-      <c r="I17" s="6" t="inlineStr">
-        <is>
-          <t>Site confirmado na busca; ano-base a confirmar.</t>
+      <c r="N17" s="13" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+      <c r="O17" s="13" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+      <c r="P17" s="14" t="inlineStr">
+        <is>
+          <t>Base do Censo 2010.</t>
+        </is>
+      </c>
+      <c r="Q17" s="6" t="inlineStr">
+        <is>
+          <t>Site confirmado na busca; faixas e ano-base a confirmar.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="13" t="inlineStr">
+      <c r="A18" s="18" t="inlineStr">
         <is>
           <t>Impacto</t>
         </is>
       </c>
-      <c r="B18" s="14" t="inlineStr">
+      <c r="B18" s="19" t="inlineStr">
         <is>
           <t>I1</t>
         </is>
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
-          <t>Mobilidade (classe da via + paradas de ônibus + interdições)</t>
+          <t>Mobilidade</t>
         </is>
       </c>
       <c r="D18" s="6" t="inlineStr">
         <is>
+          <t>Classe da via mais importante afetada pelo alagamento; +1 se houver interdição registrada pela CTTU (máximo 5)</t>
+        </is>
+      </c>
+      <c r="E18" s="7" t="inlineStr">
+        <is>
+          <t>Classe</t>
+        </is>
+      </c>
+      <c r="F18" s="8" t="inlineStr">
+        <is>
+          <t>Via local ou de pedestres</t>
+        </is>
+      </c>
+      <c r="G18" s="9" t="inlineStr">
+        <is>
+          <t>Coletora</t>
+        </is>
+      </c>
+      <c r="H18" s="10" t="inlineStr">
+        <is>
+          <t>Arterial secundária</t>
+        </is>
+      </c>
+      <c r="I18" s="11" t="inlineStr">
+        <is>
+          <t>Arterial principal</t>
+        </is>
+      </c>
+      <c r="J18" s="12" t="inlineStr">
+        <is>
+          <t>Trânsito rápido ou corredor de ônibus</t>
+        </is>
+      </c>
+      <c r="K18" s="6" t="inlineStr">
+        <is>
+          <t>Proposta Claude, a partir da classificação viária usada na planilha original</t>
+        </is>
+      </c>
+      <c r="L18" s="6" t="inlineStr">
+        <is>
           <t>Manter</t>
         </is>
       </c>
-      <c r="E18" s="6" t="inlineStr">
-        <is>
-          <t>Hierarquia viária (ESIG / CTTU); OpenStreetMap; paradas (Grande Recife Consórcio); interdições (CTTU)</t>
-        </is>
-      </c>
-      <c r="F18" s="7" t="inlineStr">
-        <is>
-          <t>Pendente</t>
-        </is>
-      </c>
-      <c r="G18" s="7" t="inlineStr">
-        <is>
-          <t>Pendente</t>
-        </is>
-      </c>
-      <c r="H18" s="8" t="inlineStr">
-        <is>
-          <t>Pedir a Antônio (CTTU): hierarquia viária, linhas e registro de interdições por alagamento.</t>
-        </is>
-      </c>
-      <c r="I18" s="6" t="inlineStr">
-        <is>
-          <t>Vias no ESIG confirmadas na busca; dados de ônibus e interdições não verificados.</t>
+      <c r="M18" s="6" t="inlineStr">
+        <is>
+          <t>Hierarquia viária (ESIG / CTTU); OSM; paradas (Grande Recife); interdições (CTTU)</t>
+        </is>
+      </c>
+      <c r="N18" s="13" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+      <c r="O18" s="13" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+      <c r="P18" s="14" t="inlineStr">
+        <is>
+          <t>Pedir a Antônio (CTTU): hierarquia viária, linhas e registro de interdições.</t>
+        </is>
+      </c>
+      <c r="Q18" s="6" t="inlineStr">
+        <is>
+          <t>Vias no ESIG confirmadas na busca; ônibus e interdições não verificados.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="13" t="inlineStr">
+      <c r="A19" s="18" t="inlineStr">
         <is>
           <t>Impacto</t>
         </is>
       </c>
-      <c r="B19" s="14" t="inlineStr">
+      <c r="B19" s="19" t="inlineStr">
         <is>
           <t>I2</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>Risco sanitário (% de domicílios sem rede de esgoto)</t>
+          <t>Risco sanitário</t>
         </is>
       </c>
       <c r="D19" s="6" t="inlineStr">
         <is>
+          <t>% de domicílios sem ligação à rede de esgoto nos setores do círculo</t>
+        </is>
+      </c>
+      <c r="E19" s="7" t="inlineStr">
+        <is>
+          <t>Quintil</t>
+        </is>
+      </c>
+      <c r="F19" s="8" t="inlineStr">
+        <is>
+          <t>Quintil 1 (20% menores)</t>
+        </is>
+      </c>
+      <c r="G19" s="9" t="inlineStr">
+        <is>
+          <t>Quintil 2</t>
+        </is>
+      </c>
+      <c r="H19" s="10" t="inlineStr">
+        <is>
+          <t>Quintil 3</t>
+        </is>
+      </c>
+      <c r="I19" s="11" t="inlineStr">
+        <is>
+          <t>Quintil 4</t>
+        </is>
+      </c>
+      <c r="J19" s="12" t="inlineStr">
+        <is>
+          <t>Quintil 5 (20% maiores)</t>
+        </is>
+      </c>
+      <c r="K19" s="6" t="inlineStr">
+        <is>
+          <t>Proposta Claude (quintis)</t>
+        </is>
+      </c>
+      <c r="L19" s="6" t="inlineStr">
+        <is>
           <t>Manter</t>
         </is>
       </c>
-      <c r="E19" s="6" t="inlineStr">
-        <is>
-          <t>IBGE — Agregados por setor censitário 2022 (esgotamento); Compesa (rede e extravasamentos)</t>
-        </is>
-      </c>
-      <c r="F19" s="7" t="inlineStr">
-        <is>
-          <t>Pendente</t>
-        </is>
-      </c>
-      <c r="G19" s="7" t="inlineStr">
-        <is>
-          <t>Pendente</t>
-        </is>
-      </c>
-      <c r="H19" s="8" t="inlineStr">
-        <is>
-          <t>Compesa complementa com extravasamentos, se fornecer.</t>
-        </is>
-      </c>
-      <c r="I19" s="6" t="inlineStr">
+      <c r="M19" s="6" t="inlineStr">
+        <is>
+          <t>IBGE — Agregados por setor 2022 (esgotamento); Compesa</t>
+        </is>
+      </c>
+      <c r="N19" s="13" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+      <c r="O19" s="13" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+      <c r="P19" s="14" t="inlineStr">
+        <is>
+          <t>Quintis porque a cobertura de esgoto no Recife é baixa e faixas fixas podem saturar.</t>
+        </is>
+      </c>
+      <c r="Q19" s="6" t="inlineStr">
         <is>
           <t>Esgotamento por setor confirmado na busca (não baixado).</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="15" t="inlineStr">
+      <c r="A21" s="20" t="inlineStr">
         <is>
           <t>Resumo</t>
         </is>
       </c>
-      <c r="F21" s="16" t="inlineStr">
+      <c r="N21" s="21" t="inlineStr">
         <is>
           <t>Fonte confirmada</t>
         </is>
       </c>
-      <c r="G21" s="16" t="inlineStr">
+      <c r="O21" s="21" t="inlineStr">
         <is>
           <t>Dado existe</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="E22" s="17" t="inlineStr">
+      <c r="M22" s="22" t="inlineStr">
         <is>
           <t>Sim</t>
         </is>
       </c>
-      <c r="F22" s="18">
-        <f>COUNTIF(F$5:F$19,$E22)</f>
+      <c r="N22" s="23">
+        <f>COUNTIF(N$5:N$19,$M22)</f>
         <v/>
       </c>
-      <c r="G22" s="18">
-        <f>COUNTIF(G$5:G$19,$E22)</f>
+      <c r="O22" s="23">
+        <f>COUNTIF(O$5:O$19,$M22)</f>
         <v/>
       </c>
     </row>
     <row r="23">
-      <c r="E23" s="17" t="inlineStr">
+      <c r="M23" s="22" t="inlineStr">
         <is>
           <t>Parcial</t>
         </is>
       </c>
-      <c r="F23" s="18">
-        <f>COUNTIF(F$5:F$19,$E23)</f>
+      <c r="N23" s="23">
+        <f>COUNTIF(N$5:N$19,$M23)</f>
         <v/>
       </c>
-      <c r="G23" s="18">
-        <f>COUNTIF(G$5:G$19,$E23)</f>
+      <c r="O23" s="23">
+        <f>COUNTIF(O$5:O$19,$M23)</f>
         <v/>
       </c>
     </row>
     <row r="24">
-      <c r="E24" s="17" t="inlineStr">
+      <c r="M24" s="22" t="inlineStr">
         <is>
           <t>Não</t>
         </is>
       </c>
-      <c r="F24" s="18">
-        <f>COUNTIF(F$5:F$19,$E24)</f>
+      <c r="N24" s="23">
+        <f>COUNTIF(N$5:N$19,$M24)</f>
         <v/>
       </c>
-      <c r="G24" s="18">
-        <f>COUNTIF(G$5:G$19,$E24)</f>
+      <c r="O24" s="23">
+        <f>COUNTIF(O$5:O$19,$M24)</f>
         <v/>
       </c>
     </row>
     <row r="25">
-      <c r="E25" s="17" t="inlineStr">
-        <is>
-          <t>Pendente</t>
-        </is>
-      </c>
-      <c r="F25" s="18">
-        <f>COUNTIF(F$5:F$19,$E25)</f>
+      <c r="M25" s="22" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+      <c r="N25" s="23">
+        <f>COUNTIF(N$5:N$19,$M25)</f>
         <v/>
       </c>
-      <c r="G25" s="18">
-        <f>COUNTIF(G$5:G$19,$E25)</f>
+      <c r="O25" s="23">
+        <f>COUNTIF(O$5:O$19,$M25)</f>
         <v/>
       </c>
     </row>
     <row r="26">
-      <c r="E26" s="19" t="inlineStr">
+      <c r="M26" s="24" t="inlineStr">
         <is>
           <t>Subcritérios com fonte e dado confirmados</t>
         </is>
       </c>
-      <c r="G26" s="20">
-        <f>COUNTIFS(F5:F19,"Sim",G5:G19,"Sim")&amp;" de "&amp;ROWS(F5:F19)</f>
+      <c r="O26" s="25">
+        <f>COUNTIFS(N5:N19,"Sim",O5:O19,"Sim")&amp;" de "&amp;ROWS(N5:N19)</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:I19"/>
+  <autoFilter ref="A4:Q19"/>
   <mergeCells count="1">
-    <mergeCell ref="A2:I2"/>
+    <mergeCell ref="A2:Q2"/>
   </mergeCells>
-  <conditionalFormatting sqref="F5:G19">
+  <conditionalFormatting sqref="N5:O19">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Sim"</formula>
     </cfRule>
@@ -1464,7 +2143,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="F5:G19" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="N5:O19" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Sim,Não,Parcial,Pendente"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Aba Glossário na planilha de checklist
63 termos em 6 grupos (modelo de risco, tipo de nota, território e SIG,
fontes de dados, checklist e órgãos), com significado e exemplo no projeto,
para compartilhar com a equipe.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018419ScLbL3ubanHMYyaBnW
</commit_message>
<xml_diff>
--- a/dados/Recife_Resiliente_Checklist_Subcriterios.xlsx
+++ b/dados/Recife_Resiliente_Checklist_Subcriterios.xlsx
@@ -8,9 +8,11 @@
   </bookViews>
   <sheets>
     <sheet name="Checklist subcritérios" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Glossário" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Checklist subcritérios'!$A$4:$Q$19</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Glossário'!$A$4:$D$67</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -71,7 +73,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="12">
+  <fills count="13">
     <fill>
       <patternFill/>
     </fill>
@@ -128,6 +130,11 @@
         <fgColor rgb="00EDE2F6"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EDEDED"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -155,7 +162,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -225,6 +232,34 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -646,7 +681,7 @@
     <row r="2" ht="44" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Proposta de 02/10/2026 (Pedro + Claude), não validada pelo grupo. Nota 5 = mais crítico. Faixa fixa = valor absoluto (provisória: calibrar com os dados reais). Quintil = nota relativa entre os 21 pontos (Quintil 1 = 20% com menor valor). Preencha as colunas amarelas (N, O e P): Sim / Não / Parcial / Pendente. 'Fonte confirmada' = a base existe e é acessível; 'Dado existe na fonte' = a variável está lá, na escala do círculo de 300 m, e cobre os 21 pontos.</t>
+          <t>Proposta de 02/10/2026 (Pedro + Claude), não validada pelo grupo. Nota 5 = mais crítico. Faixa fixa = valor absoluto (provisória: calibrar com os dados reais). Quintil = nota relativa entre os 21 pontos (Quintil 1 = 20% com menor valor). Preencha as colunas amarelas (N, O e P): Sim / Não / Parcial / Pendente. 'Fonte confirmada' = a base existe e é acessível; 'Dado existe na fonte' = a variável está lá, na escala do círculo de 300 m, e cobre os 21 pontos. Termos explicados na aba Glossário.</t>
         </is>
       </c>
     </row>
@@ -2150,4 +2185,1350 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D67"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="70" customWidth="1" min="3" max="3"/>
+    <col width="45" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Glossário — termos usados nesta planilha e no modelo de risco</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="26" t="inlineStr">
+        <is>
+          <t>Para quem não participou das discussões do modelo. Os papéis dos órgãos são uma leitura preliminar, ainda não confirmada com cada órgão.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="27" t="inlineStr">
+        <is>
+          <t>Grupo</t>
+        </is>
+      </c>
+      <c r="B4" s="27" t="inlineStr">
+        <is>
+          <t>Termo</t>
+        </is>
+      </c>
+      <c r="C4" s="27" t="inlineStr">
+        <is>
+          <t>O que significa</t>
+        </is>
+      </c>
+      <c r="D4" s="27" t="inlineStr">
+        <is>
+          <t>Exemplo no projeto</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="28" t="inlineStr">
+        <is>
+          <t>Modelo de risco</t>
+        </is>
+      </c>
+      <c r="B5" s="29" t="inlineStr">
+        <is>
+          <t>Risco</t>
+        </is>
+      </c>
+      <c r="C5" s="30" t="inlineStr">
+        <is>
+          <t>Medida de quão prioritário é um ponto para a prevenção. Calculado como Probabilidade × Consequência, numa escala de 1 a 25.</t>
+        </is>
+      </c>
+      <c r="D5" s="30" t="inlineStr">
+        <is>
+          <t>Um ponto com Probabilidade 4 e Consequência 3 tem risco 12.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="28" t="inlineStr">
+        <is>
+          <t>Modelo de risco</t>
+        </is>
+      </c>
+      <c r="B6" s="29" t="inlineStr">
+        <is>
+          <t>Critério</t>
+        </is>
+      </c>
+      <c r="C6" s="30" t="inlineStr">
+        <is>
+          <t>Um dos 4 grandes componentes do risco: Probabilidade, Exposição, Vulnerabilidade e Impacto.</t>
+        </is>
+      </c>
+      <c r="D6" s="30" t="inlineStr">
+        <is>
+          <t>Vulnerabilidade é um critério.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="28" t="inlineStr">
+        <is>
+          <t>Modelo de risco</t>
+        </is>
+      </c>
+      <c r="B7" s="29" t="inlineStr">
+        <is>
+          <t>Subcritério</t>
+        </is>
+      </c>
+      <c r="C7" s="30" t="inlineStr">
+        <is>
+          <t>Um item medível dentro de um critério. Cada subcritério recebe uma nota de 1 a 5.</t>
+        </is>
+      </c>
+      <c r="D7" s="30" t="inlineStr">
+        <is>
+          <t>População (E1) é um subcritério da Exposição.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="28" t="inlineStr">
+        <is>
+          <t>Modelo de risco</t>
+        </is>
+      </c>
+      <c r="B8" s="29" t="inlineStr">
+        <is>
+          <t>Probabilidade</t>
+        </is>
+      </c>
+      <c r="C8" s="30" t="inlineStr">
+        <is>
+          <t>Quanto e com que facilidade o ponto alaga: frequência, severidade, maré, proximidade de rio, impermeabilização.</t>
+        </is>
+      </c>
+      <c r="D8" s="30" t="inlineStr">
+        <is>
+          <t>Um ponto que alaga 7 vezes por ano tem Frequência (P1) = 5.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="28" t="inlineStr">
+        <is>
+          <t>Modelo de risco</t>
+        </is>
+      </c>
+      <c r="B9" s="29" t="inlineStr">
+        <is>
+          <t>Exposição</t>
+        </is>
+      </c>
+      <c r="C9" s="30" t="inlineStr">
+        <is>
+          <t>Quem e o que está no caminho da água dentro do círculo de 300 m: moradores, escolas, unidades de saúde, comércio.</t>
+        </is>
+      </c>
+      <c r="D9" s="30" t="inlineStr">
+        <is>
+          <t>Um ponto com muitas escolas por perto tem Equipamentos sensíveis (E2) alto.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="28" t="inlineStr">
+        <is>
+          <t>Modelo de risco</t>
+        </is>
+      </c>
+      <c r="B10" s="29" t="inlineStr">
+        <is>
+          <t>Vulnerabilidade</t>
+        </is>
+      </c>
+      <c r="C10" s="30" t="inlineStr">
+        <is>
+          <t>Quanto quem está ali tem dificuldade de lidar com o alagamento: idosos e crianças, favelas e comunidades, moradia térrea.</t>
+        </is>
+      </c>
+      <c r="D10" s="30" t="inlineStr">
+        <is>
+          <t>Área com muitas casas térreas tem Tipo de moradia (V4) alto.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="28" t="inlineStr">
+        <is>
+          <t>Modelo de risco</t>
+        </is>
+      </c>
+      <c r="B11" s="29" t="inlineStr">
+        <is>
+          <t>Impacto</t>
+        </is>
+      </c>
+      <c r="C11" s="30" t="inlineStr">
+        <is>
+          <t>Consequência que vai além do local: mobilidade da cidade e saúde pública (esgoto).</t>
+        </is>
+      </c>
+      <c r="D11" s="30" t="inlineStr">
+        <is>
+          <t>Alagamento numa avenida arterial com ônibus tem Mobilidade (I1) alta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="28" t="inlineStr">
+        <is>
+          <t>Modelo de risco</t>
+        </is>
+      </c>
+      <c r="B12" s="29" t="inlineStr">
+        <is>
+          <t>Consequência</t>
+        </is>
+      </c>
+      <c r="C12" s="30" t="inlineStr">
+        <is>
+          <t>Média ponderada de Exposição, Vulnerabilidade e Impacto, de 1 a 5. É o que multiplica a Probabilidade.</t>
+        </is>
+      </c>
+      <c r="D12" s="30" t="inlineStr">
+        <is>
+          <t>Exposição 4, Vulnerabilidade 2 e Impacto 3 com pesos iguais dão Consequência 3.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="28" t="inlineStr">
+        <is>
+          <t>Modelo de risco</t>
+        </is>
+      </c>
+      <c r="B13" s="29" t="inlineStr">
+        <is>
+          <t>Nota (1 a 5)</t>
+        </is>
+      </c>
+      <c r="C13" s="30" t="inlineStr">
+        <is>
+          <t>Valor dado a cada subcritério. 5 = mais crítico, 1 = menos crítico.</t>
+        </is>
+      </c>
+      <c r="D13" s="30" t="inlineStr">
+        <is>
+          <t>Nota 5 em Maré (P3) = o ponto alaga conforme a maré.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="28" t="inlineStr">
+        <is>
+          <t>Modelo de risco</t>
+        </is>
+      </c>
+      <c r="B14" s="29" t="inlineStr">
+        <is>
+          <t>Peso</t>
+        </is>
+      </c>
+      <c r="C14" s="30" t="inlineStr">
+        <is>
+          <t>Importância relativa de um subcritério dentro do critério, ou de um critério dentro da Consequência. Definido pelo grupo. A Probabilidade não tem peso, porque multiplica.</t>
+        </is>
+      </c>
+      <c r="D14" s="30" t="inlineStr">
+        <is>
+          <t>Frequência e Severidade terão peso maior que Proximidade de rio.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="28" t="inlineStr">
+        <is>
+          <t>Modelo de risco</t>
+        </is>
+      </c>
+      <c r="B15" s="29" t="inlineStr">
+        <is>
+          <t>Média ponderada</t>
+        </is>
+      </c>
+      <c r="C15" s="30" t="inlineStr">
+        <is>
+          <t>Média em que cada item conta conforme o seu peso.</t>
+        </is>
+      </c>
+      <c r="D15" s="30" t="inlineStr">
+        <is>
+          <t>Notas 5 (peso 2) e 2 (peso 1): (5×2 + 2×1) ÷ 3 = 4.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="28" t="inlineStr">
+        <is>
+          <t>Modelo de risco</t>
+        </is>
+      </c>
+      <c r="B16" s="29" t="inlineStr">
+        <is>
+          <t>Cobertura</t>
+        </is>
+      </c>
+      <c r="C16" s="30" t="inlineStr">
+        <is>
+          <t>Quantos subcritérios têm nota para o ponto. Nota faltante não vira zero nem média: fica de fora e a cobertura mostra a falta.</t>
+        </is>
+      </c>
+      <c r="D16" s="30" t="inlineStr">
+        <is>
+          <t>Cobertura 11/13 = faltam 2 notas para aquele ponto.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="28" t="inlineStr">
+        <is>
+          <t>Modelo de risco</t>
+        </is>
+      </c>
+      <c r="B17" s="29" t="inlineStr">
+        <is>
+          <t>Sem Probabilidade, sem risco</t>
+        </is>
+      </c>
+      <c r="C17" s="30" t="inlineStr">
+        <is>
+          <t>Como o risco é uma multiplicação, um ponto sem nota de Probabilidade não tem risco calculado nem posição no ranking.</t>
+        </is>
+      </c>
+      <c r="D17" s="30" t="inlineStr">
+        <is>
+          <t>Por isso a ficha com a EMLURB é prioritária.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="28" t="inlineStr">
+        <is>
+          <t>Modelo de risco</t>
+        </is>
+      </c>
+      <c r="B18" s="29" t="inlineStr">
+        <is>
+          <t>Tratabilidade</t>
+        </is>
+      </c>
+      <c r="C18" s="30" t="inlineStr">
+        <is>
+          <t>Se é fácil agir no ponto (governança, natureza da causa, obra ou orçamento em andamento). Fica FORA do risco. 5 = mais fácil.</t>
+        </is>
+      </c>
+      <c r="D18" s="30" t="inlineStr">
+        <is>
+          <t>Ponto com dono definido e causa de manutenção tem tratabilidade alta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="28" t="inlineStr">
+        <is>
+          <t>Modelo de risco</t>
+        </is>
+      </c>
+      <c r="B19" s="29" t="inlineStr">
+        <is>
+          <t>Matriz risco × tratabilidade</t>
+        </is>
+      </c>
+      <c r="C19" s="30" t="inlineStr">
+        <is>
+          <t>Cruza o risco (corte em 9) com a tratabilidade (corte em 3) e coloca cada ponto num de 4 quadrantes.</t>
+        </is>
+      </c>
+      <c r="D19" s="30" t="inlineStr">
+        <is>
+          <t>Risco 12 e tratabilidade 4 = quadrante Agir já.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="28" t="inlineStr">
+        <is>
+          <t>Modelo de risco</t>
+        </is>
+      </c>
+      <c r="B20" s="29" t="inlineStr">
+        <is>
+          <t>Agir já / Estruturar / Oportunidade / Monitorar</t>
+        </is>
+      </c>
+      <c r="C20" s="30" t="inlineStr">
+        <is>
+          <t>Quadrantes da matriz. Agir já: risco alto, fácil de agir. Estruturar: risco alto, difícil (exige articulação). Oportunidade: risco baixo, fácil. Monitorar: risco baixo, difícil.</t>
+        </is>
+      </c>
+      <c r="D20" s="30" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="28" t="inlineStr">
+        <is>
+          <t>Modelo de risco</t>
+        </is>
+      </c>
+      <c r="B21" s="29" t="inlineStr">
+        <is>
+          <t>Diagnóstico de causa</t>
+        </is>
+      </c>
+      <c r="C21" s="30" t="inlineStr">
+        <is>
+          <t>Por que o ponto alaga (drenagem obstruída, subdimensionada, maré, esgoto). Fica fora do risco e indica qual órgão age.</t>
+        </is>
+      </c>
+      <c r="D21" s="30" t="inlineStr">
+        <is>
+          <t>Galeria assoreada → EMLURB (manutenção).</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="28" t="inlineStr">
+        <is>
+          <t>Modelo de risco</t>
+        </is>
+      </c>
+      <c r="B22" s="29" t="inlineStr">
+        <is>
+          <t>Análise de sensibilidade</t>
+        </is>
+      </c>
+      <c r="C22" s="30" t="inlineStr">
+        <is>
+          <t>Recalcular o ranking com outros pesos (ex.: pesos iguais) para ver se o resultado depende demais dos pesos escolhidos.</t>
+        </is>
+      </c>
+      <c r="D22" s="30" t="inlineStr">
+        <is>
+          <t>Se o top 5 muda muito, avisar a alta gestão.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="31" t="inlineStr">
+        <is>
+          <t>Tipo de nota</t>
+        </is>
+      </c>
+      <c r="B23" s="29" t="inlineStr">
+        <is>
+          <t>Faixa fixa</t>
+        </is>
+      </c>
+      <c r="C23" s="30" t="inlineStr">
+        <is>
+          <t>O valor medido cai numa faixa definida antes da coleta. A nota não depende dos outros pontos.</t>
+        </is>
+      </c>
+      <c r="D23" s="30" t="inlineStr">
+        <is>
+          <t>P1: 5 alagamentos/ano cai em '5–6' = nota 4.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="31" t="inlineStr">
+        <is>
+          <t>Tipo de nota</t>
+        </is>
+      </c>
+      <c r="B24" s="29" t="inlineStr">
+        <is>
+          <t>Classe</t>
+        </is>
+      </c>
+      <c r="C24" s="30" t="inlineStr">
+        <is>
+          <t>O ponto é encaixado numa categoria descritiva, não num número.</t>
+        </is>
+      </c>
+      <c r="D24" s="30" t="inlineStr">
+        <is>
+          <t>P3: 'agrava ocasionalmente' = nota 3.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="31" t="inlineStr">
+        <is>
+          <t>Tipo de nota</t>
+        </is>
+      </c>
+      <c r="B25" s="29" t="inlineStr">
+        <is>
+          <t>Quintil</t>
+        </is>
+      </c>
+      <c r="C25" s="30" t="inlineStr">
+        <is>
+          <t>Nota relativa entre os 21 pontos: os valores são ordenados e divididos em 5 grupos de ~4 pontos. Os 20% menores recebem 1; os 20% maiores, 5.</t>
+        </is>
+      </c>
+      <c r="D25" s="30" t="inlineStr">
+        <is>
+          <t>E1: os ~4 pontos com mais moradores recebem nota 5.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="31" t="inlineStr">
+        <is>
+          <t>Tipo de nota</t>
+        </is>
+      </c>
+      <c r="B26" s="29" t="inlineStr">
+        <is>
+          <t>Quintil invertido</t>
+        </is>
+      </c>
+      <c r="C26" s="30" t="inlineStr">
+        <is>
+          <t>Igual ao quintil, mas o MENOR valor recebe a nota mais alta.</t>
+        </is>
+      </c>
+      <c r="D26" s="30" t="inlineStr">
+        <is>
+          <t>P4: o ponto mais perto do rio recebe nota 5.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="31" t="inlineStr">
+        <is>
+          <t>Tipo de nota</t>
+        </is>
+      </c>
+      <c r="B27" s="29" t="inlineStr">
+        <is>
+          <t>Faixa provisória</t>
+        </is>
+      </c>
+      <c r="C27" s="30" t="inlineStr">
+        <is>
+          <t>Faixa proposta antes de ver os dados reais. Deve ser calibrada quando os dados chegarem.</t>
+        </is>
+      </c>
+      <c r="D27" s="30" t="inlineStr">
+        <is>
+          <t>Se todos os pontos caírem na mesma faixa, ela precisa ser ajustada.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="31" t="inlineStr">
+        <is>
+          <t>Tipo de nota</t>
+        </is>
+      </c>
+      <c r="B28" s="29" t="inlineStr">
+        <is>
+          <t>Origem da faixa</t>
+        </is>
+      </c>
+      <c r="C28" s="30" t="inlineStr">
+        <is>
+          <t>De onde veio a escala: planilha original da equipe, referência oficial (ex.: Ipea) ou proposta do Claude (a revisar pelo grupo).</t>
+        </is>
+      </c>
+      <c r="D28" s="30" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="32" t="inlineStr">
+        <is>
+          <t>Território e SIG</t>
+        </is>
+      </c>
+      <c r="B29" s="29" t="inlineStr">
+        <is>
+          <t>Ponto crítico</t>
+        </is>
+      </c>
+      <c r="C29" s="30" t="inlineStr">
+        <is>
+          <t>Local da lista da EMLURB onde há alagamento recorrente. Pode ser um ponto, um trecho de rua ou vários trechos.</t>
+        </is>
+      </c>
+      <c r="D29" s="30" t="inlineStr">
+        <is>
+          <t>Ponto 24 — Ipsep, Rua Blumenau (até a maré).</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="32" t="inlineStr">
+        <is>
+          <t>Território e SIG</t>
+        </is>
+      </c>
+      <c r="B30" s="29" t="inlineStr">
+        <is>
+          <t>Trecho (Linha / Vários)</t>
+        </is>
+      </c>
+      <c r="C30" s="30" t="inlineStr">
+        <is>
+          <t>Ponto crítico que é uma extensão de rua, não um local único. 12 dos 21 pontos são trechos.</t>
+        </is>
+      </c>
+      <c r="D30" s="30" t="inlineStr">
+        <is>
+          <t>Ponto 11 — Rua Professor José Brandão (toda a extensão).</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="32" t="inlineStr">
+        <is>
+          <t>Território e SIG</t>
+        </is>
+      </c>
+      <c r="B31" s="29" t="inlineStr">
+        <is>
+          <t>RPA 6</t>
+        </is>
+      </c>
+      <c r="C31" s="30" t="inlineStr">
+        <is>
+          <t>Região Político-Administrativa 6 do Recife (Boa Viagem, Pina, Imbiribeira, Ipsep, Ibura, Jordão, entre outros bairros). Escopo do piloto.</t>
+        </is>
+      </c>
+      <c r="D31" s="30" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="32" t="inlineStr">
+        <is>
+          <t>Território e SIG</t>
+        </is>
+      </c>
+      <c r="B32" s="29" t="inlineStr">
+        <is>
+          <t>SIG</t>
+        </is>
+      </c>
+      <c r="C32" s="30" t="inlineStr">
+        <is>
+          <t>Sistema de Informação Geográfica: programa para mapas e cálculos espaciais. Usamos o ArcGIS Pro.</t>
+        </is>
+      </c>
+      <c r="D32" s="30" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="32" t="inlineStr">
+        <is>
+          <t>Território e SIG</t>
+        </is>
+      </c>
+      <c r="B33" s="29" t="inlineStr">
+        <is>
+          <t>Círculo de 300 m (buffer)</t>
+        </is>
+      </c>
+      <c r="C33" s="30" t="inlineStr">
+        <is>
+          <t>Área de 300 m em volta do ponto (ou da linha do trecho) onde se medem os subcritérios do SIG. Usado no cálculo do risco.</t>
+        </is>
+      </c>
+      <c r="D33" s="30" t="inlineStr">
+        <is>
+          <t>Moradores dentro do círculo = População (E1).</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="32" t="inlineStr">
+        <is>
+          <t>Território e SIG</t>
+        </is>
+      </c>
+      <c r="B34" s="29" t="inlineStr">
+        <is>
+          <t>Área de influência de 1 km</t>
+        </is>
+      </c>
+      <c r="C34" s="30" t="inlineStr">
+        <is>
+          <t>Círculo de 1 km mostrado no painel só como informação. Não entra no cálculo, porque com 1 km quase todos os pontos se sobrepõem.</t>
+        </is>
+      </c>
+      <c r="D34" s="30" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="32" t="inlineStr">
+        <is>
+          <t>Território e SIG</t>
+        </is>
+      </c>
+      <c r="B35" s="29" t="inlineStr">
+        <is>
+          <t>Grupo de sobreposição (G1–G5)</t>
+        </is>
+      </c>
+      <c r="C35" s="30" t="inlineStr">
+        <is>
+          <t>Pontos cujos círculos de 300 m se sobrepõem. Nesses grupos os subcritérios do SIG tendem a dar notas parecidas.</t>
+        </is>
+      </c>
+      <c r="D35" s="30" t="inlineStr">
+        <is>
+          <t>G1 = pontos 5, 6, 7, 11 e 12 (Conselheiro Aguiar).</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="32" t="inlineStr">
+        <is>
+          <t>Território e SIG</t>
+        </is>
+      </c>
+      <c r="B36" s="29" t="inlineStr">
+        <is>
+          <t>Ponderação por área</t>
+        </is>
+      </c>
+      <c r="C36" s="30" t="inlineStr">
+        <is>
+          <t>Quando uma área de dados (setor, célula) corta o círculo, conta só a parte que fica dentro dele.</t>
+        </is>
+      </c>
+      <c r="D36" s="30" t="inlineStr">
+        <is>
+          <t>Setor com 40% da área no círculo contribui com 40% da população.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="32" t="inlineStr">
+        <is>
+          <t>Território e SIG</t>
+        </is>
+      </c>
+      <c r="B37" s="29" t="inlineStr">
+        <is>
+          <t>EPSG:31985 (SIRGAS 2000 / UTM 25S)</t>
+        </is>
+      </c>
+      <c r="C37" s="30" t="inlineStr">
+        <is>
+          <t>Sistema de coordenadas usado no projeto. Todas as camadas precisam estar nele antes dos cálculos.</t>
+        </is>
+      </c>
+      <c r="D37" s="30" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="32" t="inlineStr">
+        <is>
+          <t>Território e SIG</t>
+        </is>
+      </c>
+      <c r="B38" s="29" t="inlineStr">
+        <is>
+          <t>Coordenada aproximada / verificada</t>
+        </is>
+      </c>
+      <c r="C38" s="30" t="inlineStr">
+        <is>
+          <t>Aproximada = localizada automaticamente e ainda não conferida. Verificada = conferida com a EMLURB ou por imagem de satélite.</t>
+        </is>
+      </c>
+      <c r="D38" s="30" t="inlineStr">
+        <is>
+          <t>Hoje nenhuma das 21 coordenadas está verificada.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="32" t="inlineStr">
+        <is>
+          <t>Território e SIG</t>
+        </is>
+      </c>
+      <c r="B39" s="29" t="inlineStr">
+        <is>
+          <t>Bacia / sub-bacia</t>
+        </is>
+      </c>
+      <c r="C39" s="30" t="inlineStr">
+        <is>
+          <t>Área que drena para um mesmo rio ou canal. Hierarquia do Plano de Drenagem: Bacia → Sub-bacia → Ponto crítico → Obra.</t>
+        </is>
+      </c>
+      <c r="D39" s="30" t="inlineStr">
+        <is>
+          <t>Usada para ligar obras aos pontos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="32" t="inlineStr">
+        <is>
+          <t>Território e SIG</t>
+        </is>
+      </c>
+      <c r="B40" s="29" t="inlineStr">
+        <is>
+          <t>Shapefile / GeoJSON</t>
+        </is>
+      </c>
+      <c r="C40" s="30" t="inlineStr">
+        <is>
+          <t>Formatos de arquivo de mapa que o ArcGIS abre.</t>
+        </is>
+      </c>
+      <c r="D40" s="30" t="inlineStr">
+        <is>
+          <t>dados/processados/pontos_rpa6.geojson tem os 21 pontos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="33" t="inlineStr">
+        <is>
+          <t>Fontes de dados</t>
+        </is>
+      </c>
+      <c r="B41" s="29" t="inlineStr">
+        <is>
+          <t>Censo 2022 (IBGE)</t>
+        </is>
+      </c>
+      <c r="C41" s="30" t="inlineStr">
+        <is>
+          <t>Recenseamento de 2022. Fonte de população, idade, tipo de domicílio e esgotamento.</t>
+        </is>
+      </c>
+      <c r="D41" s="30" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="33" t="inlineStr">
+        <is>
+          <t>Fontes de dados</t>
+        </is>
+      </c>
+      <c r="B42" s="29" t="inlineStr">
+        <is>
+          <t>Setor censitário</t>
+        </is>
+      </c>
+      <c r="C42" s="30" t="inlineStr">
+        <is>
+          <t>Menor área de divulgação do Censo (no Recife adensado, poucos quarteirões).</t>
+        </is>
+      </c>
+      <c r="D42" s="30" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="33" t="inlineStr">
+        <is>
+          <t>Fontes de dados</t>
+        </is>
+      </c>
+      <c r="B43" s="29" t="inlineStr">
+        <is>
+          <t>Grade Estatística (IBGE)</t>
+        </is>
+      </c>
+      <c r="C43" s="30" t="inlineStr">
+        <is>
+          <t>Malha de quadrados de 200 × 200 m (área urbana) com a população do Censo 2022.</t>
+        </is>
+      </c>
+      <c r="D43" s="30" t="inlineStr">
+        <is>
+          <t>Fonte do E1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="33" t="inlineStr">
+        <is>
+          <t>Fontes de dados</t>
+        </is>
+      </c>
+      <c r="B44" s="29" t="inlineStr">
+        <is>
+          <t>CNEFE (IBGE)</t>
+        </is>
+      </c>
+      <c r="C44" s="30" t="inlineStr">
+        <is>
+          <t>Cadastro de endereços do Censo 2022, com coordenada e tipo de uso (domicílio, ensino, saúde, outras finalidades).</t>
+        </is>
+      </c>
+      <c r="D44" s="30" t="inlineStr">
+        <is>
+          <t>Fonte do E2 e do E3.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="33" t="inlineStr">
+        <is>
+          <t>Fontes de dados</t>
+        </is>
+      </c>
+      <c r="B45" s="29" t="inlineStr">
+        <is>
+          <t>Favelas e Comunidades Urbanas (IBGE)</t>
+        </is>
+      </c>
+      <c r="C45" s="30" t="inlineStr">
+        <is>
+          <t>Mapeamento do IBGE das favelas e comunidades urbanas no Censo 2022. Publicação da malha ainda não confirmada.</t>
+        </is>
+      </c>
+      <c r="D45" s="30" t="inlineStr">
+        <is>
+          <t>Fonte do V3.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="33" t="inlineStr">
+        <is>
+          <t>Fontes de dados</t>
+        </is>
+      </c>
+      <c r="B46" s="29" t="inlineStr">
+        <is>
+          <t>IVS (Ipea)</t>
+        </is>
+      </c>
+      <c r="C46" s="30" t="inlineStr">
+        <is>
+          <t>Índice de Vulnerabilidade Social do Ipea, de 0 a 1 (quanto maior, mais vulnerável). Base do Censo 2010.</t>
+        </is>
+      </c>
+      <c r="D46" s="30" t="inlineStr">
+        <is>
+          <t>Plano B do V3.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="33" t="inlineStr">
+        <is>
+          <t>Fontes de dados</t>
+        </is>
+      </c>
+      <c r="B47" s="29" t="inlineStr">
+        <is>
+          <t>UDH</t>
+        </is>
+      </c>
+      <c r="C47" s="30" t="inlineStr">
+        <is>
+          <t>Unidade de Desenvolvimento Humano: área usada pelo Ipea, maior que o setor censitário.</t>
+        </is>
+      </c>
+      <c r="D47" s="30" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="33" t="inlineStr">
+        <is>
+          <t>Fontes de dados</t>
+        </is>
+      </c>
+      <c r="B48" s="29" t="inlineStr">
+        <is>
+          <t>MapBiomas</t>
+        </is>
+      </c>
+      <c r="C48" s="30" t="inlineStr">
+        <is>
+          <t>Mapa de cobertura do solo (vegetação, área construída etc.) com pixels de 30 m. Não verificado.</t>
+        </is>
+      </c>
+      <c r="D48" s="30" t="inlineStr">
+        <is>
+          <t>Fonte do P5.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="33" t="inlineStr">
+        <is>
+          <t>Fontes de dados</t>
+        </is>
+      </c>
+      <c r="B49" s="29" t="inlineStr">
+        <is>
+          <t>ESIG</t>
+        </is>
+      </c>
+      <c r="C49" s="30" t="inlineStr">
+        <is>
+          <t>Sistema de informações geográficas da Prefeitura do Recife (vias, lotes, edificações, recursos hídricos).</t>
+        </is>
+      </c>
+      <c r="D49" s="30" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="33" t="inlineStr">
+        <is>
+          <t>Fontes de dados</t>
+        </is>
+      </c>
+      <c r="B50" s="29" t="inlineStr">
+        <is>
+          <t>CNES / DATASUS</t>
+        </is>
+      </c>
+      <c r="C50" s="30" t="inlineStr">
+        <is>
+          <t>Cadastro Nacional de Estabelecimentos de Saúde.</t>
+        </is>
+      </c>
+      <c r="D50" s="30" t="inlineStr">
+        <is>
+          <t>Complementa o E2.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="33" t="inlineStr">
+        <is>
+          <t>Fontes de dados</t>
+        </is>
+      </c>
+      <c r="B51" s="29" t="inlineStr">
+        <is>
+          <t>APAC / Cemaden</t>
+        </is>
+      </c>
+      <c r="C51" s="30" t="inlineStr">
+        <is>
+          <t>Agência Pernambucana de Águas e Clima / Centro Nacional de Monitoramento de Desastres: dados de chuva e marés.</t>
+        </is>
+      </c>
+      <c r="D51" s="30" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="33" t="inlineStr">
+        <is>
+          <t>Fontes de dados</t>
+        </is>
+      </c>
+      <c r="B52" s="29" t="inlineStr">
+        <is>
+          <t>PMDR</t>
+        </is>
+      </c>
+      <c r="C52" s="30" t="inlineStr">
+        <is>
+          <t>Plano Municipal de Drenagem do Recife. Define bacias e sub-bacias.</t>
+        </is>
+      </c>
+      <c r="D52" s="30" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="33" t="inlineStr">
+        <is>
+          <t>Fontes de dados</t>
+        </is>
+      </c>
+      <c r="B53" s="29" t="inlineStr">
+        <is>
+          <t>Ficha EMLURB</t>
+        </is>
+      </c>
+      <c r="C53" s="30" t="inlineStr">
+        <is>
+          <t>Formulário a ser preenchido com a EMLURB, com uma linha por ponto: localização, frequência, severidade, maré e obras ligadas.</t>
+        </is>
+      </c>
+      <c r="D53" s="30" t="inlineStr">
+        <is>
+          <t>Fonte provisória de P1, P2 e P3.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="34" t="inlineStr">
+        <is>
+          <t>Checklist</t>
+        </is>
+      </c>
+      <c r="B54" s="29" t="inlineStr">
+        <is>
+          <t>Recomendação</t>
+        </is>
+      </c>
+      <c r="C54" s="30" t="inlineStr">
+        <is>
+          <t>Manter = entra no modelo. Condicional = só entra se o dado existir. Plano B = usado só se outro subcritério falhar. Peso alto / menor = sugestão para a definição dos pesos.</t>
+        </is>
+      </c>
+      <c r="D54" s="30" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="34" t="inlineStr">
+        <is>
+          <t>Checklist</t>
+        </is>
+      </c>
+      <c r="B55" s="29" t="inlineStr">
+        <is>
+          <t>Fonte confirmada?</t>
+        </is>
+      </c>
+      <c r="C55" s="30" t="inlineStr">
+        <is>
+          <t>A base de dados existe e a equipe consegue acessá-la (download ou pedido atendido).</t>
+        </is>
+      </c>
+      <c r="D55" s="30" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="34" t="inlineStr">
+        <is>
+          <t>Checklist</t>
+        </is>
+      </c>
+      <c r="B56" s="29" t="inlineStr">
+        <is>
+          <t>Dado existe na fonte?</t>
+        </is>
+      </c>
+      <c r="C56" s="30" t="inlineStr">
+        <is>
+          <t>A variável necessária está na base, na escala do círculo de 300 m, e cobre os 21 pontos.</t>
+        </is>
+      </c>
+      <c r="D56" s="30" t="inlineStr">
+        <is>
+          <t>O IBGE existe (fonte confirmada), mas falta checar se o tipo de domicílio vem por setor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="34" t="inlineStr">
+        <is>
+          <t>Checklist</t>
+        </is>
+      </c>
+      <c r="B57" s="29" t="inlineStr">
+        <is>
+          <t>Sim / Parcial / Não / Pendente</t>
+        </is>
+      </c>
+      <c r="C57" s="30" t="inlineStr">
+        <is>
+          <t>Sim = confirmado. Parcial = existe, mas com limitação (escala, cobertura, data). Não = não existe ou não é acessível. Pendente = ainda não checado.</t>
+        </is>
+      </c>
+      <c r="D57" s="30" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="34" t="inlineStr">
+        <is>
+          <t>Checklist</t>
+        </is>
+      </c>
+      <c r="B58" s="29" t="inlineStr">
+        <is>
+          <t>Busca prévia (Claude)</t>
+        </is>
+      </c>
+      <c r="C58" s="30" t="inlineStr">
+        <is>
+          <t>O que foi encontrado em busca na internet. 'Confirmado na busca' = a base aparece como publicada, mas o arquivo não foi aberto.</t>
+        </is>
+      </c>
+      <c r="D58" s="30" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="35" t="inlineStr">
+        <is>
+          <t>Órgãos</t>
+        </is>
+      </c>
+      <c r="B59" s="29" t="inlineStr">
+        <is>
+          <t>COP</t>
+        </is>
+      </c>
+      <c r="C59" s="30" t="inlineStr">
+        <is>
+          <t>Centro de Operações do Recife: monitoramento e resposta aos eventos.</t>
+        </is>
+      </c>
+      <c r="D59" s="30" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="35" t="inlineStr">
+        <is>
+          <t>Órgãos</t>
+        </is>
+      </c>
+      <c r="B60" s="29" t="inlineStr">
+        <is>
+          <t>EMLURB</t>
+        </is>
+      </c>
+      <c r="C60" s="30" t="inlineStr">
+        <is>
+          <t>Empresa de Manutenção e Limpeza Urbana: manutenção da drenagem e lista de pontos críticos.</t>
+        </is>
+      </c>
+      <c r="D60" s="30" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="35" t="inlineStr">
+        <is>
+          <t>Órgãos</t>
+        </is>
+      </c>
+      <c r="B61" s="29" t="inlineStr">
+        <is>
+          <t>Defesa Civil (Sedec)</t>
+        </is>
+      </c>
+      <c r="C61" s="30" t="inlineStr">
+        <is>
+          <t>Áreas de risco, alertas e vistorias.</t>
+        </is>
+      </c>
+      <c r="D61" s="30" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="35" t="inlineStr">
+        <is>
+          <t>Órgãos</t>
+        </is>
+      </c>
+      <c r="B62" s="29" t="inlineStr">
+        <is>
+          <t>URB</t>
+        </is>
+      </c>
+      <c r="C62" s="30" t="inlineStr">
+        <is>
+          <t>Autarquia de Urbanização do Recife: obras urbanas e de drenagem.</t>
+        </is>
+      </c>
+      <c r="D62" s="30" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="35" t="inlineStr">
+        <is>
+          <t>Órgãos</t>
+        </is>
+      </c>
+      <c r="B63" s="29" t="inlineStr">
+        <is>
+          <t>CTTU</t>
+        </is>
+      </c>
+      <c r="C63" s="30" t="inlineStr">
+        <is>
+          <t>Autarquia de Trânsito e Transporte Urbano: trânsito, vias e interdições.</t>
+        </is>
+      </c>
+      <c r="D63" s="30" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="35" t="inlineStr">
+        <is>
+          <t>Órgãos</t>
+        </is>
+      </c>
+      <c r="B64" s="29" t="inlineStr">
+        <is>
+          <t>Compesa</t>
+        </is>
+      </c>
+      <c r="C64" s="30" t="inlineStr">
+        <is>
+          <t>Companhia Pernambucana de Saneamento: água e esgoto.</t>
+        </is>
+      </c>
+      <c r="D64" s="30" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="35" t="inlineStr">
+        <is>
+          <t>Órgãos</t>
+        </is>
+      </c>
+      <c r="B65" s="29" t="inlineStr">
+        <is>
+          <t>ProMorar</t>
+        </is>
+      </c>
+      <c r="C65" s="30" t="inlineStr">
+        <is>
+          <t>Programa de urbanização de comunidades.</t>
+        </is>
+      </c>
+      <c r="D65" s="30" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="35" t="inlineStr">
+        <is>
+          <t>Órgãos</t>
+        </is>
+      </c>
+      <c r="B66" s="29" t="inlineStr">
+        <is>
+          <t>SEPLAG / SEPLAN</t>
+        </is>
+      </c>
+      <c r="C66" s="30" t="inlineStr">
+        <is>
+          <t>Planejamento e gestão. A SEPLAN não é a SEPLAG; o papel dela no projeto ainda será definido.</t>
+        </is>
+      </c>
+      <c r="D66" s="30" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="35" t="inlineStr">
+        <is>
+          <t>Órgãos</t>
+        </is>
+      </c>
+      <c r="B67" s="29" t="inlineStr">
+        <is>
+          <t>Grande Recife Consórcio</t>
+        </is>
+      </c>
+      <c r="C67" s="30" t="inlineStr">
+        <is>
+          <t>Consórcio de transporte metropolitano: linhas e paradas de ônibus.</t>
+        </is>
+      </c>
+      <c r="D67" s="30" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A4:D67"/>
+  <mergeCells count="1">
+    <mergeCell ref="A2:D2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Aba Notas dos pontos e índice de risco de 0 a 1
- Nova aba na planilha de checklist com os 21 pontos, notas de 1 a 5 por
  subcritério, linha de pesos (vazio = peso igual), nota de cada critério,
  Consequência, Risco P × C, índice de risco 0–1, posição e notas preenchidas
- Índice (Risco − 1) ÷ 24 também na saída do hierarquizar.py
- Lista de pontos enviada por Pedro guardada em dados/brutos/emlurb

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018419ScLbL3ubanHMYyaBnW
</commit_message>
<xml_diff>
--- a/dados/Recife_Resiliente_Checklist_Subcriterios.xlsx
+++ b/dados/Recife_Resiliente_Checklist_Subcriterios.xlsx
@@ -8,11 +8,12 @@
   </bookViews>
   <sheets>
     <sheet name="Checklist subcritérios" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Glossário" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Notas dos pontos" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Glossário" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Checklist subcritérios'!$A$4:$Q$19</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Glossário'!$A$4:$D$67</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Glossário'!$A$4:$D$67</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -20,8 +21,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="10">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.000"/>
+  </numFmts>
+  <fonts count="14">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -72,8 +75,28 @@
       <b val="1"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="000000FF"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="000000FF"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="13">
+  <fills count="15">
     <fill>
       <patternFill/>
     </fill>
@@ -132,6 +155,16 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00595959"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C00000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00EDEDED"/>
       </patternFill>
     </fill>
@@ -162,7 +195,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="60">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -233,6 +266,79 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="8" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="9" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="9" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="8" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -241,9 +347,6 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -258,7 +361,7 @@
     <xf numFmtId="0" fontId="8" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2191,6 +2294,1931 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:AC34"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="42" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="7" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="11" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
+    <col width="13" customWidth="1" min="12" max="12"/>
+    <col width="11" customWidth="1" min="13" max="13"/>
+    <col width="11" customWidth="1" min="14" max="14"/>
+    <col width="11" customWidth="1" min="15" max="15"/>
+    <col width="13" customWidth="1" min="16" max="16"/>
+    <col width="11" customWidth="1" min="17" max="17"/>
+    <col width="11" customWidth="1" min="18" max="18"/>
+    <col width="11" customWidth="1" min="19" max="19"/>
+    <col width="11" customWidth="1" min="20" max="20"/>
+    <col width="13" customWidth="1" min="21" max="21"/>
+    <col width="11" customWidth="1" min="22" max="22"/>
+    <col width="11" customWidth="1" min="23" max="23"/>
+    <col width="13" customWidth="1" min="24" max="24"/>
+    <col width="13" customWidth="1" min="25" max="25"/>
+    <col width="13" customWidth="1" min="26" max="26"/>
+    <col width="13" customWidth="1" min="27" max="27"/>
+    <col width="13" customWidth="1" min="28" max="28"/>
+    <col width="13" customWidth="1" min="29" max="29"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Recife Resiliente — Notas dos pontos críticos da RPA 6 e cálculo do risco</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="40" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Preencha as notas (1 a 5, 5 = mais crítico) nas células amarelas, conforme as escalas da aba 'Checklist subcritérios'. Linha 'Peso': vazia = todos os pesos iguais. Nota em branco fica fora da média (não vira zero). Sem nota de Probabilidade não há risco. P6 e V1 são condicionais: deixe em branco se não forem usados. Colunas cinza são calculadas: não edite.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="F4" s="26" t="inlineStr">
+        <is>
+          <t>Probabilidade</t>
+        </is>
+      </c>
+      <c r="M4" s="27" t="inlineStr">
+        <is>
+          <t>Exposição</t>
+        </is>
+      </c>
+      <c r="Q4" s="28" t="inlineStr">
+        <is>
+          <t>Vulnerabilidade</t>
+        </is>
+      </c>
+      <c r="V4" s="29" t="inlineStr">
+        <is>
+          <t>Impacto</t>
+        </is>
+      </c>
+      <c r="Y4" s="30" t="inlineStr">
+        <is>
+          <t>Resultado</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="E5" s="31" t="inlineStr">
+        <is>
+          <t>Peso →</t>
+        </is>
+      </c>
+      <c r="F5" s="32" t="n"/>
+      <c r="G5" s="32" t="n"/>
+      <c r="H5" s="32" t="n"/>
+      <c r="I5" s="32" t="n"/>
+      <c r="J5" s="32" t="n"/>
+      <c r="K5" s="32" t="n"/>
+      <c r="L5" s="33" t="inlineStr">
+        <is>
+          <t>(multiplica)</t>
+        </is>
+      </c>
+      <c r="M5" s="32" t="n"/>
+      <c r="N5" s="32" t="n"/>
+      <c r="O5" s="32" t="n"/>
+      <c r="P5" s="34" t="n"/>
+      <c r="Q5" s="32" t="n"/>
+      <c r="R5" s="32" t="n"/>
+      <c r="S5" s="32" t="n"/>
+      <c r="T5" s="32" t="n"/>
+      <c r="U5" s="34" t="n"/>
+      <c r="V5" s="32" t="n"/>
+      <c r="W5" s="32" t="n"/>
+      <c r="X5" s="34" t="n"/>
+    </row>
+    <row r="6" ht="54" customHeight="1">
+      <c r="A6" s="35" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B6" s="35" t="inlineStr">
+        <is>
+          <t>Bairro</t>
+        </is>
+      </c>
+      <c r="C6" s="35" t="inlineStr">
+        <is>
+          <t>Trecho</t>
+        </is>
+      </c>
+      <c r="D6" s="35" t="inlineStr">
+        <is>
+          <t>Tipo</t>
+        </is>
+      </c>
+      <c r="E6" s="35" t="inlineStr">
+        <is>
+          <t>Grupo</t>
+        </is>
+      </c>
+      <c r="F6" s="36" t="inlineStr">
+        <is>
+          <t>P1
+Frequência de alagamento</t>
+        </is>
+      </c>
+      <c r="G6" s="36" t="inlineStr">
+        <is>
+          <t>P2
+Severidade</t>
+        </is>
+      </c>
+      <c r="H6" s="36" t="inlineStr">
+        <is>
+          <t>P3
+Influência da maré</t>
+        </is>
+      </c>
+      <c r="I6" s="36" t="inlineStr">
+        <is>
+          <t>P4
+Proximidade de rio ou canal</t>
+        </is>
+      </c>
+      <c r="J6" s="36" t="inlineStr">
+        <is>
+          <t>P5
+Impermeabilização</t>
+        </is>
+      </c>
+      <c r="K6" s="36" t="inlineStr">
+        <is>
+          <t>P6
+Baixio</t>
+        </is>
+      </c>
+      <c r="L6" s="37" t="inlineStr">
+        <is>
+          <t>Nota
+Probabilidade</t>
+        </is>
+      </c>
+      <c r="M6" s="38" t="inlineStr">
+        <is>
+          <t>E1
+População</t>
+        </is>
+      </c>
+      <c r="N6" s="38" t="inlineStr">
+        <is>
+          <t>E2
+Equipamentos sensíveis</t>
+        </is>
+      </c>
+      <c r="O6" s="38" t="inlineStr">
+        <is>
+          <t>E3
+Atividade econômica</t>
+        </is>
+      </c>
+      <c r="P6" s="37" t="inlineStr">
+        <is>
+          <t>Nota
+Exposição</t>
+        </is>
+      </c>
+      <c r="Q6" s="39" t="inlineStr">
+        <is>
+          <t>V2
+Grupos sensíveis</t>
+        </is>
+      </c>
+      <c r="R6" s="39" t="inlineStr">
+        <is>
+          <t>V3
+Favelas e comunidades urbanas</t>
+        </is>
+      </c>
+      <c r="S6" s="39" t="inlineStr">
+        <is>
+          <t>V4
+Tipo de moradia</t>
+        </is>
+      </c>
+      <c r="T6" s="39" t="inlineStr">
+        <is>
+          <t>V1
+Vulnerabilidade social (IVS)</t>
+        </is>
+      </c>
+      <c r="U6" s="37" t="inlineStr">
+        <is>
+          <t>Nota
+Vulnerabilidade</t>
+        </is>
+      </c>
+      <c r="V6" s="40" t="inlineStr">
+        <is>
+          <t>I1
+Mobilidade</t>
+        </is>
+      </c>
+      <c r="W6" s="40" t="inlineStr">
+        <is>
+          <t>I2
+Risco sanitário</t>
+        </is>
+      </c>
+      <c r="X6" s="37" t="inlineStr">
+        <is>
+          <t>Nota
+Impacto</t>
+        </is>
+      </c>
+      <c r="Y6" s="41" t="inlineStr">
+        <is>
+          <t>Consequência
+(1–5)</t>
+        </is>
+      </c>
+      <c r="Z6" s="41" t="inlineStr">
+        <is>
+          <t>Risco
+P × C (1–25)</t>
+        </is>
+      </c>
+      <c r="AA6" s="41" t="inlineStr">
+        <is>
+          <t>Índice de risco
+(0–1)</t>
+        </is>
+      </c>
+      <c r="AB6" s="41" t="inlineStr">
+        <is>
+          <t>Posição</t>
+        </is>
+      </c>
+      <c r="AC6" s="41" t="inlineStr">
+        <is>
+          <t>Notas
+preenchidas</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="42" t="n">
+        <v>5</v>
+      </c>
+      <c r="B7" s="42" t="inlineStr">
+        <is>
+          <t>Boa Viagem</t>
+        </is>
+      </c>
+      <c r="C7" s="43" t="inlineStr">
+        <is>
+          <t>Avenida Conselheiro Aguiar (Interseção com a Rua Tenente João Cícero)</t>
+        </is>
+      </c>
+      <c r="D7" s="42" t="inlineStr">
+        <is>
+          <t>Ponto</t>
+        </is>
+      </c>
+      <c r="E7" s="42" t="inlineStr">
+        <is>
+          <t>G1</t>
+        </is>
+      </c>
+      <c r="F7" s="44" t="n"/>
+      <c r="G7" s="44" t="n"/>
+      <c r="H7" s="44" t="n"/>
+      <c r="I7" s="44" t="n"/>
+      <c r="J7" s="44" t="n"/>
+      <c r="K7" s="44" t="n"/>
+      <c r="L7" s="45">
+        <f>IF(COUNT(F7:K7)=0,"",IFERROR(SUMPRODUCT(F7:K7,(F$5:K$5+(F$5:K$5="")))/SUMPRODUCT((F7:K7&lt;&gt;"")*(F$5:K$5+(F$5:K$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="M7" s="44" t="n"/>
+      <c r="N7" s="44" t="n"/>
+      <c r="O7" s="44" t="n"/>
+      <c r="P7" s="45">
+        <f>IF(COUNT(M7:O7)=0,"",IFERROR(SUMPRODUCT(M7:O7,(M$5:O$5+(M$5:O$5="")))/SUMPRODUCT((M7:O7&lt;&gt;"")*(M$5:O$5+(M$5:O$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="Q7" s="44" t="n"/>
+      <c r="R7" s="44" t="n"/>
+      <c r="S7" s="44" t="n"/>
+      <c r="T7" s="44" t="n"/>
+      <c r="U7" s="45">
+        <f>IF(COUNT(Q7:T7)=0,"",IFERROR(SUMPRODUCT(Q7:T7,(Q$5:T$5+(Q$5:T$5="")))/SUMPRODUCT((Q7:T7&lt;&gt;"")*(Q$5:T$5+(Q$5:T$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="V7" s="44" t="n"/>
+      <c r="W7" s="44" t="n"/>
+      <c r="X7" s="45">
+        <f>IF(COUNT(V7:W7)=0,"",IFERROR(SUMPRODUCT(V7:W7,(V$5:W$5+(V$5:W$5="")))/SUMPRODUCT((V7:W7&lt;&gt;"")*(V$5:W$5+(V$5:W$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="Y7" s="45">
+        <f>IFERROR(IF((ISNUMBER(P7)*(P$5+(P$5=""))+ISNUMBER(U7)*(U$5+(U$5=""))+ISNUMBER(X7)*(X$5+(X$5="")))=0,"",(N(P7)*(P$5+(P$5=""))+N(U7)*(U$5+(U$5=""))+N(X7)*(X$5+(X$5="")))/(ISNUMBER(P7)*(P$5+(P$5=""))+ISNUMBER(U7)*(U$5+(U$5=""))+ISNUMBER(X7)*(X$5+(X$5="")))),"")</f>
+        <v/>
+      </c>
+      <c r="Z7" s="46">
+        <f>IF(AND(ISNUMBER(L7),ISNUMBER(Y7)),L7*Y7,"")</f>
+        <v/>
+      </c>
+      <c r="AA7" s="47">
+        <f>IF(ISNUMBER(Z7),(Z7-1)/24,"")</f>
+        <v/>
+      </c>
+      <c r="AB7" s="48">
+        <f>IF(ISNUMBER(Z7),COUNTIF(Z$7:Z$27,"&gt;"&amp;Z7)+1,"")</f>
+        <v/>
+      </c>
+      <c r="AC7" s="49">
+        <f>COUNT(F7,G7,H7,I7,J7,K7,M7,N7,O7,Q7,R7,S7,T7,V7,W7)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="42" t="n">
+        <v>6</v>
+      </c>
+      <c r="B8" s="42" t="inlineStr">
+        <is>
+          <t>Boa Viagem</t>
+        </is>
+      </c>
+      <c r="C8" s="43" t="inlineStr">
+        <is>
+          <t>Avenida Conselheiro Aguiar (Interseção com a Rua Dona Benvinda)</t>
+        </is>
+      </c>
+      <c r="D8" s="42" t="inlineStr">
+        <is>
+          <t>Ponto</t>
+        </is>
+      </c>
+      <c r="E8" s="42" t="inlineStr">
+        <is>
+          <t>G1</t>
+        </is>
+      </c>
+      <c r="F8" s="44" t="n"/>
+      <c r="G8" s="44" t="n"/>
+      <c r="H8" s="44" t="n"/>
+      <c r="I8" s="44" t="n"/>
+      <c r="J8" s="44" t="n"/>
+      <c r="K8" s="44" t="n"/>
+      <c r="L8" s="45">
+        <f>IF(COUNT(F8:K8)=0,"",IFERROR(SUMPRODUCT(F8:K8,(F$5:K$5+(F$5:K$5="")))/SUMPRODUCT((F8:K8&lt;&gt;"")*(F$5:K$5+(F$5:K$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="M8" s="44" t="n"/>
+      <c r="N8" s="44" t="n"/>
+      <c r="O8" s="44" t="n"/>
+      <c r="P8" s="45">
+        <f>IF(COUNT(M8:O8)=0,"",IFERROR(SUMPRODUCT(M8:O8,(M$5:O$5+(M$5:O$5="")))/SUMPRODUCT((M8:O8&lt;&gt;"")*(M$5:O$5+(M$5:O$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="Q8" s="44" t="n"/>
+      <c r="R8" s="44" t="n"/>
+      <c r="S8" s="44" t="n"/>
+      <c r="T8" s="44" t="n"/>
+      <c r="U8" s="45">
+        <f>IF(COUNT(Q8:T8)=0,"",IFERROR(SUMPRODUCT(Q8:T8,(Q$5:T$5+(Q$5:T$5="")))/SUMPRODUCT((Q8:T8&lt;&gt;"")*(Q$5:T$5+(Q$5:T$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="V8" s="44" t="n"/>
+      <c r="W8" s="44" t="n"/>
+      <c r="X8" s="45">
+        <f>IF(COUNT(V8:W8)=0,"",IFERROR(SUMPRODUCT(V8:W8,(V$5:W$5+(V$5:W$5="")))/SUMPRODUCT((V8:W8&lt;&gt;"")*(V$5:W$5+(V$5:W$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="Y8" s="45">
+        <f>IFERROR(IF((ISNUMBER(P8)*(P$5+(P$5=""))+ISNUMBER(U8)*(U$5+(U$5=""))+ISNUMBER(X8)*(X$5+(X$5="")))=0,"",(N(P8)*(P$5+(P$5=""))+N(U8)*(U$5+(U$5=""))+N(X8)*(X$5+(X$5="")))/(ISNUMBER(P8)*(P$5+(P$5=""))+ISNUMBER(U8)*(U$5+(U$5=""))+ISNUMBER(X8)*(X$5+(X$5="")))),"")</f>
+        <v/>
+      </c>
+      <c r="Z8" s="46">
+        <f>IF(AND(ISNUMBER(L8),ISNUMBER(Y8)),L8*Y8,"")</f>
+        <v/>
+      </c>
+      <c r="AA8" s="47">
+        <f>IF(ISNUMBER(Z8),(Z8-1)/24,"")</f>
+        <v/>
+      </c>
+      <c r="AB8" s="48">
+        <f>IF(ISNUMBER(Z8),COUNTIF(Z$7:Z$27,"&gt;"&amp;Z8)+1,"")</f>
+        <v/>
+      </c>
+      <c r="AC8" s="49">
+        <f>COUNT(F8,G8,H8,I8,J8,K8,M8,N8,O8,Q8,R8,S8,T8,V8,W8)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="42" t="n">
+        <v>7</v>
+      </c>
+      <c r="B9" s="42" t="inlineStr">
+        <is>
+          <t>Boa Viagem</t>
+        </is>
+      </c>
+      <c r="C9" s="43" t="inlineStr">
+        <is>
+          <t>Avenida Conselheiro Aguiar (Interseção com a Rua Maria Carolina)</t>
+        </is>
+      </c>
+      <c r="D9" s="42" t="inlineStr">
+        <is>
+          <t>Ponto</t>
+        </is>
+      </c>
+      <c r="E9" s="42" t="inlineStr">
+        <is>
+          <t>G1</t>
+        </is>
+      </c>
+      <c r="F9" s="44" t="n"/>
+      <c r="G9" s="44" t="n"/>
+      <c r="H9" s="44" t="n"/>
+      <c r="I9" s="44" t="n"/>
+      <c r="J9" s="44" t="n"/>
+      <c r="K9" s="44" t="n"/>
+      <c r="L9" s="45">
+        <f>IF(COUNT(F9:K9)=0,"",IFERROR(SUMPRODUCT(F9:K9,(F$5:K$5+(F$5:K$5="")))/SUMPRODUCT((F9:K9&lt;&gt;"")*(F$5:K$5+(F$5:K$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="M9" s="44" t="n"/>
+      <c r="N9" s="44" t="n"/>
+      <c r="O9" s="44" t="n"/>
+      <c r="P9" s="45">
+        <f>IF(COUNT(M9:O9)=0,"",IFERROR(SUMPRODUCT(M9:O9,(M$5:O$5+(M$5:O$5="")))/SUMPRODUCT((M9:O9&lt;&gt;"")*(M$5:O$5+(M$5:O$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="Q9" s="44" t="n"/>
+      <c r="R9" s="44" t="n"/>
+      <c r="S9" s="44" t="n"/>
+      <c r="T9" s="44" t="n"/>
+      <c r="U9" s="45">
+        <f>IF(COUNT(Q9:T9)=0,"",IFERROR(SUMPRODUCT(Q9:T9,(Q$5:T$5+(Q$5:T$5="")))/SUMPRODUCT((Q9:T9&lt;&gt;"")*(Q$5:T$5+(Q$5:T$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="V9" s="44" t="n"/>
+      <c r="W9" s="44" t="n"/>
+      <c r="X9" s="45">
+        <f>IF(COUNT(V9:W9)=0,"",IFERROR(SUMPRODUCT(V9:W9,(V$5:W$5+(V$5:W$5="")))/SUMPRODUCT((V9:W9&lt;&gt;"")*(V$5:W$5+(V$5:W$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="Y9" s="45">
+        <f>IFERROR(IF((ISNUMBER(P9)*(P$5+(P$5=""))+ISNUMBER(U9)*(U$5+(U$5=""))+ISNUMBER(X9)*(X$5+(X$5="")))=0,"",(N(P9)*(P$5+(P$5=""))+N(U9)*(U$5+(U$5=""))+N(X9)*(X$5+(X$5="")))/(ISNUMBER(P9)*(P$5+(P$5=""))+ISNUMBER(U9)*(U$5+(U$5=""))+ISNUMBER(X9)*(X$5+(X$5="")))),"")</f>
+        <v/>
+      </c>
+      <c r="Z9" s="46">
+        <f>IF(AND(ISNUMBER(L9),ISNUMBER(Y9)),L9*Y9,"")</f>
+        <v/>
+      </c>
+      <c r="AA9" s="47">
+        <f>IF(ISNUMBER(Z9),(Z9-1)/24,"")</f>
+        <v/>
+      </c>
+      <c r="AB9" s="48">
+        <f>IF(ISNUMBER(Z9),COUNTIF(Z$7:Z$27,"&gt;"&amp;Z9)+1,"")</f>
+        <v/>
+      </c>
+      <c r="AC9" s="49">
+        <f>COUNT(F9,G9,H9,I9,J9,K9,M9,N9,O9,Q9,R9,S9,T9,V9,W9)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="42" t="n">
+        <v>8</v>
+      </c>
+      <c r="B10" s="42" t="inlineStr">
+        <is>
+          <t>Boa Viagem</t>
+        </is>
+      </c>
+      <c r="C10" s="43" t="inlineStr">
+        <is>
+          <t>Avenida Conselheiro Aguiar (Do nº 1501 até a Rua Baltazar Pereira)</t>
+        </is>
+      </c>
+      <c r="D10" s="42" t="inlineStr">
+        <is>
+          <t>Linha</t>
+        </is>
+      </c>
+      <c r="E10" s="42" t="inlineStr">
+        <is>
+          <t>G2</t>
+        </is>
+      </c>
+      <c r="F10" s="44" t="n"/>
+      <c r="G10" s="44" t="n"/>
+      <c r="H10" s="44" t="n"/>
+      <c r="I10" s="44" t="n"/>
+      <c r="J10" s="44" t="n"/>
+      <c r="K10" s="44" t="n"/>
+      <c r="L10" s="45">
+        <f>IF(COUNT(F10:K10)=0,"",IFERROR(SUMPRODUCT(F10:K10,(F$5:K$5+(F$5:K$5="")))/SUMPRODUCT((F10:K10&lt;&gt;"")*(F$5:K$5+(F$5:K$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="M10" s="44" t="n"/>
+      <c r="N10" s="44" t="n"/>
+      <c r="O10" s="44" t="n"/>
+      <c r="P10" s="45">
+        <f>IF(COUNT(M10:O10)=0,"",IFERROR(SUMPRODUCT(M10:O10,(M$5:O$5+(M$5:O$5="")))/SUMPRODUCT((M10:O10&lt;&gt;"")*(M$5:O$5+(M$5:O$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="Q10" s="44" t="n"/>
+      <c r="R10" s="44" t="n"/>
+      <c r="S10" s="44" t="n"/>
+      <c r="T10" s="44" t="n"/>
+      <c r="U10" s="45">
+        <f>IF(COUNT(Q10:T10)=0,"",IFERROR(SUMPRODUCT(Q10:T10,(Q$5:T$5+(Q$5:T$5="")))/SUMPRODUCT((Q10:T10&lt;&gt;"")*(Q$5:T$5+(Q$5:T$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="V10" s="44" t="n"/>
+      <c r="W10" s="44" t="n"/>
+      <c r="X10" s="45">
+        <f>IF(COUNT(V10:W10)=0,"",IFERROR(SUMPRODUCT(V10:W10,(V$5:W$5+(V$5:W$5="")))/SUMPRODUCT((V10:W10&lt;&gt;"")*(V$5:W$5+(V$5:W$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="Y10" s="45">
+        <f>IFERROR(IF((ISNUMBER(P10)*(P$5+(P$5=""))+ISNUMBER(U10)*(U$5+(U$5=""))+ISNUMBER(X10)*(X$5+(X$5="")))=0,"",(N(P10)*(P$5+(P$5=""))+N(U10)*(U$5+(U$5=""))+N(X10)*(X$5+(X$5="")))/(ISNUMBER(P10)*(P$5+(P$5=""))+ISNUMBER(U10)*(U$5+(U$5=""))+ISNUMBER(X10)*(X$5+(X$5="")))),"")</f>
+        <v/>
+      </c>
+      <c r="Z10" s="46">
+        <f>IF(AND(ISNUMBER(L10),ISNUMBER(Y10)),L10*Y10,"")</f>
+        <v/>
+      </c>
+      <c r="AA10" s="47">
+        <f>IF(ISNUMBER(Z10),(Z10-1)/24,"")</f>
+        <v/>
+      </c>
+      <c r="AB10" s="48">
+        <f>IF(ISNUMBER(Z10),COUNTIF(Z$7:Z$27,"&gt;"&amp;Z10)+1,"")</f>
+        <v/>
+      </c>
+      <c r="AC10" s="49">
+        <f>COUNT(F10,G10,H10,I10,J10,K10,M10,N10,O10,Q10,R10,S10,T10,V10,W10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="42" t="n">
+        <v>9</v>
+      </c>
+      <c r="B11" s="42" t="inlineStr">
+        <is>
+          <t>Imbiribeira</t>
+        </is>
+      </c>
+      <c r="C11" s="43" t="inlineStr">
+        <is>
+          <t>Avenida Mascarenhas de Moraes (Da Rua General Mac Arthur até a Universo)</t>
+        </is>
+      </c>
+      <c r="D11" s="42" t="inlineStr">
+        <is>
+          <t>Linha</t>
+        </is>
+      </c>
+      <c r="E11" s="42" t="inlineStr">
+        <is>
+          <t>G3</t>
+        </is>
+      </c>
+      <c r="F11" s="44" t="n"/>
+      <c r="G11" s="44" t="n"/>
+      <c r="H11" s="44" t="n"/>
+      <c r="I11" s="44" t="n"/>
+      <c r="J11" s="44" t="n"/>
+      <c r="K11" s="44" t="n"/>
+      <c r="L11" s="45">
+        <f>IF(COUNT(F11:K11)=0,"",IFERROR(SUMPRODUCT(F11:K11,(F$5:K$5+(F$5:K$5="")))/SUMPRODUCT((F11:K11&lt;&gt;"")*(F$5:K$5+(F$5:K$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="M11" s="44" t="n"/>
+      <c r="N11" s="44" t="n"/>
+      <c r="O11" s="44" t="n"/>
+      <c r="P11" s="45">
+        <f>IF(COUNT(M11:O11)=0,"",IFERROR(SUMPRODUCT(M11:O11,(M$5:O$5+(M$5:O$5="")))/SUMPRODUCT((M11:O11&lt;&gt;"")*(M$5:O$5+(M$5:O$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="Q11" s="44" t="n"/>
+      <c r="R11" s="44" t="n"/>
+      <c r="S11" s="44" t="n"/>
+      <c r="T11" s="44" t="n"/>
+      <c r="U11" s="45">
+        <f>IF(COUNT(Q11:T11)=0,"",IFERROR(SUMPRODUCT(Q11:T11,(Q$5:T$5+(Q$5:T$5="")))/SUMPRODUCT((Q11:T11&lt;&gt;"")*(Q$5:T$5+(Q$5:T$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="V11" s="44" t="n"/>
+      <c r="W11" s="44" t="n"/>
+      <c r="X11" s="45">
+        <f>IF(COUNT(V11:W11)=0,"",IFERROR(SUMPRODUCT(V11:W11,(V$5:W$5+(V$5:W$5="")))/SUMPRODUCT((V11:W11&lt;&gt;"")*(V$5:W$5+(V$5:W$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="Y11" s="45">
+        <f>IFERROR(IF((ISNUMBER(P11)*(P$5+(P$5=""))+ISNUMBER(U11)*(U$5+(U$5=""))+ISNUMBER(X11)*(X$5+(X$5="")))=0,"",(N(P11)*(P$5+(P$5=""))+N(U11)*(U$5+(U$5=""))+N(X11)*(X$5+(X$5="")))/(ISNUMBER(P11)*(P$5+(P$5=""))+ISNUMBER(U11)*(U$5+(U$5=""))+ISNUMBER(X11)*(X$5+(X$5="")))),"")</f>
+        <v/>
+      </c>
+      <c r="Z11" s="46">
+        <f>IF(AND(ISNUMBER(L11),ISNUMBER(Y11)),L11*Y11,"")</f>
+        <v/>
+      </c>
+      <c r="AA11" s="47">
+        <f>IF(ISNUMBER(Z11),(Z11-1)/24,"")</f>
+        <v/>
+      </c>
+      <c r="AB11" s="48">
+        <f>IF(ISNUMBER(Z11),COUNTIF(Z$7:Z$27,"&gt;"&amp;Z11)+1,"")</f>
+        <v/>
+      </c>
+      <c r="AC11" s="49">
+        <f>COUNT(F11,G11,H11,I11,J11,K11,M11,N11,O11,Q11,R11,S11,T11,V11,W11)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="42" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="42" t="inlineStr">
+        <is>
+          <t>Boa Viagem</t>
+        </is>
+      </c>
+      <c r="C12" s="43" t="inlineStr">
+        <is>
+          <t>Rua Professor José Brandão (Toda a extensão)</t>
+        </is>
+      </c>
+      <c r="D12" s="42" t="inlineStr">
+        <is>
+          <t>Linha</t>
+        </is>
+      </c>
+      <c r="E12" s="42" t="inlineStr">
+        <is>
+          <t>G1</t>
+        </is>
+      </c>
+      <c r="F12" s="44" t="n"/>
+      <c r="G12" s="44" t="n"/>
+      <c r="H12" s="44" t="n"/>
+      <c r="I12" s="44" t="n"/>
+      <c r="J12" s="44" t="n"/>
+      <c r="K12" s="44" t="n"/>
+      <c r="L12" s="45">
+        <f>IF(COUNT(F12:K12)=0,"",IFERROR(SUMPRODUCT(F12:K12,(F$5:K$5+(F$5:K$5="")))/SUMPRODUCT((F12:K12&lt;&gt;"")*(F$5:K$5+(F$5:K$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="M12" s="44" t="n"/>
+      <c r="N12" s="44" t="n"/>
+      <c r="O12" s="44" t="n"/>
+      <c r="P12" s="45">
+        <f>IF(COUNT(M12:O12)=0,"",IFERROR(SUMPRODUCT(M12:O12,(M$5:O$5+(M$5:O$5="")))/SUMPRODUCT((M12:O12&lt;&gt;"")*(M$5:O$5+(M$5:O$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="Q12" s="44" t="n"/>
+      <c r="R12" s="44" t="n"/>
+      <c r="S12" s="44" t="n"/>
+      <c r="T12" s="44" t="n"/>
+      <c r="U12" s="45">
+        <f>IF(COUNT(Q12:T12)=0,"",IFERROR(SUMPRODUCT(Q12:T12,(Q$5:T$5+(Q$5:T$5="")))/SUMPRODUCT((Q12:T12&lt;&gt;"")*(Q$5:T$5+(Q$5:T$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="V12" s="44" t="n"/>
+      <c r="W12" s="44" t="n"/>
+      <c r="X12" s="45">
+        <f>IF(COUNT(V12:W12)=0,"",IFERROR(SUMPRODUCT(V12:W12,(V$5:W$5+(V$5:W$5="")))/SUMPRODUCT((V12:W12&lt;&gt;"")*(V$5:W$5+(V$5:W$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="Y12" s="45">
+        <f>IFERROR(IF((ISNUMBER(P12)*(P$5+(P$5=""))+ISNUMBER(U12)*(U$5+(U$5=""))+ISNUMBER(X12)*(X$5+(X$5="")))=0,"",(N(P12)*(P$5+(P$5=""))+N(U12)*(U$5+(U$5=""))+N(X12)*(X$5+(X$5="")))/(ISNUMBER(P12)*(P$5+(P$5=""))+ISNUMBER(U12)*(U$5+(U$5=""))+ISNUMBER(X12)*(X$5+(X$5="")))),"")</f>
+        <v/>
+      </c>
+      <c r="Z12" s="46">
+        <f>IF(AND(ISNUMBER(L12),ISNUMBER(Y12)),L12*Y12,"")</f>
+        <v/>
+      </c>
+      <c r="AA12" s="47">
+        <f>IF(ISNUMBER(Z12),(Z12-1)/24,"")</f>
+        <v/>
+      </c>
+      <c r="AB12" s="48">
+        <f>IF(ISNUMBER(Z12),COUNTIF(Z$7:Z$27,"&gt;"&amp;Z12)+1,"")</f>
+        <v/>
+      </c>
+      <c r="AC12" s="49">
+        <f>COUNT(F12,G12,H12,I12,J12,K12,M12,N12,O12,Q12,R12,S12,T12,V12,W12)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="42" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="42" t="inlineStr">
+        <is>
+          <t>Boa Viagem</t>
+        </is>
+      </c>
+      <c r="C13" s="43" t="inlineStr">
+        <is>
+          <t>Rua Padre Bernardino Pessoa (Da Avenida Conselheiro Aguiar até a Via Mangue)</t>
+        </is>
+      </c>
+      <c r="D13" s="42" t="inlineStr">
+        <is>
+          <t>Linha</t>
+        </is>
+      </c>
+      <c r="E13" s="42" t="inlineStr">
+        <is>
+          <t>G1</t>
+        </is>
+      </c>
+      <c r="F13" s="44" t="n"/>
+      <c r="G13" s="44" t="n"/>
+      <c r="H13" s="44" t="n"/>
+      <c r="I13" s="44" t="n"/>
+      <c r="J13" s="44" t="n"/>
+      <c r="K13" s="44" t="n"/>
+      <c r="L13" s="45">
+        <f>IF(COUNT(F13:K13)=0,"",IFERROR(SUMPRODUCT(F13:K13,(F$5:K$5+(F$5:K$5="")))/SUMPRODUCT((F13:K13&lt;&gt;"")*(F$5:K$5+(F$5:K$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="M13" s="44" t="n"/>
+      <c r="N13" s="44" t="n"/>
+      <c r="O13" s="44" t="n"/>
+      <c r="P13" s="45">
+        <f>IF(COUNT(M13:O13)=0,"",IFERROR(SUMPRODUCT(M13:O13,(M$5:O$5+(M$5:O$5="")))/SUMPRODUCT((M13:O13&lt;&gt;"")*(M$5:O$5+(M$5:O$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="Q13" s="44" t="n"/>
+      <c r="R13" s="44" t="n"/>
+      <c r="S13" s="44" t="n"/>
+      <c r="T13" s="44" t="n"/>
+      <c r="U13" s="45">
+        <f>IF(COUNT(Q13:T13)=0,"",IFERROR(SUMPRODUCT(Q13:T13,(Q$5:T$5+(Q$5:T$5="")))/SUMPRODUCT((Q13:T13&lt;&gt;"")*(Q$5:T$5+(Q$5:T$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="V13" s="44" t="n"/>
+      <c r="W13" s="44" t="n"/>
+      <c r="X13" s="45">
+        <f>IF(COUNT(V13:W13)=0,"",IFERROR(SUMPRODUCT(V13:W13,(V$5:W$5+(V$5:W$5="")))/SUMPRODUCT((V13:W13&lt;&gt;"")*(V$5:W$5+(V$5:W$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="Y13" s="45">
+        <f>IFERROR(IF((ISNUMBER(P13)*(P$5+(P$5=""))+ISNUMBER(U13)*(U$5+(U$5=""))+ISNUMBER(X13)*(X$5+(X$5="")))=0,"",(N(P13)*(P$5+(P$5=""))+N(U13)*(U$5+(U$5=""))+N(X13)*(X$5+(X$5="")))/(ISNUMBER(P13)*(P$5+(P$5=""))+ISNUMBER(U13)*(U$5+(U$5=""))+ISNUMBER(X13)*(X$5+(X$5="")))),"")</f>
+        <v/>
+      </c>
+      <c r="Z13" s="46">
+        <f>IF(AND(ISNUMBER(L13),ISNUMBER(Y13)),L13*Y13,"")</f>
+        <v/>
+      </c>
+      <c r="AA13" s="47">
+        <f>IF(ISNUMBER(Z13),(Z13-1)/24,"")</f>
+        <v/>
+      </c>
+      <c r="AB13" s="48">
+        <f>IF(ISNUMBER(Z13),COUNTIF(Z$7:Z$27,"&gt;"&amp;Z13)+1,"")</f>
+        <v/>
+      </c>
+      <c r="AC13" s="49">
+        <f>COUNT(F13,G13,H13,I13,J13,K13,M13,N13,O13,Q13,R13,S13,T13,V13,W13)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="42" t="n">
+        <v>18</v>
+      </c>
+      <c r="B14" s="42" t="inlineStr">
+        <is>
+          <t>Boa Viagem</t>
+        </is>
+      </c>
+      <c r="C14" s="43" t="inlineStr">
+        <is>
+          <t>Rua Jornalista Alfredo Porto Silveira (Toda a extensão)</t>
+        </is>
+      </c>
+      <c r="D14" s="42" t="inlineStr">
+        <is>
+          <t>Linha</t>
+        </is>
+      </c>
+      <c r="E14" s="42" t="inlineStr"/>
+      <c r="F14" s="44" t="n"/>
+      <c r="G14" s="44" t="n"/>
+      <c r="H14" s="44" t="n"/>
+      <c r="I14" s="44" t="n"/>
+      <c r="J14" s="44" t="n"/>
+      <c r="K14" s="44" t="n"/>
+      <c r="L14" s="45">
+        <f>IF(COUNT(F14:K14)=0,"",IFERROR(SUMPRODUCT(F14:K14,(F$5:K$5+(F$5:K$5="")))/SUMPRODUCT((F14:K14&lt;&gt;"")*(F$5:K$5+(F$5:K$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="M14" s="44" t="n"/>
+      <c r="N14" s="44" t="n"/>
+      <c r="O14" s="44" t="n"/>
+      <c r="P14" s="45">
+        <f>IF(COUNT(M14:O14)=0,"",IFERROR(SUMPRODUCT(M14:O14,(M$5:O$5+(M$5:O$5="")))/SUMPRODUCT((M14:O14&lt;&gt;"")*(M$5:O$5+(M$5:O$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="Q14" s="44" t="n"/>
+      <c r="R14" s="44" t="n"/>
+      <c r="S14" s="44" t="n"/>
+      <c r="T14" s="44" t="n"/>
+      <c r="U14" s="45">
+        <f>IF(COUNT(Q14:T14)=0,"",IFERROR(SUMPRODUCT(Q14:T14,(Q$5:T$5+(Q$5:T$5="")))/SUMPRODUCT((Q14:T14&lt;&gt;"")*(Q$5:T$5+(Q$5:T$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="V14" s="44" t="n"/>
+      <c r="W14" s="44" t="n"/>
+      <c r="X14" s="45">
+        <f>IF(COUNT(V14:W14)=0,"",IFERROR(SUMPRODUCT(V14:W14,(V$5:W$5+(V$5:W$5="")))/SUMPRODUCT((V14:W14&lt;&gt;"")*(V$5:W$5+(V$5:W$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="Y14" s="45">
+        <f>IFERROR(IF((ISNUMBER(P14)*(P$5+(P$5=""))+ISNUMBER(U14)*(U$5+(U$5=""))+ISNUMBER(X14)*(X$5+(X$5="")))=0,"",(N(P14)*(P$5+(P$5=""))+N(U14)*(U$5+(U$5=""))+N(X14)*(X$5+(X$5="")))/(ISNUMBER(P14)*(P$5+(P$5=""))+ISNUMBER(U14)*(U$5+(U$5=""))+ISNUMBER(X14)*(X$5+(X$5="")))),"")</f>
+        <v/>
+      </c>
+      <c r="Z14" s="46">
+        <f>IF(AND(ISNUMBER(L14),ISNUMBER(Y14)),L14*Y14,"")</f>
+        <v/>
+      </c>
+      <c r="AA14" s="47">
+        <f>IF(ISNUMBER(Z14),(Z14-1)/24,"")</f>
+        <v/>
+      </c>
+      <c r="AB14" s="48">
+        <f>IF(ISNUMBER(Z14),COUNTIF(Z$7:Z$27,"&gt;"&amp;Z14)+1,"")</f>
+        <v/>
+      </c>
+      <c r="AC14" s="49">
+        <f>COUNT(F14,G14,H14,I14,J14,K14,M14,N14,O14,Q14,R14,S14,T14,V14,W14)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="42" t="n">
+        <v>19</v>
+      </c>
+      <c r="B15" s="42" t="inlineStr">
+        <is>
+          <t>Pina</t>
+        </is>
+      </c>
+      <c r="C15" s="43" t="inlineStr">
+        <is>
+          <t>Rua São Luiz (Final da rua)</t>
+        </is>
+      </c>
+      <c r="D15" s="42" t="inlineStr">
+        <is>
+          <t>Ponto</t>
+        </is>
+      </c>
+      <c r="E15" s="42" t="inlineStr"/>
+      <c r="F15" s="44" t="n"/>
+      <c r="G15" s="44" t="n"/>
+      <c r="H15" s="44" t="n"/>
+      <c r="I15" s="44" t="n"/>
+      <c r="J15" s="44" t="n"/>
+      <c r="K15" s="44" t="n"/>
+      <c r="L15" s="45">
+        <f>IF(COUNT(F15:K15)=0,"",IFERROR(SUMPRODUCT(F15:K15,(F$5:K$5+(F$5:K$5="")))/SUMPRODUCT((F15:K15&lt;&gt;"")*(F$5:K$5+(F$5:K$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="M15" s="44" t="n"/>
+      <c r="N15" s="44" t="n"/>
+      <c r="O15" s="44" t="n"/>
+      <c r="P15" s="45">
+        <f>IF(COUNT(M15:O15)=0,"",IFERROR(SUMPRODUCT(M15:O15,(M$5:O$5+(M$5:O$5="")))/SUMPRODUCT((M15:O15&lt;&gt;"")*(M$5:O$5+(M$5:O$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="Q15" s="44" t="n"/>
+      <c r="R15" s="44" t="n"/>
+      <c r="S15" s="44" t="n"/>
+      <c r="T15" s="44" t="n"/>
+      <c r="U15" s="45">
+        <f>IF(COUNT(Q15:T15)=0,"",IFERROR(SUMPRODUCT(Q15:T15,(Q$5:T$5+(Q$5:T$5="")))/SUMPRODUCT((Q15:T15&lt;&gt;"")*(Q$5:T$5+(Q$5:T$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="V15" s="44" t="n"/>
+      <c r="W15" s="44" t="n"/>
+      <c r="X15" s="45">
+        <f>IF(COUNT(V15:W15)=0,"",IFERROR(SUMPRODUCT(V15:W15,(V$5:W$5+(V$5:W$5="")))/SUMPRODUCT((V15:W15&lt;&gt;"")*(V$5:W$5+(V$5:W$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="Y15" s="45">
+        <f>IFERROR(IF((ISNUMBER(P15)*(P$5+(P$5=""))+ISNUMBER(U15)*(U$5+(U$5=""))+ISNUMBER(X15)*(X$5+(X$5="")))=0,"",(N(P15)*(P$5+(P$5=""))+N(U15)*(U$5+(U$5=""))+N(X15)*(X$5+(X$5="")))/(ISNUMBER(P15)*(P$5+(P$5=""))+ISNUMBER(U15)*(U$5+(U$5=""))+ISNUMBER(X15)*(X$5+(X$5="")))),"")</f>
+        <v/>
+      </c>
+      <c r="Z15" s="46">
+        <f>IF(AND(ISNUMBER(L15),ISNUMBER(Y15)),L15*Y15,"")</f>
+        <v/>
+      </c>
+      <c r="AA15" s="47">
+        <f>IF(ISNUMBER(Z15),(Z15-1)/24,"")</f>
+        <v/>
+      </c>
+      <c r="AB15" s="48">
+        <f>IF(ISNUMBER(Z15),COUNTIF(Z$7:Z$27,"&gt;"&amp;Z15)+1,"")</f>
+        <v/>
+      </c>
+      <c r="AC15" s="49">
+        <f>COUNT(F15,G15,H15,I15,J15,K15,M15,N15,O15,Q15,R15,S15,T15,V15,W15)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="42" t="n">
+        <v>22</v>
+      </c>
+      <c r="B16" s="42" t="inlineStr">
+        <is>
+          <t>Jordão</t>
+        </is>
+      </c>
+      <c r="C16" s="43" t="inlineStr">
+        <is>
+          <t>Avenida Maria Irene (Vários trechos)</t>
+        </is>
+      </c>
+      <c r="D16" s="42" t="inlineStr">
+        <is>
+          <t>Vários</t>
+        </is>
+      </c>
+      <c r="E16" s="42" t="inlineStr"/>
+      <c r="F16" s="44" t="n"/>
+      <c r="G16" s="44" t="n"/>
+      <c r="H16" s="44" t="n"/>
+      <c r="I16" s="44" t="n"/>
+      <c r="J16" s="44" t="n"/>
+      <c r="K16" s="44" t="n"/>
+      <c r="L16" s="45">
+        <f>IF(COUNT(F16:K16)=0,"",IFERROR(SUMPRODUCT(F16:K16,(F$5:K$5+(F$5:K$5="")))/SUMPRODUCT((F16:K16&lt;&gt;"")*(F$5:K$5+(F$5:K$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="M16" s="44" t="n"/>
+      <c r="N16" s="44" t="n"/>
+      <c r="O16" s="44" t="n"/>
+      <c r="P16" s="45">
+        <f>IF(COUNT(M16:O16)=0,"",IFERROR(SUMPRODUCT(M16:O16,(M$5:O$5+(M$5:O$5="")))/SUMPRODUCT((M16:O16&lt;&gt;"")*(M$5:O$5+(M$5:O$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="Q16" s="44" t="n"/>
+      <c r="R16" s="44" t="n"/>
+      <c r="S16" s="44" t="n"/>
+      <c r="T16" s="44" t="n"/>
+      <c r="U16" s="45">
+        <f>IF(COUNT(Q16:T16)=0,"",IFERROR(SUMPRODUCT(Q16:T16,(Q$5:T$5+(Q$5:T$5="")))/SUMPRODUCT((Q16:T16&lt;&gt;"")*(Q$5:T$5+(Q$5:T$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="V16" s="44" t="n"/>
+      <c r="W16" s="44" t="n"/>
+      <c r="X16" s="45">
+        <f>IF(COUNT(V16:W16)=0,"",IFERROR(SUMPRODUCT(V16:W16,(V$5:W$5+(V$5:W$5="")))/SUMPRODUCT((V16:W16&lt;&gt;"")*(V$5:W$5+(V$5:W$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="Y16" s="45">
+        <f>IFERROR(IF((ISNUMBER(P16)*(P$5+(P$5=""))+ISNUMBER(U16)*(U$5+(U$5=""))+ISNUMBER(X16)*(X$5+(X$5="")))=0,"",(N(P16)*(P$5+(P$5=""))+N(U16)*(U$5+(U$5=""))+N(X16)*(X$5+(X$5="")))/(ISNUMBER(P16)*(P$5+(P$5=""))+ISNUMBER(U16)*(U$5+(U$5=""))+ISNUMBER(X16)*(X$5+(X$5="")))),"")</f>
+        <v/>
+      </c>
+      <c r="Z16" s="46">
+        <f>IF(AND(ISNUMBER(L16),ISNUMBER(Y16)),L16*Y16,"")</f>
+        <v/>
+      </c>
+      <c r="AA16" s="47">
+        <f>IF(ISNUMBER(Z16),(Z16-1)/24,"")</f>
+        <v/>
+      </c>
+      <c r="AB16" s="48">
+        <f>IF(ISNUMBER(Z16),COUNTIF(Z$7:Z$27,"&gt;"&amp;Z16)+1,"")</f>
+        <v/>
+      </c>
+      <c r="AC16" s="49">
+        <f>COUNT(F16,G16,H16,I16,J16,K16,M16,N16,O16,Q16,R16,S16,T16,V16,W16)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="42" t="n">
+        <v>24</v>
+      </c>
+      <c r="B17" s="42" t="inlineStr">
+        <is>
+          <t>Ipsep</t>
+        </is>
+      </c>
+      <c r="C17" s="43" t="inlineStr">
+        <is>
+          <t>Rua Blumenau (Até a maré)</t>
+        </is>
+      </c>
+      <c r="D17" s="42" t="inlineStr">
+        <is>
+          <t>Linha</t>
+        </is>
+      </c>
+      <c r="E17" s="42" t="inlineStr"/>
+      <c r="F17" s="44" t="n"/>
+      <c r="G17" s="44" t="n"/>
+      <c r="H17" s="44" t="n"/>
+      <c r="I17" s="44" t="n"/>
+      <c r="J17" s="44" t="n"/>
+      <c r="K17" s="44" t="n"/>
+      <c r="L17" s="45">
+        <f>IF(COUNT(F17:K17)=0,"",IFERROR(SUMPRODUCT(F17:K17,(F$5:K$5+(F$5:K$5="")))/SUMPRODUCT((F17:K17&lt;&gt;"")*(F$5:K$5+(F$5:K$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="M17" s="44" t="n"/>
+      <c r="N17" s="44" t="n"/>
+      <c r="O17" s="44" t="n"/>
+      <c r="P17" s="45">
+        <f>IF(COUNT(M17:O17)=0,"",IFERROR(SUMPRODUCT(M17:O17,(M$5:O$5+(M$5:O$5="")))/SUMPRODUCT((M17:O17&lt;&gt;"")*(M$5:O$5+(M$5:O$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="Q17" s="44" t="n"/>
+      <c r="R17" s="44" t="n"/>
+      <c r="S17" s="44" t="n"/>
+      <c r="T17" s="44" t="n"/>
+      <c r="U17" s="45">
+        <f>IF(COUNT(Q17:T17)=0,"",IFERROR(SUMPRODUCT(Q17:T17,(Q$5:T$5+(Q$5:T$5="")))/SUMPRODUCT((Q17:T17&lt;&gt;"")*(Q$5:T$5+(Q$5:T$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="V17" s="44" t="n"/>
+      <c r="W17" s="44" t="n"/>
+      <c r="X17" s="45">
+        <f>IF(COUNT(V17:W17)=0,"",IFERROR(SUMPRODUCT(V17:W17,(V$5:W$5+(V$5:W$5="")))/SUMPRODUCT((V17:W17&lt;&gt;"")*(V$5:W$5+(V$5:W$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="Y17" s="45">
+        <f>IFERROR(IF((ISNUMBER(P17)*(P$5+(P$5=""))+ISNUMBER(U17)*(U$5+(U$5=""))+ISNUMBER(X17)*(X$5+(X$5="")))=0,"",(N(P17)*(P$5+(P$5=""))+N(U17)*(U$5+(U$5=""))+N(X17)*(X$5+(X$5="")))/(ISNUMBER(P17)*(P$5+(P$5=""))+ISNUMBER(U17)*(U$5+(U$5=""))+ISNUMBER(X17)*(X$5+(X$5="")))),"")</f>
+        <v/>
+      </c>
+      <c r="Z17" s="46">
+        <f>IF(AND(ISNUMBER(L17),ISNUMBER(Y17)),L17*Y17,"")</f>
+        <v/>
+      </c>
+      <c r="AA17" s="47">
+        <f>IF(ISNUMBER(Z17),(Z17-1)/24,"")</f>
+        <v/>
+      </c>
+      <c r="AB17" s="48">
+        <f>IF(ISNUMBER(Z17),COUNTIF(Z$7:Z$27,"&gt;"&amp;Z17)+1,"")</f>
+        <v/>
+      </c>
+      <c r="AC17" s="49">
+        <f>COUNT(F17,G17,H17,I17,J17,K17,M17,N17,O17,Q17,R17,S17,T17,V17,W17)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="42" t="n">
+        <v>25</v>
+      </c>
+      <c r="B18" s="42" t="inlineStr">
+        <is>
+          <t>Ipsep</t>
+        </is>
+      </c>
+      <c r="C18" s="43" t="inlineStr">
+        <is>
+          <t>Rua Raimundo Diniz (Vários trechos)</t>
+        </is>
+      </c>
+      <c r="D18" s="42" t="inlineStr">
+        <is>
+          <t>Vários</t>
+        </is>
+      </c>
+      <c r="E18" s="42" t="inlineStr"/>
+      <c r="F18" s="44" t="n"/>
+      <c r="G18" s="44" t="n"/>
+      <c r="H18" s="44" t="n"/>
+      <c r="I18" s="44" t="n"/>
+      <c r="J18" s="44" t="n"/>
+      <c r="K18" s="44" t="n"/>
+      <c r="L18" s="45">
+        <f>IF(COUNT(F18:K18)=0,"",IFERROR(SUMPRODUCT(F18:K18,(F$5:K$5+(F$5:K$5="")))/SUMPRODUCT((F18:K18&lt;&gt;"")*(F$5:K$5+(F$5:K$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="M18" s="44" t="n"/>
+      <c r="N18" s="44" t="n"/>
+      <c r="O18" s="44" t="n"/>
+      <c r="P18" s="45">
+        <f>IF(COUNT(M18:O18)=0,"",IFERROR(SUMPRODUCT(M18:O18,(M$5:O$5+(M$5:O$5="")))/SUMPRODUCT((M18:O18&lt;&gt;"")*(M$5:O$5+(M$5:O$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="Q18" s="44" t="n"/>
+      <c r="R18" s="44" t="n"/>
+      <c r="S18" s="44" t="n"/>
+      <c r="T18" s="44" t="n"/>
+      <c r="U18" s="45">
+        <f>IF(COUNT(Q18:T18)=0,"",IFERROR(SUMPRODUCT(Q18:T18,(Q$5:T$5+(Q$5:T$5="")))/SUMPRODUCT((Q18:T18&lt;&gt;"")*(Q$5:T$5+(Q$5:T$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="V18" s="44" t="n"/>
+      <c r="W18" s="44" t="n"/>
+      <c r="X18" s="45">
+        <f>IF(COUNT(V18:W18)=0,"",IFERROR(SUMPRODUCT(V18:W18,(V$5:W$5+(V$5:W$5="")))/SUMPRODUCT((V18:W18&lt;&gt;"")*(V$5:W$5+(V$5:W$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="Y18" s="45">
+        <f>IFERROR(IF((ISNUMBER(P18)*(P$5+(P$5=""))+ISNUMBER(U18)*(U$5+(U$5=""))+ISNUMBER(X18)*(X$5+(X$5="")))=0,"",(N(P18)*(P$5+(P$5=""))+N(U18)*(U$5+(U$5=""))+N(X18)*(X$5+(X$5="")))/(ISNUMBER(P18)*(P$5+(P$5=""))+ISNUMBER(U18)*(U$5+(U$5=""))+ISNUMBER(X18)*(X$5+(X$5="")))),"")</f>
+        <v/>
+      </c>
+      <c r="Z18" s="46">
+        <f>IF(AND(ISNUMBER(L18),ISNUMBER(Y18)),L18*Y18,"")</f>
+        <v/>
+      </c>
+      <c r="AA18" s="47">
+        <f>IF(ISNUMBER(Z18),(Z18-1)/24,"")</f>
+        <v/>
+      </c>
+      <c r="AB18" s="48">
+        <f>IF(ISNUMBER(Z18),COUNTIF(Z$7:Z$27,"&gt;"&amp;Z18)+1,"")</f>
+        <v/>
+      </c>
+      <c r="AC18" s="49">
+        <f>COUNT(F18,G18,H18,I18,J18,K18,M18,N18,O18,Q18,R18,S18,T18,V18,W18)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="42" t="n">
+        <v>26</v>
+      </c>
+      <c r="B19" s="42" t="inlineStr">
+        <is>
+          <t>Boa Viagem</t>
+        </is>
+      </c>
+      <c r="C19" s="43" t="inlineStr">
+        <is>
+          <t>Avenida Boa Viagem (Antes da Rua Baltazar Passos)</t>
+        </is>
+      </c>
+      <c r="D19" s="42" t="inlineStr">
+        <is>
+          <t>Ponto</t>
+        </is>
+      </c>
+      <c r="E19" s="42" t="inlineStr"/>
+      <c r="F19" s="44" t="n"/>
+      <c r="G19" s="44" t="n"/>
+      <c r="H19" s="44" t="n"/>
+      <c r="I19" s="44" t="n"/>
+      <c r="J19" s="44" t="n"/>
+      <c r="K19" s="44" t="n"/>
+      <c r="L19" s="45">
+        <f>IF(COUNT(F19:K19)=0,"",IFERROR(SUMPRODUCT(F19:K19,(F$5:K$5+(F$5:K$5="")))/SUMPRODUCT((F19:K19&lt;&gt;"")*(F$5:K$5+(F$5:K$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="M19" s="44" t="n"/>
+      <c r="N19" s="44" t="n"/>
+      <c r="O19" s="44" t="n"/>
+      <c r="P19" s="45">
+        <f>IF(COUNT(M19:O19)=0,"",IFERROR(SUMPRODUCT(M19:O19,(M$5:O$5+(M$5:O$5="")))/SUMPRODUCT((M19:O19&lt;&gt;"")*(M$5:O$5+(M$5:O$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="Q19" s="44" t="n"/>
+      <c r="R19" s="44" t="n"/>
+      <c r="S19" s="44" t="n"/>
+      <c r="T19" s="44" t="n"/>
+      <c r="U19" s="45">
+        <f>IF(COUNT(Q19:T19)=0,"",IFERROR(SUMPRODUCT(Q19:T19,(Q$5:T$5+(Q$5:T$5="")))/SUMPRODUCT((Q19:T19&lt;&gt;"")*(Q$5:T$5+(Q$5:T$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="V19" s="44" t="n"/>
+      <c r="W19" s="44" t="n"/>
+      <c r="X19" s="45">
+        <f>IF(COUNT(V19:W19)=0,"",IFERROR(SUMPRODUCT(V19:W19,(V$5:W$5+(V$5:W$5="")))/SUMPRODUCT((V19:W19&lt;&gt;"")*(V$5:W$5+(V$5:W$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="Y19" s="45">
+        <f>IFERROR(IF((ISNUMBER(P19)*(P$5+(P$5=""))+ISNUMBER(U19)*(U$5+(U$5=""))+ISNUMBER(X19)*(X$5+(X$5="")))=0,"",(N(P19)*(P$5+(P$5=""))+N(U19)*(U$5+(U$5=""))+N(X19)*(X$5+(X$5="")))/(ISNUMBER(P19)*(P$5+(P$5=""))+ISNUMBER(U19)*(U$5+(U$5=""))+ISNUMBER(X19)*(X$5+(X$5="")))),"")</f>
+        <v/>
+      </c>
+      <c r="Z19" s="46">
+        <f>IF(AND(ISNUMBER(L19),ISNUMBER(Y19)),L19*Y19,"")</f>
+        <v/>
+      </c>
+      <c r="AA19" s="47">
+        <f>IF(ISNUMBER(Z19),(Z19-1)/24,"")</f>
+        <v/>
+      </c>
+      <c r="AB19" s="48">
+        <f>IF(ISNUMBER(Z19),COUNTIF(Z$7:Z$27,"&gt;"&amp;Z19)+1,"")</f>
+        <v/>
+      </c>
+      <c r="AC19" s="49">
+        <f>COUNT(F19,G19,H19,I19,J19,K19,M19,N19,O19,Q19,R19,S19,T19,V19,W19)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="42" t="n">
+        <v>33</v>
+      </c>
+      <c r="B20" s="42" t="inlineStr">
+        <is>
+          <t>Ibura</t>
+        </is>
+      </c>
+      <c r="C20" s="43" t="inlineStr">
+        <is>
+          <t>Avenida Dois Rios (Interseção da Avenida Dois Rios com a Rua Rio Pajeú até a Rua Ecoporanga / interseção da Avenida Dois Rios com a Rua Rio Prado)</t>
+        </is>
+      </c>
+      <c r="D20" s="42" t="inlineStr">
+        <is>
+          <t>Linha</t>
+        </is>
+      </c>
+      <c r="E20" s="42" t="inlineStr">
+        <is>
+          <t>G4</t>
+        </is>
+      </c>
+      <c r="F20" s="44" t="n"/>
+      <c r="G20" s="44" t="n"/>
+      <c r="H20" s="44" t="n"/>
+      <c r="I20" s="44" t="n"/>
+      <c r="J20" s="44" t="n"/>
+      <c r="K20" s="44" t="n"/>
+      <c r="L20" s="45">
+        <f>IF(COUNT(F20:K20)=0,"",IFERROR(SUMPRODUCT(F20:K20,(F$5:K$5+(F$5:K$5="")))/SUMPRODUCT((F20:K20&lt;&gt;"")*(F$5:K$5+(F$5:K$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="M20" s="44" t="n"/>
+      <c r="N20" s="44" t="n"/>
+      <c r="O20" s="44" t="n"/>
+      <c r="P20" s="45">
+        <f>IF(COUNT(M20:O20)=0,"",IFERROR(SUMPRODUCT(M20:O20,(M$5:O$5+(M$5:O$5="")))/SUMPRODUCT((M20:O20&lt;&gt;"")*(M$5:O$5+(M$5:O$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="Q20" s="44" t="n"/>
+      <c r="R20" s="44" t="n"/>
+      <c r="S20" s="44" t="n"/>
+      <c r="T20" s="44" t="n"/>
+      <c r="U20" s="45">
+        <f>IF(COUNT(Q20:T20)=0,"",IFERROR(SUMPRODUCT(Q20:T20,(Q$5:T$5+(Q$5:T$5="")))/SUMPRODUCT((Q20:T20&lt;&gt;"")*(Q$5:T$5+(Q$5:T$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="V20" s="44" t="n"/>
+      <c r="W20" s="44" t="n"/>
+      <c r="X20" s="45">
+        <f>IF(COUNT(V20:W20)=0,"",IFERROR(SUMPRODUCT(V20:W20,(V$5:W$5+(V$5:W$5="")))/SUMPRODUCT((V20:W20&lt;&gt;"")*(V$5:W$5+(V$5:W$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="Y20" s="45">
+        <f>IFERROR(IF((ISNUMBER(P20)*(P$5+(P$5=""))+ISNUMBER(U20)*(U$5+(U$5=""))+ISNUMBER(X20)*(X$5+(X$5="")))=0,"",(N(P20)*(P$5+(P$5=""))+N(U20)*(U$5+(U$5=""))+N(X20)*(X$5+(X$5="")))/(ISNUMBER(P20)*(P$5+(P$5=""))+ISNUMBER(U20)*(U$5+(U$5=""))+ISNUMBER(X20)*(X$5+(X$5="")))),"")</f>
+        <v/>
+      </c>
+      <c r="Z20" s="46">
+        <f>IF(AND(ISNUMBER(L20),ISNUMBER(Y20)),L20*Y20,"")</f>
+        <v/>
+      </c>
+      <c r="AA20" s="47">
+        <f>IF(ISNUMBER(Z20),(Z20-1)/24,"")</f>
+        <v/>
+      </c>
+      <c r="AB20" s="48">
+        <f>IF(ISNUMBER(Z20),COUNTIF(Z$7:Z$27,"&gt;"&amp;Z20)+1,"")</f>
+        <v/>
+      </c>
+      <c r="AC20" s="49">
+        <f>COUNT(F20,G20,H20,I20,J20,K20,M20,N20,O20,Q20,R20,S20,T20,V20,W20)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="42" t="n">
+        <v>34</v>
+      </c>
+      <c r="B21" s="42" t="inlineStr">
+        <is>
+          <t>Ibura</t>
+        </is>
+      </c>
+      <c r="C21" s="43" t="inlineStr">
+        <is>
+          <t>Avenida Dom Helder Câmara (Interseção da Avenida Dom Helder Câmara com a Rua Achiles Amorim)</t>
+        </is>
+      </c>
+      <c r="D21" s="42" t="inlineStr">
+        <is>
+          <t>Ponto</t>
+        </is>
+      </c>
+      <c r="E21" s="42" t="inlineStr">
+        <is>
+          <t>G5</t>
+        </is>
+      </c>
+      <c r="F21" s="44" t="n"/>
+      <c r="G21" s="44" t="n"/>
+      <c r="H21" s="44" t="n"/>
+      <c r="I21" s="44" t="n"/>
+      <c r="J21" s="44" t="n"/>
+      <c r="K21" s="44" t="n"/>
+      <c r="L21" s="45">
+        <f>IF(COUNT(F21:K21)=0,"",IFERROR(SUMPRODUCT(F21:K21,(F$5:K$5+(F$5:K$5="")))/SUMPRODUCT((F21:K21&lt;&gt;"")*(F$5:K$5+(F$5:K$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="M21" s="44" t="n"/>
+      <c r="N21" s="44" t="n"/>
+      <c r="O21" s="44" t="n"/>
+      <c r="P21" s="45">
+        <f>IF(COUNT(M21:O21)=0,"",IFERROR(SUMPRODUCT(M21:O21,(M$5:O$5+(M$5:O$5="")))/SUMPRODUCT((M21:O21&lt;&gt;"")*(M$5:O$5+(M$5:O$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="Q21" s="44" t="n"/>
+      <c r="R21" s="44" t="n"/>
+      <c r="S21" s="44" t="n"/>
+      <c r="T21" s="44" t="n"/>
+      <c r="U21" s="45">
+        <f>IF(COUNT(Q21:T21)=0,"",IFERROR(SUMPRODUCT(Q21:T21,(Q$5:T$5+(Q$5:T$5="")))/SUMPRODUCT((Q21:T21&lt;&gt;"")*(Q$5:T$5+(Q$5:T$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="V21" s="44" t="n"/>
+      <c r="W21" s="44" t="n"/>
+      <c r="X21" s="45">
+        <f>IF(COUNT(V21:W21)=0,"",IFERROR(SUMPRODUCT(V21:W21,(V$5:W$5+(V$5:W$5="")))/SUMPRODUCT((V21:W21&lt;&gt;"")*(V$5:W$5+(V$5:W$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="Y21" s="45">
+        <f>IFERROR(IF((ISNUMBER(P21)*(P$5+(P$5=""))+ISNUMBER(U21)*(U$5+(U$5=""))+ISNUMBER(X21)*(X$5+(X$5="")))=0,"",(N(P21)*(P$5+(P$5=""))+N(U21)*(U$5+(U$5=""))+N(X21)*(X$5+(X$5="")))/(ISNUMBER(P21)*(P$5+(P$5=""))+ISNUMBER(U21)*(U$5+(U$5=""))+ISNUMBER(X21)*(X$5+(X$5="")))),"")</f>
+        <v/>
+      </c>
+      <c r="Z21" s="46">
+        <f>IF(AND(ISNUMBER(L21),ISNUMBER(Y21)),L21*Y21,"")</f>
+        <v/>
+      </c>
+      <c r="AA21" s="47">
+        <f>IF(ISNUMBER(Z21),(Z21-1)/24,"")</f>
+        <v/>
+      </c>
+      <c r="AB21" s="48">
+        <f>IF(ISNUMBER(Z21),COUNTIF(Z$7:Z$27,"&gt;"&amp;Z21)+1,"")</f>
+        <v/>
+      </c>
+      <c r="AC21" s="49">
+        <f>COUNT(F21,G21,H21,I21,J21,K21,M21,N21,O21,Q21,R21,S21,T21,V21,W21)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="42" t="n">
+        <v>35</v>
+      </c>
+      <c r="B22" s="42" t="inlineStr">
+        <is>
+          <t>Ibura</t>
+        </is>
+      </c>
+      <c r="C22" s="43" t="inlineStr">
+        <is>
+          <t>Avenida Dois Rios (Próximo ao SESI)</t>
+        </is>
+      </c>
+      <c r="D22" s="42" t="inlineStr">
+        <is>
+          <t>Ponto</t>
+        </is>
+      </c>
+      <c r="E22" s="42" t="inlineStr">
+        <is>
+          <t>G4</t>
+        </is>
+      </c>
+      <c r="F22" s="44" t="n"/>
+      <c r="G22" s="44" t="n"/>
+      <c r="H22" s="44" t="n"/>
+      <c r="I22" s="44" t="n"/>
+      <c r="J22" s="44" t="n"/>
+      <c r="K22" s="44" t="n"/>
+      <c r="L22" s="45">
+        <f>IF(COUNT(F22:K22)=0,"",IFERROR(SUMPRODUCT(F22:K22,(F$5:K$5+(F$5:K$5="")))/SUMPRODUCT((F22:K22&lt;&gt;"")*(F$5:K$5+(F$5:K$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="M22" s="44" t="n"/>
+      <c r="N22" s="44" t="n"/>
+      <c r="O22" s="44" t="n"/>
+      <c r="P22" s="45">
+        <f>IF(COUNT(M22:O22)=0,"",IFERROR(SUMPRODUCT(M22:O22,(M$5:O$5+(M$5:O$5="")))/SUMPRODUCT((M22:O22&lt;&gt;"")*(M$5:O$5+(M$5:O$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="Q22" s="44" t="n"/>
+      <c r="R22" s="44" t="n"/>
+      <c r="S22" s="44" t="n"/>
+      <c r="T22" s="44" t="n"/>
+      <c r="U22" s="45">
+        <f>IF(COUNT(Q22:T22)=0,"",IFERROR(SUMPRODUCT(Q22:T22,(Q$5:T$5+(Q$5:T$5="")))/SUMPRODUCT((Q22:T22&lt;&gt;"")*(Q$5:T$5+(Q$5:T$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="V22" s="44" t="n"/>
+      <c r="W22" s="44" t="n"/>
+      <c r="X22" s="45">
+        <f>IF(COUNT(V22:W22)=0,"",IFERROR(SUMPRODUCT(V22:W22,(V$5:W$5+(V$5:W$5="")))/SUMPRODUCT((V22:W22&lt;&gt;"")*(V$5:W$5+(V$5:W$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="Y22" s="45">
+        <f>IFERROR(IF((ISNUMBER(P22)*(P$5+(P$5=""))+ISNUMBER(U22)*(U$5+(U$5=""))+ISNUMBER(X22)*(X$5+(X$5="")))=0,"",(N(P22)*(P$5+(P$5=""))+N(U22)*(U$5+(U$5=""))+N(X22)*(X$5+(X$5="")))/(ISNUMBER(P22)*(P$5+(P$5=""))+ISNUMBER(U22)*(U$5+(U$5=""))+ISNUMBER(X22)*(X$5+(X$5="")))),"")</f>
+        <v/>
+      </c>
+      <c r="Z22" s="46">
+        <f>IF(AND(ISNUMBER(L22),ISNUMBER(Y22)),L22*Y22,"")</f>
+        <v/>
+      </c>
+      <c r="AA22" s="47">
+        <f>IF(ISNUMBER(Z22),(Z22-1)/24,"")</f>
+        <v/>
+      </c>
+      <c r="AB22" s="48">
+        <f>IF(ISNUMBER(Z22),COUNTIF(Z$7:Z$27,"&gt;"&amp;Z22)+1,"")</f>
+        <v/>
+      </c>
+      <c r="AC22" s="49">
+        <f>COUNT(F22,G22,H22,I22,J22,K22,M22,N22,O22,Q22,R22,S22,T22,V22,W22)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="42" t="n">
+        <v>36</v>
+      </c>
+      <c r="B23" s="42" t="inlineStr">
+        <is>
+          <t>Imbiribeira</t>
+        </is>
+      </c>
+      <c r="C23" s="43" t="inlineStr">
+        <is>
+          <t>Avenida Mascarenhas de Moraes (Trecho da Ferreira Costa)</t>
+        </is>
+      </c>
+      <c r="D23" s="42" t="inlineStr">
+        <is>
+          <t>Ponto</t>
+        </is>
+      </c>
+      <c r="E23" s="42" t="inlineStr">
+        <is>
+          <t>G3</t>
+        </is>
+      </c>
+      <c r="F23" s="44" t="n"/>
+      <c r="G23" s="44" t="n"/>
+      <c r="H23" s="44" t="n"/>
+      <c r="I23" s="44" t="n"/>
+      <c r="J23" s="44" t="n"/>
+      <c r="K23" s="44" t="n"/>
+      <c r="L23" s="45">
+        <f>IF(COUNT(F23:K23)=0,"",IFERROR(SUMPRODUCT(F23:K23,(F$5:K$5+(F$5:K$5="")))/SUMPRODUCT((F23:K23&lt;&gt;"")*(F$5:K$5+(F$5:K$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="M23" s="44" t="n"/>
+      <c r="N23" s="44" t="n"/>
+      <c r="O23" s="44" t="n"/>
+      <c r="P23" s="45">
+        <f>IF(COUNT(M23:O23)=0,"",IFERROR(SUMPRODUCT(M23:O23,(M$5:O$5+(M$5:O$5="")))/SUMPRODUCT((M23:O23&lt;&gt;"")*(M$5:O$5+(M$5:O$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="Q23" s="44" t="n"/>
+      <c r="R23" s="44" t="n"/>
+      <c r="S23" s="44" t="n"/>
+      <c r="T23" s="44" t="n"/>
+      <c r="U23" s="45">
+        <f>IF(COUNT(Q23:T23)=0,"",IFERROR(SUMPRODUCT(Q23:T23,(Q$5:T$5+(Q$5:T$5="")))/SUMPRODUCT((Q23:T23&lt;&gt;"")*(Q$5:T$5+(Q$5:T$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="V23" s="44" t="n"/>
+      <c r="W23" s="44" t="n"/>
+      <c r="X23" s="45">
+        <f>IF(COUNT(V23:W23)=0,"",IFERROR(SUMPRODUCT(V23:W23,(V$5:W$5+(V$5:W$5="")))/SUMPRODUCT((V23:W23&lt;&gt;"")*(V$5:W$5+(V$5:W$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="Y23" s="45">
+        <f>IFERROR(IF((ISNUMBER(P23)*(P$5+(P$5=""))+ISNUMBER(U23)*(U$5+(U$5=""))+ISNUMBER(X23)*(X$5+(X$5="")))=0,"",(N(P23)*(P$5+(P$5=""))+N(U23)*(U$5+(U$5=""))+N(X23)*(X$5+(X$5="")))/(ISNUMBER(P23)*(P$5+(P$5=""))+ISNUMBER(U23)*(U$5+(U$5=""))+ISNUMBER(X23)*(X$5+(X$5="")))),"")</f>
+        <v/>
+      </c>
+      <c r="Z23" s="46">
+        <f>IF(AND(ISNUMBER(L23),ISNUMBER(Y23)),L23*Y23,"")</f>
+        <v/>
+      </c>
+      <c r="AA23" s="47">
+        <f>IF(ISNUMBER(Z23),(Z23-1)/24,"")</f>
+        <v/>
+      </c>
+      <c r="AB23" s="48">
+        <f>IF(ISNUMBER(Z23),COUNTIF(Z$7:Z$27,"&gt;"&amp;Z23)+1,"")</f>
+        <v/>
+      </c>
+      <c r="AC23" s="49">
+        <f>COUNT(F23,G23,H23,I23,J23,K23,M23,N23,O23,Q23,R23,S23,T23,V23,W23)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="42" t="n">
+        <v>37</v>
+      </c>
+      <c r="B24" s="42" t="inlineStr">
+        <is>
+          <t>Ipsep</t>
+        </is>
+      </c>
+      <c r="C24" s="43" t="inlineStr">
+        <is>
+          <t>Avenida Recife (Da Avenida Dom Helder Câmara até o Rio Tejipió)</t>
+        </is>
+      </c>
+      <c r="D24" s="42" t="inlineStr">
+        <is>
+          <t>Linha</t>
+        </is>
+      </c>
+      <c r="E24" s="42" t="inlineStr">
+        <is>
+          <t>G5</t>
+        </is>
+      </c>
+      <c r="F24" s="44" t="n"/>
+      <c r="G24" s="44" t="n"/>
+      <c r="H24" s="44" t="n"/>
+      <c r="I24" s="44" t="n"/>
+      <c r="J24" s="44" t="n"/>
+      <c r="K24" s="44" t="n"/>
+      <c r="L24" s="45">
+        <f>IF(COUNT(F24:K24)=0,"",IFERROR(SUMPRODUCT(F24:K24,(F$5:K$5+(F$5:K$5="")))/SUMPRODUCT((F24:K24&lt;&gt;"")*(F$5:K$5+(F$5:K$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="M24" s="44" t="n"/>
+      <c r="N24" s="44" t="n"/>
+      <c r="O24" s="44" t="n"/>
+      <c r="P24" s="45">
+        <f>IF(COUNT(M24:O24)=0,"",IFERROR(SUMPRODUCT(M24:O24,(M$5:O$5+(M$5:O$5="")))/SUMPRODUCT((M24:O24&lt;&gt;"")*(M$5:O$5+(M$5:O$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="Q24" s="44" t="n"/>
+      <c r="R24" s="44" t="n"/>
+      <c r="S24" s="44" t="n"/>
+      <c r="T24" s="44" t="n"/>
+      <c r="U24" s="45">
+        <f>IF(COUNT(Q24:T24)=0,"",IFERROR(SUMPRODUCT(Q24:T24,(Q$5:T$5+(Q$5:T$5="")))/SUMPRODUCT((Q24:T24&lt;&gt;"")*(Q$5:T$5+(Q$5:T$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="V24" s="44" t="n"/>
+      <c r="W24" s="44" t="n"/>
+      <c r="X24" s="45">
+        <f>IF(COUNT(V24:W24)=0,"",IFERROR(SUMPRODUCT(V24:W24,(V$5:W$5+(V$5:W$5="")))/SUMPRODUCT((V24:W24&lt;&gt;"")*(V$5:W$5+(V$5:W$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="Y24" s="45">
+        <f>IFERROR(IF((ISNUMBER(P24)*(P$5+(P$5=""))+ISNUMBER(U24)*(U$5+(U$5=""))+ISNUMBER(X24)*(X$5+(X$5="")))=0,"",(N(P24)*(P$5+(P$5=""))+N(U24)*(U$5+(U$5=""))+N(X24)*(X$5+(X$5="")))/(ISNUMBER(P24)*(P$5+(P$5=""))+ISNUMBER(U24)*(U$5+(U$5=""))+ISNUMBER(X24)*(X$5+(X$5="")))),"")</f>
+        <v/>
+      </c>
+      <c r="Z24" s="46">
+        <f>IF(AND(ISNUMBER(L24),ISNUMBER(Y24)),L24*Y24,"")</f>
+        <v/>
+      </c>
+      <c r="AA24" s="47">
+        <f>IF(ISNUMBER(Z24),(Z24-1)/24,"")</f>
+        <v/>
+      </c>
+      <c r="AB24" s="48">
+        <f>IF(ISNUMBER(Z24),COUNTIF(Z$7:Z$27,"&gt;"&amp;Z24)+1,"")</f>
+        <v/>
+      </c>
+      <c r="AC24" s="49">
+        <f>COUNT(F24,G24,H24,I24,J24,K24,M24,N24,O24,Q24,R24,S24,T24,V24,W24)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="42" t="n">
+        <v>41</v>
+      </c>
+      <c r="B25" s="42" t="inlineStr">
+        <is>
+          <t>Boa Viagem</t>
+        </is>
+      </c>
+      <c r="C25" s="43" t="inlineStr">
+        <is>
+          <t>Rua Thomé Gibson (Da Avenida Encanta Moça até a Via Mangue)</t>
+        </is>
+      </c>
+      <c r="D25" s="42" t="inlineStr">
+        <is>
+          <t>Linha</t>
+        </is>
+      </c>
+      <c r="E25" s="42" t="inlineStr">
+        <is>
+          <t>G2</t>
+        </is>
+      </c>
+      <c r="F25" s="44" t="n"/>
+      <c r="G25" s="44" t="n"/>
+      <c r="H25" s="44" t="n"/>
+      <c r="I25" s="44" t="n"/>
+      <c r="J25" s="44" t="n"/>
+      <c r="K25" s="44" t="n"/>
+      <c r="L25" s="45">
+        <f>IF(COUNT(F25:K25)=0,"",IFERROR(SUMPRODUCT(F25:K25,(F$5:K$5+(F$5:K$5="")))/SUMPRODUCT((F25:K25&lt;&gt;"")*(F$5:K$5+(F$5:K$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="M25" s="44" t="n"/>
+      <c r="N25" s="44" t="n"/>
+      <c r="O25" s="44" t="n"/>
+      <c r="P25" s="45">
+        <f>IF(COUNT(M25:O25)=0,"",IFERROR(SUMPRODUCT(M25:O25,(M$5:O$5+(M$5:O$5="")))/SUMPRODUCT((M25:O25&lt;&gt;"")*(M$5:O$5+(M$5:O$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="Q25" s="44" t="n"/>
+      <c r="R25" s="44" t="n"/>
+      <c r="S25" s="44" t="n"/>
+      <c r="T25" s="44" t="n"/>
+      <c r="U25" s="45">
+        <f>IF(COUNT(Q25:T25)=0,"",IFERROR(SUMPRODUCT(Q25:T25,(Q$5:T$5+(Q$5:T$5="")))/SUMPRODUCT((Q25:T25&lt;&gt;"")*(Q$5:T$5+(Q$5:T$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="V25" s="44" t="n"/>
+      <c r="W25" s="44" t="n"/>
+      <c r="X25" s="45">
+        <f>IF(COUNT(V25:W25)=0,"",IFERROR(SUMPRODUCT(V25:W25,(V$5:W$5+(V$5:W$5="")))/SUMPRODUCT((V25:W25&lt;&gt;"")*(V$5:W$5+(V$5:W$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="Y25" s="45">
+        <f>IFERROR(IF((ISNUMBER(P25)*(P$5+(P$5=""))+ISNUMBER(U25)*(U$5+(U$5=""))+ISNUMBER(X25)*(X$5+(X$5="")))=0,"",(N(P25)*(P$5+(P$5=""))+N(U25)*(U$5+(U$5=""))+N(X25)*(X$5+(X$5="")))/(ISNUMBER(P25)*(P$5+(P$5=""))+ISNUMBER(U25)*(U$5+(U$5=""))+ISNUMBER(X25)*(X$5+(X$5="")))),"")</f>
+        <v/>
+      </c>
+      <c r="Z25" s="46">
+        <f>IF(AND(ISNUMBER(L25),ISNUMBER(Y25)),L25*Y25,"")</f>
+        <v/>
+      </c>
+      <c r="AA25" s="47">
+        <f>IF(ISNUMBER(Z25),(Z25-1)/24,"")</f>
+        <v/>
+      </c>
+      <c r="AB25" s="48">
+        <f>IF(ISNUMBER(Z25),COUNTIF(Z$7:Z$27,"&gt;"&amp;Z25)+1,"")</f>
+        <v/>
+      </c>
+      <c r="AC25" s="49">
+        <f>COUNT(F25,G25,H25,I25,J25,K25,M25,N25,O25,Q25,R25,S25,T25,V25,W25)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="42" t="n">
+        <v>51</v>
+      </c>
+      <c r="B26" s="42" t="inlineStr">
+        <is>
+          <t>Pina</t>
+        </is>
+      </c>
+      <c r="C26" s="43" t="inlineStr">
+        <is>
+          <t>Avenida Antônio de Góes (Da saída da Via Mangue até a Bacia do Pina (Rio Capibaribe) e cruzamento com a Avenida Conselheiro Aguiar)</t>
+        </is>
+      </c>
+      <c r="D26" s="42" t="inlineStr">
+        <is>
+          <t>Linha</t>
+        </is>
+      </c>
+      <c r="E26" s="42" t="inlineStr"/>
+      <c r="F26" s="44" t="n"/>
+      <c r="G26" s="44" t="n"/>
+      <c r="H26" s="44" t="n"/>
+      <c r="I26" s="44" t="n"/>
+      <c r="J26" s="44" t="n"/>
+      <c r="K26" s="44" t="n"/>
+      <c r="L26" s="45">
+        <f>IF(COUNT(F26:K26)=0,"",IFERROR(SUMPRODUCT(F26:K26,(F$5:K$5+(F$5:K$5="")))/SUMPRODUCT((F26:K26&lt;&gt;"")*(F$5:K$5+(F$5:K$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="M26" s="44" t="n"/>
+      <c r="N26" s="44" t="n"/>
+      <c r="O26" s="44" t="n"/>
+      <c r="P26" s="45">
+        <f>IF(COUNT(M26:O26)=0,"",IFERROR(SUMPRODUCT(M26:O26,(M$5:O$5+(M$5:O$5="")))/SUMPRODUCT((M26:O26&lt;&gt;"")*(M$5:O$5+(M$5:O$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="Q26" s="44" t="n"/>
+      <c r="R26" s="44" t="n"/>
+      <c r="S26" s="44" t="n"/>
+      <c r="T26" s="44" t="n"/>
+      <c r="U26" s="45">
+        <f>IF(COUNT(Q26:T26)=0,"",IFERROR(SUMPRODUCT(Q26:T26,(Q$5:T$5+(Q$5:T$5="")))/SUMPRODUCT((Q26:T26&lt;&gt;"")*(Q$5:T$5+(Q$5:T$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="V26" s="44" t="n"/>
+      <c r="W26" s="44" t="n"/>
+      <c r="X26" s="45">
+        <f>IF(COUNT(V26:W26)=0,"",IFERROR(SUMPRODUCT(V26:W26,(V$5:W$5+(V$5:W$5="")))/SUMPRODUCT((V26:W26&lt;&gt;"")*(V$5:W$5+(V$5:W$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="Y26" s="45">
+        <f>IFERROR(IF((ISNUMBER(P26)*(P$5+(P$5=""))+ISNUMBER(U26)*(U$5+(U$5=""))+ISNUMBER(X26)*(X$5+(X$5="")))=0,"",(N(P26)*(P$5+(P$5=""))+N(U26)*(U$5+(U$5=""))+N(X26)*(X$5+(X$5="")))/(ISNUMBER(P26)*(P$5+(P$5=""))+ISNUMBER(U26)*(U$5+(U$5=""))+ISNUMBER(X26)*(X$5+(X$5="")))),"")</f>
+        <v/>
+      </c>
+      <c r="Z26" s="46">
+        <f>IF(AND(ISNUMBER(L26),ISNUMBER(Y26)),L26*Y26,"")</f>
+        <v/>
+      </c>
+      <c r="AA26" s="47">
+        <f>IF(ISNUMBER(Z26),(Z26-1)/24,"")</f>
+        <v/>
+      </c>
+      <c r="AB26" s="48">
+        <f>IF(ISNUMBER(Z26),COUNTIF(Z$7:Z$27,"&gt;"&amp;Z26)+1,"")</f>
+        <v/>
+      </c>
+      <c r="AC26" s="49">
+        <f>COUNT(F26,G26,H26,I26,J26,K26,M26,N26,O26,Q26,R26,S26,T26,V26,W26)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="42" t="n">
+        <v>54</v>
+      </c>
+      <c r="B27" s="42" t="inlineStr">
+        <is>
+          <t>Ibura</t>
+        </is>
+      </c>
+      <c r="C27" s="43" t="inlineStr">
+        <is>
+          <t>Rua Rio Prado (Interseção da Rua Rio Prado com a Rua Rio Brígida)</t>
+        </is>
+      </c>
+      <c r="D27" s="42" t="inlineStr">
+        <is>
+          <t>Ponto</t>
+        </is>
+      </c>
+      <c r="E27" s="42" t="inlineStr">
+        <is>
+          <t>G4</t>
+        </is>
+      </c>
+      <c r="F27" s="44" t="n"/>
+      <c r="G27" s="44" t="n"/>
+      <c r="H27" s="44" t="n"/>
+      <c r="I27" s="44" t="n"/>
+      <c r="J27" s="44" t="n"/>
+      <c r="K27" s="44" t="n"/>
+      <c r="L27" s="45">
+        <f>IF(COUNT(F27:K27)=0,"",IFERROR(SUMPRODUCT(F27:K27,(F$5:K$5+(F$5:K$5="")))/SUMPRODUCT((F27:K27&lt;&gt;"")*(F$5:K$5+(F$5:K$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="M27" s="44" t="n"/>
+      <c r="N27" s="44" t="n"/>
+      <c r="O27" s="44" t="n"/>
+      <c r="P27" s="45">
+        <f>IF(COUNT(M27:O27)=0,"",IFERROR(SUMPRODUCT(M27:O27,(M$5:O$5+(M$5:O$5="")))/SUMPRODUCT((M27:O27&lt;&gt;"")*(M$5:O$5+(M$5:O$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="Q27" s="44" t="n"/>
+      <c r="R27" s="44" t="n"/>
+      <c r="S27" s="44" t="n"/>
+      <c r="T27" s="44" t="n"/>
+      <c r="U27" s="45">
+        <f>IF(COUNT(Q27:T27)=0,"",IFERROR(SUMPRODUCT(Q27:T27,(Q$5:T$5+(Q$5:T$5="")))/SUMPRODUCT((Q27:T27&lt;&gt;"")*(Q$5:T$5+(Q$5:T$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="V27" s="44" t="n"/>
+      <c r="W27" s="44" t="n"/>
+      <c r="X27" s="45">
+        <f>IF(COUNT(V27:W27)=0,"",IFERROR(SUMPRODUCT(V27:W27,(V$5:W$5+(V$5:W$5="")))/SUMPRODUCT((V27:W27&lt;&gt;"")*(V$5:W$5+(V$5:W$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="Y27" s="45">
+        <f>IFERROR(IF((ISNUMBER(P27)*(P$5+(P$5=""))+ISNUMBER(U27)*(U$5+(U$5=""))+ISNUMBER(X27)*(X$5+(X$5="")))=0,"",(N(P27)*(P$5+(P$5=""))+N(U27)*(U$5+(U$5=""))+N(X27)*(X$5+(X$5="")))/(ISNUMBER(P27)*(P$5+(P$5=""))+ISNUMBER(U27)*(U$5+(U$5=""))+ISNUMBER(X27)*(X$5+(X$5="")))),"")</f>
+        <v/>
+      </c>
+      <c r="Z27" s="46">
+        <f>IF(AND(ISNUMBER(L27),ISNUMBER(Y27)),L27*Y27,"")</f>
+        <v/>
+      </c>
+      <c r="AA27" s="47">
+        <f>IF(ISNUMBER(Z27),(Z27-1)/24,"")</f>
+        <v/>
+      </c>
+      <c r="AB27" s="48">
+        <f>IF(ISNUMBER(Z27),COUNTIF(Z$7:Z$27,"&gt;"&amp;Z27)+1,"")</f>
+        <v/>
+      </c>
+      <c r="AC27" s="49">
+        <f>COUNT(F27,G27,H27,I27,J27,K27,M27,N27,O27,Q27,R27,S27,T27,V27,W27)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="21" t="inlineStr">
+        <is>
+          <t>Como o cálculo funciona:</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="50" t="inlineStr">
+        <is>
+          <t>• Nota do critério = média ponderada das notas dos subcritérios preenchidos (pesos da linha 5; vazio = 1).</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="50" t="inlineStr">
+        <is>
+          <t>• Consequência = média ponderada das notas de Exposição, Vulnerabilidade e Impacto (pesos da linha 5 nas colunas cinza 'Nota').</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="50" t="inlineStr">
+        <is>
+          <t>• Risco = nota da Probabilidade × Consequência (1 a 25).</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="50" t="inlineStr">
+        <is>
+          <t>• Índice de risco (0–1) = (Risco − 1) ÷ 24. 0 = risco mínimo (P = 1 e C = 1); 1 = risco máximo (P = 5 e C = 5). Corte da matriz (risco 9) = índice 0,333. O ranking é o mesmo do Risco.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="50" t="inlineStr">
+        <is>
+          <t>• Posição = ranking pelo Risco (1 = maior risco). Empates recebem a mesma posição.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="Y4:AC4"/>
+    <mergeCell ref="M4:P4"/>
+    <mergeCell ref="F4:L4"/>
+    <mergeCell ref="V4:X4"/>
+    <mergeCell ref="Q4:U4"/>
+  </mergeCells>
+  <conditionalFormatting sqref="AA7:AA27">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0.3333333333333333"/>
+        <cfvo type="num" val="1"/>
+        <color rgb="00FFFFFF"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="00F8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="2">
+    <dataValidation sqref="F7:F27 G7:G27 H7:H27 I7:I27 J7:J27 K7:K27 M7:M27 N7:N27 O7:O27 Q7:Q27 R7:R27 S7:S27 T7:T27 V7:V27 W7:W27" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Nota inválida" error="Use um número inteiro de 1 a 5 (5 = mais crítico)." type="whole" operator="between">
+      <formula1>1</formula1>
+      <formula2>5</formula2>
+    </dataValidation>
+    <dataValidation sqref="F5 G5 H5 I5 J5 K5 M5 N5 O5 P5 Q5 R5 S5 T5 U5 V5 W5 X5" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Peso deve ser um número maior ou igual a zero." type="decimal" operator="greaterThanOrEqual">
+      <formula1>0</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:D67"/>
@@ -2210,1319 +4238,1319 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="26" t="inlineStr">
+      <c r="A2" s="51" t="inlineStr">
         <is>
           <t>Para quem não participou das discussões do modelo. Os papéis dos órgãos são uma leitura preliminar, ainda não confirmada com cada órgão.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="27" t="inlineStr">
+      <c r="A4" s="52" t="inlineStr">
         <is>
           <t>Grupo</t>
         </is>
       </c>
-      <c r="B4" s="27" t="inlineStr">
+      <c r="B4" s="52" t="inlineStr">
         <is>
           <t>Termo</t>
         </is>
       </c>
-      <c r="C4" s="27" t="inlineStr">
+      <c r="C4" s="52" t="inlineStr">
         <is>
           <t>O que significa</t>
         </is>
       </c>
-      <c r="D4" s="27" t="inlineStr">
+      <c r="D4" s="52" t="inlineStr">
         <is>
           <t>Exemplo no projeto</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="28" t="inlineStr">
+      <c r="A5" s="53" t="inlineStr">
         <is>
           <t>Modelo de risco</t>
         </is>
       </c>
-      <c r="B5" s="29" t="inlineStr">
+      <c r="B5" s="54" t="inlineStr">
         <is>
           <t>Risco</t>
         </is>
       </c>
-      <c r="C5" s="30" t="inlineStr">
+      <c r="C5" s="43" t="inlineStr">
         <is>
           <t>Medida de quão prioritário é um ponto para a prevenção. Calculado como Probabilidade × Consequência, numa escala de 1 a 25.</t>
         </is>
       </c>
-      <c r="D5" s="30" t="inlineStr">
+      <c r="D5" s="43" t="inlineStr">
         <is>
           <t>Um ponto com Probabilidade 4 e Consequência 3 tem risco 12.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="28" t="inlineStr">
+      <c r="A6" s="53" t="inlineStr">
         <is>
           <t>Modelo de risco</t>
         </is>
       </c>
-      <c r="B6" s="29" t="inlineStr">
+      <c r="B6" s="54" t="inlineStr">
         <is>
           <t>Critério</t>
         </is>
       </c>
-      <c r="C6" s="30" t="inlineStr">
+      <c r="C6" s="43" t="inlineStr">
         <is>
           <t>Um dos 4 grandes componentes do risco: Probabilidade, Exposição, Vulnerabilidade e Impacto.</t>
         </is>
       </c>
-      <c r="D6" s="30" t="inlineStr">
+      <c r="D6" s="43" t="inlineStr">
         <is>
           <t>Vulnerabilidade é um critério.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="28" t="inlineStr">
+      <c r="A7" s="53" t="inlineStr">
         <is>
           <t>Modelo de risco</t>
         </is>
       </c>
-      <c r="B7" s="29" t="inlineStr">
+      <c r="B7" s="54" t="inlineStr">
         <is>
           <t>Subcritério</t>
         </is>
       </c>
-      <c r="C7" s="30" t="inlineStr">
+      <c r="C7" s="43" t="inlineStr">
         <is>
           <t>Um item medível dentro de um critério. Cada subcritério recebe uma nota de 1 a 5.</t>
         </is>
       </c>
-      <c r="D7" s="30" t="inlineStr">
+      <c r="D7" s="43" t="inlineStr">
         <is>
           <t>População (E1) é um subcritério da Exposição.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="28" t="inlineStr">
+      <c r="A8" s="53" t="inlineStr">
         <is>
           <t>Modelo de risco</t>
         </is>
       </c>
-      <c r="B8" s="29" t="inlineStr">
+      <c r="B8" s="54" t="inlineStr">
         <is>
           <t>Probabilidade</t>
         </is>
       </c>
-      <c r="C8" s="30" t="inlineStr">
+      <c r="C8" s="43" t="inlineStr">
         <is>
           <t>Quanto e com que facilidade o ponto alaga: frequência, severidade, maré, proximidade de rio, impermeabilização.</t>
         </is>
       </c>
-      <c r="D8" s="30" t="inlineStr">
+      <c r="D8" s="43" t="inlineStr">
         <is>
           <t>Um ponto que alaga 7 vezes por ano tem Frequência (P1) = 5.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="28" t="inlineStr">
+      <c r="A9" s="53" t="inlineStr">
         <is>
           <t>Modelo de risco</t>
         </is>
       </c>
-      <c r="B9" s="29" t="inlineStr">
+      <c r="B9" s="54" t="inlineStr">
         <is>
           <t>Exposição</t>
         </is>
       </c>
-      <c r="C9" s="30" t="inlineStr">
+      <c r="C9" s="43" t="inlineStr">
         <is>
           <t>Quem e o que está no caminho da água dentro do círculo de 300 m: moradores, escolas, unidades de saúde, comércio.</t>
         </is>
       </c>
-      <c r="D9" s="30" t="inlineStr">
+      <c r="D9" s="43" t="inlineStr">
         <is>
           <t>Um ponto com muitas escolas por perto tem Equipamentos sensíveis (E2) alto.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="28" t="inlineStr">
+      <c r="A10" s="53" t="inlineStr">
         <is>
           <t>Modelo de risco</t>
         </is>
       </c>
-      <c r="B10" s="29" t="inlineStr">
+      <c r="B10" s="54" t="inlineStr">
         <is>
           <t>Vulnerabilidade</t>
         </is>
       </c>
-      <c r="C10" s="30" t="inlineStr">
+      <c r="C10" s="43" t="inlineStr">
         <is>
           <t>Quanto quem está ali tem dificuldade de lidar com o alagamento: idosos e crianças, favelas e comunidades, moradia térrea.</t>
         </is>
       </c>
-      <c r="D10" s="30" t="inlineStr">
+      <c r="D10" s="43" t="inlineStr">
         <is>
           <t>Área com muitas casas térreas tem Tipo de moradia (V4) alto.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="28" t="inlineStr">
+      <c r="A11" s="53" t="inlineStr">
         <is>
           <t>Modelo de risco</t>
         </is>
       </c>
-      <c r="B11" s="29" t="inlineStr">
+      <c r="B11" s="54" t="inlineStr">
         <is>
           <t>Impacto</t>
         </is>
       </c>
-      <c r="C11" s="30" t="inlineStr">
+      <c r="C11" s="43" t="inlineStr">
         <is>
           <t>Consequência que vai além do local: mobilidade da cidade e saúde pública (esgoto).</t>
         </is>
       </c>
-      <c r="D11" s="30" t="inlineStr">
+      <c r="D11" s="43" t="inlineStr">
         <is>
           <t>Alagamento numa avenida arterial com ônibus tem Mobilidade (I1) alta.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="28" t="inlineStr">
+      <c r="A12" s="53" t="inlineStr">
         <is>
           <t>Modelo de risco</t>
         </is>
       </c>
-      <c r="B12" s="29" t="inlineStr">
+      <c r="B12" s="54" t="inlineStr">
         <is>
           <t>Consequência</t>
         </is>
       </c>
-      <c r="C12" s="30" t="inlineStr">
+      <c r="C12" s="43" t="inlineStr">
         <is>
           <t>Média ponderada de Exposição, Vulnerabilidade e Impacto, de 1 a 5. É o que multiplica a Probabilidade.</t>
         </is>
       </c>
-      <c r="D12" s="30" t="inlineStr">
+      <c r="D12" s="43" t="inlineStr">
         <is>
           <t>Exposição 4, Vulnerabilidade 2 e Impacto 3 com pesos iguais dão Consequência 3.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="28" t="inlineStr">
+      <c r="A13" s="53" t="inlineStr">
         <is>
           <t>Modelo de risco</t>
         </is>
       </c>
-      <c r="B13" s="29" t="inlineStr">
+      <c r="B13" s="54" t="inlineStr">
         <is>
           <t>Nota (1 a 5)</t>
         </is>
       </c>
-      <c r="C13" s="30" t="inlineStr">
+      <c r="C13" s="43" t="inlineStr">
         <is>
           <t>Valor dado a cada subcritério. 5 = mais crítico, 1 = menos crítico.</t>
         </is>
       </c>
-      <c r="D13" s="30" t="inlineStr">
+      <c r="D13" s="43" t="inlineStr">
         <is>
           <t>Nota 5 em Maré (P3) = o ponto alaga conforme a maré.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="28" t="inlineStr">
+      <c r="A14" s="53" t="inlineStr">
         <is>
           <t>Modelo de risco</t>
         </is>
       </c>
-      <c r="B14" s="29" t="inlineStr">
+      <c r="B14" s="54" t="inlineStr">
         <is>
           <t>Peso</t>
         </is>
       </c>
-      <c r="C14" s="30" t="inlineStr">
+      <c r="C14" s="43" t="inlineStr">
         <is>
           <t>Importância relativa de um subcritério dentro do critério, ou de um critério dentro da Consequência. Definido pelo grupo. A Probabilidade não tem peso, porque multiplica.</t>
         </is>
       </c>
-      <c r="D14" s="30" t="inlineStr">
+      <c r="D14" s="43" t="inlineStr">
         <is>
           <t>Frequência e Severidade terão peso maior que Proximidade de rio.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="28" t="inlineStr">
+      <c r="A15" s="53" t="inlineStr">
         <is>
           <t>Modelo de risco</t>
         </is>
       </c>
-      <c r="B15" s="29" t="inlineStr">
+      <c r="B15" s="54" t="inlineStr">
         <is>
           <t>Média ponderada</t>
         </is>
       </c>
-      <c r="C15" s="30" t="inlineStr">
+      <c r="C15" s="43" t="inlineStr">
         <is>
           <t>Média em que cada item conta conforme o seu peso.</t>
         </is>
       </c>
-      <c r="D15" s="30" t="inlineStr">
+      <c r="D15" s="43" t="inlineStr">
         <is>
           <t>Notas 5 (peso 2) e 2 (peso 1): (5×2 + 2×1) ÷ 3 = 4.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="28" t="inlineStr">
+      <c r="A16" s="53" t="inlineStr">
         <is>
           <t>Modelo de risco</t>
         </is>
       </c>
-      <c r="B16" s="29" t="inlineStr">
+      <c r="B16" s="54" t="inlineStr">
         <is>
           <t>Cobertura</t>
         </is>
       </c>
-      <c r="C16" s="30" t="inlineStr">
+      <c r="C16" s="43" t="inlineStr">
         <is>
           <t>Quantos subcritérios têm nota para o ponto. Nota faltante não vira zero nem média: fica de fora e a cobertura mostra a falta.</t>
         </is>
       </c>
-      <c r="D16" s="30" t="inlineStr">
+      <c r="D16" s="43" t="inlineStr">
         <is>
           <t>Cobertura 11/13 = faltam 2 notas para aquele ponto.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="28" t="inlineStr">
+      <c r="A17" s="53" t="inlineStr">
         <is>
           <t>Modelo de risco</t>
         </is>
       </c>
-      <c r="B17" s="29" t="inlineStr">
+      <c r="B17" s="54" t="inlineStr">
         <is>
           <t>Sem Probabilidade, sem risco</t>
         </is>
       </c>
-      <c r="C17" s="30" t="inlineStr">
+      <c r="C17" s="43" t="inlineStr">
         <is>
           <t>Como o risco é uma multiplicação, um ponto sem nota de Probabilidade não tem risco calculado nem posição no ranking.</t>
         </is>
       </c>
-      <c r="D17" s="30" t="inlineStr">
+      <c r="D17" s="43" t="inlineStr">
         <is>
           <t>Por isso a ficha com a EMLURB é prioritária.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="28" t="inlineStr">
+      <c r="A18" s="53" t="inlineStr">
         <is>
           <t>Modelo de risco</t>
         </is>
       </c>
-      <c r="B18" s="29" t="inlineStr">
+      <c r="B18" s="54" t="inlineStr">
         <is>
           <t>Tratabilidade</t>
         </is>
       </c>
-      <c r="C18" s="30" t="inlineStr">
+      <c r="C18" s="43" t="inlineStr">
         <is>
           <t>Se é fácil agir no ponto (governança, natureza da causa, obra ou orçamento em andamento). Fica FORA do risco. 5 = mais fácil.</t>
         </is>
       </c>
-      <c r="D18" s="30" t="inlineStr">
+      <c r="D18" s="43" t="inlineStr">
         <is>
           <t>Ponto com dono definido e causa de manutenção tem tratabilidade alta.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="28" t="inlineStr">
+      <c r="A19" s="53" t="inlineStr">
         <is>
           <t>Modelo de risco</t>
         </is>
       </c>
-      <c r="B19" s="29" t="inlineStr">
+      <c r="B19" s="54" t="inlineStr">
         <is>
           <t>Matriz risco × tratabilidade</t>
         </is>
       </c>
-      <c r="C19" s="30" t="inlineStr">
+      <c r="C19" s="43" t="inlineStr">
         <is>
           <t>Cruza o risco (corte em 9) com a tratabilidade (corte em 3) e coloca cada ponto num de 4 quadrantes.</t>
         </is>
       </c>
-      <c r="D19" s="30" t="inlineStr">
+      <c r="D19" s="43" t="inlineStr">
         <is>
           <t>Risco 12 e tratabilidade 4 = quadrante Agir já.</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="28" t="inlineStr">
+      <c r="A20" s="53" t="inlineStr">
         <is>
           <t>Modelo de risco</t>
         </is>
       </c>
-      <c r="B20" s="29" t="inlineStr">
+      <c r="B20" s="54" t="inlineStr">
         <is>
           <t>Agir já / Estruturar / Oportunidade / Monitorar</t>
         </is>
       </c>
-      <c r="C20" s="30" t="inlineStr">
+      <c r="C20" s="43" t="inlineStr">
         <is>
           <t>Quadrantes da matriz. Agir já: risco alto, fácil de agir. Estruturar: risco alto, difícil (exige articulação). Oportunidade: risco baixo, fácil. Monitorar: risco baixo, difícil.</t>
         </is>
       </c>
-      <c r="D20" s="30" t="inlineStr"/>
+      <c r="D20" s="43" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" s="28" t="inlineStr">
+      <c r="A21" s="53" t="inlineStr">
         <is>
           <t>Modelo de risco</t>
         </is>
       </c>
-      <c r="B21" s="29" t="inlineStr">
+      <c r="B21" s="54" t="inlineStr">
         <is>
           <t>Diagnóstico de causa</t>
         </is>
       </c>
-      <c r="C21" s="30" t="inlineStr">
+      <c r="C21" s="43" t="inlineStr">
         <is>
           <t>Por que o ponto alaga (drenagem obstruída, subdimensionada, maré, esgoto). Fica fora do risco e indica qual órgão age.</t>
         </is>
       </c>
-      <c r="D21" s="30" t="inlineStr">
+      <c r="D21" s="43" t="inlineStr">
         <is>
           <t>Galeria assoreada → EMLURB (manutenção).</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="28" t="inlineStr">
+      <c r="A22" s="53" t="inlineStr">
         <is>
           <t>Modelo de risco</t>
         </is>
       </c>
-      <c r="B22" s="29" t="inlineStr">
+      <c r="B22" s="54" t="inlineStr">
         <is>
           <t>Análise de sensibilidade</t>
         </is>
       </c>
-      <c r="C22" s="30" t="inlineStr">
+      <c r="C22" s="43" t="inlineStr">
         <is>
           <t>Recalcular o ranking com outros pesos (ex.: pesos iguais) para ver se o resultado depende demais dos pesos escolhidos.</t>
         </is>
       </c>
-      <c r="D22" s="30" t="inlineStr">
+      <c r="D22" s="43" t="inlineStr">
         <is>
           <t>Se o top 5 muda muito, avisar a alta gestão.</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="31" t="inlineStr">
+      <c r="A23" s="55" t="inlineStr">
         <is>
           <t>Tipo de nota</t>
         </is>
       </c>
-      <c r="B23" s="29" t="inlineStr">
+      <c r="B23" s="54" t="inlineStr">
         <is>
           <t>Faixa fixa</t>
         </is>
       </c>
-      <c r="C23" s="30" t="inlineStr">
+      <c r="C23" s="43" t="inlineStr">
         <is>
           <t>O valor medido cai numa faixa definida antes da coleta. A nota não depende dos outros pontos.</t>
         </is>
       </c>
-      <c r="D23" s="30" t="inlineStr">
+      <c r="D23" s="43" t="inlineStr">
         <is>
           <t>P1: 5 alagamentos/ano cai em '5–6' = nota 4.</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="31" t="inlineStr">
+      <c r="A24" s="55" t="inlineStr">
         <is>
           <t>Tipo de nota</t>
         </is>
       </c>
-      <c r="B24" s="29" t="inlineStr">
+      <c r="B24" s="54" t="inlineStr">
         <is>
           <t>Classe</t>
         </is>
       </c>
-      <c r="C24" s="30" t="inlineStr">
+      <c r="C24" s="43" t="inlineStr">
         <is>
           <t>O ponto é encaixado numa categoria descritiva, não num número.</t>
         </is>
       </c>
-      <c r="D24" s="30" t="inlineStr">
+      <c r="D24" s="43" t="inlineStr">
         <is>
           <t>P3: 'agrava ocasionalmente' = nota 3.</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="31" t="inlineStr">
+      <c r="A25" s="55" t="inlineStr">
         <is>
           <t>Tipo de nota</t>
         </is>
       </c>
-      <c r="B25" s="29" t="inlineStr">
+      <c r="B25" s="54" t="inlineStr">
         <is>
           <t>Quintil</t>
         </is>
       </c>
-      <c r="C25" s="30" t="inlineStr">
+      <c r="C25" s="43" t="inlineStr">
         <is>
           <t>Nota relativa entre os 21 pontos: os valores são ordenados e divididos em 5 grupos de ~4 pontos. Os 20% menores recebem 1; os 20% maiores, 5.</t>
         </is>
       </c>
-      <c r="D25" s="30" t="inlineStr">
+      <c r="D25" s="43" t="inlineStr">
         <is>
           <t>E1: os ~4 pontos com mais moradores recebem nota 5.</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="31" t="inlineStr">
+      <c r="A26" s="55" t="inlineStr">
         <is>
           <t>Tipo de nota</t>
         </is>
       </c>
-      <c r="B26" s="29" t="inlineStr">
+      <c r="B26" s="54" t="inlineStr">
         <is>
           <t>Quintil invertido</t>
         </is>
       </c>
-      <c r="C26" s="30" t="inlineStr">
+      <c r="C26" s="43" t="inlineStr">
         <is>
           <t>Igual ao quintil, mas o MENOR valor recebe a nota mais alta.</t>
         </is>
       </c>
-      <c r="D26" s="30" t="inlineStr">
+      <c r="D26" s="43" t="inlineStr">
         <is>
           <t>P4: o ponto mais perto do rio recebe nota 5.</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="31" t="inlineStr">
+      <c r="A27" s="55" t="inlineStr">
         <is>
           <t>Tipo de nota</t>
         </is>
       </c>
-      <c r="B27" s="29" t="inlineStr">
+      <c r="B27" s="54" t="inlineStr">
         <is>
           <t>Faixa provisória</t>
         </is>
       </c>
-      <c r="C27" s="30" t="inlineStr">
+      <c r="C27" s="43" t="inlineStr">
         <is>
           <t>Faixa proposta antes de ver os dados reais. Deve ser calibrada quando os dados chegarem.</t>
         </is>
       </c>
-      <c r="D27" s="30" t="inlineStr">
+      <c r="D27" s="43" t="inlineStr">
         <is>
           <t>Se todos os pontos caírem na mesma faixa, ela precisa ser ajustada.</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="31" t="inlineStr">
+      <c r="A28" s="55" t="inlineStr">
         <is>
           <t>Tipo de nota</t>
         </is>
       </c>
-      <c r="B28" s="29" t="inlineStr">
+      <c r="B28" s="54" t="inlineStr">
         <is>
           <t>Origem da faixa</t>
         </is>
       </c>
-      <c r="C28" s="30" t="inlineStr">
+      <c r="C28" s="43" t="inlineStr">
         <is>
           <t>De onde veio a escala: planilha original da equipe, referência oficial (ex.: Ipea) ou proposta do Claude (a revisar pelo grupo).</t>
         </is>
       </c>
-      <c r="D28" s="30" t="inlineStr"/>
+      <c r="D28" s="43" t="inlineStr"/>
     </row>
     <row r="29">
-      <c r="A29" s="32" t="inlineStr">
+      <c r="A29" s="56" t="inlineStr">
         <is>
           <t>Território e SIG</t>
         </is>
       </c>
-      <c r="B29" s="29" t="inlineStr">
+      <c r="B29" s="54" t="inlineStr">
         <is>
           <t>Ponto crítico</t>
         </is>
       </c>
-      <c r="C29" s="30" t="inlineStr">
+      <c r="C29" s="43" t="inlineStr">
         <is>
           <t>Local da lista da EMLURB onde há alagamento recorrente. Pode ser um ponto, um trecho de rua ou vários trechos.</t>
         </is>
       </c>
-      <c r="D29" s="30" t="inlineStr">
+      <c r="D29" s="43" t="inlineStr">
         <is>
           <t>Ponto 24 — Ipsep, Rua Blumenau (até a maré).</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="32" t="inlineStr">
+      <c r="A30" s="56" t="inlineStr">
         <is>
           <t>Território e SIG</t>
         </is>
       </c>
-      <c r="B30" s="29" t="inlineStr">
+      <c r="B30" s="54" t="inlineStr">
         <is>
           <t>Trecho (Linha / Vários)</t>
         </is>
       </c>
-      <c r="C30" s="30" t="inlineStr">
+      <c r="C30" s="43" t="inlineStr">
         <is>
           <t>Ponto crítico que é uma extensão de rua, não um local único. 12 dos 21 pontos são trechos.</t>
         </is>
       </c>
-      <c r="D30" s="30" t="inlineStr">
+      <c r="D30" s="43" t="inlineStr">
         <is>
           <t>Ponto 11 — Rua Professor José Brandão (toda a extensão).</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="32" t="inlineStr">
+      <c r="A31" s="56" t="inlineStr">
         <is>
           <t>Território e SIG</t>
         </is>
       </c>
-      <c r="B31" s="29" t="inlineStr">
+      <c r="B31" s="54" t="inlineStr">
         <is>
           <t>RPA 6</t>
         </is>
       </c>
-      <c r="C31" s="30" t="inlineStr">
+      <c r="C31" s="43" t="inlineStr">
         <is>
           <t>Região Político-Administrativa 6 do Recife (Boa Viagem, Pina, Imbiribeira, Ipsep, Ibura, Jordão, entre outros bairros). Escopo do piloto.</t>
         </is>
       </c>
-      <c r="D31" s="30" t="inlineStr"/>
+      <c r="D31" s="43" t="inlineStr"/>
     </row>
     <row r="32">
-      <c r="A32" s="32" t="inlineStr">
+      <c r="A32" s="56" t="inlineStr">
         <is>
           <t>Território e SIG</t>
         </is>
       </c>
-      <c r="B32" s="29" t="inlineStr">
+      <c r="B32" s="54" t="inlineStr">
         <is>
           <t>SIG</t>
         </is>
       </c>
-      <c r="C32" s="30" t="inlineStr">
+      <c r="C32" s="43" t="inlineStr">
         <is>
           <t>Sistema de Informação Geográfica: programa para mapas e cálculos espaciais. Usamos o ArcGIS Pro.</t>
         </is>
       </c>
-      <c r="D32" s="30" t="inlineStr"/>
+      <c r="D32" s="43" t="inlineStr"/>
     </row>
     <row r="33">
-      <c r="A33" s="32" t="inlineStr">
+      <c r="A33" s="56" t="inlineStr">
         <is>
           <t>Território e SIG</t>
         </is>
       </c>
-      <c r="B33" s="29" t="inlineStr">
+      <c r="B33" s="54" t="inlineStr">
         <is>
           <t>Círculo de 300 m (buffer)</t>
         </is>
       </c>
-      <c r="C33" s="30" t="inlineStr">
+      <c r="C33" s="43" t="inlineStr">
         <is>
           <t>Área de 300 m em volta do ponto (ou da linha do trecho) onde se medem os subcritérios do SIG. Usado no cálculo do risco.</t>
         </is>
       </c>
-      <c r="D33" s="30" t="inlineStr">
+      <c r="D33" s="43" t="inlineStr">
         <is>
           <t>Moradores dentro do círculo = População (E1).</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="32" t="inlineStr">
+      <c r="A34" s="56" t="inlineStr">
         <is>
           <t>Território e SIG</t>
         </is>
       </c>
-      <c r="B34" s="29" t="inlineStr">
+      <c r="B34" s="54" t="inlineStr">
         <is>
           <t>Área de influência de 1 km</t>
         </is>
       </c>
-      <c r="C34" s="30" t="inlineStr">
+      <c r="C34" s="43" t="inlineStr">
         <is>
           <t>Círculo de 1 km mostrado no painel só como informação. Não entra no cálculo, porque com 1 km quase todos os pontos se sobrepõem.</t>
         </is>
       </c>
-      <c r="D34" s="30" t="inlineStr"/>
+      <c r="D34" s="43" t="inlineStr"/>
     </row>
     <row r="35">
-      <c r="A35" s="32" t="inlineStr">
+      <c r="A35" s="56" t="inlineStr">
         <is>
           <t>Território e SIG</t>
         </is>
       </c>
-      <c r="B35" s="29" t="inlineStr">
+      <c r="B35" s="54" t="inlineStr">
         <is>
           <t>Grupo de sobreposição (G1–G5)</t>
         </is>
       </c>
-      <c r="C35" s="30" t="inlineStr">
+      <c r="C35" s="43" t="inlineStr">
         <is>
           <t>Pontos cujos círculos de 300 m se sobrepõem. Nesses grupos os subcritérios do SIG tendem a dar notas parecidas.</t>
         </is>
       </c>
-      <c r="D35" s="30" t="inlineStr">
+      <c r="D35" s="43" t="inlineStr">
         <is>
           <t>G1 = pontos 5, 6, 7, 11 e 12 (Conselheiro Aguiar).</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="32" t="inlineStr">
+      <c r="A36" s="56" t="inlineStr">
         <is>
           <t>Território e SIG</t>
         </is>
       </c>
-      <c r="B36" s="29" t="inlineStr">
+      <c r="B36" s="54" t="inlineStr">
         <is>
           <t>Ponderação por área</t>
         </is>
       </c>
-      <c r="C36" s="30" t="inlineStr">
+      <c r="C36" s="43" t="inlineStr">
         <is>
           <t>Quando uma área de dados (setor, célula) corta o círculo, conta só a parte que fica dentro dele.</t>
         </is>
       </c>
-      <c r="D36" s="30" t="inlineStr">
+      <c r="D36" s="43" t="inlineStr">
         <is>
           <t>Setor com 40% da área no círculo contribui com 40% da população.</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="32" t="inlineStr">
+      <c r="A37" s="56" t="inlineStr">
         <is>
           <t>Território e SIG</t>
         </is>
       </c>
-      <c r="B37" s="29" t="inlineStr">
+      <c r="B37" s="54" t="inlineStr">
         <is>
           <t>EPSG:31985 (SIRGAS 2000 / UTM 25S)</t>
         </is>
       </c>
-      <c r="C37" s="30" t="inlineStr">
+      <c r="C37" s="43" t="inlineStr">
         <is>
           <t>Sistema de coordenadas usado no projeto. Todas as camadas precisam estar nele antes dos cálculos.</t>
         </is>
       </c>
-      <c r="D37" s="30" t="inlineStr"/>
+      <c r="D37" s="43" t="inlineStr"/>
     </row>
     <row r="38">
-      <c r="A38" s="32" t="inlineStr">
+      <c r="A38" s="56" t="inlineStr">
         <is>
           <t>Território e SIG</t>
         </is>
       </c>
-      <c r="B38" s="29" t="inlineStr">
+      <c r="B38" s="54" t="inlineStr">
         <is>
           <t>Coordenada aproximada / verificada</t>
         </is>
       </c>
-      <c r="C38" s="30" t="inlineStr">
+      <c r="C38" s="43" t="inlineStr">
         <is>
           <t>Aproximada = localizada automaticamente e ainda não conferida. Verificada = conferida com a EMLURB ou por imagem de satélite.</t>
         </is>
       </c>
-      <c r="D38" s="30" t="inlineStr">
+      <c r="D38" s="43" t="inlineStr">
         <is>
           <t>Hoje nenhuma das 21 coordenadas está verificada.</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="32" t="inlineStr">
+      <c r="A39" s="56" t="inlineStr">
         <is>
           <t>Território e SIG</t>
         </is>
       </c>
-      <c r="B39" s="29" t="inlineStr">
+      <c r="B39" s="54" t="inlineStr">
         <is>
           <t>Bacia / sub-bacia</t>
         </is>
       </c>
-      <c r="C39" s="30" t="inlineStr">
+      <c r="C39" s="43" t="inlineStr">
         <is>
           <t>Área que drena para um mesmo rio ou canal. Hierarquia do Plano de Drenagem: Bacia → Sub-bacia → Ponto crítico → Obra.</t>
         </is>
       </c>
-      <c r="D39" s="30" t="inlineStr">
+      <c r="D39" s="43" t="inlineStr">
         <is>
           <t>Usada para ligar obras aos pontos.</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="32" t="inlineStr">
+      <c r="A40" s="56" t="inlineStr">
         <is>
           <t>Território e SIG</t>
         </is>
       </c>
-      <c r="B40" s="29" t="inlineStr">
+      <c r="B40" s="54" t="inlineStr">
         <is>
           <t>Shapefile / GeoJSON</t>
         </is>
       </c>
-      <c r="C40" s="30" t="inlineStr">
+      <c r="C40" s="43" t="inlineStr">
         <is>
           <t>Formatos de arquivo de mapa que o ArcGIS abre.</t>
         </is>
       </c>
-      <c r="D40" s="30" t="inlineStr">
+      <c r="D40" s="43" t="inlineStr">
         <is>
           <t>dados/processados/pontos_rpa6.geojson tem os 21 pontos.</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="33" t="inlineStr">
+      <c r="A41" s="57" t="inlineStr">
         <is>
           <t>Fontes de dados</t>
         </is>
       </c>
-      <c r="B41" s="29" t="inlineStr">
+      <c r="B41" s="54" t="inlineStr">
         <is>
           <t>Censo 2022 (IBGE)</t>
         </is>
       </c>
-      <c r="C41" s="30" t="inlineStr">
+      <c r="C41" s="43" t="inlineStr">
         <is>
           <t>Recenseamento de 2022. Fonte de população, idade, tipo de domicílio e esgotamento.</t>
         </is>
       </c>
-      <c r="D41" s="30" t="inlineStr"/>
+      <c r="D41" s="43" t="inlineStr"/>
     </row>
     <row r="42">
-      <c r="A42" s="33" t="inlineStr">
+      <c r="A42" s="57" t="inlineStr">
         <is>
           <t>Fontes de dados</t>
         </is>
       </c>
-      <c r="B42" s="29" t="inlineStr">
+      <c r="B42" s="54" t="inlineStr">
         <is>
           <t>Setor censitário</t>
         </is>
       </c>
-      <c r="C42" s="30" t="inlineStr">
+      <c r="C42" s="43" t="inlineStr">
         <is>
           <t>Menor área de divulgação do Censo (no Recife adensado, poucos quarteirões).</t>
         </is>
       </c>
-      <c r="D42" s="30" t="inlineStr"/>
+      <c r="D42" s="43" t="inlineStr"/>
     </row>
     <row r="43">
-      <c r="A43" s="33" t="inlineStr">
+      <c r="A43" s="57" t="inlineStr">
         <is>
           <t>Fontes de dados</t>
         </is>
       </c>
-      <c r="B43" s="29" t="inlineStr">
+      <c r="B43" s="54" t="inlineStr">
         <is>
           <t>Grade Estatística (IBGE)</t>
         </is>
       </c>
-      <c r="C43" s="30" t="inlineStr">
+      <c r="C43" s="43" t="inlineStr">
         <is>
           <t>Malha de quadrados de 200 × 200 m (área urbana) com a população do Censo 2022.</t>
         </is>
       </c>
-      <c r="D43" s="30" t="inlineStr">
+      <c r="D43" s="43" t="inlineStr">
         <is>
           <t>Fonte do E1.</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="33" t="inlineStr">
+      <c r="A44" s="57" t="inlineStr">
         <is>
           <t>Fontes de dados</t>
         </is>
       </c>
-      <c r="B44" s="29" t="inlineStr">
+      <c r="B44" s="54" t="inlineStr">
         <is>
           <t>CNEFE (IBGE)</t>
         </is>
       </c>
-      <c r="C44" s="30" t="inlineStr">
+      <c r="C44" s="43" t="inlineStr">
         <is>
           <t>Cadastro de endereços do Censo 2022, com coordenada e tipo de uso (domicílio, ensino, saúde, outras finalidades).</t>
         </is>
       </c>
-      <c r="D44" s="30" t="inlineStr">
+      <c r="D44" s="43" t="inlineStr">
         <is>
           <t>Fonte do E2 e do E3.</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="33" t="inlineStr">
+      <c r="A45" s="57" t="inlineStr">
         <is>
           <t>Fontes de dados</t>
         </is>
       </c>
-      <c r="B45" s="29" t="inlineStr">
+      <c r="B45" s="54" t="inlineStr">
         <is>
           <t>Favelas e Comunidades Urbanas (IBGE)</t>
         </is>
       </c>
-      <c r="C45" s="30" t="inlineStr">
+      <c r="C45" s="43" t="inlineStr">
         <is>
           <t>Mapeamento do IBGE das favelas e comunidades urbanas no Censo 2022. Publicação da malha ainda não confirmada.</t>
         </is>
       </c>
-      <c r="D45" s="30" t="inlineStr">
+      <c r="D45" s="43" t="inlineStr">
         <is>
           <t>Fonte do V3.</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="33" t="inlineStr">
+      <c r="A46" s="57" t="inlineStr">
         <is>
           <t>Fontes de dados</t>
         </is>
       </c>
-      <c r="B46" s="29" t="inlineStr">
+      <c r="B46" s="54" t="inlineStr">
         <is>
           <t>IVS (Ipea)</t>
         </is>
       </c>
-      <c r="C46" s="30" t="inlineStr">
+      <c r="C46" s="43" t="inlineStr">
         <is>
           <t>Índice de Vulnerabilidade Social do Ipea, de 0 a 1 (quanto maior, mais vulnerável). Base do Censo 2010.</t>
         </is>
       </c>
-      <c r="D46" s="30" t="inlineStr">
+      <c r="D46" s="43" t="inlineStr">
         <is>
           <t>Plano B do V3.</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="33" t="inlineStr">
+      <c r="A47" s="57" t="inlineStr">
         <is>
           <t>Fontes de dados</t>
         </is>
       </c>
-      <c r="B47" s="29" t="inlineStr">
+      <c r="B47" s="54" t="inlineStr">
         <is>
           <t>UDH</t>
         </is>
       </c>
-      <c r="C47" s="30" t="inlineStr">
+      <c r="C47" s="43" t="inlineStr">
         <is>
           <t>Unidade de Desenvolvimento Humano: área usada pelo Ipea, maior que o setor censitário.</t>
         </is>
       </c>
-      <c r="D47" s="30" t="inlineStr"/>
+      <c r="D47" s="43" t="inlineStr"/>
     </row>
     <row r="48">
-      <c r="A48" s="33" t="inlineStr">
+      <c r="A48" s="57" t="inlineStr">
         <is>
           <t>Fontes de dados</t>
         </is>
       </c>
-      <c r="B48" s="29" t="inlineStr">
+      <c r="B48" s="54" t="inlineStr">
         <is>
           <t>MapBiomas</t>
         </is>
       </c>
-      <c r="C48" s="30" t="inlineStr">
+      <c r="C48" s="43" t="inlineStr">
         <is>
           <t>Mapa de cobertura do solo (vegetação, área construída etc.) com pixels de 30 m. Não verificado.</t>
         </is>
       </c>
-      <c r="D48" s="30" t="inlineStr">
+      <c r="D48" s="43" t="inlineStr">
         <is>
           <t>Fonte do P5.</t>
         </is>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="33" t="inlineStr">
+      <c r="A49" s="57" t="inlineStr">
         <is>
           <t>Fontes de dados</t>
         </is>
       </c>
-      <c r="B49" s="29" t="inlineStr">
+      <c r="B49" s="54" t="inlineStr">
         <is>
           <t>ESIG</t>
         </is>
       </c>
-      <c r="C49" s="30" t="inlineStr">
+      <c r="C49" s="43" t="inlineStr">
         <is>
           <t>Sistema de informações geográficas da Prefeitura do Recife (vias, lotes, edificações, recursos hídricos).</t>
         </is>
       </c>
-      <c r="D49" s="30" t="inlineStr"/>
+      <c r="D49" s="43" t="inlineStr"/>
     </row>
     <row r="50">
-      <c r="A50" s="33" t="inlineStr">
+      <c r="A50" s="57" t="inlineStr">
         <is>
           <t>Fontes de dados</t>
         </is>
       </c>
-      <c r="B50" s="29" t="inlineStr">
+      <c r="B50" s="54" t="inlineStr">
         <is>
           <t>CNES / DATASUS</t>
         </is>
       </c>
-      <c r="C50" s="30" t="inlineStr">
+      <c r="C50" s="43" t="inlineStr">
         <is>
           <t>Cadastro Nacional de Estabelecimentos de Saúde.</t>
         </is>
       </c>
-      <c r="D50" s="30" t="inlineStr">
+      <c r="D50" s="43" t="inlineStr">
         <is>
           <t>Complementa o E2.</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="33" t="inlineStr">
+      <c r="A51" s="57" t="inlineStr">
         <is>
           <t>Fontes de dados</t>
         </is>
       </c>
-      <c r="B51" s="29" t="inlineStr">
+      <c r="B51" s="54" t="inlineStr">
         <is>
           <t>APAC / Cemaden</t>
         </is>
       </c>
-      <c r="C51" s="30" t="inlineStr">
+      <c r="C51" s="43" t="inlineStr">
         <is>
           <t>Agência Pernambucana de Águas e Clima / Centro Nacional de Monitoramento de Desastres: dados de chuva e marés.</t>
         </is>
       </c>
-      <c r="D51" s="30" t="inlineStr"/>
+      <c r="D51" s="43" t="inlineStr"/>
     </row>
     <row r="52">
-      <c r="A52" s="33" t="inlineStr">
+      <c r="A52" s="57" t="inlineStr">
         <is>
           <t>Fontes de dados</t>
         </is>
       </c>
-      <c r="B52" s="29" t="inlineStr">
+      <c r="B52" s="54" t="inlineStr">
         <is>
           <t>PMDR</t>
         </is>
       </c>
-      <c r="C52" s="30" t="inlineStr">
+      <c r="C52" s="43" t="inlineStr">
         <is>
           <t>Plano Municipal de Drenagem do Recife. Define bacias e sub-bacias.</t>
         </is>
       </c>
-      <c r="D52" s="30" t="inlineStr"/>
+      <c r="D52" s="43" t="inlineStr"/>
     </row>
     <row r="53">
-      <c r="A53" s="33" t="inlineStr">
+      <c r="A53" s="57" t="inlineStr">
         <is>
           <t>Fontes de dados</t>
         </is>
       </c>
-      <c r="B53" s="29" t="inlineStr">
+      <c r="B53" s="54" t="inlineStr">
         <is>
           <t>Ficha EMLURB</t>
         </is>
       </c>
-      <c r="C53" s="30" t="inlineStr">
+      <c r="C53" s="43" t="inlineStr">
         <is>
           <t>Formulário a ser preenchido com a EMLURB, com uma linha por ponto: localização, frequência, severidade, maré e obras ligadas.</t>
         </is>
       </c>
-      <c r="D53" s="30" t="inlineStr">
+      <c r="D53" s="43" t="inlineStr">
         <is>
           <t>Fonte provisória de P1, P2 e P3.</t>
         </is>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="34" t="inlineStr">
+      <c r="A54" s="58" t="inlineStr">
         <is>
           <t>Checklist</t>
         </is>
       </c>
-      <c r="B54" s="29" t="inlineStr">
+      <c r="B54" s="54" t="inlineStr">
         <is>
           <t>Recomendação</t>
         </is>
       </c>
-      <c r="C54" s="30" t="inlineStr">
+      <c r="C54" s="43" t="inlineStr">
         <is>
           <t>Manter = entra no modelo. Condicional = só entra se o dado existir. Plano B = usado só se outro subcritério falhar. Peso alto / menor = sugestão para a definição dos pesos.</t>
         </is>
       </c>
-      <c r="D54" s="30" t="inlineStr"/>
+      <c r="D54" s="43" t="inlineStr"/>
     </row>
     <row r="55">
-      <c r="A55" s="34" t="inlineStr">
+      <c r="A55" s="58" t="inlineStr">
         <is>
           <t>Checklist</t>
         </is>
       </c>
-      <c r="B55" s="29" t="inlineStr">
+      <c r="B55" s="54" t="inlineStr">
         <is>
           <t>Fonte confirmada?</t>
         </is>
       </c>
-      <c r="C55" s="30" t="inlineStr">
+      <c r="C55" s="43" t="inlineStr">
         <is>
           <t>A base de dados existe e a equipe consegue acessá-la (download ou pedido atendido).</t>
         </is>
       </c>
-      <c r="D55" s="30" t="inlineStr"/>
+      <c r="D55" s="43" t="inlineStr"/>
     </row>
     <row r="56">
-      <c r="A56" s="34" t="inlineStr">
+      <c r="A56" s="58" t="inlineStr">
         <is>
           <t>Checklist</t>
         </is>
       </c>
-      <c r="B56" s="29" t="inlineStr">
+      <c r="B56" s="54" t="inlineStr">
         <is>
           <t>Dado existe na fonte?</t>
         </is>
       </c>
-      <c r="C56" s="30" t="inlineStr">
+      <c r="C56" s="43" t="inlineStr">
         <is>
           <t>A variável necessária está na base, na escala do círculo de 300 m, e cobre os 21 pontos.</t>
         </is>
       </c>
-      <c r="D56" s="30" t="inlineStr">
+      <c r="D56" s="43" t="inlineStr">
         <is>
           <t>O IBGE existe (fonte confirmada), mas falta checar se o tipo de domicílio vem por setor.</t>
         </is>
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="34" t="inlineStr">
+      <c r="A57" s="58" t="inlineStr">
         <is>
           <t>Checklist</t>
         </is>
       </c>
-      <c r="B57" s="29" t="inlineStr">
+      <c r="B57" s="54" t="inlineStr">
         <is>
           <t>Sim / Parcial / Não / Pendente</t>
         </is>
       </c>
-      <c r="C57" s="30" t="inlineStr">
+      <c r="C57" s="43" t="inlineStr">
         <is>
           <t>Sim = confirmado. Parcial = existe, mas com limitação (escala, cobertura, data). Não = não existe ou não é acessível. Pendente = ainda não checado.</t>
         </is>
       </c>
-      <c r="D57" s="30" t="inlineStr"/>
+      <c r="D57" s="43" t="inlineStr"/>
     </row>
     <row r="58">
-      <c r="A58" s="34" t="inlineStr">
+      <c r="A58" s="58" t="inlineStr">
         <is>
           <t>Checklist</t>
         </is>
       </c>
-      <c r="B58" s="29" t="inlineStr">
+      <c r="B58" s="54" t="inlineStr">
         <is>
           <t>Busca prévia (Claude)</t>
         </is>
       </c>
-      <c r="C58" s="30" t="inlineStr">
+      <c r="C58" s="43" t="inlineStr">
         <is>
           <t>O que foi encontrado em busca na internet. 'Confirmado na busca' = a base aparece como publicada, mas o arquivo não foi aberto.</t>
         </is>
       </c>
-      <c r="D58" s="30" t="inlineStr"/>
+      <c r="D58" s="43" t="inlineStr"/>
     </row>
     <row r="59">
-      <c r="A59" s="35" t="inlineStr">
+      <c r="A59" s="59" t="inlineStr">
         <is>
           <t>Órgãos</t>
         </is>
       </c>
-      <c r="B59" s="29" t="inlineStr">
+      <c r="B59" s="54" t="inlineStr">
         <is>
           <t>COP</t>
         </is>
       </c>
-      <c r="C59" s="30" t="inlineStr">
+      <c r="C59" s="43" t="inlineStr">
         <is>
           <t>Centro de Operações do Recife: monitoramento e resposta aos eventos.</t>
         </is>
       </c>
-      <c r="D59" s="30" t="inlineStr"/>
+      <c r="D59" s="43" t="inlineStr"/>
     </row>
     <row r="60">
-      <c r="A60" s="35" t="inlineStr">
+      <c r="A60" s="59" t="inlineStr">
         <is>
           <t>Órgãos</t>
         </is>
       </c>
-      <c r="B60" s="29" t="inlineStr">
+      <c r="B60" s="54" t="inlineStr">
         <is>
           <t>EMLURB</t>
         </is>
       </c>
-      <c r="C60" s="30" t="inlineStr">
+      <c r="C60" s="43" t="inlineStr">
         <is>
           <t>Empresa de Manutenção e Limpeza Urbana: manutenção da drenagem e lista de pontos críticos.</t>
         </is>
       </c>
-      <c r="D60" s="30" t="inlineStr"/>
+      <c r="D60" s="43" t="inlineStr"/>
     </row>
     <row r="61">
-      <c r="A61" s="35" t="inlineStr">
+      <c r="A61" s="59" t="inlineStr">
         <is>
           <t>Órgãos</t>
         </is>
       </c>
-      <c r="B61" s="29" t="inlineStr">
+      <c r="B61" s="54" t="inlineStr">
         <is>
           <t>Defesa Civil (Sedec)</t>
         </is>
       </c>
-      <c r="C61" s="30" t="inlineStr">
+      <c r="C61" s="43" t="inlineStr">
         <is>
           <t>Áreas de risco, alertas e vistorias.</t>
         </is>
       </c>
-      <c r="D61" s="30" t="inlineStr"/>
+      <c r="D61" s="43" t="inlineStr"/>
     </row>
     <row r="62">
-      <c r="A62" s="35" t="inlineStr">
+      <c r="A62" s="59" t="inlineStr">
         <is>
           <t>Órgãos</t>
         </is>
       </c>
-      <c r="B62" s="29" t="inlineStr">
+      <c r="B62" s="54" t="inlineStr">
         <is>
           <t>URB</t>
         </is>
       </c>
-      <c r="C62" s="30" t="inlineStr">
+      <c r="C62" s="43" t="inlineStr">
         <is>
           <t>Autarquia de Urbanização do Recife: obras urbanas e de drenagem.</t>
         </is>
       </c>
-      <c r="D62" s="30" t="inlineStr"/>
+      <c r="D62" s="43" t="inlineStr"/>
     </row>
     <row r="63">
-      <c r="A63" s="35" t="inlineStr">
+      <c r="A63" s="59" t="inlineStr">
         <is>
           <t>Órgãos</t>
         </is>
       </c>
-      <c r="B63" s="29" t="inlineStr">
+      <c r="B63" s="54" t="inlineStr">
         <is>
           <t>CTTU</t>
         </is>
       </c>
-      <c r="C63" s="30" t="inlineStr">
+      <c r="C63" s="43" t="inlineStr">
         <is>
           <t>Autarquia de Trânsito e Transporte Urbano: trânsito, vias e interdições.</t>
         </is>
       </c>
-      <c r="D63" s="30" t="inlineStr"/>
+      <c r="D63" s="43" t="inlineStr"/>
     </row>
     <row r="64">
-      <c r="A64" s="35" t="inlineStr">
+      <c r="A64" s="59" t="inlineStr">
         <is>
           <t>Órgãos</t>
         </is>
       </c>
-      <c r="B64" s="29" t="inlineStr">
+      <c r="B64" s="54" t="inlineStr">
         <is>
           <t>Compesa</t>
         </is>
       </c>
-      <c r="C64" s="30" t="inlineStr">
+      <c r="C64" s="43" t="inlineStr">
         <is>
           <t>Companhia Pernambucana de Saneamento: água e esgoto.</t>
         </is>
       </c>
-      <c r="D64" s="30" t="inlineStr"/>
+      <c r="D64" s="43" t="inlineStr"/>
     </row>
     <row r="65">
-      <c r="A65" s="35" t="inlineStr">
+      <c r="A65" s="59" t="inlineStr">
         <is>
           <t>Órgãos</t>
         </is>
       </c>
-      <c r="B65" s="29" t="inlineStr">
+      <c r="B65" s="54" t="inlineStr">
         <is>
           <t>ProMorar</t>
         </is>
       </c>
-      <c r="C65" s="30" t="inlineStr">
+      <c r="C65" s="43" t="inlineStr">
         <is>
           <t>Programa de urbanização de comunidades.</t>
         </is>
       </c>
-      <c r="D65" s="30" t="inlineStr"/>
+      <c r="D65" s="43" t="inlineStr"/>
     </row>
     <row r="66">
-      <c r="A66" s="35" t="inlineStr">
+      <c r="A66" s="59" t="inlineStr">
         <is>
           <t>Órgãos</t>
         </is>
       </c>
-      <c r="B66" s="29" t="inlineStr">
+      <c r="B66" s="54" t="inlineStr">
         <is>
           <t>SEPLAG / SEPLAN</t>
         </is>
       </c>
-      <c r="C66" s="30" t="inlineStr">
+      <c r="C66" s="43" t="inlineStr">
         <is>
           <t>Planejamento e gestão. A SEPLAN não é a SEPLAG; o papel dela no projeto ainda será definido.</t>
         </is>
       </c>
-      <c r="D66" s="30" t="inlineStr"/>
+      <c r="D66" s="43" t="inlineStr"/>
     </row>
     <row r="67">
-      <c r="A67" s="35" t="inlineStr">
+      <c r="A67" s="59" t="inlineStr">
         <is>
           <t>Órgãos</t>
         </is>
       </c>
-      <c r="B67" s="29" t="inlineStr">
+      <c r="B67" s="54" t="inlineStr">
         <is>
           <t>Grande Recife Consórcio</t>
         </is>
       </c>
-      <c r="C67" s="30" t="inlineStr">
+      <c r="C67" s="43" t="inlineStr">
         <is>
           <t>Consórcio de transporte metropolitano: linhas e paradas de ônibus.</t>
         </is>
       </c>
-      <c r="D67" s="30" t="inlineStr"/>
+      <c r="D67" s="43" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A4:D67"/>

</xml_diff>

<commit_message>
Renomeia a coluna Grupo para Grupo de sobreposição na aba de notas
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018419ScLbL3ubanHMYyaBnW
</commit_message>
<xml_diff>
--- a/dados/Recife_Resiliente_Checklist_Subcriterios.xlsx
+++ b/dados/Recife_Resiliente_Checklist_Subcriterios.xlsx
@@ -2303,7 +2303,7 @@
     <col width="13" customWidth="1" min="2" max="2"/>
     <col width="42" customWidth="1" min="3" max="3"/>
     <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="7" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
     <col width="11" customWidth="1" min="6" max="6"/>
     <col width="11" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
@@ -2340,7 +2340,7 @@
     <row r="2" ht="40" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Preencha as notas (1 a 5, 5 = mais crítico) nas células amarelas, conforme as escalas da aba 'Checklist subcritérios'. Linha 'Peso': vazia = todos os pesos iguais. Nota em branco fica fora da média (não vira zero). Sem nota de Probabilidade não há risco. P6 e V1 são condicionais: deixe em branco se não forem usados. Colunas cinza são calculadas: não edite.</t>
+          <t>Preencha as notas (1 a 5, 5 = mais crítico) nas células amarelas, conforme as escalas da aba 'Checklist subcritérios'. Linha 'Peso': vazia = todos os pesos iguais. Nota em branco fica fora da média (não vira zero). Sem nota de Probabilidade não há risco. P6 e V1 são condicionais: deixe em branco se não forem usados. Colunas cinza são calculadas: não edite. 'Grupo de sobreposição' (G1–G5) = pontos cujos círculos de 300 m se sobrepõem; vazio = ponto isolado.</t>
         </is>
       </c>
     </row>
@@ -2424,7 +2424,8 @@
       </c>
       <c r="E6" s="35" t="inlineStr">
         <is>
-          <t>Grupo</t>
+          <t>Grupo de
+sobreposição</t>
         </is>
       </c>
       <c r="F6" s="36" t="inlineStr">

</xml_diff>

<commit_message>
Coordenadas e precisão na aba Notas dos pontos
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018419ScLbL3ubanHMYyaBnW
</commit_message>
<xml_diff>
--- a/dados/Recife_Resiliente_Checklist_Subcriterios.xlsx
+++ b/dados/Recife_Resiliente_Checklist_Subcriterios.xlsx
@@ -21,8 +21,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="0.000"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="0.000000"/>
+    <numFmt numFmtId="165" formatCode="0.000"/>
   </numFmts>
   <fonts count="14">
     <font>
@@ -195,7 +196,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="60">
+  <cellXfs count="61">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -320,6 +321,9 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -329,7 +333,7 @@
     <xf numFmtId="2" fontId="9" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="9" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="1" fontId="9" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -2296,7 +2300,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AC34"/>
+  <dimension ref="A1:AF34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -2306,28 +2310,31 @@
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="11" customWidth="1" min="6" max="6"/>
     <col width="11" customWidth="1" min="7" max="7"/>
-    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
     <col width="11" customWidth="1" min="9" max="9"/>
     <col width="11" customWidth="1" min="10" max="10"/>
     <col width="11" customWidth="1" min="11" max="11"/>
-    <col width="13" customWidth="1" min="12" max="12"/>
+    <col width="11" customWidth="1" min="12" max="12"/>
     <col width="11" customWidth="1" min="13" max="13"/>
     <col width="11" customWidth="1" min="14" max="14"/>
-    <col width="11" customWidth="1" min="15" max="15"/>
-    <col width="13" customWidth="1" min="16" max="16"/>
+    <col width="13" customWidth="1" min="15" max="15"/>
+    <col width="11" customWidth="1" min="16" max="16"/>
     <col width="11" customWidth="1" min="17" max="17"/>
     <col width="11" customWidth="1" min="18" max="18"/>
-    <col width="11" customWidth="1" min="19" max="19"/>
+    <col width="13" customWidth="1" min="19" max="19"/>
     <col width="11" customWidth="1" min="20" max="20"/>
-    <col width="13" customWidth="1" min="21" max="21"/>
+    <col width="11" customWidth="1" min="21" max="21"/>
     <col width="11" customWidth="1" min="22" max="22"/>
     <col width="11" customWidth="1" min="23" max="23"/>
     <col width="13" customWidth="1" min="24" max="24"/>
-    <col width="13" customWidth="1" min="25" max="25"/>
-    <col width="13" customWidth="1" min="26" max="26"/>
+    <col width="11" customWidth="1" min="25" max="25"/>
+    <col width="11" customWidth="1" min="26" max="26"/>
     <col width="13" customWidth="1" min="27" max="27"/>
     <col width="13" customWidth="1" min="28" max="28"/>
     <col width="13" customWidth="1" min="29" max="29"/>
+    <col width="13" customWidth="1" min="30" max="30"/>
+    <col width="13" customWidth="1" min="31" max="31"/>
+    <col width="13" customWidth="1" min="32" max="32"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2340,66 +2347,66 @@
     <row r="2" ht="40" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Preencha as notas (1 a 5, 5 = mais crítico) nas células amarelas, conforme as escalas da aba 'Checklist subcritérios'. Linha 'Peso': vazia = todos os pesos iguais. Nota em branco fica fora da média (não vira zero). Sem nota de Probabilidade não há risco. P6 e V1 são condicionais: deixe em branco se não forem usados. Colunas cinza são calculadas: não edite. 'Grupo de sobreposição' (G1–G5) = pontos cujos círculos de 300 m se sobrepõem; vazio = ponto isolado.</t>
+          <t>Preencha as notas (1 a 5, 5 = mais crítico) nas células amarelas, conforme as escalas da aba 'Checklist subcritérios'. Linha 'Peso': vazia = todos os pesos iguais. Nota em branco fica fora da média (não vira zero). Sem nota de Probabilidade não há risco. P6 e V1 são condicionais: deixe em branco se não forem usados. Colunas cinza são calculadas: não edite. 'Grupo de sobreposição' (G1–G5) = pontos cujos círculos de 300 m se sobrepõem; vazio = ponto isolado. Coordenadas em graus decimais (WGS 84), ainda NÃO verificadas: 'Aproximado' e 'Interseção' foram localizadas automaticamente pelo OpenStreetMap.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="F4" s="26" t="inlineStr">
+      <c r="I4" s="26" t="inlineStr">
         <is>
           <t>Probabilidade</t>
         </is>
       </c>
-      <c r="M4" s="27" t="inlineStr">
+      <c r="P4" s="27" t="inlineStr">
         <is>
           <t>Exposição</t>
         </is>
       </c>
-      <c r="Q4" s="28" t="inlineStr">
+      <c r="T4" s="28" t="inlineStr">
         <is>
           <t>Vulnerabilidade</t>
         </is>
       </c>
-      <c r="V4" s="29" t="inlineStr">
+      <c r="Y4" s="29" t="inlineStr">
         <is>
           <t>Impacto</t>
         </is>
       </c>
-      <c r="Y4" s="30" t="inlineStr">
+      <c r="AB4" s="30" t="inlineStr">
         <is>
           <t>Resultado</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="E5" s="31" t="inlineStr">
+      <c r="H5" s="31" t="inlineStr">
         <is>
           <t>Peso →</t>
         </is>
       </c>
-      <c r="F5" s="32" t="n"/>
-      <c r="G5" s="32" t="n"/>
-      <c r="H5" s="32" t="n"/>
       <c r="I5" s="32" t="n"/>
       <c r="J5" s="32" t="n"/>
       <c r="K5" s="32" t="n"/>
-      <c r="L5" s="33" t="inlineStr">
-        <is>
-          <t>(multiplica)</t>
-        </is>
-      </c>
+      <c r="L5" s="32" t="n"/>
       <c r="M5" s="32" t="n"/>
       <c r="N5" s="32" t="n"/>
-      <c r="O5" s="32" t="n"/>
-      <c r="P5" s="34" t="n"/>
+      <c r="O5" s="33" t="inlineStr">
+        <is>
+          <t>(multiplica)</t>
+        </is>
+      </c>
+      <c r="P5" s="32" t="n"/>
       <c r="Q5" s="32" t="n"/>
       <c r="R5" s="32" t="n"/>
-      <c r="S5" s="32" t="n"/>
+      <c r="S5" s="34" t="n"/>
       <c r="T5" s="32" t="n"/>
-      <c r="U5" s="34" t="n"/>
+      <c r="U5" s="32" t="n"/>
       <c r="V5" s="32" t="n"/>
       <c r="W5" s="32" t="n"/>
       <c r="X5" s="34" t="n"/>
+      <c r="Y5" s="32" t="n"/>
+      <c r="Z5" s="32" t="n"/>
+      <c r="AA5" s="34" t="n"/>
     </row>
     <row r="6" ht="54" customHeight="1">
       <c r="A6" s="35" t="inlineStr">
@@ -2428,144 +2435,160 @@
 sobreposição</t>
         </is>
       </c>
-      <c r="F6" s="36" t="inlineStr">
+      <c r="F6" s="35" t="inlineStr">
+        <is>
+          <t>Latitude</t>
+        </is>
+      </c>
+      <c r="G6" s="35" t="inlineStr">
+        <is>
+          <t>Longitude</t>
+        </is>
+      </c>
+      <c r="H6" s="35" t="inlineStr">
+        <is>
+          <t>Precisão da
+coordenada</t>
+        </is>
+      </c>
+      <c r="I6" s="36" t="inlineStr">
         <is>
           <t>P1
 Frequência de alagamento</t>
         </is>
       </c>
-      <c r="G6" s="36" t="inlineStr">
+      <c r="J6" s="36" t="inlineStr">
         <is>
           <t>P2
 Severidade</t>
         </is>
       </c>
-      <c r="H6" s="36" t="inlineStr">
+      <c r="K6" s="36" t="inlineStr">
         <is>
           <t>P3
 Influência da maré</t>
         </is>
       </c>
-      <c r="I6" s="36" t="inlineStr">
+      <c r="L6" s="36" t="inlineStr">
         <is>
           <t>P4
 Proximidade de rio ou canal</t>
         </is>
       </c>
-      <c r="J6" s="36" t="inlineStr">
+      <c r="M6" s="36" t="inlineStr">
         <is>
           <t>P5
 Impermeabilização</t>
         </is>
       </c>
-      <c r="K6" s="36" t="inlineStr">
+      <c r="N6" s="36" t="inlineStr">
         <is>
           <t>P6
 Baixio</t>
         </is>
       </c>
-      <c r="L6" s="37" t="inlineStr">
+      <c r="O6" s="37" t="inlineStr">
         <is>
           <t>Nota
 Probabilidade</t>
         </is>
       </c>
-      <c r="M6" s="38" t="inlineStr">
+      <c r="P6" s="38" t="inlineStr">
         <is>
           <t>E1
 População</t>
         </is>
       </c>
-      <c r="N6" s="38" t="inlineStr">
+      <c r="Q6" s="38" t="inlineStr">
         <is>
           <t>E2
 Equipamentos sensíveis</t>
         </is>
       </c>
-      <c r="O6" s="38" t="inlineStr">
+      <c r="R6" s="38" t="inlineStr">
         <is>
           <t>E3
 Atividade econômica</t>
         </is>
       </c>
-      <c r="P6" s="37" t="inlineStr">
+      <c r="S6" s="37" t="inlineStr">
         <is>
           <t>Nota
 Exposição</t>
         </is>
       </c>
-      <c r="Q6" s="39" t="inlineStr">
+      <c r="T6" s="39" t="inlineStr">
         <is>
           <t>V2
 Grupos sensíveis</t>
         </is>
       </c>
-      <c r="R6" s="39" t="inlineStr">
+      <c r="U6" s="39" t="inlineStr">
         <is>
           <t>V3
 Favelas e comunidades urbanas</t>
         </is>
       </c>
-      <c r="S6" s="39" t="inlineStr">
+      <c r="V6" s="39" t="inlineStr">
         <is>
           <t>V4
 Tipo de moradia</t>
         </is>
       </c>
-      <c r="T6" s="39" t="inlineStr">
+      <c r="W6" s="39" t="inlineStr">
         <is>
           <t>V1
 Vulnerabilidade social (IVS)</t>
         </is>
       </c>
-      <c r="U6" s="37" t="inlineStr">
+      <c r="X6" s="37" t="inlineStr">
         <is>
           <t>Nota
 Vulnerabilidade</t>
         </is>
       </c>
-      <c r="V6" s="40" t="inlineStr">
+      <c r="Y6" s="40" t="inlineStr">
         <is>
           <t>I1
 Mobilidade</t>
         </is>
       </c>
-      <c r="W6" s="40" t="inlineStr">
+      <c r="Z6" s="40" t="inlineStr">
         <is>
           <t>I2
 Risco sanitário</t>
         </is>
       </c>
-      <c r="X6" s="37" t="inlineStr">
+      <c r="AA6" s="37" t="inlineStr">
         <is>
           <t>Nota
 Impacto</t>
         </is>
       </c>
-      <c r="Y6" s="41" t="inlineStr">
+      <c r="AB6" s="41" t="inlineStr">
         <is>
           <t>Consequência
 (1–5)</t>
         </is>
       </c>
-      <c r="Z6" s="41" t="inlineStr">
+      <c r="AC6" s="41" t="inlineStr">
         <is>
           <t>Risco
 P × C (1–25)</t>
         </is>
       </c>
-      <c r="AA6" s="41" t="inlineStr">
+      <c r="AD6" s="41" t="inlineStr">
         <is>
           <t>Índice de risco
 (0–1)</t>
         </is>
       </c>
-      <c r="AB6" s="41" t="inlineStr">
+      <c r="AE6" s="41" t="inlineStr">
         <is>
           <t>Posição</t>
         </is>
       </c>
-      <c r="AC6" s="41" t="inlineStr">
+      <c r="AF6" s="41" t="inlineStr">
         <is>
           <t>Notas
 preenchidas</t>
@@ -2596,55 +2619,66 @@
           <t>G1</t>
         </is>
       </c>
-      <c r="F7" s="44" t="n"/>
-      <c r="G7" s="44" t="n"/>
-      <c r="H7" s="44" t="n"/>
-      <c r="I7" s="44" t="n"/>
-      <c r="J7" s="44" t="n"/>
-      <c r="K7" s="44" t="n"/>
-      <c r="L7" s="45">
-        <f>IF(COUNT(F7:K7)=0,"",IFERROR(SUMPRODUCT(F7:K7,(F$5:K$5+(F$5:K$5="")))/SUMPRODUCT((F7:K7&lt;&gt;"")*(F$5:K$5+(F$5:K$5=""))),""))</f>
-        <v/>
-      </c>
-      <c r="M7" s="44" t="n"/>
-      <c r="N7" s="44" t="n"/>
-      <c r="O7" s="44" t="n"/>
-      <c r="P7" s="45">
-        <f>IF(COUNT(M7:O7)=0,"",IFERROR(SUMPRODUCT(M7:O7,(M$5:O$5+(M$5:O$5="")))/SUMPRODUCT((M7:O7&lt;&gt;"")*(M$5:O$5+(M$5:O$5=""))),""))</f>
-        <v/>
-      </c>
-      <c r="Q7" s="44" t="n"/>
-      <c r="R7" s="44" t="n"/>
-      <c r="S7" s="44" t="n"/>
-      <c r="T7" s="44" t="n"/>
-      <c r="U7" s="45">
-        <f>IF(COUNT(Q7:T7)=0,"",IFERROR(SUMPRODUCT(Q7:T7,(Q$5:T$5+(Q$5:T$5="")))/SUMPRODUCT((Q7:T7&lt;&gt;"")*(Q$5:T$5+(Q$5:T$5=""))),""))</f>
-        <v/>
-      </c>
-      <c r="V7" s="44" t="n"/>
-      <c r="W7" s="44" t="n"/>
-      <c r="X7" s="45">
-        <f>IF(COUNT(V7:W7)=0,"",IFERROR(SUMPRODUCT(V7:W7,(V$5:W$5+(V$5:W$5="")))/SUMPRODUCT((V7:W7&lt;&gt;"")*(V$5:W$5+(V$5:W$5=""))),""))</f>
-        <v/>
-      </c>
-      <c r="Y7" s="45">
-        <f>IFERROR(IF((ISNUMBER(P7)*(P$5+(P$5=""))+ISNUMBER(U7)*(U$5+(U$5=""))+ISNUMBER(X7)*(X$5+(X$5="")))=0,"",(N(P7)*(P$5+(P$5=""))+N(U7)*(U$5+(U$5=""))+N(X7)*(X$5+(X$5="")))/(ISNUMBER(P7)*(P$5+(P$5=""))+ISNUMBER(U7)*(U$5+(U$5=""))+ISNUMBER(X7)*(X$5+(X$5="")))),"")</f>
-        <v/>
-      </c>
-      <c r="Z7" s="46">
-        <f>IF(AND(ISNUMBER(L7),ISNUMBER(Y7)),L7*Y7,"")</f>
-        <v/>
-      </c>
-      <c r="AA7" s="47">
-        <f>IF(ISNUMBER(Z7),(Z7-1)/24,"")</f>
-        <v/>
-      </c>
-      <c r="AB7" s="48">
-        <f>IF(ISNUMBER(Z7),COUNTIF(Z$7:Z$27,"&gt;"&amp;Z7)+1,"")</f>
-        <v/>
-      </c>
-      <c r="AC7" s="49">
-        <f>COUNT(F7,G7,H7,I7,J7,K7,M7,N7,O7,Q7,R7,S7,T7,V7,W7)</f>
+      <c r="F7" s="44" t="n">
+        <v>-8.113732000000001</v>
+      </c>
+      <c r="G7" s="44" t="n">
+        <v>-34.893163</v>
+      </c>
+      <c r="H7" s="42" t="inlineStr">
+        <is>
+          <t>Interseção</t>
+        </is>
+      </c>
+      <c r="I7" s="45" t="n"/>
+      <c r="J7" s="45" t="n"/>
+      <c r="K7" s="45" t="n"/>
+      <c r="L7" s="45" t="n"/>
+      <c r="M7" s="45" t="n"/>
+      <c r="N7" s="45" t="n"/>
+      <c r="O7" s="46">
+        <f>IF(COUNT(I7:N7)=0,"",IFERROR(SUMPRODUCT(I7:N7,(I$5:N$5+(I$5:N$5="")))/SUMPRODUCT((I7:N7&lt;&gt;"")*(I$5:N$5+(I$5:N$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="P7" s="45" t="n"/>
+      <c r="Q7" s="45" t="n"/>
+      <c r="R7" s="45" t="n"/>
+      <c r="S7" s="46">
+        <f>IF(COUNT(P7:R7)=0,"",IFERROR(SUMPRODUCT(P7:R7,(P$5:R$5+(P$5:R$5="")))/SUMPRODUCT((P7:R7&lt;&gt;"")*(P$5:R$5+(P$5:R$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="T7" s="45" t="n"/>
+      <c r="U7" s="45" t="n"/>
+      <c r="V7" s="45" t="n"/>
+      <c r="W7" s="45" t="n"/>
+      <c r="X7" s="46">
+        <f>IF(COUNT(T7:W7)=0,"",IFERROR(SUMPRODUCT(T7:W7,(T$5:W$5+(T$5:W$5="")))/SUMPRODUCT((T7:W7&lt;&gt;"")*(T$5:W$5+(T$5:W$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="Y7" s="45" t="n"/>
+      <c r="Z7" s="45" t="n"/>
+      <c r="AA7" s="46">
+        <f>IF(COUNT(Y7:Z7)=0,"",IFERROR(SUMPRODUCT(Y7:Z7,(Y$5:Z$5+(Y$5:Z$5="")))/SUMPRODUCT((Y7:Z7&lt;&gt;"")*(Y$5:Z$5+(Y$5:Z$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="AB7" s="46">
+        <f>IFERROR(IF((ISNUMBER(S7)*(S$5+(S$5=""))+ISNUMBER(X7)*(X$5+(X$5=""))+ISNUMBER(AA7)*(AA$5+(AA$5="")))=0,"",(N(S7)*(S$5+(S$5=""))+N(X7)*(X$5+(X$5=""))+N(AA7)*(AA$5+(AA$5="")))/(ISNUMBER(S7)*(S$5+(S$5=""))+ISNUMBER(X7)*(X$5+(X$5=""))+ISNUMBER(AA7)*(AA$5+(AA$5="")))),"")</f>
+        <v/>
+      </c>
+      <c r="AC7" s="47">
+        <f>IF(AND(ISNUMBER(O7),ISNUMBER(AB7)),O7*AB7,"")</f>
+        <v/>
+      </c>
+      <c r="AD7" s="48">
+        <f>IF(ISNUMBER(AC7),(AC7-1)/24,"")</f>
+        <v/>
+      </c>
+      <c r="AE7" s="49">
+        <f>IF(ISNUMBER(AC7),COUNTIF(AC$7:AC$27,"&gt;"&amp;AC7)+1,"")</f>
+        <v/>
+      </c>
+      <c r="AF7" s="50">
+        <f>COUNT(I7,J7,K7,L7,M7,N7,P7,Q7,R7,T7,U7,V7,W7,Y7,Z7)</f>
         <v/>
       </c>
     </row>
@@ -2672,55 +2706,66 @@
           <t>G1</t>
         </is>
       </c>
-      <c r="F8" s="44" t="n"/>
-      <c r="G8" s="44" t="n"/>
-      <c r="H8" s="44" t="n"/>
-      <c r="I8" s="44" t="n"/>
-      <c r="J8" s="44" t="n"/>
-      <c r="K8" s="44" t="n"/>
-      <c r="L8" s="45">
-        <f>IF(COUNT(F8:K8)=0,"",IFERROR(SUMPRODUCT(F8:K8,(F$5:K$5+(F$5:K$5="")))/SUMPRODUCT((F8:K8&lt;&gt;"")*(F$5:K$5+(F$5:K$5=""))),""))</f>
-        <v/>
-      </c>
-      <c r="M8" s="44" t="n"/>
-      <c r="N8" s="44" t="n"/>
-      <c r="O8" s="44" t="n"/>
-      <c r="P8" s="45">
-        <f>IF(COUNT(M8:O8)=0,"",IFERROR(SUMPRODUCT(M8:O8,(M$5:O$5+(M$5:O$5="")))/SUMPRODUCT((M8:O8&lt;&gt;"")*(M$5:O$5+(M$5:O$5=""))),""))</f>
-        <v/>
-      </c>
-      <c r="Q8" s="44" t="n"/>
-      <c r="R8" s="44" t="n"/>
-      <c r="S8" s="44" t="n"/>
-      <c r="T8" s="44" t="n"/>
-      <c r="U8" s="45">
-        <f>IF(COUNT(Q8:T8)=0,"",IFERROR(SUMPRODUCT(Q8:T8,(Q$5:T$5+(Q$5:T$5="")))/SUMPRODUCT((Q8:T8&lt;&gt;"")*(Q$5:T$5+(Q$5:T$5=""))),""))</f>
-        <v/>
-      </c>
-      <c r="V8" s="44" t="n"/>
-      <c r="W8" s="44" t="n"/>
-      <c r="X8" s="45">
-        <f>IF(COUNT(V8:W8)=0,"",IFERROR(SUMPRODUCT(V8:W8,(V$5:W$5+(V$5:W$5="")))/SUMPRODUCT((V8:W8&lt;&gt;"")*(V$5:W$5+(V$5:W$5=""))),""))</f>
-        <v/>
-      </c>
-      <c r="Y8" s="45">
-        <f>IFERROR(IF((ISNUMBER(P8)*(P$5+(P$5=""))+ISNUMBER(U8)*(U$5+(U$5=""))+ISNUMBER(X8)*(X$5+(X$5="")))=0,"",(N(P8)*(P$5+(P$5=""))+N(U8)*(U$5+(U$5=""))+N(X8)*(X$5+(X$5="")))/(ISNUMBER(P8)*(P$5+(P$5=""))+ISNUMBER(U8)*(U$5+(U$5=""))+ISNUMBER(X8)*(X$5+(X$5="")))),"")</f>
-        <v/>
-      </c>
-      <c r="Z8" s="46">
-        <f>IF(AND(ISNUMBER(L8),ISNUMBER(Y8)),L8*Y8,"")</f>
-        <v/>
-      </c>
-      <c r="AA8" s="47">
-        <f>IF(ISNUMBER(Z8),(Z8-1)/24,"")</f>
-        <v/>
-      </c>
-      <c r="AB8" s="48">
-        <f>IF(ISNUMBER(Z8),COUNTIF(Z$7:Z$27,"&gt;"&amp;Z8)+1,"")</f>
-        <v/>
-      </c>
-      <c r="AC8" s="49">
-        <f>COUNT(F8,G8,H8,I8,J8,K8,M8,N8,O8,Q8,R8,S8,T8,V8,W8)</f>
+      <c r="F8" s="44" t="n">
+        <v>-8.111008999999999</v>
+      </c>
+      <c r="G8" s="44" t="n">
+        <v>-34.891491</v>
+      </c>
+      <c r="H8" s="42" t="inlineStr">
+        <is>
+          <t>Interseção</t>
+        </is>
+      </c>
+      <c r="I8" s="45" t="n"/>
+      <c r="J8" s="45" t="n"/>
+      <c r="K8" s="45" t="n"/>
+      <c r="L8" s="45" t="n"/>
+      <c r="M8" s="45" t="n"/>
+      <c r="N8" s="45" t="n"/>
+      <c r="O8" s="46">
+        <f>IF(COUNT(I8:N8)=0,"",IFERROR(SUMPRODUCT(I8:N8,(I$5:N$5+(I$5:N$5="")))/SUMPRODUCT((I8:N8&lt;&gt;"")*(I$5:N$5+(I$5:N$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="P8" s="45" t="n"/>
+      <c r="Q8" s="45" t="n"/>
+      <c r="R8" s="45" t="n"/>
+      <c r="S8" s="46">
+        <f>IF(COUNT(P8:R8)=0,"",IFERROR(SUMPRODUCT(P8:R8,(P$5:R$5+(P$5:R$5="")))/SUMPRODUCT((P8:R8&lt;&gt;"")*(P$5:R$5+(P$5:R$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="T8" s="45" t="n"/>
+      <c r="U8" s="45" t="n"/>
+      <c r="V8" s="45" t="n"/>
+      <c r="W8" s="45" t="n"/>
+      <c r="X8" s="46">
+        <f>IF(COUNT(T8:W8)=0,"",IFERROR(SUMPRODUCT(T8:W8,(T$5:W$5+(T$5:W$5="")))/SUMPRODUCT((T8:W8&lt;&gt;"")*(T$5:W$5+(T$5:W$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="Y8" s="45" t="n"/>
+      <c r="Z8" s="45" t="n"/>
+      <c r="AA8" s="46">
+        <f>IF(COUNT(Y8:Z8)=0,"",IFERROR(SUMPRODUCT(Y8:Z8,(Y$5:Z$5+(Y$5:Z$5="")))/SUMPRODUCT((Y8:Z8&lt;&gt;"")*(Y$5:Z$5+(Y$5:Z$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="AB8" s="46">
+        <f>IFERROR(IF((ISNUMBER(S8)*(S$5+(S$5=""))+ISNUMBER(X8)*(X$5+(X$5=""))+ISNUMBER(AA8)*(AA$5+(AA$5="")))=0,"",(N(S8)*(S$5+(S$5=""))+N(X8)*(X$5+(X$5=""))+N(AA8)*(AA$5+(AA$5="")))/(ISNUMBER(S8)*(S$5+(S$5=""))+ISNUMBER(X8)*(X$5+(X$5=""))+ISNUMBER(AA8)*(AA$5+(AA$5="")))),"")</f>
+        <v/>
+      </c>
+      <c r="AC8" s="47">
+        <f>IF(AND(ISNUMBER(O8),ISNUMBER(AB8)),O8*AB8,"")</f>
+        <v/>
+      </c>
+      <c r="AD8" s="48">
+        <f>IF(ISNUMBER(AC8),(AC8-1)/24,"")</f>
+        <v/>
+      </c>
+      <c r="AE8" s="49">
+        <f>IF(ISNUMBER(AC8),COUNTIF(AC$7:AC$27,"&gt;"&amp;AC8)+1,"")</f>
+        <v/>
+      </c>
+      <c r="AF8" s="50">
+        <f>COUNT(I8,J8,K8,L8,M8,N8,P8,Q8,R8,T8,U8,V8,W8,Y8,Z8)</f>
         <v/>
       </c>
     </row>
@@ -2748,55 +2793,66 @@
           <t>G1</t>
         </is>
       </c>
-      <c r="F9" s="44" t="n"/>
-      <c r="G9" s="44" t="n"/>
-      <c r="H9" s="44" t="n"/>
-      <c r="I9" s="44" t="n"/>
-      <c r="J9" s="44" t="n"/>
-      <c r="K9" s="44" t="n"/>
-      <c r="L9" s="45">
-        <f>IF(COUNT(F9:K9)=0,"",IFERROR(SUMPRODUCT(F9:K9,(F$5:K$5+(F$5:K$5="")))/SUMPRODUCT((F9:K9&lt;&gt;"")*(F$5:K$5+(F$5:K$5=""))),""))</f>
-        <v/>
-      </c>
-      <c r="M9" s="44" t="n"/>
-      <c r="N9" s="44" t="n"/>
-      <c r="O9" s="44" t="n"/>
-      <c r="P9" s="45">
-        <f>IF(COUNT(M9:O9)=0,"",IFERROR(SUMPRODUCT(M9:O9,(M$5:O$5+(M$5:O$5="")))/SUMPRODUCT((M9:O9&lt;&gt;"")*(M$5:O$5+(M$5:O$5=""))),""))</f>
-        <v/>
-      </c>
-      <c r="Q9" s="44" t="n"/>
-      <c r="R9" s="44" t="n"/>
-      <c r="S9" s="44" t="n"/>
-      <c r="T9" s="44" t="n"/>
-      <c r="U9" s="45">
-        <f>IF(COUNT(Q9:T9)=0,"",IFERROR(SUMPRODUCT(Q9:T9,(Q$5:T$5+(Q$5:T$5="")))/SUMPRODUCT((Q9:T9&lt;&gt;"")*(Q$5:T$5+(Q$5:T$5=""))),""))</f>
-        <v/>
-      </c>
-      <c r="V9" s="44" t="n"/>
-      <c r="W9" s="44" t="n"/>
-      <c r="X9" s="45">
-        <f>IF(COUNT(V9:W9)=0,"",IFERROR(SUMPRODUCT(V9:W9,(V$5:W$5+(V$5:W$5="")))/SUMPRODUCT((V9:W9&lt;&gt;"")*(V$5:W$5+(V$5:W$5=""))),""))</f>
-        <v/>
-      </c>
-      <c r="Y9" s="45">
-        <f>IFERROR(IF((ISNUMBER(P9)*(P$5+(P$5=""))+ISNUMBER(U9)*(U$5+(U$5=""))+ISNUMBER(X9)*(X$5+(X$5="")))=0,"",(N(P9)*(P$5+(P$5=""))+N(U9)*(U$5+(U$5=""))+N(X9)*(X$5+(X$5="")))/(ISNUMBER(P9)*(P$5+(P$5=""))+ISNUMBER(U9)*(U$5+(U$5=""))+ISNUMBER(X9)*(X$5+(X$5="")))),"")</f>
-        <v/>
-      </c>
-      <c r="Z9" s="46">
-        <f>IF(AND(ISNUMBER(L9),ISNUMBER(Y9)),L9*Y9,"")</f>
-        <v/>
-      </c>
-      <c r="AA9" s="47">
-        <f>IF(ISNUMBER(Z9),(Z9-1)/24,"")</f>
-        <v/>
-      </c>
-      <c r="AB9" s="48">
-        <f>IF(ISNUMBER(Z9),COUNTIF(Z$7:Z$27,"&gt;"&amp;Z9)+1,"")</f>
-        <v/>
-      </c>
-      <c r="AC9" s="49">
-        <f>COUNT(F9,G9,H9,I9,J9,K9,M9,N9,O9,Q9,R9,S9,T9,V9,W9)</f>
+      <c r="F9" s="44" t="n">
+        <v>-8.11538</v>
+      </c>
+      <c r="G9" s="44" t="n">
+        <v>-34.894176</v>
+      </c>
+      <c r="H9" s="42" t="inlineStr">
+        <is>
+          <t>Interseção</t>
+        </is>
+      </c>
+      <c r="I9" s="45" t="n"/>
+      <c r="J9" s="45" t="n"/>
+      <c r="K9" s="45" t="n"/>
+      <c r="L9" s="45" t="n"/>
+      <c r="M9" s="45" t="n"/>
+      <c r="N9" s="45" t="n"/>
+      <c r="O9" s="46">
+        <f>IF(COUNT(I9:N9)=0,"",IFERROR(SUMPRODUCT(I9:N9,(I$5:N$5+(I$5:N$5="")))/SUMPRODUCT((I9:N9&lt;&gt;"")*(I$5:N$5+(I$5:N$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="P9" s="45" t="n"/>
+      <c r="Q9" s="45" t="n"/>
+      <c r="R9" s="45" t="n"/>
+      <c r="S9" s="46">
+        <f>IF(COUNT(P9:R9)=0,"",IFERROR(SUMPRODUCT(P9:R9,(P$5:R$5+(P$5:R$5="")))/SUMPRODUCT((P9:R9&lt;&gt;"")*(P$5:R$5+(P$5:R$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="T9" s="45" t="n"/>
+      <c r="U9" s="45" t="n"/>
+      <c r="V9" s="45" t="n"/>
+      <c r="W9" s="45" t="n"/>
+      <c r="X9" s="46">
+        <f>IF(COUNT(T9:W9)=0,"",IFERROR(SUMPRODUCT(T9:W9,(T$5:W$5+(T$5:W$5="")))/SUMPRODUCT((T9:W9&lt;&gt;"")*(T$5:W$5+(T$5:W$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="Y9" s="45" t="n"/>
+      <c r="Z9" s="45" t="n"/>
+      <c r="AA9" s="46">
+        <f>IF(COUNT(Y9:Z9)=0,"",IFERROR(SUMPRODUCT(Y9:Z9,(Y$5:Z$5+(Y$5:Z$5="")))/SUMPRODUCT((Y9:Z9&lt;&gt;"")*(Y$5:Z$5+(Y$5:Z$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="AB9" s="46">
+        <f>IFERROR(IF((ISNUMBER(S9)*(S$5+(S$5=""))+ISNUMBER(X9)*(X$5+(X$5=""))+ISNUMBER(AA9)*(AA$5+(AA$5="")))=0,"",(N(S9)*(S$5+(S$5=""))+N(X9)*(X$5+(X$5=""))+N(AA9)*(AA$5+(AA$5="")))/(ISNUMBER(S9)*(S$5+(S$5=""))+ISNUMBER(X9)*(X$5+(X$5=""))+ISNUMBER(AA9)*(AA$5+(AA$5="")))),"")</f>
+        <v/>
+      </c>
+      <c r="AC9" s="47">
+        <f>IF(AND(ISNUMBER(O9),ISNUMBER(AB9)),O9*AB9,"")</f>
+        <v/>
+      </c>
+      <c r="AD9" s="48">
+        <f>IF(ISNUMBER(AC9),(AC9-1)/24,"")</f>
+        <v/>
+      </c>
+      <c r="AE9" s="49">
+        <f>IF(ISNUMBER(AC9),COUNTIF(AC$7:AC$27,"&gt;"&amp;AC9)+1,"")</f>
+        <v/>
+      </c>
+      <c r="AF9" s="50">
+        <f>COUNT(I9,J9,K9,L9,M9,N9,P9,Q9,R9,T9,U9,V9,W9,Y9,Z9)</f>
         <v/>
       </c>
     </row>
@@ -2824,55 +2880,66 @@
           <t>G2</t>
         </is>
       </c>
-      <c r="F10" s="44" t="n"/>
-      <c r="G10" s="44" t="n"/>
-      <c r="H10" s="44" t="n"/>
-      <c r="I10" s="44" t="n"/>
-      <c r="J10" s="44" t="n"/>
-      <c r="K10" s="44" t="n"/>
-      <c r="L10" s="45">
-        <f>IF(COUNT(F10:K10)=0,"",IFERROR(SUMPRODUCT(F10:K10,(F$5:K$5+(F$5:K$5="")))/SUMPRODUCT((F10:K10&lt;&gt;"")*(F$5:K$5+(F$5:K$5=""))),""))</f>
-        <v/>
-      </c>
-      <c r="M10" s="44" t="n"/>
-      <c r="N10" s="44" t="n"/>
-      <c r="O10" s="44" t="n"/>
-      <c r="P10" s="45">
-        <f>IF(COUNT(M10:O10)=0,"",IFERROR(SUMPRODUCT(M10:O10,(M$5:O$5+(M$5:O$5="")))/SUMPRODUCT((M10:O10&lt;&gt;"")*(M$5:O$5+(M$5:O$5=""))),""))</f>
-        <v/>
-      </c>
-      <c r="Q10" s="44" t="n"/>
-      <c r="R10" s="44" t="n"/>
-      <c r="S10" s="44" t="n"/>
-      <c r="T10" s="44" t="n"/>
-      <c r="U10" s="45">
-        <f>IF(COUNT(Q10:T10)=0,"",IFERROR(SUMPRODUCT(Q10:T10,(Q$5:T$5+(Q$5:T$5="")))/SUMPRODUCT((Q10:T10&lt;&gt;"")*(Q$5:T$5+(Q$5:T$5=""))),""))</f>
-        <v/>
-      </c>
-      <c r="V10" s="44" t="n"/>
-      <c r="W10" s="44" t="n"/>
-      <c r="X10" s="45">
-        <f>IF(COUNT(V10:W10)=0,"",IFERROR(SUMPRODUCT(V10:W10,(V$5:W$5+(V$5:W$5="")))/SUMPRODUCT((V10:W10&lt;&gt;"")*(V$5:W$5+(V$5:W$5=""))),""))</f>
-        <v/>
-      </c>
-      <c r="Y10" s="45">
-        <f>IFERROR(IF((ISNUMBER(P10)*(P$5+(P$5=""))+ISNUMBER(U10)*(U$5+(U$5=""))+ISNUMBER(X10)*(X$5+(X$5="")))=0,"",(N(P10)*(P$5+(P$5=""))+N(U10)*(U$5+(U$5=""))+N(X10)*(X$5+(X$5="")))/(ISNUMBER(P10)*(P$5+(P$5=""))+ISNUMBER(U10)*(U$5+(U$5=""))+ISNUMBER(X10)*(X$5+(X$5="")))),"")</f>
-        <v/>
-      </c>
-      <c r="Z10" s="46">
-        <f>IF(AND(ISNUMBER(L10),ISNUMBER(Y10)),L10*Y10,"")</f>
-        <v/>
-      </c>
-      <c r="AA10" s="47">
-        <f>IF(ISNUMBER(Z10),(Z10-1)/24,"")</f>
-        <v/>
-      </c>
-      <c r="AB10" s="48">
-        <f>IF(ISNUMBER(Z10),COUNTIF(Z$7:Z$27,"&gt;"&amp;Z10)+1,"")</f>
-        <v/>
-      </c>
-      <c r="AC10" s="49">
-        <f>COUNT(F10,G10,H10,I10,J10,K10,M10,N10,O10,Q10,R10,S10,T10,V10,W10)</f>
+      <c r="F10" s="44" t="n">
+        <v>-8.101065999999999</v>
+      </c>
+      <c r="G10" s="44" t="n">
+        <v>-34.886765</v>
+      </c>
+      <c r="H10" s="42" t="inlineStr">
+        <is>
+          <t>Interseção</t>
+        </is>
+      </c>
+      <c r="I10" s="45" t="n"/>
+      <c r="J10" s="45" t="n"/>
+      <c r="K10" s="45" t="n"/>
+      <c r="L10" s="45" t="n"/>
+      <c r="M10" s="45" t="n"/>
+      <c r="N10" s="45" t="n"/>
+      <c r="O10" s="46">
+        <f>IF(COUNT(I10:N10)=0,"",IFERROR(SUMPRODUCT(I10:N10,(I$5:N$5+(I$5:N$5="")))/SUMPRODUCT((I10:N10&lt;&gt;"")*(I$5:N$5+(I$5:N$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="P10" s="45" t="n"/>
+      <c r="Q10" s="45" t="n"/>
+      <c r="R10" s="45" t="n"/>
+      <c r="S10" s="46">
+        <f>IF(COUNT(P10:R10)=0,"",IFERROR(SUMPRODUCT(P10:R10,(P$5:R$5+(P$5:R$5="")))/SUMPRODUCT((P10:R10&lt;&gt;"")*(P$5:R$5+(P$5:R$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="T10" s="45" t="n"/>
+      <c r="U10" s="45" t="n"/>
+      <c r="V10" s="45" t="n"/>
+      <c r="W10" s="45" t="n"/>
+      <c r="X10" s="46">
+        <f>IF(COUNT(T10:W10)=0,"",IFERROR(SUMPRODUCT(T10:W10,(T$5:W$5+(T$5:W$5="")))/SUMPRODUCT((T10:W10&lt;&gt;"")*(T$5:W$5+(T$5:W$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="Y10" s="45" t="n"/>
+      <c r="Z10" s="45" t="n"/>
+      <c r="AA10" s="46">
+        <f>IF(COUNT(Y10:Z10)=0,"",IFERROR(SUMPRODUCT(Y10:Z10,(Y$5:Z$5+(Y$5:Z$5="")))/SUMPRODUCT((Y10:Z10&lt;&gt;"")*(Y$5:Z$5+(Y$5:Z$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="AB10" s="46">
+        <f>IFERROR(IF((ISNUMBER(S10)*(S$5+(S$5=""))+ISNUMBER(X10)*(X$5+(X$5=""))+ISNUMBER(AA10)*(AA$5+(AA$5="")))=0,"",(N(S10)*(S$5+(S$5=""))+N(X10)*(X$5+(X$5=""))+N(AA10)*(AA$5+(AA$5="")))/(ISNUMBER(S10)*(S$5+(S$5=""))+ISNUMBER(X10)*(X$5+(X$5=""))+ISNUMBER(AA10)*(AA$5+(AA$5="")))),"")</f>
+        <v/>
+      </c>
+      <c r="AC10" s="47">
+        <f>IF(AND(ISNUMBER(O10),ISNUMBER(AB10)),O10*AB10,"")</f>
+        <v/>
+      </c>
+      <c r="AD10" s="48">
+        <f>IF(ISNUMBER(AC10),(AC10-1)/24,"")</f>
+        <v/>
+      </c>
+      <c r="AE10" s="49">
+        <f>IF(ISNUMBER(AC10),COUNTIF(AC$7:AC$27,"&gt;"&amp;AC10)+1,"")</f>
+        <v/>
+      </c>
+      <c r="AF10" s="50">
+        <f>COUNT(I10,J10,K10,L10,M10,N10,P10,Q10,R10,T10,U10,V10,W10,Y10,Z10)</f>
         <v/>
       </c>
     </row>
@@ -2900,55 +2967,66 @@
           <t>G3</t>
         </is>
       </c>
-      <c r="F11" s="44" t="n"/>
-      <c r="G11" s="44" t="n"/>
-      <c r="H11" s="44" t="n"/>
-      <c r="I11" s="44" t="n"/>
-      <c r="J11" s="44" t="n"/>
-      <c r="K11" s="44" t="n"/>
-      <c r="L11" s="45">
-        <f>IF(COUNT(F11:K11)=0,"",IFERROR(SUMPRODUCT(F11:K11,(F$5:K$5+(F$5:K$5="")))/SUMPRODUCT((F11:K11&lt;&gt;"")*(F$5:K$5+(F$5:K$5=""))),""))</f>
-        <v/>
-      </c>
-      <c r="M11" s="44" t="n"/>
-      <c r="N11" s="44" t="n"/>
-      <c r="O11" s="44" t="n"/>
-      <c r="P11" s="45">
-        <f>IF(COUNT(M11:O11)=0,"",IFERROR(SUMPRODUCT(M11:O11,(M$5:O$5+(M$5:O$5="")))/SUMPRODUCT((M11:O11&lt;&gt;"")*(M$5:O$5+(M$5:O$5=""))),""))</f>
-        <v/>
-      </c>
-      <c r="Q11" s="44" t="n"/>
-      <c r="R11" s="44" t="n"/>
-      <c r="S11" s="44" t="n"/>
-      <c r="T11" s="44" t="n"/>
-      <c r="U11" s="45">
-        <f>IF(COUNT(Q11:T11)=0,"",IFERROR(SUMPRODUCT(Q11:T11,(Q$5:T$5+(Q$5:T$5="")))/SUMPRODUCT((Q11:T11&lt;&gt;"")*(Q$5:T$5+(Q$5:T$5=""))),""))</f>
-        <v/>
-      </c>
-      <c r="V11" s="44" t="n"/>
-      <c r="W11" s="44" t="n"/>
-      <c r="X11" s="45">
-        <f>IF(COUNT(V11:W11)=0,"",IFERROR(SUMPRODUCT(V11:W11,(V$5:W$5+(V$5:W$5="")))/SUMPRODUCT((V11:W11&lt;&gt;"")*(V$5:W$5+(V$5:W$5=""))),""))</f>
-        <v/>
-      </c>
-      <c r="Y11" s="45">
-        <f>IFERROR(IF((ISNUMBER(P11)*(P$5+(P$5=""))+ISNUMBER(U11)*(U$5+(U$5=""))+ISNUMBER(X11)*(X$5+(X$5="")))=0,"",(N(P11)*(P$5+(P$5=""))+N(U11)*(U$5+(U$5=""))+N(X11)*(X$5+(X$5="")))/(ISNUMBER(P11)*(P$5+(P$5=""))+ISNUMBER(U11)*(U$5+(U$5=""))+ISNUMBER(X11)*(X$5+(X$5="")))),"")</f>
-        <v/>
-      </c>
-      <c r="Z11" s="46">
-        <f>IF(AND(ISNUMBER(L11),ISNUMBER(Y11)),L11*Y11,"")</f>
-        <v/>
-      </c>
-      <c r="AA11" s="47">
-        <f>IF(ISNUMBER(Z11),(Z11-1)/24,"")</f>
-        <v/>
-      </c>
-      <c r="AB11" s="48">
-        <f>IF(ISNUMBER(Z11),COUNTIF(Z$7:Z$27,"&gt;"&amp;Z11)+1,"")</f>
-        <v/>
-      </c>
-      <c r="AC11" s="49">
-        <f>COUNT(F11,G11,H11,I11,J11,K11,M11,N11,O11,Q11,R11,S11,T11,V11,W11)</f>
+      <c r="F11" s="44" t="n">
+        <v>-8.108934</v>
+      </c>
+      <c r="G11" s="44" t="n">
+        <v>-34.911777</v>
+      </c>
+      <c r="H11" s="42" t="inlineStr">
+        <is>
+          <t>Interseção</t>
+        </is>
+      </c>
+      <c r="I11" s="45" t="n"/>
+      <c r="J11" s="45" t="n"/>
+      <c r="K11" s="45" t="n"/>
+      <c r="L11" s="45" t="n"/>
+      <c r="M11" s="45" t="n"/>
+      <c r="N11" s="45" t="n"/>
+      <c r="O11" s="46">
+        <f>IF(COUNT(I11:N11)=0,"",IFERROR(SUMPRODUCT(I11:N11,(I$5:N$5+(I$5:N$5="")))/SUMPRODUCT((I11:N11&lt;&gt;"")*(I$5:N$5+(I$5:N$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="P11" s="45" t="n"/>
+      <c r="Q11" s="45" t="n"/>
+      <c r="R11" s="45" t="n"/>
+      <c r="S11" s="46">
+        <f>IF(COUNT(P11:R11)=0,"",IFERROR(SUMPRODUCT(P11:R11,(P$5:R$5+(P$5:R$5="")))/SUMPRODUCT((P11:R11&lt;&gt;"")*(P$5:R$5+(P$5:R$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="T11" s="45" t="n"/>
+      <c r="U11" s="45" t="n"/>
+      <c r="V11" s="45" t="n"/>
+      <c r="W11" s="45" t="n"/>
+      <c r="X11" s="46">
+        <f>IF(COUNT(T11:W11)=0,"",IFERROR(SUMPRODUCT(T11:W11,(T$5:W$5+(T$5:W$5="")))/SUMPRODUCT((T11:W11&lt;&gt;"")*(T$5:W$5+(T$5:W$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="Y11" s="45" t="n"/>
+      <c r="Z11" s="45" t="n"/>
+      <c r="AA11" s="46">
+        <f>IF(COUNT(Y11:Z11)=0,"",IFERROR(SUMPRODUCT(Y11:Z11,(Y$5:Z$5+(Y$5:Z$5="")))/SUMPRODUCT((Y11:Z11&lt;&gt;"")*(Y$5:Z$5+(Y$5:Z$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="AB11" s="46">
+        <f>IFERROR(IF((ISNUMBER(S11)*(S$5+(S$5=""))+ISNUMBER(X11)*(X$5+(X$5=""))+ISNUMBER(AA11)*(AA$5+(AA$5="")))=0,"",(N(S11)*(S$5+(S$5=""))+N(X11)*(X$5+(X$5=""))+N(AA11)*(AA$5+(AA$5="")))/(ISNUMBER(S11)*(S$5+(S$5=""))+ISNUMBER(X11)*(X$5+(X$5=""))+ISNUMBER(AA11)*(AA$5+(AA$5="")))),"")</f>
+        <v/>
+      </c>
+      <c r="AC11" s="47">
+        <f>IF(AND(ISNUMBER(O11),ISNUMBER(AB11)),O11*AB11,"")</f>
+        <v/>
+      </c>
+      <c r="AD11" s="48">
+        <f>IF(ISNUMBER(AC11),(AC11-1)/24,"")</f>
+        <v/>
+      </c>
+      <c r="AE11" s="49">
+        <f>IF(ISNUMBER(AC11),COUNTIF(AC$7:AC$27,"&gt;"&amp;AC11)+1,"")</f>
+        <v/>
+      </c>
+      <c r="AF11" s="50">
+        <f>COUNT(I11,J11,K11,L11,M11,N11,P11,Q11,R11,T11,U11,V11,W11,Y11,Z11)</f>
         <v/>
       </c>
     </row>
@@ -2976,55 +3054,66 @@
           <t>G1</t>
         </is>
       </c>
-      <c r="F12" s="44" t="n"/>
-      <c r="G12" s="44" t="n"/>
-      <c r="H12" s="44" t="n"/>
-      <c r="I12" s="44" t="n"/>
-      <c r="J12" s="44" t="n"/>
-      <c r="K12" s="44" t="n"/>
-      <c r="L12" s="45">
-        <f>IF(COUNT(F12:K12)=0,"",IFERROR(SUMPRODUCT(F12:K12,(F$5:K$5+(F$5:K$5="")))/SUMPRODUCT((F12:K12&lt;&gt;"")*(F$5:K$5+(F$5:K$5=""))),""))</f>
-        <v/>
-      </c>
-      <c r="M12" s="44" t="n"/>
-      <c r="N12" s="44" t="n"/>
-      <c r="O12" s="44" t="n"/>
-      <c r="P12" s="45">
-        <f>IF(COUNT(M12:O12)=0,"",IFERROR(SUMPRODUCT(M12:O12,(M$5:O$5+(M$5:O$5="")))/SUMPRODUCT((M12:O12&lt;&gt;"")*(M$5:O$5+(M$5:O$5=""))),""))</f>
-        <v/>
-      </c>
-      <c r="Q12" s="44" t="n"/>
-      <c r="R12" s="44" t="n"/>
-      <c r="S12" s="44" t="n"/>
-      <c r="T12" s="44" t="n"/>
-      <c r="U12" s="45">
-        <f>IF(COUNT(Q12:T12)=0,"",IFERROR(SUMPRODUCT(Q12:T12,(Q$5:T$5+(Q$5:T$5="")))/SUMPRODUCT((Q12:T12&lt;&gt;"")*(Q$5:T$5+(Q$5:T$5=""))),""))</f>
-        <v/>
-      </c>
-      <c r="V12" s="44" t="n"/>
-      <c r="W12" s="44" t="n"/>
-      <c r="X12" s="45">
-        <f>IF(COUNT(V12:W12)=0,"",IFERROR(SUMPRODUCT(V12:W12,(V$5:W$5+(V$5:W$5="")))/SUMPRODUCT((V12:W12&lt;&gt;"")*(V$5:W$5+(V$5:W$5=""))),""))</f>
-        <v/>
-      </c>
-      <c r="Y12" s="45">
-        <f>IFERROR(IF((ISNUMBER(P12)*(P$5+(P$5=""))+ISNUMBER(U12)*(U$5+(U$5=""))+ISNUMBER(X12)*(X$5+(X$5="")))=0,"",(N(P12)*(P$5+(P$5=""))+N(U12)*(U$5+(U$5=""))+N(X12)*(X$5+(X$5="")))/(ISNUMBER(P12)*(P$5+(P$5=""))+ISNUMBER(U12)*(U$5+(U$5=""))+ISNUMBER(X12)*(X$5+(X$5="")))),"")</f>
-        <v/>
-      </c>
-      <c r="Z12" s="46">
-        <f>IF(AND(ISNUMBER(L12),ISNUMBER(Y12)),L12*Y12,"")</f>
-        <v/>
-      </c>
-      <c r="AA12" s="47">
-        <f>IF(ISNUMBER(Z12),(Z12-1)/24,"")</f>
-        <v/>
-      </c>
-      <c r="AB12" s="48">
-        <f>IF(ISNUMBER(Z12),COUNTIF(Z$7:Z$27,"&gt;"&amp;Z12)+1,"")</f>
-        <v/>
-      </c>
-      <c r="AC12" s="49">
-        <f>COUNT(F12,G12,H12,I12,J12,K12,M12,N12,O12,Q12,R12,S12,T12,V12,W12)</f>
+      <c r="F12" s="44" t="n">
+        <v>-8.111815999999999</v>
+      </c>
+      <c r="G12" s="44" t="n">
+        <v>-34.894789</v>
+      </c>
+      <c r="H12" s="42" t="inlineStr">
+        <is>
+          <t>Aproximado</t>
+        </is>
+      </c>
+      <c r="I12" s="45" t="n"/>
+      <c r="J12" s="45" t="n"/>
+      <c r="K12" s="45" t="n"/>
+      <c r="L12" s="45" t="n"/>
+      <c r="M12" s="45" t="n"/>
+      <c r="N12" s="45" t="n"/>
+      <c r="O12" s="46">
+        <f>IF(COUNT(I12:N12)=0,"",IFERROR(SUMPRODUCT(I12:N12,(I$5:N$5+(I$5:N$5="")))/SUMPRODUCT((I12:N12&lt;&gt;"")*(I$5:N$5+(I$5:N$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="P12" s="45" t="n"/>
+      <c r="Q12" s="45" t="n"/>
+      <c r="R12" s="45" t="n"/>
+      <c r="S12" s="46">
+        <f>IF(COUNT(P12:R12)=0,"",IFERROR(SUMPRODUCT(P12:R12,(P$5:R$5+(P$5:R$5="")))/SUMPRODUCT((P12:R12&lt;&gt;"")*(P$5:R$5+(P$5:R$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="T12" s="45" t="n"/>
+      <c r="U12" s="45" t="n"/>
+      <c r="V12" s="45" t="n"/>
+      <c r="W12" s="45" t="n"/>
+      <c r="X12" s="46">
+        <f>IF(COUNT(T12:W12)=0,"",IFERROR(SUMPRODUCT(T12:W12,(T$5:W$5+(T$5:W$5="")))/SUMPRODUCT((T12:W12&lt;&gt;"")*(T$5:W$5+(T$5:W$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="Y12" s="45" t="n"/>
+      <c r="Z12" s="45" t="n"/>
+      <c r="AA12" s="46">
+        <f>IF(COUNT(Y12:Z12)=0,"",IFERROR(SUMPRODUCT(Y12:Z12,(Y$5:Z$5+(Y$5:Z$5="")))/SUMPRODUCT((Y12:Z12&lt;&gt;"")*(Y$5:Z$5+(Y$5:Z$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="AB12" s="46">
+        <f>IFERROR(IF((ISNUMBER(S12)*(S$5+(S$5=""))+ISNUMBER(X12)*(X$5+(X$5=""))+ISNUMBER(AA12)*(AA$5+(AA$5="")))=0,"",(N(S12)*(S$5+(S$5=""))+N(X12)*(X$5+(X$5=""))+N(AA12)*(AA$5+(AA$5="")))/(ISNUMBER(S12)*(S$5+(S$5=""))+ISNUMBER(X12)*(X$5+(X$5=""))+ISNUMBER(AA12)*(AA$5+(AA$5="")))),"")</f>
+        <v/>
+      </c>
+      <c r="AC12" s="47">
+        <f>IF(AND(ISNUMBER(O12),ISNUMBER(AB12)),O12*AB12,"")</f>
+        <v/>
+      </c>
+      <c r="AD12" s="48">
+        <f>IF(ISNUMBER(AC12),(AC12-1)/24,"")</f>
+        <v/>
+      </c>
+      <c r="AE12" s="49">
+        <f>IF(ISNUMBER(AC12),COUNTIF(AC$7:AC$27,"&gt;"&amp;AC12)+1,"")</f>
+        <v/>
+      </c>
+      <c r="AF12" s="50">
+        <f>COUNT(I12,J12,K12,L12,M12,N12,P12,Q12,R12,T12,U12,V12,W12,Y12,Z12)</f>
         <v/>
       </c>
     </row>
@@ -3052,55 +3141,66 @@
           <t>G1</t>
         </is>
       </c>
-      <c r="F13" s="44" t="n"/>
-      <c r="G13" s="44" t="n"/>
-      <c r="H13" s="44" t="n"/>
-      <c r="I13" s="44" t="n"/>
-      <c r="J13" s="44" t="n"/>
-      <c r="K13" s="44" t="n"/>
-      <c r="L13" s="45">
-        <f>IF(COUNT(F13:K13)=0,"",IFERROR(SUMPRODUCT(F13:K13,(F$5:K$5+(F$5:K$5="")))/SUMPRODUCT((F13:K13&lt;&gt;"")*(F$5:K$5+(F$5:K$5=""))),""))</f>
-        <v/>
-      </c>
-      <c r="M13" s="44" t="n"/>
-      <c r="N13" s="44" t="n"/>
-      <c r="O13" s="44" t="n"/>
-      <c r="P13" s="45">
-        <f>IF(COUNT(M13:O13)=0,"",IFERROR(SUMPRODUCT(M13:O13,(M$5:O$5+(M$5:O$5="")))/SUMPRODUCT((M13:O13&lt;&gt;"")*(M$5:O$5+(M$5:O$5=""))),""))</f>
-        <v/>
-      </c>
-      <c r="Q13" s="44" t="n"/>
-      <c r="R13" s="44" t="n"/>
-      <c r="S13" s="44" t="n"/>
-      <c r="T13" s="44" t="n"/>
-      <c r="U13" s="45">
-        <f>IF(COUNT(Q13:T13)=0,"",IFERROR(SUMPRODUCT(Q13:T13,(Q$5:T$5+(Q$5:T$5="")))/SUMPRODUCT((Q13:T13&lt;&gt;"")*(Q$5:T$5+(Q$5:T$5=""))),""))</f>
-        <v/>
-      </c>
-      <c r="V13" s="44" t="n"/>
-      <c r="W13" s="44" t="n"/>
-      <c r="X13" s="45">
-        <f>IF(COUNT(V13:W13)=0,"",IFERROR(SUMPRODUCT(V13:W13,(V$5:W$5+(V$5:W$5="")))/SUMPRODUCT((V13:W13&lt;&gt;"")*(V$5:W$5+(V$5:W$5=""))),""))</f>
-        <v/>
-      </c>
-      <c r="Y13" s="45">
-        <f>IFERROR(IF((ISNUMBER(P13)*(P$5+(P$5=""))+ISNUMBER(U13)*(U$5+(U$5=""))+ISNUMBER(X13)*(X$5+(X$5="")))=0,"",(N(P13)*(P$5+(P$5=""))+N(U13)*(U$5+(U$5=""))+N(X13)*(X$5+(X$5="")))/(ISNUMBER(P13)*(P$5+(P$5=""))+ISNUMBER(U13)*(U$5+(U$5=""))+ISNUMBER(X13)*(X$5+(X$5="")))),"")</f>
-        <v/>
-      </c>
-      <c r="Z13" s="46">
-        <f>IF(AND(ISNUMBER(L13),ISNUMBER(Y13)),L13*Y13,"")</f>
-        <v/>
-      </c>
-      <c r="AA13" s="47">
-        <f>IF(ISNUMBER(Z13),(Z13-1)/24,"")</f>
-        <v/>
-      </c>
-      <c r="AB13" s="48">
-        <f>IF(ISNUMBER(Z13),COUNTIF(Z$7:Z$27,"&gt;"&amp;Z13)+1,"")</f>
-        <v/>
-      </c>
-      <c r="AC13" s="49">
-        <f>COUNT(F13,G13,H13,I13,J13,K13,M13,N13,O13,Q13,R13,S13,T13,V13,W13)</f>
+      <c r="F13" s="44" t="n">
+        <v>-8.112935</v>
+      </c>
+      <c r="G13" s="44" t="n">
+        <v>-34.896796</v>
+      </c>
+      <c r="H13" s="42" t="inlineStr">
+        <is>
+          <t>Aproximado</t>
+        </is>
+      </c>
+      <c r="I13" s="45" t="n"/>
+      <c r="J13" s="45" t="n"/>
+      <c r="K13" s="45" t="n"/>
+      <c r="L13" s="45" t="n"/>
+      <c r="M13" s="45" t="n"/>
+      <c r="N13" s="45" t="n"/>
+      <c r="O13" s="46">
+        <f>IF(COUNT(I13:N13)=0,"",IFERROR(SUMPRODUCT(I13:N13,(I$5:N$5+(I$5:N$5="")))/SUMPRODUCT((I13:N13&lt;&gt;"")*(I$5:N$5+(I$5:N$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="P13" s="45" t="n"/>
+      <c r="Q13" s="45" t="n"/>
+      <c r="R13" s="45" t="n"/>
+      <c r="S13" s="46">
+        <f>IF(COUNT(P13:R13)=0,"",IFERROR(SUMPRODUCT(P13:R13,(P$5:R$5+(P$5:R$5="")))/SUMPRODUCT((P13:R13&lt;&gt;"")*(P$5:R$5+(P$5:R$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="T13" s="45" t="n"/>
+      <c r="U13" s="45" t="n"/>
+      <c r="V13" s="45" t="n"/>
+      <c r="W13" s="45" t="n"/>
+      <c r="X13" s="46">
+        <f>IF(COUNT(T13:W13)=0,"",IFERROR(SUMPRODUCT(T13:W13,(T$5:W$5+(T$5:W$5="")))/SUMPRODUCT((T13:W13&lt;&gt;"")*(T$5:W$5+(T$5:W$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="Y13" s="45" t="n"/>
+      <c r="Z13" s="45" t="n"/>
+      <c r="AA13" s="46">
+        <f>IF(COUNT(Y13:Z13)=0,"",IFERROR(SUMPRODUCT(Y13:Z13,(Y$5:Z$5+(Y$5:Z$5="")))/SUMPRODUCT((Y13:Z13&lt;&gt;"")*(Y$5:Z$5+(Y$5:Z$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="AB13" s="46">
+        <f>IFERROR(IF((ISNUMBER(S13)*(S$5+(S$5=""))+ISNUMBER(X13)*(X$5+(X$5=""))+ISNUMBER(AA13)*(AA$5+(AA$5="")))=0,"",(N(S13)*(S$5+(S$5=""))+N(X13)*(X$5+(X$5=""))+N(AA13)*(AA$5+(AA$5="")))/(ISNUMBER(S13)*(S$5+(S$5=""))+ISNUMBER(X13)*(X$5+(X$5=""))+ISNUMBER(AA13)*(AA$5+(AA$5="")))),"")</f>
+        <v/>
+      </c>
+      <c r="AC13" s="47">
+        <f>IF(AND(ISNUMBER(O13),ISNUMBER(AB13)),O13*AB13,"")</f>
+        <v/>
+      </c>
+      <c r="AD13" s="48">
+        <f>IF(ISNUMBER(AC13),(AC13-1)/24,"")</f>
+        <v/>
+      </c>
+      <c r="AE13" s="49">
+        <f>IF(ISNUMBER(AC13),COUNTIF(AC$7:AC$27,"&gt;"&amp;AC13)+1,"")</f>
+        <v/>
+      </c>
+      <c r="AF13" s="50">
+        <f>COUNT(I13,J13,K13,L13,M13,N13,P13,Q13,R13,T13,U13,V13,W13,Y13,Z13)</f>
         <v/>
       </c>
     </row>
@@ -3124,55 +3224,66 @@
         </is>
       </c>
       <c r="E14" s="42" t="inlineStr"/>
-      <c r="F14" s="44" t="n"/>
-      <c r="G14" s="44" t="n"/>
-      <c r="H14" s="44" t="n"/>
-      <c r="I14" s="44" t="n"/>
-      <c r="J14" s="44" t="n"/>
-      <c r="K14" s="44" t="n"/>
-      <c r="L14" s="45">
-        <f>IF(COUNT(F14:K14)=0,"",IFERROR(SUMPRODUCT(F14:K14,(F$5:K$5+(F$5:K$5="")))/SUMPRODUCT((F14:K14&lt;&gt;"")*(F$5:K$5+(F$5:K$5=""))),""))</f>
-        <v/>
-      </c>
-      <c r="M14" s="44" t="n"/>
-      <c r="N14" s="44" t="n"/>
-      <c r="O14" s="44" t="n"/>
-      <c r="P14" s="45">
-        <f>IF(COUNT(M14:O14)=0,"",IFERROR(SUMPRODUCT(M14:O14,(M$5:O$5+(M$5:O$5="")))/SUMPRODUCT((M14:O14&lt;&gt;"")*(M$5:O$5+(M$5:O$5=""))),""))</f>
-        <v/>
-      </c>
-      <c r="Q14" s="44" t="n"/>
-      <c r="R14" s="44" t="n"/>
-      <c r="S14" s="44" t="n"/>
-      <c r="T14" s="44" t="n"/>
-      <c r="U14" s="45">
-        <f>IF(COUNT(Q14:T14)=0,"",IFERROR(SUMPRODUCT(Q14:T14,(Q$5:T$5+(Q$5:T$5="")))/SUMPRODUCT((Q14:T14&lt;&gt;"")*(Q$5:T$5+(Q$5:T$5=""))),""))</f>
-        <v/>
-      </c>
-      <c r="V14" s="44" t="n"/>
-      <c r="W14" s="44" t="n"/>
-      <c r="X14" s="45">
-        <f>IF(COUNT(V14:W14)=0,"",IFERROR(SUMPRODUCT(V14:W14,(V$5:W$5+(V$5:W$5="")))/SUMPRODUCT((V14:W14&lt;&gt;"")*(V$5:W$5+(V$5:W$5=""))),""))</f>
-        <v/>
-      </c>
-      <c r="Y14" s="45">
-        <f>IFERROR(IF((ISNUMBER(P14)*(P$5+(P$5=""))+ISNUMBER(U14)*(U$5+(U$5=""))+ISNUMBER(X14)*(X$5+(X$5="")))=0,"",(N(P14)*(P$5+(P$5=""))+N(U14)*(U$5+(U$5=""))+N(X14)*(X$5+(X$5="")))/(ISNUMBER(P14)*(P$5+(P$5=""))+ISNUMBER(U14)*(U$5+(U$5=""))+ISNUMBER(X14)*(X$5+(X$5="")))),"")</f>
-        <v/>
-      </c>
-      <c r="Z14" s="46">
-        <f>IF(AND(ISNUMBER(L14),ISNUMBER(Y14)),L14*Y14,"")</f>
-        <v/>
-      </c>
-      <c r="AA14" s="47">
-        <f>IF(ISNUMBER(Z14),(Z14-1)/24,"")</f>
-        <v/>
-      </c>
-      <c r="AB14" s="48">
-        <f>IF(ISNUMBER(Z14),COUNTIF(Z$7:Z$27,"&gt;"&amp;Z14)+1,"")</f>
-        <v/>
-      </c>
-      <c r="AC14" s="49">
-        <f>COUNT(F14,G14,H14,I14,J14,K14,M14,N14,O14,Q14,R14,S14,T14,V14,W14)</f>
+      <c r="F14" s="44" t="n">
+        <v>-8.138795999999999</v>
+      </c>
+      <c r="G14" s="44" t="n">
+        <v>-34.913979</v>
+      </c>
+      <c r="H14" s="42" t="inlineStr">
+        <is>
+          <t>Aproximado</t>
+        </is>
+      </c>
+      <c r="I14" s="45" t="n"/>
+      <c r="J14" s="45" t="n"/>
+      <c r="K14" s="45" t="n"/>
+      <c r="L14" s="45" t="n"/>
+      <c r="M14" s="45" t="n"/>
+      <c r="N14" s="45" t="n"/>
+      <c r="O14" s="46">
+        <f>IF(COUNT(I14:N14)=0,"",IFERROR(SUMPRODUCT(I14:N14,(I$5:N$5+(I$5:N$5="")))/SUMPRODUCT((I14:N14&lt;&gt;"")*(I$5:N$5+(I$5:N$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="P14" s="45" t="n"/>
+      <c r="Q14" s="45" t="n"/>
+      <c r="R14" s="45" t="n"/>
+      <c r="S14" s="46">
+        <f>IF(COUNT(P14:R14)=0,"",IFERROR(SUMPRODUCT(P14:R14,(P$5:R$5+(P$5:R$5="")))/SUMPRODUCT((P14:R14&lt;&gt;"")*(P$5:R$5+(P$5:R$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="T14" s="45" t="n"/>
+      <c r="U14" s="45" t="n"/>
+      <c r="V14" s="45" t="n"/>
+      <c r="W14" s="45" t="n"/>
+      <c r="X14" s="46">
+        <f>IF(COUNT(T14:W14)=0,"",IFERROR(SUMPRODUCT(T14:W14,(T$5:W$5+(T$5:W$5="")))/SUMPRODUCT((T14:W14&lt;&gt;"")*(T$5:W$5+(T$5:W$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="Y14" s="45" t="n"/>
+      <c r="Z14" s="45" t="n"/>
+      <c r="AA14" s="46">
+        <f>IF(COUNT(Y14:Z14)=0,"",IFERROR(SUMPRODUCT(Y14:Z14,(Y$5:Z$5+(Y$5:Z$5="")))/SUMPRODUCT((Y14:Z14&lt;&gt;"")*(Y$5:Z$5+(Y$5:Z$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="AB14" s="46">
+        <f>IFERROR(IF((ISNUMBER(S14)*(S$5+(S$5=""))+ISNUMBER(X14)*(X$5+(X$5=""))+ISNUMBER(AA14)*(AA$5+(AA$5="")))=0,"",(N(S14)*(S$5+(S$5=""))+N(X14)*(X$5+(X$5=""))+N(AA14)*(AA$5+(AA$5="")))/(ISNUMBER(S14)*(S$5+(S$5=""))+ISNUMBER(X14)*(X$5+(X$5=""))+ISNUMBER(AA14)*(AA$5+(AA$5="")))),"")</f>
+        <v/>
+      </c>
+      <c r="AC14" s="47">
+        <f>IF(AND(ISNUMBER(O14),ISNUMBER(AB14)),O14*AB14,"")</f>
+        <v/>
+      </c>
+      <c r="AD14" s="48">
+        <f>IF(ISNUMBER(AC14),(AC14-1)/24,"")</f>
+        <v/>
+      </c>
+      <c r="AE14" s="49">
+        <f>IF(ISNUMBER(AC14),COUNTIF(AC$7:AC$27,"&gt;"&amp;AC14)+1,"")</f>
+        <v/>
+      </c>
+      <c r="AF14" s="50">
+        <f>COUNT(I14,J14,K14,L14,M14,N14,P14,Q14,R14,T14,U14,V14,W14,Y14,Z14)</f>
         <v/>
       </c>
     </row>
@@ -3196,55 +3307,66 @@
         </is>
       </c>
       <c r="E15" s="42" t="inlineStr"/>
-      <c r="F15" s="44" t="n"/>
-      <c r="G15" s="44" t="n"/>
-      <c r="H15" s="44" t="n"/>
-      <c r="I15" s="44" t="n"/>
-      <c r="J15" s="44" t="n"/>
-      <c r="K15" s="44" t="n"/>
-      <c r="L15" s="45">
-        <f>IF(COUNT(F15:K15)=0,"",IFERROR(SUMPRODUCT(F15:K15,(F$5:K$5+(F$5:K$5="")))/SUMPRODUCT((F15:K15&lt;&gt;"")*(F$5:K$5+(F$5:K$5=""))),""))</f>
-        <v/>
-      </c>
-      <c r="M15" s="44" t="n"/>
-      <c r="N15" s="44" t="n"/>
-      <c r="O15" s="44" t="n"/>
-      <c r="P15" s="45">
-        <f>IF(COUNT(M15:O15)=0,"",IFERROR(SUMPRODUCT(M15:O15,(M$5:O$5+(M$5:O$5="")))/SUMPRODUCT((M15:O15&lt;&gt;"")*(M$5:O$5+(M$5:O$5=""))),""))</f>
-        <v/>
-      </c>
-      <c r="Q15" s="44" t="n"/>
-      <c r="R15" s="44" t="n"/>
-      <c r="S15" s="44" t="n"/>
-      <c r="T15" s="44" t="n"/>
-      <c r="U15" s="45">
-        <f>IF(COUNT(Q15:T15)=0,"",IFERROR(SUMPRODUCT(Q15:T15,(Q$5:T$5+(Q$5:T$5="")))/SUMPRODUCT((Q15:T15&lt;&gt;"")*(Q$5:T$5+(Q$5:T$5=""))),""))</f>
-        <v/>
-      </c>
-      <c r="V15" s="44" t="n"/>
-      <c r="W15" s="44" t="n"/>
-      <c r="X15" s="45">
-        <f>IF(COUNT(V15:W15)=0,"",IFERROR(SUMPRODUCT(V15:W15,(V$5:W$5+(V$5:W$5="")))/SUMPRODUCT((V15:W15&lt;&gt;"")*(V$5:W$5+(V$5:W$5=""))),""))</f>
-        <v/>
-      </c>
-      <c r="Y15" s="45">
-        <f>IFERROR(IF((ISNUMBER(P15)*(P$5+(P$5=""))+ISNUMBER(U15)*(U$5+(U$5=""))+ISNUMBER(X15)*(X$5+(X$5="")))=0,"",(N(P15)*(P$5+(P$5=""))+N(U15)*(U$5+(U$5=""))+N(X15)*(X$5+(X$5="")))/(ISNUMBER(P15)*(P$5+(P$5=""))+ISNUMBER(U15)*(U$5+(U$5=""))+ISNUMBER(X15)*(X$5+(X$5="")))),"")</f>
-        <v/>
-      </c>
-      <c r="Z15" s="46">
-        <f>IF(AND(ISNUMBER(L15),ISNUMBER(Y15)),L15*Y15,"")</f>
-        <v/>
-      </c>
-      <c r="AA15" s="47">
-        <f>IF(ISNUMBER(Z15),(Z15-1)/24,"")</f>
-        <v/>
-      </c>
-      <c r="AB15" s="48">
-        <f>IF(ISNUMBER(Z15),COUNTIF(Z$7:Z$27,"&gt;"&amp;Z15)+1,"")</f>
-        <v/>
-      </c>
-      <c r="AC15" s="49">
-        <f>COUNT(F15,G15,H15,I15,J15,K15,M15,N15,O15,Q15,R15,S15,T15,V15,W15)</f>
+      <c r="F15" s="44" t="n">
+        <v>-8.089715999999999</v>
+      </c>
+      <c r="G15" s="44" t="n">
+        <v>-34.888275</v>
+      </c>
+      <c r="H15" s="42" t="inlineStr">
+        <is>
+          <t>Aproximado</t>
+        </is>
+      </c>
+      <c r="I15" s="45" t="n"/>
+      <c r="J15" s="45" t="n"/>
+      <c r="K15" s="45" t="n"/>
+      <c r="L15" s="45" t="n"/>
+      <c r="M15" s="45" t="n"/>
+      <c r="N15" s="45" t="n"/>
+      <c r="O15" s="46">
+        <f>IF(COUNT(I15:N15)=0,"",IFERROR(SUMPRODUCT(I15:N15,(I$5:N$5+(I$5:N$5="")))/SUMPRODUCT((I15:N15&lt;&gt;"")*(I$5:N$5+(I$5:N$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="P15" s="45" t="n"/>
+      <c r="Q15" s="45" t="n"/>
+      <c r="R15" s="45" t="n"/>
+      <c r="S15" s="46">
+        <f>IF(COUNT(P15:R15)=0,"",IFERROR(SUMPRODUCT(P15:R15,(P$5:R$5+(P$5:R$5="")))/SUMPRODUCT((P15:R15&lt;&gt;"")*(P$5:R$5+(P$5:R$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="T15" s="45" t="n"/>
+      <c r="U15" s="45" t="n"/>
+      <c r="V15" s="45" t="n"/>
+      <c r="W15" s="45" t="n"/>
+      <c r="X15" s="46">
+        <f>IF(COUNT(T15:W15)=0,"",IFERROR(SUMPRODUCT(T15:W15,(T$5:W$5+(T$5:W$5="")))/SUMPRODUCT((T15:W15&lt;&gt;"")*(T$5:W$5+(T$5:W$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="Y15" s="45" t="n"/>
+      <c r="Z15" s="45" t="n"/>
+      <c r="AA15" s="46">
+        <f>IF(COUNT(Y15:Z15)=0,"",IFERROR(SUMPRODUCT(Y15:Z15,(Y$5:Z$5+(Y$5:Z$5="")))/SUMPRODUCT((Y15:Z15&lt;&gt;"")*(Y$5:Z$5+(Y$5:Z$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="AB15" s="46">
+        <f>IFERROR(IF((ISNUMBER(S15)*(S$5+(S$5=""))+ISNUMBER(X15)*(X$5+(X$5=""))+ISNUMBER(AA15)*(AA$5+(AA$5="")))=0,"",(N(S15)*(S$5+(S$5=""))+N(X15)*(X$5+(X$5=""))+N(AA15)*(AA$5+(AA$5="")))/(ISNUMBER(S15)*(S$5+(S$5=""))+ISNUMBER(X15)*(X$5+(X$5=""))+ISNUMBER(AA15)*(AA$5+(AA$5="")))),"")</f>
+        <v/>
+      </c>
+      <c r="AC15" s="47">
+        <f>IF(AND(ISNUMBER(O15),ISNUMBER(AB15)),O15*AB15,"")</f>
+        <v/>
+      </c>
+      <c r="AD15" s="48">
+        <f>IF(ISNUMBER(AC15),(AC15-1)/24,"")</f>
+        <v/>
+      </c>
+      <c r="AE15" s="49">
+        <f>IF(ISNUMBER(AC15),COUNTIF(AC$7:AC$27,"&gt;"&amp;AC15)+1,"")</f>
+        <v/>
+      </c>
+      <c r="AF15" s="50">
+        <f>COUNT(I15,J15,K15,L15,M15,N15,P15,Q15,R15,T15,U15,V15,W15,Y15,Z15)</f>
         <v/>
       </c>
     </row>
@@ -3268,55 +3390,66 @@
         </is>
       </c>
       <c r="E16" s="42" t="inlineStr"/>
-      <c r="F16" s="44" t="n"/>
-      <c r="G16" s="44" t="n"/>
-      <c r="H16" s="44" t="n"/>
-      <c r="I16" s="44" t="n"/>
-      <c r="J16" s="44" t="n"/>
-      <c r="K16" s="44" t="n"/>
-      <c r="L16" s="45">
-        <f>IF(COUNT(F16:K16)=0,"",IFERROR(SUMPRODUCT(F16:K16,(F$5:K$5+(F$5:K$5="")))/SUMPRODUCT((F16:K16&lt;&gt;"")*(F$5:K$5+(F$5:K$5=""))),""))</f>
-        <v/>
-      </c>
-      <c r="M16" s="44" t="n"/>
-      <c r="N16" s="44" t="n"/>
-      <c r="O16" s="44" t="n"/>
-      <c r="P16" s="45">
-        <f>IF(COUNT(M16:O16)=0,"",IFERROR(SUMPRODUCT(M16:O16,(M$5:O$5+(M$5:O$5="")))/SUMPRODUCT((M16:O16&lt;&gt;"")*(M$5:O$5+(M$5:O$5=""))),""))</f>
-        <v/>
-      </c>
-      <c r="Q16" s="44" t="n"/>
-      <c r="R16" s="44" t="n"/>
-      <c r="S16" s="44" t="n"/>
-      <c r="T16" s="44" t="n"/>
-      <c r="U16" s="45">
-        <f>IF(COUNT(Q16:T16)=0,"",IFERROR(SUMPRODUCT(Q16:T16,(Q$5:T$5+(Q$5:T$5="")))/SUMPRODUCT((Q16:T16&lt;&gt;"")*(Q$5:T$5+(Q$5:T$5=""))),""))</f>
-        <v/>
-      </c>
-      <c r="V16" s="44" t="n"/>
-      <c r="W16" s="44" t="n"/>
-      <c r="X16" s="45">
-        <f>IF(COUNT(V16:W16)=0,"",IFERROR(SUMPRODUCT(V16:W16,(V$5:W$5+(V$5:W$5="")))/SUMPRODUCT((V16:W16&lt;&gt;"")*(V$5:W$5+(V$5:W$5=""))),""))</f>
-        <v/>
-      </c>
-      <c r="Y16" s="45">
-        <f>IFERROR(IF((ISNUMBER(P16)*(P$5+(P$5=""))+ISNUMBER(U16)*(U$5+(U$5=""))+ISNUMBER(X16)*(X$5+(X$5="")))=0,"",(N(P16)*(P$5+(P$5=""))+N(U16)*(U$5+(U$5=""))+N(X16)*(X$5+(X$5="")))/(ISNUMBER(P16)*(P$5+(P$5=""))+ISNUMBER(U16)*(U$5+(U$5=""))+ISNUMBER(X16)*(X$5+(X$5="")))),"")</f>
-        <v/>
-      </c>
-      <c r="Z16" s="46">
-        <f>IF(AND(ISNUMBER(L16),ISNUMBER(Y16)),L16*Y16,"")</f>
-        <v/>
-      </c>
-      <c r="AA16" s="47">
-        <f>IF(ISNUMBER(Z16),(Z16-1)/24,"")</f>
-        <v/>
-      </c>
-      <c r="AB16" s="48">
-        <f>IF(ISNUMBER(Z16),COUNTIF(Z$7:Z$27,"&gt;"&amp;Z16)+1,"")</f>
-        <v/>
-      </c>
-      <c r="AC16" s="49">
-        <f>COUNT(F16,G16,H16,I16,J16,K16,M16,N16,O16,Q16,R16,S16,T16,V16,W16)</f>
+      <c r="F16" s="44" t="n">
+        <v>-8.140504999999999</v>
+      </c>
+      <c r="G16" s="44" t="n">
+        <v>-34.927358</v>
+      </c>
+      <c r="H16" s="42" t="inlineStr">
+        <is>
+          <t>Aproximado</t>
+        </is>
+      </c>
+      <c r="I16" s="45" t="n"/>
+      <c r="J16" s="45" t="n"/>
+      <c r="K16" s="45" t="n"/>
+      <c r="L16" s="45" t="n"/>
+      <c r="M16" s="45" t="n"/>
+      <c r="N16" s="45" t="n"/>
+      <c r="O16" s="46">
+        <f>IF(COUNT(I16:N16)=0,"",IFERROR(SUMPRODUCT(I16:N16,(I$5:N$5+(I$5:N$5="")))/SUMPRODUCT((I16:N16&lt;&gt;"")*(I$5:N$5+(I$5:N$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="P16" s="45" t="n"/>
+      <c r="Q16" s="45" t="n"/>
+      <c r="R16" s="45" t="n"/>
+      <c r="S16" s="46">
+        <f>IF(COUNT(P16:R16)=0,"",IFERROR(SUMPRODUCT(P16:R16,(P$5:R$5+(P$5:R$5="")))/SUMPRODUCT((P16:R16&lt;&gt;"")*(P$5:R$5+(P$5:R$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="T16" s="45" t="n"/>
+      <c r="U16" s="45" t="n"/>
+      <c r="V16" s="45" t="n"/>
+      <c r="W16" s="45" t="n"/>
+      <c r="X16" s="46">
+        <f>IF(COUNT(T16:W16)=0,"",IFERROR(SUMPRODUCT(T16:W16,(T$5:W$5+(T$5:W$5="")))/SUMPRODUCT((T16:W16&lt;&gt;"")*(T$5:W$5+(T$5:W$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="Y16" s="45" t="n"/>
+      <c r="Z16" s="45" t="n"/>
+      <c r="AA16" s="46">
+        <f>IF(COUNT(Y16:Z16)=0,"",IFERROR(SUMPRODUCT(Y16:Z16,(Y$5:Z$5+(Y$5:Z$5="")))/SUMPRODUCT((Y16:Z16&lt;&gt;"")*(Y$5:Z$5+(Y$5:Z$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="AB16" s="46">
+        <f>IFERROR(IF((ISNUMBER(S16)*(S$5+(S$5=""))+ISNUMBER(X16)*(X$5+(X$5=""))+ISNUMBER(AA16)*(AA$5+(AA$5="")))=0,"",(N(S16)*(S$5+(S$5=""))+N(X16)*(X$5+(X$5=""))+N(AA16)*(AA$5+(AA$5="")))/(ISNUMBER(S16)*(S$5+(S$5=""))+ISNUMBER(X16)*(X$5+(X$5=""))+ISNUMBER(AA16)*(AA$5+(AA$5="")))),"")</f>
+        <v/>
+      </c>
+      <c r="AC16" s="47">
+        <f>IF(AND(ISNUMBER(O16),ISNUMBER(AB16)),O16*AB16,"")</f>
+        <v/>
+      </c>
+      <c r="AD16" s="48">
+        <f>IF(ISNUMBER(AC16),(AC16-1)/24,"")</f>
+        <v/>
+      </c>
+      <c r="AE16" s="49">
+        <f>IF(ISNUMBER(AC16),COUNTIF(AC$7:AC$27,"&gt;"&amp;AC16)+1,"")</f>
+        <v/>
+      </c>
+      <c r="AF16" s="50">
+        <f>COUNT(I16,J16,K16,L16,M16,N16,P16,Q16,R16,T16,U16,V16,W16,Y16,Z16)</f>
         <v/>
       </c>
     </row>
@@ -3340,55 +3473,66 @@
         </is>
       </c>
       <c r="E17" s="42" t="inlineStr"/>
-      <c r="F17" s="44" t="n"/>
-      <c r="G17" s="44" t="n"/>
-      <c r="H17" s="44" t="n"/>
-      <c r="I17" s="44" t="n"/>
-      <c r="J17" s="44" t="n"/>
-      <c r="K17" s="44" t="n"/>
-      <c r="L17" s="45">
-        <f>IF(COUNT(F17:K17)=0,"",IFERROR(SUMPRODUCT(F17:K17,(F$5:K$5+(F$5:K$5="")))/SUMPRODUCT((F17:K17&lt;&gt;"")*(F$5:K$5+(F$5:K$5=""))),""))</f>
-        <v/>
-      </c>
-      <c r="M17" s="44" t="n"/>
-      <c r="N17" s="44" t="n"/>
-      <c r="O17" s="44" t="n"/>
-      <c r="P17" s="45">
-        <f>IF(COUNT(M17:O17)=0,"",IFERROR(SUMPRODUCT(M17:O17,(M$5:O$5+(M$5:O$5="")))/SUMPRODUCT((M17:O17&lt;&gt;"")*(M$5:O$5+(M$5:O$5=""))),""))</f>
-        <v/>
-      </c>
-      <c r="Q17" s="44" t="n"/>
-      <c r="R17" s="44" t="n"/>
-      <c r="S17" s="44" t="n"/>
-      <c r="T17" s="44" t="n"/>
-      <c r="U17" s="45">
-        <f>IF(COUNT(Q17:T17)=0,"",IFERROR(SUMPRODUCT(Q17:T17,(Q$5:T$5+(Q$5:T$5="")))/SUMPRODUCT((Q17:T17&lt;&gt;"")*(Q$5:T$5+(Q$5:T$5=""))),""))</f>
-        <v/>
-      </c>
-      <c r="V17" s="44" t="n"/>
-      <c r="W17" s="44" t="n"/>
-      <c r="X17" s="45">
-        <f>IF(COUNT(V17:W17)=0,"",IFERROR(SUMPRODUCT(V17:W17,(V$5:W$5+(V$5:W$5="")))/SUMPRODUCT((V17:W17&lt;&gt;"")*(V$5:W$5+(V$5:W$5=""))),""))</f>
-        <v/>
-      </c>
-      <c r="Y17" s="45">
-        <f>IFERROR(IF((ISNUMBER(P17)*(P$5+(P$5=""))+ISNUMBER(U17)*(U$5+(U$5=""))+ISNUMBER(X17)*(X$5+(X$5="")))=0,"",(N(P17)*(P$5+(P$5=""))+N(U17)*(U$5+(U$5=""))+N(X17)*(X$5+(X$5="")))/(ISNUMBER(P17)*(P$5+(P$5=""))+ISNUMBER(U17)*(U$5+(U$5=""))+ISNUMBER(X17)*(X$5+(X$5="")))),"")</f>
-        <v/>
-      </c>
-      <c r="Z17" s="46">
-        <f>IF(AND(ISNUMBER(L17),ISNUMBER(Y17)),L17*Y17,"")</f>
-        <v/>
-      </c>
-      <c r="AA17" s="47">
-        <f>IF(ISNUMBER(Z17),(Z17-1)/24,"")</f>
-        <v/>
-      </c>
-      <c r="AB17" s="48">
-        <f>IF(ISNUMBER(Z17),COUNTIF(Z$7:Z$27,"&gt;"&amp;Z17)+1,"")</f>
-        <v/>
-      </c>
-      <c r="AC17" s="49">
-        <f>COUNT(F17,G17,H17,I17,J17,K17,M17,N17,O17,Q17,R17,S17,T17,V17,W17)</f>
+      <c r="F17" s="44" t="n">
+        <v>-8.107611</v>
+      </c>
+      <c r="G17" s="44" t="n">
+        <v>-34.920256</v>
+      </c>
+      <c r="H17" s="42" t="inlineStr">
+        <is>
+          <t>Aproximado</t>
+        </is>
+      </c>
+      <c r="I17" s="45" t="n"/>
+      <c r="J17" s="45" t="n"/>
+      <c r="K17" s="45" t="n"/>
+      <c r="L17" s="45" t="n"/>
+      <c r="M17" s="45" t="n"/>
+      <c r="N17" s="45" t="n"/>
+      <c r="O17" s="46">
+        <f>IF(COUNT(I17:N17)=0,"",IFERROR(SUMPRODUCT(I17:N17,(I$5:N$5+(I$5:N$5="")))/SUMPRODUCT((I17:N17&lt;&gt;"")*(I$5:N$5+(I$5:N$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="P17" s="45" t="n"/>
+      <c r="Q17" s="45" t="n"/>
+      <c r="R17" s="45" t="n"/>
+      <c r="S17" s="46">
+        <f>IF(COUNT(P17:R17)=0,"",IFERROR(SUMPRODUCT(P17:R17,(P$5:R$5+(P$5:R$5="")))/SUMPRODUCT((P17:R17&lt;&gt;"")*(P$5:R$5+(P$5:R$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="T17" s="45" t="n"/>
+      <c r="U17" s="45" t="n"/>
+      <c r="V17" s="45" t="n"/>
+      <c r="W17" s="45" t="n"/>
+      <c r="X17" s="46">
+        <f>IF(COUNT(T17:W17)=0,"",IFERROR(SUMPRODUCT(T17:W17,(T$5:W$5+(T$5:W$5="")))/SUMPRODUCT((T17:W17&lt;&gt;"")*(T$5:W$5+(T$5:W$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="Y17" s="45" t="n"/>
+      <c r="Z17" s="45" t="n"/>
+      <c r="AA17" s="46">
+        <f>IF(COUNT(Y17:Z17)=0,"",IFERROR(SUMPRODUCT(Y17:Z17,(Y$5:Z$5+(Y$5:Z$5="")))/SUMPRODUCT((Y17:Z17&lt;&gt;"")*(Y$5:Z$5+(Y$5:Z$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="AB17" s="46">
+        <f>IFERROR(IF((ISNUMBER(S17)*(S$5+(S$5=""))+ISNUMBER(X17)*(X$5+(X$5=""))+ISNUMBER(AA17)*(AA$5+(AA$5="")))=0,"",(N(S17)*(S$5+(S$5=""))+N(X17)*(X$5+(X$5=""))+N(AA17)*(AA$5+(AA$5="")))/(ISNUMBER(S17)*(S$5+(S$5=""))+ISNUMBER(X17)*(X$5+(X$5=""))+ISNUMBER(AA17)*(AA$5+(AA$5="")))),"")</f>
+        <v/>
+      </c>
+      <c r="AC17" s="47">
+        <f>IF(AND(ISNUMBER(O17),ISNUMBER(AB17)),O17*AB17,"")</f>
+        <v/>
+      </c>
+      <c r="AD17" s="48">
+        <f>IF(ISNUMBER(AC17),(AC17-1)/24,"")</f>
+        <v/>
+      </c>
+      <c r="AE17" s="49">
+        <f>IF(ISNUMBER(AC17),COUNTIF(AC$7:AC$27,"&gt;"&amp;AC17)+1,"")</f>
+        <v/>
+      </c>
+      <c r="AF17" s="50">
+        <f>COUNT(I17,J17,K17,L17,M17,N17,P17,Q17,R17,T17,U17,V17,W17,Y17,Z17)</f>
         <v/>
       </c>
     </row>
@@ -3412,55 +3556,66 @@
         </is>
       </c>
       <c r="E18" s="42" t="inlineStr"/>
-      <c r="F18" s="44" t="n"/>
-      <c r="G18" s="44" t="n"/>
-      <c r="H18" s="44" t="n"/>
-      <c r="I18" s="44" t="n"/>
-      <c r="J18" s="44" t="n"/>
-      <c r="K18" s="44" t="n"/>
-      <c r="L18" s="45">
-        <f>IF(COUNT(F18:K18)=0,"",IFERROR(SUMPRODUCT(F18:K18,(F$5:K$5+(F$5:K$5="")))/SUMPRODUCT((F18:K18&lt;&gt;"")*(F$5:K$5+(F$5:K$5=""))),""))</f>
-        <v/>
-      </c>
-      <c r="M18" s="44" t="n"/>
-      <c r="N18" s="44" t="n"/>
-      <c r="O18" s="44" t="n"/>
-      <c r="P18" s="45">
-        <f>IF(COUNT(M18:O18)=0,"",IFERROR(SUMPRODUCT(M18:O18,(M$5:O$5+(M$5:O$5="")))/SUMPRODUCT((M18:O18&lt;&gt;"")*(M$5:O$5+(M$5:O$5=""))),""))</f>
-        <v/>
-      </c>
-      <c r="Q18" s="44" t="n"/>
-      <c r="R18" s="44" t="n"/>
-      <c r="S18" s="44" t="n"/>
-      <c r="T18" s="44" t="n"/>
-      <c r="U18" s="45">
-        <f>IF(COUNT(Q18:T18)=0,"",IFERROR(SUMPRODUCT(Q18:T18,(Q$5:T$5+(Q$5:T$5="")))/SUMPRODUCT((Q18:T18&lt;&gt;"")*(Q$5:T$5+(Q$5:T$5=""))),""))</f>
-        <v/>
-      </c>
-      <c r="V18" s="44" t="n"/>
-      <c r="W18" s="44" t="n"/>
-      <c r="X18" s="45">
-        <f>IF(COUNT(V18:W18)=0,"",IFERROR(SUMPRODUCT(V18:W18,(V$5:W$5+(V$5:W$5="")))/SUMPRODUCT((V18:W18&lt;&gt;"")*(V$5:W$5+(V$5:W$5=""))),""))</f>
-        <v/>
-      </c>
-      <c r="Y18" s="45">
-        <f>IFERROR(IF((ISNUMBER(P18)*(P$5+(P$5=""))+ISNUMBER(U18)*(U$5+(U$5=""))+ISNUMBER(X18)*(X$5+(X$5="")))=0,"",(N(P18)*(P$5+(P$5=""))+N(U18)*(U$5+(U$5=""))+N(X18)*(X$5+(X$5="")))/(ISNUMBER(P18)*(P$5+(P$5=""))+ISNUMBER(U18)*(U$5+(U$5=""))+ISNUMBER(X18)*(X$5+(X$5="")))),"")</f>
-        <v/>
-      </c>
-      <c r="Z18" s="46">
-        <f>IF(AND(ISNUMBER(L18),ISNUMBER(Y18)),L18*Y18,"")</f>
-        <v/>
-      </c>
-      <c r="AA18" s="47">
-        <f>IF(ISNUMBER(Z18),(Z18-1)/24,"")</f>
-        <v/>
-      </c>
-      <c r="AB18" s="48">
-        <f>IF(ISNUMBER(Z18),COUNTIF(Z$7:Z$27,"&gt;"&amp;Z18)+1,"")</f>
-        <v/>
-      </c>
-      <c r="AC18" s="49">
-        <f>COUNT(F18,G18,H18,I18,J18,K18,M18,N18,O18,Q18,R18,S18,T18,V18,W18)</f>
+      <c r="F18" s="44" t="n">
+        <v>-8.114288</v>
+      </c>
+      <c r="G18" s="44" t="n">
+        <v>-34.921465</v>
+      </c>
+      <c r="H18" s="42" t="inlineStr">
+        <is>
+          <t>Aproximado</t>
+        </is>
+      </c>
+      <c r="I18" s="45" t="n"/>
+      <c r="J18" s="45" t="n"/>
+      <c r="K18" s="45" t="n"/>
+      <c r="L18" s="45" t="n"/>
+      <c r="M18" s="45" t="n"/>
+      <c r="N18" s="45" t="n"/>
+      <c r="O18" s="46">
+        <f>IF(COUNT(I18:N18)=0,"",IFERROR(SUMPRODUCT(I18:N18,(I$5:N$5+(I$5:N$5="")))/SUMPRODUCT((I18:N18&lt;&gt;"")*(I$5:N$5+(I$5:N$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="P18" s="45" t="n"/>
+      <c r="Q18" s="45" t="n"/>
+      <c r="R18" s="45" t="n"/>
+      <c r="S18" s="46">
+        <f>IF(COUNT(P18:R18)=0,"",IFERROR(SUMPRODUCT(P18:R18,(P$5:R$5+(P$5:R$5="")))/SUMPRODUCT((P18:R18&lt;&gt;"")*(P$5:R$5+(P$5:R$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="T18" s="45" t="n"/>
+      <c r="U18" s="45" t="n"/>
+      <c r="V18" s="45" t="n"/>
+      <c r="W18" s="45" t="n"/>
+      <c r="X18" s="46">
+        <f>IF(COUNT(T18:W18)=0,"",IFERROR(SUMPRODUCT(T18:W18,(T$5:W$5+(T$5:W$5="")))/SUMPRODUCT((T18:W18&lt;&gt;"")*(T$5:W$5+(T$5:W$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="Y18" s="45" t="n"/>
+      <c r="Z18" s="45" t="n"/>
+      <c r="AA18" s="46">
+        <f>IF(COUNT(Y18:Z18)=0,"",IFERROR(SUMPRODUCT(Y18:Z18,(Y$5:Z$5+(Y$5:Z$5="")))/SUMPRODUCT((Y18:Z18&lt;&gt;"")*(Y$5:Z$5+(Y$5:Z$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="AB18" s="46">
+        <f>IFERROR(IF((ISNUMBER(S18)*(S$5+(S$5=""))+ISNUMBER(X18)*(X$5+(X$5=""))+ISNUMBER(AA18)*(AA$5+(AA$5="")))=0,"",(N(S18)*(S$5+(S$5=""))+N(X18)*(X$5+(X$5=""))+N(AA18)*(AA$5+(AA$5="")))/(ISNUMBER(S18)*(S$5+(S$5=""))+ISNUMBER(X18)*(X$5+(X$5=""))+ISNUMBER(AA18)*(AA$5+(AA$5="")))),"")</f>
+        <v/>
+      </c>
+      <c r="AC18" s="47">
+        <f>IF(AND(ISNUMBER(O18),ISNUMBER(AB18)),O18*AB18,"")</f>
+        <v/>
+      </c>
+      <c r="AD18" s="48">
+        <f>IF(ISNUMBER(AC18),(AC18-1)/24,"")</f>
+        <v/>
+      </c>
+      <c r="AE18" s="49">
+        <f>IF(ISNUMBER(AC18),COUNTIF(AC$7:AC$27,"&gt;"&amp;AC18)+1,"")</f>
+        <v/>
+      </c>
+      <c r="AF18" s="50">
+        <f>COUNT(I18,J18,K18,L18,M18,N18,P18,Q18,R18,T18,U18,V18,W18,Y18,Z18)</f>
         <v/>
       </c>
     </row>
@@ -3484,55 +3639,66 @@
         </is>
       </c>
       <c r="E19" s="42" t="inlineStr"/>
-      <c r="F19" s="44" t="n"/>
-      <c r="G19" s="44" t="n"/>
-      <c r="H19" s="44" t="n"/>
-      <c r="I19" s="44" t="n"/>
-      <c r="J19" s="44" t="n"/>
-      <c r="K19" s="44" t="n"/>
-      <c r="L19" s="45">
-        <f>IF(COUNT(F19:K19)=0,"",IFERROR(SUMPRODUCT(F19:K19,(F$5:K$5+(F$5:K$5="")))/SUMPRODUCT((F19:K19&lt;&gt;"")*(F$5:K$5+(F$5:K$5=""))),""))</f>
-        <v/>
-      </c>
-      <c r="M19" s="44" t="n"/>
-      <c r="N19" s="44" t="n"/>
-      <c r="O19" s="44" t="n"/>
-      <c r="P19" s="45">
-        <f>IF(COUNT(M19:O19)=0,"",IFERROR(SUMPRODUCT(M19:O19,(M$5:O$5+(M$5:O$5="")))/SUMPRODUCT((M19:O19&lt;&gt;"")*(M$5:O$5+(M$5:O$5=""))),""))</f>
-        <v/>
-      </c>
-      <c r="Q19" s="44" t="n"/>
-      <c r="R19" s="44" t="n"/>
-      <c r="S19" s="44" t="n"/>
-      <c r="T19" s="44" t="n"/>
-      <c r="U19" s="45">
-        <f>IF(COUNT(Q19:T19)=0,"",IFERROR(SUMPRODUCT(Q19:T19,(Q$5:T$5+(Q$5:T$5="")))/SUMPRODUCT((Q19:T19&lt;&gt;"")*(Q$5:T$5+(Q$5:T$5=""))),""))</f>
-        <v/>
-      </c>
-      <c r="V19" s="44" t="n"/>
-      <c r="W19" s="44" t="n"/>
-      <c r="X19" s="45">
-        <f>IF(COUNT(V19:W19)=0,"",IFERROR(SUMPRODUCT(V19:W19,(V$5:W$5+(V$5:W$5="")))/SUMPRODUCT((V19:W19&lt;&gt;"")*(V$5:W$5+(V$5:W$5=""))),""))</f>
-        <v/>
-      </c>
-      <c r="Y19" s="45">
-        <f>IFERROR(IF((ISNUMBER(P19)*(P$5+(P$5=""))+ISNUMBER(U19)*(U$5+(U$5=""))+ISNUMBER(X19)*(X$5+(X$5="")))=0,"",(N(P19)*(P$5+(P$5=""))+N(U19)*(U$5+(U$5=""))+N(X19)*(X$5+(X$5="")))/(ISNUMBER(P19)*(P$5+(P$5=""))+ISNUMBER(U19)*(U$5+(U$5=""))+ISNUMBER(X19)*(X$5+(X$5="")))),"")</f>
-        <v/>
-      </c>
-      <c r="Z19" s="46">
-        <f>IF(AND(ISNUMBER(L19),ISNUMBER(Y19)),L19*Y19,"")</f>
-        <v/>
-      </c>
-      <c r="AA19" s="47">
-        <f>IF(ISNUMBER(Z19),(Z19-1)/24,"")</f>
-        <v/>
-      </c>
-      <c r="AB19" s="48">
-        <f>IF(ISNUMBER(Z19),COUNTIF(Z$7:Z$27,"&gt;"&amp;Z19)+1,"")</f>
-        <v/>
-      </c>
-      <c r="AC19" s="49">
-        <f>COUNT(F19,G19,H19,I19,J19,K19,M19,N19,O19,Q19,R19,S19,T19,V19,W19)</f>
+      <c r="F19" s="44" t="n">
+        <v>-8.145054999999999</v>
+      </c>
+      <c r="G19" s="44" t="n">
+        <v>-34.905114</v>
+      </c>
+      <c r="H19" s="42" t="inlineStr">
+        <is>
+          <t>Interseção</t>
+        </is>
+      </c>
+      <c r="I19" s="45" t="n"/>
+      <c r="J19" s="45" t="n"/>
+      <c r="K19" s="45" t="n"/>
+      <c r="L19" s="45" t="n"/>
+      <c r="M19" s="45" t="n"/>
+      <c r="N19" s="45" t="n"/>
+      <c r="O19" s="46">
+        <f>IF(COUNT(I19:N19)=0,"",IFERROR(SUMPRODUCT(I19:N19,(I$5:N$5+(I$5:N$5="")))/SUMPRODUCT((I19:N19&lt;&gt;"")*(I$5:N$5+(I$5:N$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="P19" s="45" t="n"/>
+      <c r="Q19" s="45" t="n"/>
+      <c r="R19" s="45" t="n"/>
+      <c r="S19" s="46">
+        <f>IF(COUNT(P19:R19)=0,"",IFERROR(SUMPRODUCT(P19:R19,(P$5:R$5+(P$5:R$5="")))/SUMPRODUCT((P19:R19&lt;&gt;"")*(P$5:R$5+(P$5:R$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="T19" s="45" t="n"/>
+      <c r="U19" s="45" t="n"/>
+      <c r="V19" s="45" t="n"/>
+      <c r="W19" s="45" t="n"/>
+      <c r="X19" s="46">
+        <f>IF(COUNT(T19:W19)=0,"",IFERROR(SUMPRODUCT(T19:W19,(T$5:W$5+(T$5:W$5="")))/SUMPRODUCT((T19:W19&lt;&gt;"")*(T$5:W$5+(T$5:W$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="Y19" s="45" t="n"/>
+      <c r="Z19" s="45" t="n"/>
+      <c r="AA19" s="46">
+        <f>IF(COUNT(Y19:Z19)=0,"",IFERROR(SUMPRODUCT(Y19:Z19,(Y$5:Z$5+(Y$5:Z$5="")))/SUMPRODUCT((Y19:Z19&lt;&gt;"")*(Y$5:Z$5+(Y$5:Z$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="AB19" s="46">
+        <f>IFERROR(IF((ISNUMBER(S19)*(S$5+(S$5=""))+ISNUMBER(X19)*(X$5+(X$5=""))+ISNUMBER(AA19)*(AA$5+(AA$5="")))=0,"",(N(S19)*(S$5+(S$5=""))+N(X19)*(X$5+(X$5=""))+N(AA19)*(AA$5+(AA$5="")))/(ISNUMBER(S19)*(S$5+(S$5=""))+ISNUMBER(X19)*(X$5+(X$5=""))+ISNUMBER(AA19)*(AA$5+(AA$5="")))),"")</f>
+        <v/>
+      </c>
+      <c r="AC19" s="47">
+        <f>IF(AND(ISNUMBER(O19),ISNUMBER(AB19)),O19*AB19,"")</f>
+        <v/>
+      </c>
+      <c r="AD19" s="48">
+        <f>IF(ISNUMBER(AC19),(AC19-1)/24,"")</f>
+        <v/>
+      </c>
+      <c r="AE19" s="49">
+        <f>IF(ISNUMBER(AC19),COUNTIF(AC$7:AC$27,"&gt;"&amp;AC19)+1,"")</f>
+        <v/>
+      </c>
+      <c r="AF19" s="50">
+        <f>COUNT(I19,J19,K19,L19,M19,N19,P19,Q19,R19,T19,U19,V19,W19,Y19,Z19)</f>
         <v/>
       </c>
     </row>
@@ -3560,55 +3726,66 @@
           <t>G4</t>
         </is>
       </c>
-      <c r="F20" s="44" t="n"/>
-      <c r="G20" s="44" t="n"/>
-      <c r="H20" s="44" t="n"/>
-      <c r="I20" s="44" t="n"/>
-      <c r="J20" s="44" t="n"/>
-      <c r="K20" s="44" t="n"/>
-      <c r="L20" s="45">
-        <f>IF(COUNT(F20:K20)=0,"",IFERROR(SUMPRODUCT(F20:K20,(F$5:K$5+(F$5:K$5="")))/SUMPRODUCT((F20:K20&lt;&gt;"")*(F$5:K$5+(F$5:K$5=""))),""))</f>
-        <v/>
-      </c>
-      <c r="M20" s="44" t="n"/>
-      <c r="N20" s="44" t="n"/>
-      <c r="O20" s="44" t="n"/>
-      <c r="P20" s="45">
-        <f>IF(COUNT(M20:O20)=0,"",IFERROR(SUMPRODUCT(M20:O20,(M$5:O$5+(M$5:O$5="")))/SUMPRODUCT((M20:O20&lt;&gt;"")*(M$5:O$5+(M$5:O$5=""))),""))</f>
-        <v/>
-      </c>
-      <c r="Q20" s="44" t="n"/>
-      <c r="R20" s="44" t="n"/>
-      <c r="S20" s="44" t="n"/>
-      <c r="T20" s="44" t="n"/>
-      <c r="U20" s="45">
-        <f>IF(COUNT(Q20:T20)=0,"",IFERROR(SUMPRODUCT(Q20:T20,(Q$5:T$5+(Q$5:T$5="")))/SUMPRODUCT((Q20:T20&lt;&gt;"")*(Q$5:T$5+(Q$5:T$5=""))),""))</f>
-        <v/>
-      </c>
-      <c r="V20" s="44" t="n"/>
-      <c r="W20" s="44" t="n"/>
-      <c r="X20" s="45">
-        <f>IF(COUNT(V20:W20)=0,"",IFERROR(SUMPRODUCT(V20:W20,(V$5:W$5+(V$5:W$5="")))/SUMPRODUCT((V20:W20&lt;&gt;"")*(V$5:W$5+(V$5:W$5=""))),""))</f>
-        <v/>
-      </c>
-      <c r="Y20" s="45">
-        <f>IFERROR(IF((ISNUMBER(P20)*(P$5+(P$5=""))+ISNUMBER(U20)*(U$5+(U$5=""))+ISNUMBER(X20)*(X$5+(X$5="")))=0,"",(N(P20)*(P$5+(P$5=""))+N(U20)*(U$5+(U$5=""))+N(X20)*(X$5+(X$5="")))/(ISNUMBER(P20)*(P$5+(P$5=""))+ISNUMBER(U20)*(U$5+(U$5=""))+ISNUMBER(X20)*(X$5+(X$5="")))),"")</f>
-        <v/>
-      </c>
-      <c r="Z20" s="46">
-        <f>IF(AND(ISNUMBER(L20),ISNUMBER(Y20)),L20*Y20,"")</f>
-        <v/>
-      </c>
-      <c r="AA20" s="47">
-        <f>IF(ISNUMBER(Z20),(Z20-1)/24,"")</f>
-        <v/>
-      </c>
-      <c r="AB20" s="48">
-        <f>IF(ISNUMBER(Z20),COUNTIF(Z$7:Z$27,"&gt;"&amp;Z20)+1,"")</f>
-        <v/>
-      </c>
-      <c r="AC20" s="49">
-        <f>COUNT(F20,G20,H20,I20,J20,K20,M20,N20,O20,Q20,R20,S20,T20,V20,W20)</f>
+      <c r="F20" s="44" t="n">
+        <v>-8.113526</v>
+      </c>
+      <c r="G20" s="44" t="n">
+        <v>-34.939007</v>
+      </c>
+      <c r="H20" s="42" t="inlineStr">
+        <is>
+          <t>Interseção</t>
+        </is>
+      </c>
+      <c r="I20" s="45" t="n"/>
+      <c r="J20" s="45" t="n"/>
+      <c r="K20" s="45" t="n"/>
+      <c r="L20" s="45" t="n"/>
+      <c r="M20" s="45" t="n"/>
+      <c r="N20" s="45" t="n"/>
+      <c r="O20" s="46">
+        <f>IF(COUNT(I20:N20)=0,"",IFERROR(SUMPRODUCT(I20:N20,(I$5:N$5+(I$5:N$5="")))/SUMPRODUCT((I20:N20&lt;&gt;"")*(I$5:N$5+(I$5:N$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="P20" s="45" t="n"/>
+      <c r="Q20" s="45" t="n"/>
+      <c r="R20" s="45" t="n"/>
+      <c r="S20" s="46">
+        <f>IF(COUNT(P20:R20)=0,"",IFERROR(SUMPRODUCT(P20:R20,(P$5:R$5+(P$5:R$5="")))/SUMPRODUCT((P20:R20&lt;&gt;"")*(P$5:R$5+(P$5:R$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="T20" s="45" t="n"/>
+      <c r="U20" s="45" t="n"/>
+      <c r="V20" s="45" t="n"/>
+      <c r="W20" s="45" t="n"/>
+      <c r="X20" s="46">
+        <f>IF(COUNT(T20:W20)=0,"",IFERROR(SUMPRODUCT(T20:W20,(T$5:W$5+(T$5:W$5="")))/SUMPRODUCT((T20:W20&lt;&gt;"")*(T$5:W$5+(T$5:W$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="Y20" s="45" t="n"/>
+      <c r="Z20" s="45" t="n"/>
+      <c r="AA20" s="46">
+        <f>IF(COUNT(Y20:Z20)=0,"",IFERROR(SUMPRODUCT(Y20:Z20,(Y$5:Z$5+(Y$5:Z$5="")))/SUMPRODUCT((Y20:Z20&lt;&gt;"")*(Y$5:Z$5+(Y$5:Z$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="AB20" s="46">
+        <f>IFERROR(IF((ISNUMBER(S20)*(S$5+(S$5=""))+ISNUMBER(X20)*(X$5+(X$5=""))+ISNUMBER(AA20)*(AA$5+(AA$5="")))=0,"",(N(S20)*(S$5+(S$5=""))+N(X20)*(X$5+(X$5=""))+N(AA20)*(AA$5+(AA$5="")))/(ISNUMBER(S20)*(S$5+(S$5=""))+ISNUMBER(X20)*(X$5+(X$5=""))+ISNUMBER(AA20)*(AA$5+(AA$5="")))),"")</f>
+        <v/>
+      </c>
+      <c r="AC20" s="47">
+        <f>IF(AND(ISNUMBER(O20),ISNUMBER(AB20)),O20*AB20,"")</f>
+        <v/>
+      </c>
+      <c r="AD20" s="48">
+        <f>IF(ISNUMBER(AC20),(AC20-1)/24,"")</f>
+        <v/>
+      </c>
+      <c r="AE20" s="49">
+        <f>IF(ISNUMBER(AC20),COUNTIF(AC$7:AC$27,"&gt;"&amp;AC20)+1,"")</f>
+        <v/>
+      </c>
+      <c r="AF20" s="50">
+        <f>COUNT(I20,J20,K20,L20,M20,N20,P20,Q20,R20,T20,U20,V20,W20,Y20,Z20)</f>
         <v/>
       </c>
     </row>
@@ -3636,55 +3813,66 @@
           <t>G5</t>
         </is>
       </c>
-      <c r="F21" s="44" t="n"/>
-      <c r="G21" s="44" t="n"/>
-      <c r="H21" s="44" t="n"/>
-      <c r="I21" s="44" t="n"/>
-      <c r="J21" s="44" t="n"/>
-      <c r="K21" s="44" t="n"/>
-      <c r="L21" s="45">
-        <f>IF(COUNT(F21:K21)=0,"",IFERROR(SUMPRODUCT(F21:K21,(F$5:K$5+(F$5:K$5="")))/SUMPRODUCT((F21:K21&lt;&gt;"")*(F$5:K$5+(F$5:K$5=""))),""))</f>
-        <v/>
-      </c>
-      <c r="M21" s="44" t="n"/>
-      <c r="N21" s="44" t="n"/>
-      <c r="O21" s="44" t="n"/>
-      <c r="P21" s="45">
-        <f>IF(COUNT(M21:O21)=0,"",IFERROR(SUMPRODUCT(M21:O21,(M$5:O$5+(M$5:O$5="")))/SUMPRODUCT((M21:O21&lt;&gt;"")*(M$5:O$5+(M$5:O$5=""))),""))</f>
-        <v/>
-      </c>
-      <c r="Q21" s="44" t="n"/>
-      <c r="R21" s="44" t="n"/>
-      <c r="S21" s="44" t="n"/>
-      <c r="T21" s="44" t="n"/>
-      <c r="U21" s="45">
-        <f>IF(COUNT(Q21:T21)=0,"",IFERROR(SUMPRODUCT(Q21:T21,(Q$5:T$5+(Q$5:T$5="")))/SUMPRODUCT((Q21:T21&lt;&gt;"")*(Q$5:T$5+(Q$5:T$5=""))),""))</f>
-        <v/>
-      </c>
-      <c r="V21" s="44" t="n"/>
-      <c r="W21" s="44" t="n"/>
-      <c r="X21" s="45">
-        <f>IF(COUNT(V21:W21)=0,"",IFERROR(SUMPRODUCT(V21:W21,(V$5:W$5+(V$5:W$5="")))/SUMPRODUCT((V21:W21&lt;&gt;"")*(V$5:W$5+(V$5:W$5=""))),""))</f>
-        <v/>
-      </c>
-      <c r="Y21" s="45">
-        <f>IFERROR(IF((ISNUMBER(P21)*(P$5+(P$5=""))+ISNUMBER(U21)*(U$5+(U$5=""))+ISNUMBER(X21)*(X$5+(X$5="")))=0,"",(N(P21)*(P$5+(P$5=""))+N(U21)*(U$5+(U$5=""))+N(X21)*(X$5+(X$5="")))/(ISNUMBER(P21)*(P$5+(P$5=""))+ISNUMBER(U21)*(U$5+(U$5=""))+ISNUMBER(X21)*(X$5+(X$5="")))),"")</f>
-        <v/>
-      </c>
-      <c r="Z21" s="46">
-        <f>IF(AND(ISNUMBER(L21),ISNUMBER(Y21)),L21*Y21,"")</f>
-        <v/>
-      </c>
-      <c r="AA21" s="47">
-        <f>IF(ISNUMBER(Z21),(Z21-1)/24,"")</f>
-        <v/>
-      </c>
-      <c r="AB21" s="48">
-        <f>IF(ISNUMBER(Z21),COUNTIF(Z$7:Z$27,"&gt;"&amp;Z21)+1,"")</f>
-        <v/>
-      </c>
-      <c r="AC21" s="49">
-        <f>COUNT(F21,G21,H21,I21,J21,K21,M21,N21,O21,Q21,R21,S21,T21,V21,W21)</f>
+      <c r="F21" s="44" t="n">
+        <v>-8.107493</v>
+      </c>
+      <c r="G21" s="44" t="n">
+        <v>-34.929853</v>
+      </c>
+      <c r="H21" s="42" t="inlineStr">
+        <is>
+          <t>Interseção</t>
+        </is>
+      </c>
+      <c r="I21" s="45" t="n"/>
+      <c r="J21" s="45" t="n"/>
+      <c r="K21" s="45" t="n"/>
+      <c r="L21" s="45" t="n"/>
+      <c r="M21" s="45" t="n"/>
+      <c r="N21" s="45" t="n"/>
+      <c r="O21" s="46">
+        <f>IF(COUNT(I21:N21)=0,"",IFERROR(SUMPRODUCT(I21:N21,(I$5:N$5+(I$5:N$5="")))/SUMPRODUCT((I21:N21&lt;&gt;"")*(I$5:N$5+(I$5:N$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="P21" s="45" t="n"/>
+      <c r="Q21" s="45" t="n"/>
+      <c r="R21" s="45" t="n"/>
+      <c r="S21" s="46">
+        <f>IF(COUNT(P21:R21)=0,"",IFERROR(SUMPRODUCT(P21:R21,(P$5:R$5+(P$5:R$5="")))/SUMPRODUCT((P21:R21&lt;&gt;"")*(P$5:R$5+(P$5:R$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="T21" s="45" t="n"/>
+      <c r="U21" s="45" t="n"/>
+      <c r="V21" s="45" t="n"/>
+      <c r="W21" s="45" t="n"/>
+      <c r="X21" s="46">
+        <f>IF(COUNT(T21:W21)=0,"",IFERROR(SUMPRODUCT(T21:W21,(T$5:W$5+(T$5:W$5="")))/SUMPRODUCT((T21:W21&lt;&gt;"")*(T$5:W$5+(T$5:W$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="Y21" s="45" t="n"/>
+      <c r="Z21" s="45" t="n"/>
+      <c r="AA21" s="46">
+        <f>IF(COUNT(Y21:Z21)=0,"",IFERROR(SUMPRODUCT(Y21:Z21,(Y$5:Z$5+(Y$5:Z$5="")))/SUMPRODUCT((Y21:Z21&lt;&gt;"")*(Y$5:Z$5+(Y$5:Z$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="AB21" s="46">
+        <f>IFERROR(IF((ISNUMBER(S21)*(S$5+(S$5=""))+ISNUMBER(X21)*(X$5+(X$5=""))+ISNUMBER(AA21)*(AA$5+(AA$5="")))=0,"",(N(S21)*(S$5+(S$5=""))+N(X21)*(X$5+(X$5=""))+N(AA21)*(AA$5+(AA$5="")))/(ISNUMBER(S21)*(S$5+(S$5=""))+ISNUMBER(X21)*(X$5+(X$5=""))+ISNUMBER(AA21)*(AA$5+(AA$5="")))),"")</f>
+        <v/>
+      </c>
+      <c r="AC21" s="47">
+        <f>IF(AND(ISNUMBER(O21),ISNUMBER(AB21)),O21*AB21,"")</f>
+        <v/>
+      </c>
+      <c r="AD21" s="48">
+        <f>IF(ISNUMBER(AC21),(AC21-1)/24,"")</f>
+        <v/>
+      </c>
+      <c r="AE21" s="49">
+        <f>IF(ISNUMBER(AC21),COUNTIF(AC$7:AC$27,"&gt;"&amp;AC21)+1,"")</f>
+        <v/>
+      </c>
+      <c r="AF21" s="50">
+        <f>COUNT(I21,J21,K21,L21,M21,N21,P21,Q21,R21,T21,U21,V21,W21,Y21,Z21)</f>
         <v/>
       </c>
     </row>
@@ -3712,55 +3900,66 @@
           <t>G4</t>
         </is>
       </c>
-      <c r="F22" s="44" t="n"/>
-      <c r="G22" s="44" t="n"/>
-      <c r="H22" s="44" t="n"/>
-      <c r="I22" s="44" t="n"/>
-      <c r="J22" s="44" t="n"/>
-      <c r="K22" s="44" t="n"/>
-      <c r="L22" s="45">
-        <f>IF(COUNT(F22:K22)=0,"",IFERROR(SUMPRODUCT(F22:K22,(F$5:K$5+(F$5:K$5="")))/SUMPRODUCT((F22:K22&lt;&gt;"")*(F$5:K$5+(F$5:K$5=""))),""))</f>
-        <v/>
-      </c>
-      <c r="M22" s="44" t="n"/>
-      <c r="N22" s="44" t="n"/>
-      <c r="O22" s="44" t="n"/>
-      <c r="P22" s="45">
-        <f>IF(COUNT(M22:O22)=0,"",IFERROR(SUMPRODUCT(M22:O22,(M$5:O$5+(M$5:O$5="")))/SUMPRODUCT((M22:O22&lt;&gt;"")*(M$5:O$5+(M$5:O$5=""))),""))</f>
-        <v/>
-      </c>
-      <c r="Q22" s="44" t="n"/>
-      <c r="R22" s="44" t="n"/>
-      <c r="S22" s="44" t="n"/>
-      <c r="T22" s="44" t="n"/>
-      <c r="U22" s="45">
-        <f>IF(COUNT(Q22:T22)=0,"",IFERROR(SUMPRODUCT(Q22:T22,(Q$5:T$5+(Q$5:T$5="")))/SUMPRODUCT((Q22:T22&lt;&gt;"")*(Q$5:T$5+(Q$5:T$5=""))),""))</f>
-        <v/>
-      </c>
-      <c r="V22" s="44" t="n"/>
-      <c r="W22" s="44" t="n"/>
-      <c r="X22" s="45">
-        <f>IF(COUNT(V22:W22)=0,"",IFERROR(SUMPRODUCT(V22:W22,(V$5:W$5+(V$5:W$5="")))/SUMPRODUCT((V22:W22&lt;&gt;"")*(V$5:W$5+(V$5:W$5=""))),""))</f>
-        <v/>
-      </c>
-      <c r="Y22" s="45">
-        <f>IFERROR(IF((ISNUMBER(P22)*(P$5+(P$5=""))+ISNUMBER(U22)*(U$5+(U$5=""))+ISNUMBER(X22)*(X$5+(X$5="")))=0,"",(N(P22)*(P$5+(P$5=""))+N(U22)*(U$5+(U$5=""))+N(X22)*(X$5+(X$5="")))/(ISNUMBER(P22)*(P$5+(P$5=""))+ISNUMBER(U22)*(U$5+(U$5=""))+ISNUMBER(X22)*(X$5+(X$5="")))),"")</f>
-        <v/>
-      </c>
-      <c r="Z22" s="46">
-        <f>IF(AND(ISNUMBER(L22),ISNUMBER(Y22)),L22*Y22,"")</f>
-        <v/>
-      </c>
-      <c r="AA22" s="47">
-        <f>IF(ISNUMBER(Z22),(Z22-1)/24,"")</f>
-        <v/>
-      </c>
-      <c r="AB22" s="48">
-        <f>IF(ISNUMBER(Z22),COUNTIF(Z$7:Z$27,"&gt;"&amp;Z22)+1,"")</f>
-        <v/>
-      </c>
-      <c r="AC22" s="49">
-        <f>COUNT(F22,G22,H22,I22,J22,K22,M22,N22,O22,Q22,R22,S22,T22,V22,W22)</f>
+      <c r="F22" s="44" t="n">
+        <v>-8.110391</v>
+      </c>
+      <c r="G22" s="44" t="n">
+        <v>-34.93687</v>
+      </c>
+      <c r="H22" s="42" t="inlineStr">
+        <is>
+          <t>Aproximado</t>
+        </is>
+      </c>
+      <c r="I22" s="45" t="n"/>
+      <c r="J22" s="45" t="n"/>
+      <c r="K22" s="45" t="n"/>
+      <c r="L22" s="45" t="n"/>
+      <c r="M22" s="45" t="n"/>
+      <c r="N22" s="45" t="n"/>
+      <c r="O22" s="46">
+        <f>IF(COUNT(I22:N22)=0,"",IFERROR(SUMPRODUCT(I22:N22,(I$5:N$5+(I$5:N$5="")))/SUMPRODUCT((I22:N22&lt;&gt;"")*(I$5:N$5+(I$5:N$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="P22" s="45" t="n"/>
+      <c r="Q22" s="45" t="n"/>
+      <c r="R22" s="45" t="n"/>
+      <c r="S22" s="46">
+        <f>IF(COUNT(P22:R22)=0,"",IFERROR(SUMPRODUCT(P22:R22,(P$5:R$5+(P$5:R$5="")))/SUMPRODUCT((P22:R22&lt;&gt;"")*(P$5:R$5+(P$5:R$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="T22" s="45" t="n"/>
+      <c r="U22" s="45" t="n"/>
+      <c r="V22" s="45" t="n"/>
+      <c r="W22" s="45" t="n"/>
+      <c r="X22" s="46">
+        <f>IF(COUNT(T22:W22)=0,"",IFERROR(SUMPRODUCT(T22:W22,(T$5:W$5+(T$5:W$5="")))/SUMPRODUCT((T22:W22&lt;&gt;"")*(T$5:W$5+(T$5:W$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="Y22" s="45" t="n"/>
+      <c r="Z22" s="45" t="n"/>
+      <c r="AA22" s="46">
+        <f>IF(COUNT(Y22:Z22)=0,"",IFERROR(SUMPRODUCT(Y22:Z22,(Y$5:Z$5+(Y$5:Z$5="")))/SUMPRODUCT((Y22:Z22&lt;&gt;"")*(Y$5:Z$5+(Y$5:Z$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="AB22" s="46">
+        <f>IFERROR(IF((ISNUMBER(S22)*(S$5+(S$5=""))+ISNUMBER(X22)*(X$5+(X$5=""))+ISNUMBER(AA22)*(AA$5+(AA$5="")))=0,"",(N(S22)*(S$5+(S$5=""))+N(X22)*(X$5+(X$5=""))+N(AA22)*(AA$5+(AA$5="")))/(ISNUMBER(S22)*(S$5+(S$5=""))+ISNUMBER(X22)*(X$5+(X$5=""))+ISNUMBER(AA22)*(AA$5+(AA$5="")))),"")</f>
+        <v/>
+      </c>
+      <c r="AC22" s="47">
+        <f>IF(AND(ISNUMBER(O22),ISNUMBER(AB22)),O22*AB22,"")</f>
+        <v/>
+      </c>
+      <c r="AD22" s="48">
+        <f>IF(ISNUMBER(AC22),(AC22-1)/24,"")</f>
+        <v/>
+      </c>
+      <c r="AE22" s="49">
+        <f>IF(ISNUMBER(AC22),COUNTIF(AC$7:AC$27,"&gt;"&amp;AC22)+1,"")</f>
+        <v/>
+      </c>
+      <c r="AF22" s="50">
+        <f>COUNT(I22,J22,K22,L22,M22,N22,P22,Q22,R22,T22,U22,V22,W22,Y22,Z22)</f>
         <v/>
       </c>
     </row>
@@ -3788,55 +3987,66 @@
           <t>G3</t>
         </is>
       </c>
-      <c r="F23" s="44" t="n"/>
-      <c r="G23" s="44" t="n"/>
-      <c r="H23" s="44" t="n"/>
-      <c r="I23" s="44" t="n"/>
-      <c r="J23" s="44" t="n"/>
-      <c r="K23" s="44" t="n"/>
-      <c r="L23" s="45">
-        <f>IF(COUNT(F23:K23)=0,"",IFERROR(SUMPRODUCT(F23:K23,(F$5:K$5+(F$5:K$5="")))/SUMPRODUCT((F23:K23&lt;&gt;"")*(F$5:K$5+(F$5:K$5=""))),""))</f>
-        <v/>
-      </c>
-      <c r="M23" s="44" t="n"/>
-      <c r="N23" s="44" t="n"/>
-      <c r="O23" s="44" t="n"/>
-      <c r="P23" s="45">
-        <f>IF(COUNT(M23:O23)=0,"",IFERROR(SUMPRODUCT(M23:O23,(M$5:O$5+(M$5:O$5="")))/SUMPRODUCT((M23:O23&lt;&gt;"")*(M$5:O$5+(M$5:O$5=""))),""))</f>
-        <v/>
-      </c>
-      <c r="Q23" s="44" t="n"/>
-      <c r="R23" s="44" t="n"/>
-      <c r="S23" s="44" t="n"/>
-      <c r="T23" s="44" t="n"/>
-      <c r="U23" s="45">
-        <f>IF(COUNT(Q23:T23)=0,"",IFERROR(SUMPRODUCT(Q23:T23,(Q$5:T$5+(Q$5:T$5="")))/SUMPRODUCT((Q23:T23&lt;&gt;"")*(Q$5:T$5+(Q$5:T$5=""))),""))</f>
-        <v/>
-      </c>
-      <c r="V23" s="44" t="n"/>
-      <c r="W23" s="44" t="n"/>
-      <c r="X23" s="45">
-        <f>IF(COUNT(V23:W23)=0,"",IFERROR(SUMPRODUCT(V23:W23,(V$5:W$5+(V$5:W$5="")))/SUMPRODUCT((V23:W23&lt;&gt;"")*(V$5:W$5+(V$5:W$5=""))),""))</f>
-        <v/>
-      </c>
-      <c r="Y23" s="45">
-        <f>IFERROR(IF((ISNUMBER(P23)*(P$5+(P$5=""))+ISNUMBER(U23)*(U$5+(U$5=""))+ISNUMBER(X23)*(X$5+(X$5="")))=0,"",(N(P23)*(P$5+(P$5=""))+N(U23)*(U$5+(U$5=""))+N(X23)*(X$5+(X$5="")))/(ISNUMBER(P23)*(P$5+(P$5=""))+ISNUMBER(U23)*(U$5+(U$5=""))+ISNUMBER(X23)*(X$5+(X$5="")))),"")</f>
-        <v/>
-      </c>
-      <c r="Z23" s="46">
-        <f>IF(AND(ISNUMBER(L23),ISNUMBER(Y23)),L23*Y23,"")</f>
-        <v/>
-      </c>
-      <c r="AA23" s="47">
-        <f>IF(ISNUMBER(Z23),(Z23-1)/24,"")</f>
-        <v/>
-      </c>
-      <c r="AB23" s="48">
-        <f>IF(ISNUMBER(Z23),COUNTIF(Z$7:Z$27,"&gt;"&amp;Z23)+1,"")</f>
-        <v/>
-      </c>
-      <c r="AC23" s="49">
-        <f>COUNT(F23,G23,H23,I23,J23,K23,M23,N23,O23,Q23,R23,S23,T23,V23,W23)</f>
+      <c r="F23" s="44" t="n">
+        <v>-8.111915</v>
+      </c>
+      <c r="G23" s="44" t="n">
+        <v>-34.912386</v>
+      </c>
+      <c r="H23" s="42" t="inlineStr">
+        <is>
+          <t>Aproximado</t>
+        </is>
+      </c>
+      <c r="I23" s="45" t="n"/>
+      <c r="J23" s="45" t="n"/>
+      <c r="K23" s="45" t="n"/>
+      <c r="L23" s="45" t="n"/>
+      <c r="M23" s="45" t="n"/>
+      <c r="N23" s="45" t="n"/>
+      <c r="O23" s="46">
+        <f>IF(COUNT(I23:N23)=0,"",IFERROR(SUMPRODUCT(I23:N23,(I$5:N$5+(I$5:N$5="")))/SUMPRODUCT((I23:N23&lt;&gt;"")*(I$5:N$5+(I$5:N$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="P23" s="45" t="n"/>
+      <c r="Q23" s="45" t="n"/>
+      <c r="R23" s="45" t="n"/>
+      <c r="S23" s="46">
+        <f>IF(COUNT(P23:R23)=0,"",IFERROR(SUMPRODUCT(P23:R23,(P$5:R$5+(P$5:R$5="")))/SUMPRODUCT((P23:R23&lt;&gt;"")*(P$5:R$5+(P$5:R$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="T23" s="45" t="n"/>
+      <c r="U23" s="45" t="n"/>
+      <c r="V23" s="45" t="n"/>
+      <c r="W23" s="45" t="n"/>
+      <c r="X23" s="46">
+        <f>IF(COUNT(T23:W23)=0,"",IFERROR(SUMPRODUCT(T23:W23,(T$5:W$5+(T$5:W$5="")))/SUMPRODUCT((T23:W23&lt;&gt;"")*(T$5:W$5+(T$5:W$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="Y23" s="45" t="n"/>
+      <c r="Z23" s="45" t="n"/>
+      <c r="AA23" s="46">
+        <f>IF(COUNT(Y23:Z23)=0,"",IFERROR(SUMPRODUCT(Y23:Z23,(Y$5:Z$5+(Y$5:Z$5="")))/SUMPRODUCT((Y23:Z23&lt;&gt;"")*(Y$5:Z$5+(Y$5:Z$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="AB23" s="46">
+        <f>IFERROR(IF((ISNUMBER(S23)*(S$5+(S$5=""))+ISNUMBER(X23)*(X$5+(X$5=""))+ISNUMBER(AA23)*(AA$5+(AA$5="")))=0,"",(N(S23)*(S$5+(S$5=""))+N(X23)*(X$5+(X$5=""))+N(AA23)*(AA$5+(AA$5="")))/(ISNUMBER(S23)*(S$5+(S$5=""))+ISNUMBER(X23)*(X$5+(X$5=""))+ISNUMBER(AA23)*(AA$5+(AA$5="")))),"")</f>
+        <v/>
+      </c>
+      <c r="AC23" s="47">
+        <f>IF(AND(ISNUMBER(O23),ISNUMBER(AB23)),O23*AB23,"")</f>
+        <v/>
+      </c>
+      <c r="AD23" s="48">
+        <f>IF(ISNUMBER(AC23),(AC23-1)/24,"")</f>
+        <v/>
+      </c>
+      <c r="AE23" s="49">
+        <f>IF(ISNUMBER(AC23),COUNTIF(AC$7:AC$27,"&gt;"&amp;AC23)+1,"")</f>
+        <v/>
+      </c>
+      <c r="AF23" s="50">
+        <f>COUNT(I23,J23,K23,L23,M23,N23,P23,Q23,R23,T23,U23,V23,W23,Y23,Z23)</f>
         <v/>
       </c>
     </row>
@@ -3864,55 +4074,66 @@
           <t>G5</t>
         </is>
       </c>
-      <c r="F24" s="44" t="n"/>
-      <c r="G24" s="44" t="n"/>
-      <c r="H24" s="44" t="n"/>
-      <c r="I24" s="44" t="n"/>
-      <c r="J24" s="44" t="n"/>
-      <c r="K24" s="44" t="n"/>
-      <c r="L24" s="45">
-        <f>IF(COUNT(F24:K24)=0,"",IFERROR(SUMPRODUCT(F24:K24,(F$5:K$5+(F$5:K$5="")))/SUMPRODUCT((F24:K24&lt;&gt;"")*(F$5:K$5+(F$5:K$5=""))),""))</f>
-        <v/>
-      </c>
-      <c r="M24" s="44" t="n"/>
-      <c r="N24" s="44" t="n"/>
-      <c r="O24" s="44" t="n"/>
-      <c r="P24" s="45">
-        <f>IF(COUNT(M24:O24)=0,"",IFERROR(SUMPRODUCT(M24:O24,(M$5:O$5+(M$5:O$5="")))/SUMPRODUCT((M24:O24&lt;&gt;"")*(M$5:O$5+(M$5:O$5=""))),""))</f>
-        <v/>
-      </c>
-      <c r="Q24" s="44" t="n"/>
-      <c r="R24" s="44" t="n"/>
-      <c r="S24" s="44" t="n"/>
-      <c r="T24" s="44" t="n"/>
-      <c r="U24" s="45">
-        <f>IF(COUNT(Q24:T24)=0,"",IFERROR(SUMPRODUCT(Q24:T24,(Q$5:T$5+(Q$5:T$5="")))/SUMPRODUCT((Q24:T24&lt;&gt;"")*(Q$5:T$5+(Q$5:T$5=""))),""))</f>
-        <v/>
-      </c>
-      <c r="V24" s="44" t="n"/>
-      <c r="W24" s="44" t="n"/>
-      <c r="X24" s="45">
-        <f>IF(COUNT(V24:W24)=0,"",IFERROR(SUMPRODUCT(V24:W24,(V$5:W$5+(V$5:W$5="")))/SUMPRODUCT((V24:W24&lt;&gt;"")*(V$5:W$5+(V$5:W$5=""))),""))</f>
-        <v/>
-      </c>
-      <c r="Y24" s="45">
-        <f>IFERROR(IF((ISNUMBER(P24)*(P$5+(P$5=""))+ISNUMBER(U24)*(U$5+(U$5=""))+ISNUMBER(X24)*(X$5+(X$5="")))=0,"",(N(P24)*(P$5+(P$5=""))+N(U24)*(U$5+(U$5=""))+N(X24)*(X$5+(X$5="")))/(ISNUMBER(P24)*(P$5+(P$5=""))+ISNUMBER(U24)*(U$5+(U$5=""))+ISNUMBER(X24)*(X$5+(X$5="")))),"")</f>
-        <v/>
-      </c>
-      <c r="Z24" s="46">
-        <f>IF(AND(ISNUMBER(L24),ISNUMBER(Y24)),L24*Y24,"")</f>
-        <v/>
-      </c>
-      <c r="AA24" s="47">
-        <f>IF(ISNUMBER(Z24),(Z24-1)/24,"")</f>
-        <v/>
-      </c>
-      <c r="AB24" s="48">
-        <f>IF(ISNUMBER(Z24),COUNTIF(Z$7:Z$27,"&gt;"&amp;Z24)+1,"")</f>
-        <v/>
-      </c>
-      <c r="AC24" s="49">
-        <f>COUNT(F24,G24,H24,I24,J24,K24,M24,N24,O24,Q24,R24,S24,T24,V24,W24)</f>
+      <c r="F24" s="44" t="n">
+        <v>-8.105179</v>
+      </c>
+      <c r="G24" s="44" t="n">
+        <v>-34.927549</v>
+      </c>
+      <c r="H24" s="42" t="inlineStr">
+        <is>
+          <t>Aproximado</t>
+        </is>
+      </c>
+      <c r="I24" s="45" t="n"/>
+      <c r="J24" s="45" t="n"/>
+      <c r="K24" s="45" t="n"/>
+      <c r="L24" s="45" t="n"/>
+      <c r="M24" s="45" t="n"/>
+      <c r="N24" s="45" t="n"/>
+      <c r="O24" s="46">
+        <f>IF(COUNT(I24:N24)=0,"",IFERROR(SUMPRODUCT(I24:N24,(I$5:N$5+(I$5:N$5="")))/SUMPRODUCT((I24:N24&lt;&gt;"")*(I$5:N$5+(I$5:N$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="P24" s="45" t="n"/>
+      <c r="Q24" s="45" t="n"/>
+      <c r="R24" s="45" t="n"/>
+      <c r="S24" s="46">
+        <f>IF(COUNT(P24:R24)=0,"",IFERROR(SUMPRODUCT(P24:R24,(P$5:R$5+(P$5:R$5="")))/SUMPRODUCT((P24:R24&lt;&gt;"")*(P$5:R$5+(P$5:R$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="T24" s="45" t="n"/>
+      <c r="U24" s="45" t="n"/>
+      <c r="V24" s="45" t="n"/>
+      <c r="W24" s="45" t="n"/>
+      <c r="X24" s="46">
+        <f>IF(COUNT(T24:W24)=0,"",IFERROR(SUMPRODUCT(T24:W24,(T$5:W$5+(T$5:W$5="")))/SUMPRODUCT((T24:W24&lt;&gt;"")*(T$5:W$5+(T$5:W$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="Y24" s="45" t="n"/>
+      <c r="Z24" s="45" t="n"/>
+      <c r="AA24" s="46">
+        <f>IF(COUNT(Y24:Z24)=0,"",IFERROR(SUMPRODUCT(Y24:Z24,(Y$5:Z$5+(Y$5:Z$5="")))/SUMPRODUCT((Y24:Z24&lt;&gt;"")*(Y$5:Z$5+(Y$5:Z$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="AB24" s="46">
+        <f>IFERROR(IF((ISNUMBER(S24)*(S$5+(S$5=""))+ISNUMBER(X24)*(X$5+(X$5=""))+ISNUMBER(AA24)*(AA$5+(AA$5="")))=0,"",(N(S24)*(S$5+(S$5=""))+N(X24)*(X$5+(X$5=""))+N(AA24)*(AA$5+(AA$5="")))/(ISNUMBER(S24)*(S$5+(S$5=""))+ISNUMBER(X24)*(X$5+(X$5=""))+ISNUMBER(AA24)*(AA$5+(AA$5="")))),"")</f>
+        <v/>
+      </c>
+      <c r="AC24" s="47">
+        <f>IF(AND(ISNUMBER(O24),ISNUMBER(AB24)),O24*AB24,"")</f>
+        <v/>
+      </c>
+      <c r="AD24" s="48">
+        <f>IF(ISNUMBER(AC24),(AC24-1)/24,"")</f>
+        <v/>
+      </c>
+      <c r="AE24" s="49">
+        <f>IF(ISNUMBER(AC24),COUNTIF(AC$7:AC$27,"&gt;"&amp;AC24)+1,"")</f>
+        <v/>
+      </c>
+      <c r="AF24" s="50">
+        <f>COUNT(I24,J24,K24,L24,M24,N24,P24,Q24,R24,T24,U24,V24,W24,Y24,Z24)</f>
         <v/>
       </c>
     </row>
@@ -3940,55 +4161,66 @@
           <t>G2</t>
         </is>
       </c>
-      <c r="F25" s="44" t="n"/>
-      <c r="G25" s="44" t="n"/>
-      <c r="H25" s="44" t="n"/>
-      <c r="I25" s="44" t="n"/>
-      <c r="J25" s="44" t="n"/>
-      <c r="K25" s="44" t="n"/>
-      <c r="L25" s="45">
-        <f>IF(COUNT(F25:K25)=0,"",IFERROR(SUMPRODUCT(F25:K25,(F$5:K$5+(F$5:K$5="")))/SUMPRODUCT((F25:K25&lt;&gt;"")*(F$5:K$5+(F$5:K$5=""))),""))</f>
-        <v/>
-      </c>
-      <c r="M25" s="44" t="n"/>
-      <c r="N25" s="44" t="n"/>
-      <c r="O25" s="44" t="n"/>
-      <c r="P25" s="45">
-        <f>IF(COUNT(M25:O25)=0,"",IFERROR(SUMPRODUCT(M25:O25,(M$5:O$5+(M$5:O$5="")))/SUMPRODUCT((M25:O25&lt;&gt;"")*(M$5:O$5+(M$5:O$5=""))),""))</f>
-        <v/>
-      </c>
-      <c r="Q25" s="44" t="n"/>
-      <c r="R25" s="44" t="n"/>
-      <c r="S25" s="44" t="n"/>
-      <c r="T25" s="44" t="n"/>
-      <c r="U25" s="45">
-        <f>IF(COUNT(Q25:T25)=0,"",IFERROR(SUMPRODUCT(Q25:T25,(Q$5:T$5+(Q$5:T$5="")))/SUMPRODUCT((Q25:T25&lt;&gt;"")*(Q$5:T$5+(Q$5:T$5=""))),""))</f>
-        <v/>
-      </c>
-      <c r="V25" s="44" t="n"/>
-      <c r="W25" s="44" t="n"/>
-      <c r="X25" s="45">
-        <f>IF(COUNT(V25:W25)=0,"",IFERROR(SUMPRODUCT(V25:W25,(V$5:W$5+(V$5:W$5="")))/SUMPRODUCT((V25:W25&lt;&gt;"")*(V$5:W$5+(V$5:W$5=""))),""))</f>
-        <v/>
-      </c>
-      <c r="Y25" s="45">
-        <f>IFERROR(IF((ISNUMBER(P25)*(P$5+(P$5=""))+ISNUMBER(U25)*(U$5+(U$5=""))+ISNUMBER(X25)*(X$5+(X$5="")))=0,"",(N(P25)*(P$5+(P$5=""))+N(U25)*(U$5+(U$5=""))+N(X25)*(X$5+(X$5="")))/(ISNUMBER(P25)*(P$5+(P$5=""))+ISNUMBER(U25)*(U$5+(U$5=""))+ISNUMBER(X25)*(X$5+(X$5="")))),"")</f>
-        <v/>
-      </c>
-      <c r="Z25" s="46">
-        <f>IF(AND(ISNUMBER(L25),ISNUMBER(Y25)),L25*Y25,"")</f>
-        <v/>
-      </c>
-      <c r="AA25" s="47">
-        <f>IF(ISNUMBER(Z25),(Z25-1)/24,"")</f>
-        <v/>
-      </c>
-      <c r="AB25" s="48">
-        <f>IF(ISNUMBER(Z25),COUNTIF(Z$7:Z$27,"&gt;"&amp;Z25)+1,"")</f>
-        <v/>
-      </c>
-      <c r="AC25" s="49">
-        <f>COUNT(F25,G25,H25,I25,J25,K25,M25,N25,O25,Q25,R25,S25,T25,V25,W25)</f>
+      <c r="F25" s="44" t="n">
+        <v>-8.098065999999999</v>
+      </c>
+      <c r="G25" s="44" t="n">
+        <v>-34.888129</v>
+      </c>
+      <c r="H25" s="42" t="inlineStr">
+        <is>
+          <t>Aproximado</t>
+        </is>
+      </c>
+      <c r="I25" s="45" t="n"/>
+      <c r="J25" s="45" t="n"/>
+      <c r="K25" s="45" t="n"/>
+      <c r="L25" s="45" t="n"/>
+      <c r="M25" s="45" t="n"/>
+      <c r="N25" s="45" t="n"/>
+      <c r="O25" s="46">
+        <f>IF(COUNT(I25:N25)=0,"",IFERROR(SUMPRODUCT(I25:N25,(I$5:N$5+(I$5:N$5="")))/SUMPRODUCT((I25:N25&lt;&gt;"")*(I$5:N$5+(I$5:N$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="P25" s="45" t="n"/>
+      <c r="Q25" s="45" t="n"/>
+      <c r="R25" s="45" t="n"/>
+      <c r="S25" s="46">
+        <f>IF(COUNT(P25:R25)=0,"",IFERROR(SUMPRODUCT(P25:R25,(P$5:R$5+(P$5:R$5="")))/SUMPRODUCT((P25:R25&lt;&gt;"")*(P$5:R$5+(P$5:R$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="T25" s="45" t="n"/>
+      <c r="U25" s="45" t="n"/>
+      <c r="V25" s="45" t="n"/>
+      <c r="W25" s="45" t="n"/>
+      <c r="X25" s="46">
+        <f>IF(COUNT(T25:W25)=0,"",IFERROR(SUMPRODUCT(T25:W25,(T$5:W$5+(T$5:W$5="")))/SUMPRODUCT((T25:W25&lt;&gt;"")*(T$5:W$5+(T$5:W$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="Y25" s="45" t="n"/>
+      <c r="Z25" s="45" t="n"/>
+      <c r="AA25" s="46">
+        <f>IF(COUNT(Y25:Z25)=0,"",IFERROR(SUMPRODUCT(Y25:Z25,(Y$5:Z$5+(Y$5:Z$5="")))/SUMPRODUCT((Y25:Z25&lt;&gt;"")*(Y$5:Z$5+(Y$5:Z$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="AB25" s="46">
+        <f>IFERROR(IF((ISNUMBER(S25)*(S$5+(S$5=""))+ISNUMBER(X25)*(X$5+(X$5=""))+ISNUMBER(AA25)*(AA$5+(AA$5="")))=0,"",(N(S25)*(S$5+(S$5=""))+N(X25)*(X$5+(X$5=""))+N(AA25)*(AA$5+(AA$5="")))/(ISNUMBER(S25)*(S$5+(S$5=""))+ISNUMBER(X25)*(X$5+(X$5=""))+ISNUMBER(AA25)*(AA$5+(AA$5="")))),"")</f>
+        <v/>
+      </c>
+      <c r="AC25" s="47">
+        <f>IF(AND(ISNUMBER(O25),ISNUMBER(AB25)),O25*AB25,"")</f>
+        <v/>
+      </c>
+      <c r="AD25" s="48">
+        <f>IF(ISNUMBER(AC25),(AC25-1)/24,"")</f>
+        <v/>
+      </c>
+      <c r="AE25" s="49">
+        <f>IF(ISNUMBER(AC25),COUNTIF(AC$7:AC$27,"&gt;"&amp;AC25)+1,"")</f>
+        <v/>
+      </c>
+      <c r="AF25" s="50">
+        <f>COUNT(I25,J25,K25,L25,M25,N25,P25,Q25,R25,T25,U25,V25,W25,Y25,Z25)</f>
         <v/>
       </c>
     </row>
@@ -4012,55 +4244,66 @@
         </is>
       </c>
       <c r="E26" s="42" t="inlineStr"/>
-      <c r="F26" s="44" t="n"/>
-      <c r="G26" s="44" t="n"/>
-      <c r="H26" s="44" t="n"/>
-      <c r="I26" s="44" t="n"/>
-      <c r="J26" s="44" t="n"/>
-      <c r="K26" s="44" t="n"/>
-      <c r="L26" s="45">
-        <f>IF(COUNT(F26:K26)=0,"",IFERROR(SUMPRODUCT(F26:K26,(F$5:K$5+(F$5:K$5="")))/SUMPRODUCT((F26:K26&lt;&gt;"")*(F$5:K$5+(F$5:K$5=""))),""))</f>
-        <v/>
-      </c>
-      <c r="M26" s="44" t="n"/>
-      <c r="N26" s="44" t="n"/>
-      <c r="O26" s="44" t="n"/>
-      <c r="P26" s="45">
-        <f>IF(COUNT(M26:O26)=0,"",IFERROR(SUMPRODUCT(M26:O26,(M$5:O$5+(M$5:O$5="")))/SUMPRODUCT((M26:O26&lt;&gt;"")*(M$5:O$5+(M$5:O$5=""))),""))</f>
-        <v/>
-      </c>
-      <c r="Q26" s="44" t="n"/>
-      <c r="R26" s="44" t="n"/>
-      <c r="S26" s="44" t="n"/>
-      <c r="T26" s="44" t="n"/>
-      <c r="U26" s="45">
-        <f>IF(COUNT(Q26:T26)=0,"",IFERROR(SUMPRODUCT(Q26:T26,(Q$5:T$5+(Q$5:T$5="")))/SUMPRODUCT((Q26:T26&lt;&gt;"")*(Q$5:T$5+(Q$5:T$5=""))),""))</f>
-        <v/>
-      </c>
-      <c r="V26" s="44" t="n"/>
-      <c r="W26" s="44" t="n"/>
-      <c r="X26" s="45">
-        <f>IF(COUNT(V26:W26)=0,"",IFERROR(SUMPRODUCT(V26:W26,(V$5:W$5+(V$5:W$5="")))/SUMPRODUCT((V26:W26&lt;&gt;"")*(V$5:W$5+(V$5:W$5=""))),""))</f>
-        <v/>
-      </c>
-      <c r="Y26" s="45">
-        <f>IFERROR(IF((ISNUMBER(P26)*(P$5+(P$5=""))+ISNUMBER(U26)*(U$5+(U$5=""))+ISNUMBER(X26)*(X$5+(X$5="")))=0,"",(N(P26)*(P$5+(P$5=""))+N(U26)*(U$5+(U$5=""))+N(X26)*(X$5+(X$5="")))/(ISNUMBER(P26)*(P$5+(P$5=""))+ISNUMBER(U26)*(U$5+(U$5=""))+ISNUMBER(X26)*(X$5+(X$5="")))),"")</f>
-        <v/>
-      </c>
-      <c r="Z26" s="46">
-        <f>IF(AND(ISNUMBER(L26),ISNUMBER(Y26)),L26*Y26,"")</f>
-        <v/>
-      </c>
-      <c r="AA26" s="47">
-        <f>IF(ISNUMBER(Z26),(Z26-1)/24,"")</f>
-        <v/>
-      </c>
-      <c r="AB26" s="48">
-        <f>IF(ISNUMBER(Z26),COUNTIF(Z$7:Z$27,"&gt;"&amp;Z26)+1,"")</f>
-        <v/>
-      </c>
-      <c r="AC26" s="49">
-        <f>COUNT(F26,G26,H26,I26,J26,K26,M26,N26,O26,Q26,R26,S26,T26,V26,W26)</f>
+      <c r="F26" s="44" t="n">
+        <v>-8.089423</v>
+      </c>
+      <c r="G26" s="44" t="n">
+        <v>-34.882717</v>
+      </c>
+      <c r="H26" s="42" t="inlineStr">
+        <is>
+          <t>Interseção</t>
+        </is>
+      </c>
+      <c r="I26" s="45" t="n"/>
+      <c r="J26" s="45" t="n"/>
+      <c r="K26" s="45" t="n"/>
+      <c r="L26" s="45" t="n"/>
+      <c r="M26" s="45" t="n"/>
+      <c r="N26" s="45" t="n"/>
+      <c r="O26" s="46">
+        <f>IF(COUNT(I26:N26)=0,"",IFERROR(SUMPRODUCT(I26:N26,(I$5:N$5+(I$5:N$5="")))/SUMPRODUCT((I26:N26&lt;&gt;"")*(I$5:N$5+(I$5:N$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="P26" s="45" t="n"/>
+      <c r="Q26" s="45" t="n"/>
+      <c r="R26" s="45" t="n"/>
+      <c r="S26" s="46">
+        <f>IF(COUNT(P26:R26)=0,"",IFERROR(SUMPRODUCT(P26:R26,(P$5:R$5+(P$5:R$5="")))/SUMPRODUCT((P26:R26&lt;&gt;"")*(P$5:R$5+(P$5:R$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="T26" s="45" t="n"/>
+      <c r="U26" s="45" t="n"/>
+      <c r="V26" s="45" t="n"/>
+      <c r="W26" s="45" t="n"/>
+      <c r="X26" s="46">
+        <f>IF(COUNT(T26:W26)=0,"",IFERROR(SUMPRODUCT(T26:W26,(T$5:W$5+(T$5:W$5="")))/SUMPRODUCT((T26:W26&lt;&gt;"")*(T$5:W$5+(T$5:W$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="Y26" s="45" t="n"/>
+      <c r="Z26" s="45" t="n"/>
+      <c r="AA26" s="46">
+        <f>IF(COUNT(Y26:Z26)=0,"",IFERROR(SUMPRODUCT(Y26:Z26,(Y$5:Z$5+(Y$5:Z$5="")))/SUMPRODUCT((Y26:Z26&lt;&gt;"")*(Y$5:Z$5+(Y$5:Z$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="AB26" s="46">
+        <f>IFERROR(IF((ISNUMBER(S26)*(S$5+(S$5=""))+ISNUMBER(X26)*(X$5+(X$5=""))+ISNUMBER(AA26)*(AA$5+(AA$5="")))=0,"",(N(S26)*(S$5+(S$5=""))+N(X26)*(X$5+(X$5=""))+N(AA26)*(AA$5+(AA$5="")))/(ISNUMBER(S26)*(S$5+(S$5=""))+ISNUMBER(X26)*(X$5+(X$5=""))+ISNUMBER(AA26)*(AA$5+(AA$5="")))),"")</f>
+        <v/>
+      </c>
+      <c r="AC26" s="47">
+        <f>IF(AND(ISNUMBER(O26),ISNUMBER(AB26)),O26*AB26,"")</f>
+        <v/>
+      </c>
+      <c r="AD26" s="48">
+        <f>IF(ISNUMBER(AC26),(AC26-1)/24,"")</f>
+        <v/>
+      </c>
+      <c r="AE26" s="49">
+        <f>IF(ISNUMBER(AC26),COUNTIF(AC$7:AC$27,"&gt;"&amp;AC26)+1,"")</f>
+        <v/>
+      </c>
+      <c r="AF26" s="50">
+        <f>COUNT(I26,J26,K26,L26,M26,N26,P26,Q26,R26,T26,U26,V26,W26,Y26,Z26)</f>
         <v/>
       </c>
     </row>
@@ -4088,55 +4331,66 @@
           <t>G4</t>
         </is>
       </c>
-      <c r="F27" s="44" t="n"/>
-      <c r="G27" s="44" t="n"/>
-      <c r="H27" s="44" t="n"/>
-      <c r="I27" s="44" t="n"/>
-      <c r="J27" s="44" t="n"/>
-      <c r="K27" s="44" t="n"/>
-      <c r="L27" s="45">
-        <f>IF(COUNT(F27:K27)=0,"",IFERROR(SUMPRODUCT(F27:K27,(F$5:K$5+(F$5:K$5="")))/SUMPRODUCT((F27:K27&lt;&gt;"")*(F$5:K$5+(F$5:K$5=""))),""))</f>
-        <v/>
-      </c>
-      <c r="M27" s="44" t="n"/>
-      <c r="N27" s="44" t="n"/>
-      <c r="O27" s="44" t="n"/>
-      <c r="P27" s="45">
-        <f>IF(COUNT(M27:O27)=0,"",IFERROR(SUMPRODUCT(M27:O27,(M$5:O$5+(M$5:O$5="")))/SUMPRODUCT((M27:O27&lt;&gt;"")*(M$5:O$5+(M$5:O$5=""))),""))</f>
-        <v/>
-      </c>
-      <c r="Q27" s="44" t="n"/>
-      <c r="R27" s="44" t="n"/>
-      <c r="S27" s="44" t="n"/>
-      <c r="T27" s="44" t="n"/>
-      <c r="U27" s="45">
-        <f>IF(COUNT(Q27:T27)=0,"",IFERROR(SUMPRODUCT(Q27:T27,(Q$5:T$5+(Q$5:T$5="")))/SUMPRODUCT((Q27:T27&lt;&gt;"")*(Q$5:T$5+(Q$5:T$5=""))),""))</f>
-        <v/>
-      </c>
-      <c r="V27" s="44" t="n"/>
-      <c r="W27" s="44" t="n"/>
-      <c r="X27" s="45">
-        <f>IF(COUNT(V27:W27)=0,"",IFERROR(SUMPRODUCT(V27:W27,(V$5:W$5+(V$5:W$5="")))/SUMPRODUCT((V27:W27&lt;&gt;"")*(V$5:W$5+(V$5:W$5=""))),""))</f>
-        <v/>
-      </c>
-      <c r="Y27" s="45">
-        <f>IFERROR(IF((ISNUMBER(P27)*(P$5+(P$5=""))+ISNUMBER(U27)*(U$5+(U$5=""))+ISNUMBER(X27)*(X$5+(X$5="")))=0,"",(N(P27)*(P$5+(P$5=""))+N(U27)*(U$5+(U$5=""))+N(X27)*(X$5+(X$5="")))/(ISNUMBER(P27)*(P$5+(P$5=""))+ISNUMBER(U27)*(U$5+(U$5=""))+ISNUMBER(X27)*(X$5+(X$5="")))),"")</f>
-        <v/>
-      </c>
-      <c r="Z27" s="46">
-        <f>IF(AND(ISNUMBER(L27),ISNUMBER(Y27)),L27*Y27,"")</f>
-        <v/>
-      </c>
-      <c r="AA27" s="47">
-        <f>IF(ISNUMBER(Z27),(Z27-1)/24,"")</f>
-        <v/>
-      </c>
-      <c r="AB27" s="48">
-        <f>IF(ISNUMBER(Z27),COUNTIF(Z$7:Z$27,"&gt;"&amp;Z27)+1,"")</f>
-        <v/>
-      </c>
-      <c r="AC27" s="49">
-        <f>COUNT(F27,G27,H27,I27,J27,K27,M27,N27,O27,Q27,R27,S27,T27,V27,W27)</f>
+      <c r="F27" s="44" t="n">
+        <v>-8.113868999999999</v>
+      </c>
+      <c r="G27" s="44" t="n">
+        <v>-34.940702</v>
+      </c>
+      <c r="H27" s="42" t="inlineStr">
+        <is>
+          <t>Interseção</t>
+        </is>
+      </c>
+      <c r="I27" s="45" t="n"/>
+      <c r="J27" s="45" t="n"/>
+      <c r="K27" s="45" t="n"/>
+      <c r="L27" s="45" t="n"/>
+      <c r="M27" s="45" t="n"/>
+      <c r="N27" s="45" t="n"/>
+      <c r="O27" s="46">
+        <f>IF(COUNT(I27:N27)=0,"",IFERROR(SUMPRODUCT(I27:N27,(I$5:N$5+(I$5:N$5="")))/SUMPRODUCT((I27:N27&lt;&gt;"")*(I$5:N$5+(I$5:N$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="P27" s="45" t="n"/>
+      <c r="Q27" s="45" t="n"/>
+      <c r="R27" s="45" t="n"/>
+      <c r="S27" s="46">
+        <f>IF(COUNT(P27:R27)=0,"",IFERROR(SUMPRODUCT(P27:R27,(P$5:R$5+(P$5:R$5="")))/SUMPRODUCT((P27:R27&lt;&gt;"")*(P$5:R$5+(P$5:R$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="T27" s="45" t="n"/>
+      <c r="U27" s="45" t="n"/>
+      <c r="V27" s="45" t="n"/>
+      <c r="W27" s="45" t="n"/>
+      <c r="X27" s="46">
+        <f>IF(COUNT(T27:W27)=0,"",IFERROR(SUMPRODUCT(T27:W27,(T$5:W$5+(T$5:W$5="")))/SUMPRODUCT((T27:W27&lt;&gt;"")*(T$5:W$5+(T$5:W$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="Y27" s="45" t="n"/>
+      <c r="Z27" s="45" t="n"/>
+      <c r="AA27" s="46">
+        <f>IF(COUNT(Y27:Z27)=0,"",IFERROR(SUMPRODUCT(Y27:Z27,(Y$5:Z$5+(Y$5:Z$5="")))/SUMPRODUCT((Y27:Z27&lt;&gt;"")*(Y$5:Z$5+(Y$5:Z$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="AB27" s="46">
+        <f>IFERROR(IF((ISNUMBER(S27)*(S$5+(S$5=""))+ISNUMBER(X27)*(X$5+(X$5=""))+ISNUMBER(AA27)*(AA$5+(AA$5="")))=0,"",(N(S27)*(S$5+(S$5=""))+N(X27)*(X$5+(X$5=""))+N(AA27)*(AA$5+(AA$5="")))/(ISNUMBER(S27)*(S$5+(S$5=""))+ISNUMBER(X27)*(X$5+(X$5=""))+ISNUMBER(AA27)*(AA$5+(AA$5="")))),"")</f>
+        <v/>
+      </c>
+      <c r="AC27" s="47">
+        <f>IF(AND(ISNUMBER(O27),ISNUMBER(AB27)),O27*AB27,"")</f>
+        <v/>
+      </c>
+      <c r="AD27" s="48">
+        <f>IF(ISNUMBER(AC27),(AC27-1)/24,"")</f>
+        <v/>
+      </c>
+      <c r="AE27" s="49">
+        <f>IF(ISNUMBER(AC27),COUNTIF(AC$7:AC$27,"&gt;"&amp;AC27)+1,"")</f>
+        <v/>
+      </c>
+      <c r="AF27" s="50">
+        <f>COUNT(I27,J27,K27,L27,M27,N27,P27,Q27,R27,T27,U27,V27,W27,Y27,Z27)</f>
         <v/>
       </c>
     </row>
@@ -4148,35 +4402,35 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="50" t="inlineStr">
+      <c r="A30" s="51" t="inlineStr">
         <is>
           <t>• Nota do critério = média ponderada das notas dos subcritérios preenchidos (pesos da linha 5; vazio = 1).</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="50" t="inlineStr">
+      <c r="A31" s="51" t="inlineStr">
         <is>
           <t>• Consequência = média ponderada das notas de Exposição, Vulnerabilidade e Impacto (pesos da linha 5 nas colunas cinza 'Nota').</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="50" t="inlineStr">
+      <c r="A32" s="51" t="inlineStr">
         <is>
           <t>• Risco = nota da Probabilidade × Consequência (1 a 25).</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="50" t="inlineStr">
+      <c r="A33" s="51" t="inlineStr">
         <is>
           <t>• Índice de risco (0–1) = (Risco − 1) ÷ 24. 0 = risco mínimo (P = 1 e C = 1); 1 = risco máximo (P = 5 e C = 5). Corte da matriz (risco 9) = índice 0,333. O ranking é o mesmo do Risco.</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="50" t="inlineStr">
+      <c r="A34" s="51" t="inlineStr">
         <is>
           <t>• Posição = ranking pelo Risco (1 = maior risco). Empates recebem a mesma posição.</t>
         </is>
@@ -4184,13 +4438,13 @@
     </row>
   </sheetData>
   <mergeCells count="5">
-    <mergeCell ref="Y4:AC4"/>
-    <mergeCell ref="M4:P4"/>
-    <mergeCell ref="F4:L4"/>
-    <mergeCell ref="V4:X4"/>
-    <mergeCell ref="Q4:U4"/>
+    <mergeCell ref="AB4:AF4"/>
+    <mergeCell ref="I4:O4"/>
+    <mergeCell ref="P4:S4"/>
+    <mergeCell ref="Y4:AA4"/>
+    <mergeCell ref="T4:X4"/>
   </mergeCells>
-  <conditionalFormatting sqref="AA7:AA27">
+  <conditionalFormatting sqref="AD7:AD27">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="num" val="0"/>
@@ -4203,11 +4457,11 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="F7:F27 G7:G27 H7:H27 I7:I27 J7:J27 K7:K27 M7:M27 N7:N27 O7:O27 Q7:Q27 R7:R27 S7:S27 T7:T27 V7:V27 W7:W27" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Nota inválida" error="Use um número inteiro de 1 a 5 (5 = mais crítico)." type="whole" operator="between">
+    <dataValidation sqref="I7:I27 J7:J27 K7:K27 L7:L27 M7:M27 N7:N27 P7:P27 Q7:Q27 R7:R27 T7:T27 U7:U27 V7:V27 W7:W27 Y7:Y27 Z7:Z27" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Nota inválida" error="Use um número inteiro de 1 a 5 (5 = mais crítico)." type="whole" operator="between">
       <formula1>1</formula1>
       <formula2>5</formula2>
     </dataValidation>
-    <dataValidation sqref="F5 G5 H5 I5 J5 K5 M5 N5 O5 P5 Q5 R5 S5 T5 U5 V5 W5 X5" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Peso deve ser um número maior ou igual a zero." type="decimal" operator="greaterThanOrEqual">
+    <dataValidation sqref="I5 J5 K5 L5 M5 N5 P5 Q5 R5 S5 T5 U5 V5 W5 X5 Y5 Z5 AA5" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Peso deve ser um número maior ou igual a zero." type="decimal" operator="greaterThanOrEqual">
       <formula1>0</formula1>
     </dataValidation>
   </dataValidations>
@@ -4239,41 +4493,41 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="51" t="inlineStr">
+      <c r="A2" s="52" t="inlineStr">
         <is>
           <t>Para quem não participou das discussões do modelo. Os papéis dos órgãos são uma leitura preliminar, ainda não confirmada com cada órgão.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="52" t="inlineStr">
+      <c r="A4" s="53" t="inlineStr">
         <is>
           <t>Grupo</t>
         </is>
       </c>
-      <c r="B4" s="52" t="inlineStr">
+      <c r="B4" s="53" t="inlineStr">
         <is>
           <t>Termo</t>
         </is>
       </c>
-      <c r="C4" s="52" t="inlineStr">
+      <c r="C4" s="53" t="inlineStr">
         <is>
           <t>O que significa</t>
         </is>
       </c>
-      <c r="D4" s="52" t="inlineStr">
+      <c r="D4" s="53" t="inlineStr">
         <is>
           <t>Exemplo no projeto</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="53" t="inlineStr">
+      <c r="A5" s="54" t="inlineStr">
         <is>
           <t>Modelo de risco</t>
         </is>
       </c>
-      <c r="B5" s="54" t="inlineStr">
+      <c r="B5" s="55" t="inlineStr">
         <is>
           <t>Risco</t>
         </is>
@@ -4290,12 +4544,12 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="53" t="inlineStr">
+      <c r="A6" s="54" t="inlineStr">
         <is>
           <t>Modelo de risco</t>
         </is>
       </c>
-      <c r="B6" s="54" t="inlineStr">
+      <c r="B6" s="55" t="inlineStr">
         <is>
           <t>Critério</t>
         </is>
@@ -4312,12 +4566,12 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="53" t="inlineStr">
+      <c r="A7" s="54" t="inlineStr">
         <is>
           <t>Modelo de risco</t>
         </is>
       </c>
-      <c r="B7" s="54" t="inlineStr">
+      <c r="B7" s="55" t="inlineStr">
         <is>
           <t>Subcritério</t>
         </is>
@@ -4334,12 +4588,12 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="53" t="inlineStr">
+      <c r="A8" s="54" t="inlineStr">
         <is>
           <t>Modelo de risco</t>
         </is>
       </c>
-      <c r="B8" s="54" t="inlineStr">
+      <c r="B8" s="55" t="inlineStr">
         <is>
           <t>Probabilidade</t>
         </is>
@@ -4356,12 +4610,12 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="53" t="inlineStr">
+      <c r="A9" s="54" t="inlineStr">
         <is>
           <t>Modelo de risco</t>
         </is>
       </c>
-      <c r="B9" s="54" t="inlineStr">
+      <c r="B9" s="55" t="inlineStr">
         <is>
           <t>Exposição</t>
         </is>
@@ -4378,12 +4632,12 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="53" t="inlineStr">
+      <c r="A10" s="54" t="inlineStr">
         <is>
           <t>Modelo de risco</t>
         </is>
       </c>
-      <c r="B10" s="54" t="inlineStr">
+      <c r="B10" s="55" t="inlineStr">
         <is>
           <t>Vulnerabilidade</t>
         </is>
@@ -4400,12 +4654,12 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="53" t="inlineStr">
+      <c r="A11" s="54" t="inlineStr">
         <is>
           <t>Modelo de risco</t>
         </is>
       </c>
-      <c r="B11" s="54" t="inlineStr">
+      <c r="B11" s="55" t="inlineStr">
         <is>
           <t>Impacto</t>
         </is>
@@ -4422,12 +4676,12 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="53" t="inlineStr">
+      <c r="A12" s="54" t="inlineStr">
         <is>
           <t>Modelo de risco</t>
         </is>
       </c>
-      <c r="B12" s="54" t="inlineStr">
+      <c r="B12" s="55" t="inlineStr">
         <is>
           <t>Consequência</t>
         </is>
@@ -4444,12 +4698,12 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="53" t="inlineStr">
+      <c r="A13" s="54" t="inlineStr">
         <is>
           <t>Modelo de risco</t>
         </is>
       </c>
-      <c r="B13" s="54" t="inlineStr">
+      <c r="B13" s="55" t="inlineStr">
         <is>
           <t>Nota (1 a 5)</t>
         </is>
@@ -4466,12 +4720,12 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="53" t="inlineStr">
+      <c r="A14" s="54" t="inlineStr">
         <is>
           <t>Modelo de risco</t>
         </is>
       </c>
-      <c r="B14" s="54" t="inlineStr">
+      <c r="B14" s="55" t="inlineStr">
         <is>
           <t>Peso</t>
         </is>
@@ -4488,12 +4742,12 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="53" t="inlineStr">
+      <c r="A15" s="54" t="inlineStr">
         <is>
           <t>Modelo de risco</t>
         </is>
       </c>
-      <c r="B15" s="54" t="inlineStr">
+      <c r="B15" s="55" t="inlineStr">
         <is>
           <t>Média ponderada</t>
         </is>
@@ -4510,12 +4764,12 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="53" t="inlineStr">
+      <c r="A16" s="54" t="inlineStr">
         <is>
           <t>Modelo de risco</t>
         </is>
       </c>
-      <c r="B16" s="54" t="inlineStr">
+      <c r="B16" s="55" t="inlineStr">
         <is>
           <t>Cobertura</t>
         </is>
@@ -4532,12 +4786,12 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="53" t="inlineStr">
+      <c r="A17" s="54" t="inlineStr">
         <is>
           <t>Modelo de risco</t>
         </is>
       </c>
-      <c r="B17" s="54" t="inlineStr">
+      <c r="B17" s="55" t="inlineStr">
         <is>
           <t>Sem Probabilidade, sem risco</t>
         </is>
@@ -4554,12 +4808,12 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="53" t="inlineStr">
+      <c r="A18" s="54" t="inlineStr">
         <is>
           <t>Modelo de risco</t>
         </is>
       </c>
-      <c r="B18" s="54" t="inlineStr">
+      <c r="B18" s="55" t="inlineStr">
         <is>
           <t>Tratabilidade</t>
         </is>
@@ -4576,12 +4830,12 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="53" t="inlineStr">
+      <c r="A19" s="54" t="inlineStr">
         <is>
           <t>Modelo de risco</t>
         </is>
       </c>
-      <c r="B19" s="54" t="inlineStr">
+      <c r="B19" s="55" t="inlineStr">
         <is>
           <t>Matriz risco × tratabilidade</t>
         </is>
@@ -4598,12 +4852,12 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="53" t="inlineStr">
+      <c r="A20" s="54" t="inlineStr">
         <is>
           <t>Modelo de risco</t>
         </is>
       </c>
-      <c r="B20" s="54" t="inlineStr">
+      <c r="B20" s="55" t="inlineStr">
         <is>
           <t>Agir já / Estruturar / Oportunidade / Monitorar</t>
         </is>
@@ -4616,12 +4870,12 @@
       <c r="D20" s="43" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" s="53" t="inlineStr">
+      <c r="A21" s="54" t="inlineStr">
         <is>
           <t>Modelo de risco</t>
         </is>
       </c>
-      <c r="B21" s="54" t="inlineStr">
+      <c r="B21" s="55" t="inlineStr">
         <is>
           <t>Diagnóstico de causa</t>
         </is>
@@ -4638,12 +4892,12 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="53" t="inlineStr">
+      <c r="A22" s="54" t="inlineStr">
         <is>
           <t>Modelo de risco</t>
         </is>
       </c>
-      <c r="B22" s="54" t="inlineStr">
+      <c r="B22" s="55" t="inlineStr">
         <is>
           <t>Análise de sensibilidade</t>
         </is>
@@ -4660,12 +4914,12 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="55" t="inlineStr">
+      <c r="A23" s="56" t="inlineStr">
         <is>
           <t>Tipo de nota</t>
         </is>
       </c>
-      <c r="B23" s="54" t="inlineStr">
+      <c r="B23" s="55" t="inlineStr">
         <is>
           <t>Faixa fixa</t>
         </is>
@@ -4682,12 +4936,12 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="55" t="inlineStr">
+      <c r="A24" s="56" t="inlineStr">
         <is>
           <t>Tipo de nota</t>
         </is>
       </c>
-      <c r="B24" s="54" t="inlineStr">
+      <c r="B24" s="55" t="inlineStr">
         <is>
           <t>Classe</t>
         </is>
@@ -4704,12 +4958,12 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="55" t="inlineStr">
+      <c r="A25" s="56" t="inlineStr">
         <is>
           <t>Tipo de nota</t>
         </is>
       </c>
-      <c r="B25" s="54" t="inlineStr">
+      <c r="B25" s="55" t="inlineStr">
         <is>
           <t>Quintil</t>
         </is>
@@ -4726,12 +4980,12 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="55" t="inlineStr">
+      <c r="A26" s="56" t="inlineStr">
         <is>
           <t>Tipo de nota</t>
         </is>
       </c>
-      <c r="B26" s="54" t="inlineStr">
+      <c r="B26" s="55" t="inlineStr">
         <is>
           <t>Quintil invertido</t>
         </is>
@@ -4748,12 +5002,12 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="55" t="inlineStr">
+      <c r="A27" s="56" t="inlineStr">
         <is>
           <t>Tipo de nota</t>
         </is>
       </c>
-      <c r="B27" s="54" t="inlineStr">
+      <c r="B27" s="55" t="inlineStr">
         <is>
           <t>Faixa provisória</t>
         </is>
@@ -4770,12 +5024,12 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="55" t="inlineStr">
+      <c r="A28" s="56" t="inlineStr">
         <is>
           <t>Tipo de nota</t>
         </is>
       </c>
-      <c r="B28" s="54" t="inlineStr">
+      <c r="B28" s="55" t="inlineStr">
         <is>
           <t>Origem da faixa</t>
         </is>
@@ -4788,12 +5042,12 @@
       <c r="D28" s="43" t="inlineStr"/>
     </row>
     <row r="29">
-      <c r="A29" s="56" t="inlineStr">
+      <c r="A29" s="57" t="inlineStr">
         <is>
           <t>Território e SIG</t>
         </is>
       </c>
-      <c r="B29" s="54" t="inlineStr">
+      <c r="B29" s="55" t="inlineStr">
         <is>
           <t>Ponto crítico</t>
         </is>
@@ -4810,12 +5064,12 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="56" t="inlineStr">
+      <c r="A30" s="57" t="inlineStr">
         <is>
           <t>Território e SIG</t>
         </is>
       </c>
-      <c r="B30" s="54" t="inlineStr">
+      <c r="B30" s="55" t="inlineStr">
         <is>
           <t>Trecho (Linha / Vários)</t>
         </is>
@@ -4832,12 +5086,12 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="56" t="inlineStr">
+      <c r="A31" s="57" t="inlineStr">
         <is>
           <t>Território e SIG</t>
         </is>
       </c>
-      <c r="B31" s="54" t="inlineStr">
+      <c r="B31" s="55" t="inlineStr">
         <is>
           <t>RPA 6</t>
         </is>
@@ -4850,12 +5104,12 @@
       <c r="D31" s="43" t="inlineStr"/>
     </row>
     <row r="32">
-      <c r="A32" s="56" t="inlineStr">
+      <c r="A32" s="57" t="inlineStr">
         <is>
           <t>Território e SIG</t>
         </is>
       </c>
-      <c r="B32" s="54" t="inlineStr">
+      <c r="B32" s="55" t="inlineStr">
         <is>
           <t>SIG</t>
         </is>
@@ -4868,12 +5122,12 @@
       <c r="D32" s="43" t="inlineStr"/>
     </row>
     <row r="33">
-      <c r="A33" s="56" t="inlineStr">
+      <c r="A33" s="57" t="inlineStr">
         <is>
           <t>Território e SIG</t>
         </is>
       </c>
-      <c r="B33" s="54" t="inlineStr">
+      <c r="B33" s="55" t="inlineStr">
         <is>
           <t>Círculo de 300 m (buffer)</t>
         </is>
@@ -4890,12 +5144,12 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="56" t="inlineStr">
+      <c r="A34" s="57" t="inlineStr">
         <is>
           <t>Território e SIG</t>
         </is>
       </c>
-      <c r="B34" s="54" t="inlineStr">
+      <c r="B34" s="55" t="inlineStr">
         <is>
           <t>Área de influência de 1 km</t>
         </is>
@@ -4908,12 +5162,12 @@
       <c r="D34" s="43" t="inlineStr"/>
     </row>
     <row r="35">
-      <c r="A35" s="56" t="inlineStr">
+      <c r="A35" s="57" t="inlineStr">
         <is>
           <t>Território e SIG</t>
         </is>
       </c>
-      <c r="B35" s="54" t="inlineStr">
+      <c r="B35" s="55" t="inlineStr">
         <is>
           <t>Grupo de sobreposição (G1–G5)</t>
         </is>
@@ -4930,12 +5184,12 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="56" t="inlineStr">
+      <c r="A36" s="57" t="inlineStr">
         <is>
           <t>Território e SIG</t>
         </is>
       </c>
-      <c r="B36" s="54" t="inlineStr">
+      <c r="B36" s="55" t="inlineStr">
         <is>
           <t>Ponderação por área</t>
         </is>
@@ -4952,12 +5206,12 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="56" t="inlineStr">
+      <c r="A37" s="57" t="inlineStr">
         <is>
           <t>Território e SIG</t>
         </is>
       </c>
-      <c r="B37" s="54" t="inlineStr">
+      <c r="B37" s="55" t="inlineStr">
         <is>
           <t>EPSG:31985 (SIRGAS 2000 / UTM 25S)</t>
         </is>
@@ -4970,12 +5224,12 @@
       <c r="D37" s="43" t="inlineStr"/>
     </row>
     <row r="38">
-      <c r="A38" s="56" t="inlineStr">
+      <c r="A38" s="57" t="inlineStr">
         <is>
           <t>Território e SIG</t>
         </is>
       </c>
-      <c r="B38" s="54" t="inlineStr">
+      <c r="B38" s="55" t="inlineStr">
         <is>
           <t>Coordenada aproximada / verificada</t>
         </is>
@@ -4992,12 +5246,12 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="56" t="inlineStr">
+      <c r="A39" s="57" t="inlineStr">
         <is>
           <t>Território e SIG</t>
         </is>
       </c>
-      <c r="B39" s="54" t="inlineStr">
+      <c r="B39" s="55" t="inlineStr">
         <is>
           <t>Bacia / sub-bacia</t>
         </is>
@@ -5014,12 +5268,12 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="56" t="inlineStr">
+      <c r="A40" s="57" t="inlineStr">
         <is>
           <t>Território e SIG</t>
         </is>
       </c>
-      <c r="B40" s="54" t="inlineStr">
+      <c r="B40" s="55" t="inlineStr">
         <is>
           <t>Shapefile / GeoJSON</t>
         </is>
@@ -5036,12 +5290,12 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="57" t="inlineStr">
+      <c r="A41" s="58" t="inlineStr">
         <is>
           <t>Fontes de dados</t>
         </is>
       </c>
-      <c r="B41" s="54" t="inlineStr">
+      <c r="B41" s="55" t="inlineStr">
         <is>
           <t>Censo 2022 (IBGE)</t>
         </is>
@@ -5054,12 +5308,12 @@
       <c r="D41" s="43" t="inlineStr"/>
     </row>
     <row r="42">
-      <c r="A42" s="57" t="inlineStr">
+      <c r="A42" s="58" t="inlineStr">
         <is>
           <t>Fontes de dados</t>
         </is>
       </c>
-      <c r="B42" s="54" t="inlineStr">
+      <c r="B42" s="55" t="inlineStr">
         <is>
           <t>Setor censitário</t>
         </is>
@@ -5072,12 +5326,12 @@
       <c r="D42" s="43" t="inlineStr"/>
     </row>
     <row r="43">
-      <c r="A43" s="57" t="inlineStr">
+      <c r="A43" s="58" t="inlineStr">
         <is>
           <t>Fontes de dados</t>
         </is>
       </c>
-      <c r="B43" s="54" t="inlineStr">
+      <c r="B43" s="55" t="inlineStr">
         <is>
           <t>Grade Estatística (IBGE)</t>
         </is>
@@ -5094,12 +5348,12 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="57" t="inlineStr">
+      <c r="A44" s="58" t="inlineStr">
         <is>
           <t>Fontes de dados</t>
         </is>
       </c>
-      <c r="B44" s="54" t="inlineStr">
+      <c r="B44" s="55" t="inlineStr">
         <is>
           <t>CNEFE (IBGE)</t>
         </is>
@@ -5116,12 +5370,12 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="57" t="inlineStr">
+      <c r="A45" s="58" t="inlineStr">
         <is>
           <t>Fontes de dados</t>
         </is>
       </c>
-      <c r="B45" s="54" t="inlineStr">
+      <c r="B45" s="55" t="inlineStr">
         <is>
           <t>Favelas e Comunidades Urbanas (IBGE)</t>
         </is>
@@ -5138,12 +5392,12 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="57" t="inlineStr">
+      <c r="A46" s="58" t="inlineStr">
         <is>
           <t>Fontes de dados</t>
         </is>
       </c>
-      <c r="B46" s="54" t="inlineStr">
+      <c r="B46" s="55" t="inlineStr">
         <is>
           <t>IVS (Ipea)</t>
         </is>
@@ -5160,12 +5414,12 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="57" t="inlineStr">
+      <c r="A47" s="58" t="inlineStr">
         <is>
           <t>Fontes de dados</t>
         </is>
       </c>
-      <c r="B47" s="54" t="inlineStr">
+      <c r="B47" s="55" t="inlineStr">
         <is>
           <t>UDH</t>
         </is>
@@ -5178,12 +5432,12 @@
       <c r="D47" s="43" t="inlineStr"/>
     </row>
     <row r="48">
-      <c r="A48" s="57" t="inlineStr">
+      <c r="A48" s="58" t="inlineStr">
         <is>
           <t>Fontes de dados</t>
         </is>
       </c>
-      <c r="B48" s="54" t="inlineStr">
+      <c r="B48" s="55" t="inlineStr">
         <is>
           <t>MapBiomas</t>
         </is>
@@ -5200,12 +5454,12 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="57" t="inlineStr">
+      <c r="A49" s="58" t="inlineStr">
         <is>
           <t>Fontes de dados</t>
         </is>
       </c>
-      <c r="B49" s="54" t="inlineStr">
+      <c r="B49" s="55" t="inlineStr">
         <is>
           <t>ESIG</t>
         </is>
@@ -5218,12 +5472,12 @@
       <c r="D49" s="43" t="inlineStr"/>
     </row>
     <row r="50">
-      <c r="A50" s="57" t="inlineStr">
+      <c r="A50" s="58" t="inlineStr">
         <is>
           <t>Fontes de dados</t>
         </is>
       </c>
-      <c r="B50" s="54" t="inlineStr">
+      <c r="B50" s="55" t="inlineStr">
         <is>
           <t>CNES / DATASUS</t>
         </is>
@@ -5240,12 +5494,12 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="57" t="inlineStr">
+      <c r="A51" s="58" t="inlineStr">
         <is>
           <t>Fontes de dados</t>
         </is>
       </c>
-      <c r="B51" s="54" t="inlineStr">
+      <c r="B51" s="55" t="inlineStr">
         <is>
           <t>APAC / Cemaden</t>
         </is>
@@ -5258,12 +5512,12 @@
       <c r="D51" s="43" t="inlineStr"/>
     </row>
     <row r="52">
-      <c r="A52" s="57" t="inlineStr">
+      <c r="A52" s="58" t="inlineStr">
         <is>
           <t>Fontes de dados</t>
         </is>
       </c>
-      <c r="B52" s="54" t="inlineStr">
+      <c r="B52" s="55" t="inlineStr">
         <is>
           <t>PMDR</t>
         </is>
@@ -5276,12 +5530,12 @@
       <c r="D52" s="43" t="inlineStr"/>
     </row>
     <row r="53">
-      <c r="A53" s="57" t="inlineStr">
+      <c r="A53" s="58" t="inlineStr">
         <is>
           <t>Fontes de dados</t>
         </is>
       </c>
-      <c r="B53" s="54" t="inlineStr">
+      <c r="B53" s="55" t="inlineStr">
         <is>
           <t>Ficha EMLURB</t>
         </is>
@@ -5298,12 +5552,12 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="58" t="inlineStr">
+      <c r="A54" s="59" t="inlineStr">
         <is>
           <t>Checklist</t>
         </is>
       </c>
-      <c r="B54" s="54" t="inlineStr">
+      <c r="B54" s="55" t="inlineStr">
         <is>
           <t>Recomendação</t>
         </is>
@@ -5316,12 +5570,12 @@
       <c r="D54" s="43" t="inlineStr"/>
     </row>
     <row r="55">
-      <c r="A55" s="58" t="inlineStr">
+      <c r="A55" s="59" t="inlineStr">
         <is>
           <t>Checklist</t>
         </is>
       </c>
-      <c r="B55" s="54" t="inlineStr">
+      <c r="B55" s="55" t="inlineStr">
         <is>
           <t>Fonte confirmada?</t>
         </is>
@@ -5334,12 +5588,12 @@
       <c r="D55" s="43" t="inlineStr"/>
     </row>
     <row r="56">
-      <c r="A56" s="58" t="inlineStr">
+      <c r="A56" s="59" t="inlineStr">
         <is>
           <t>Checklist</t>
         </is>
       </c>
-      <c r="B56" s="54" t="inlineStr">
+      <c r="B56" s="55" t="inlineStr">
         <is>
           <t>Dado existe na fonte?</t>
         </is>
@@ -5356,12 +5610,12 @@
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="58" t="inlineStr">
+      <c r="A57" s="59" t="inlineStr">
         <is>
           <t>Checklist</t>
         </is>
       </c>
-      <c r="B57" s="54" t="inlineStr">
+      <c r="B57" s="55" t="inlineStr">
         <is>
           <t>Sim / Parcial / Não / Pendente</t>
         </is>
@@ -5374,12 +5628,12 @@
       <c r="D57" s="43" t="inlineStr"/>
     </row>
     <row r="58">
-      <c r="A58" s="58" t="inlineStr">
+      <c r="A58" s="59" t="inlineStr">
         <is>
           <t>Checklist</t>
         </is>
       </c>
-      <c r="B58" s="54" t="inlineStr">
+      <c r="B58" s="55" t="inlineStr">
         <is>
           <t>Busca prévia (Claude)</t>
         </is>
@@ -5392,12 +5646,12 @@
       <c r="D58" s="43" t="inlineStr"/>
     </row>
     <row r="59">
-      <c r="A59" s="59" t="inlineStr">
+      <c r="A59" s="60" t="inlineStr">
         <is>
           <t>Órgãos</t>
         </is>
       </c>
-      <c r="B59" s="54" t="inlineStr">
+      <c r="B59" s="55" t="inlineStr">
         <is>
           <t>COP</t>
         </is>
@@ -5410,12 +5664,12 @@
       <c r="D59" s="43" t="inlineStr"/>
     </row>
     <row r="60">
-      <c r="A60" s="59" t="inlineStr">
+      <c r="A60" s="60" t="inlineStr">
         <is>
           <t>Órgãos</t>
         </is>
       </c>
-      <c r="B60" s="54" t="inlineStr">
+      <c r="B60" s="55" t="inlineStr">
         <is>
           <t>EMLURB</t>
         </is>
@@ -5428,12 +5682,12 @@
       <c r="D60" s="43" t="inlineStr"/>
     </row>
     <row r="61">
-      <c r="A61" s="59" t="inlineStr">
+      <c r="A61" s="60" t="inlineStr">
         <is>
           <t>Órgãos</t>
         </is>
       </c>
-      <c r="B61" s="54" t="inlineStr">
+      <c r="B61" s="55" t="inlineStr">
         <is>
           <t>Defesa Civil (Sedec)</t>
         </is>
@@ -5446,12 +5700,12 @@
       <c r="D61" s="43" t="inlineStr"/>
     </row>
     <row r="62">
-      <c r="A62" s="59" t="inlineStr">
+      <c r="A62" s="60" t="inlineStr">
         <is>
           <t>Órgãos</t>
         </is>
       </c>
-      <c r="B62" s="54" t="inlineStr">
+      <c r="B62" s="55" t="inlineStr">
         <is>
           <t>URB</t>
         </is>
@@ -5464,12 +5718,12 @@
       <c r="D62" s="43" t="inlineStr"/>
     </row>
     <row r="63">
-      <c r="A63" s="59" t="inlineStr">
+      <c r="A63" s="60" t="inlineStr">
         <is>
           <t>Órgãos</t>
         </is>
       </c>
-      <c r="B63" s="54" t="inlineStr">
+      <c r="B63" s="55" t="inlineStr">
         <is>
           <t>CTTU</t>
         </is>
@@ -5482,12 +5736,12 @@
       <c r="D63" s="43" t="inlineStr"/>
     </row>
     <row r="64">
-      <c r="A64" s="59" t="inlineStr">
+      <c r="A64" s="60" t="inlineStr">
         <is>
           <t>Órgãos</t>
         </is>
       </c>
-      <c r="B64" s="54" t="inlineStr">
+      <c r="B64" s="55" t="inlineStr">
         <is>
           <t>Compesa</t>
         </is>
@@ -5500,12 +5754,12 @@
       <c r="D64" s="43" t="inlineStr"/>
     </row>
     <row r="65">
-      <c r="A65" s="59" t="inlineStr">
+      <c r="A65" s="60" t="inlineStr">
         <is>
           <t>Órgãos</t>
         </is>
       </c>
-      <c r="B65" s="54" t="inlineStr">
+      <c r="B65" s="55" t="inlineStr">
         <is>
           <t>ProMorar</t>
         </is>
@@ -5518,12 +5772,12 @@
       <c r="D65" s="43" t="inlineStr"/>
     </row>
     <row r="66">
-      <c r="A66" s="59" t="inlineStr">
+      <c r="A66" s="60" t="inlineStr">
         <is>
           <t>Órgãos</t>
         </is>
       </c>
-      <c r="B66" s="54" t="inlineStr">
+      <c r="B66" s="55" t="inlineStr">
         <is>
           <t>SEPLAG / SEPLAN</t>
         </is>
@@ -5536,12 +5790,12 @@
       <c r="D66" s="43" t="inlineStr"/>
     </row>
     <row r="67">
-      <c r="A67" s="59" t="inlineStr">
+      <c r="A67" s="60" t="inlineStr">
         <is>
           <t>Órgãos</t>
         </is>
       </c>
-      <c r="B67" s="54" t="inlineStr">
+      <c r="B67" s="55" t="inlineStr">
         <is>
           <t>Grande Recife Consórcio</t>
         </is>

</xml_diff>

<commit_message>
Subcritérios: lista de 03/10 com o documento da equipe (nomes novos; I3, V5 e V6 sem definição); checklist, painel e docs atualizados
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R5swnHARNHJ12oc84LP2b9
</commit_message>
<xml_diff>
--- a/dados/Recife_Resiliente_Checklist_Subcriterios.xlsx
+++ b/dados/Recife_Resiliente_Checklist_Subcriterios.xlsx
@@ -12,8 +12,8 @@
     <sheet name="Glossário" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Checklist subcritérios'!$A$4:$Q$19</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Glossário'!$A$4:$D$67</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Checklist subcritérios'!$A$4:$Q$22</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Glossário'!$A$4:$D$68</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -756,7 +756,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:Q26"/>
+  <dimension ref="A1:Q29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -788,7 +788,7 @@
     <row r="2" ht="44" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Proposta de 02/10/2026 (Pedro + Claude), não validada pelo grupo. Nota 5 = mais crítico. Faixa fixa = valor absoluto (provisória: calibrar com os dados reais). Quintil = nota relativa entre os 21 pontos (Quintil 1 = 20% com menor valor). Preencha as colunas amarelas (N, O e P): Sim / Não / Parcial / Pendente. 'Fonte confirmada' = a base existe e é acessível; 'Dado existe na fonte' = a variável está lá, na escala do círculo de 300 m, e cobre os 21 pontos. Termos explicados na aba Glossário.</t>
+          <t>Proposta de 02/10/2026 (Pedro + Claude), atualizada em 03/10/2026 com o documento da equipe (Hellis); não validada pelo grupo. I3, V5 e V6 são novas e ainda sem definição nem escala. Nota 5 = mais crítico. Faixa fixa = valor absoluto (provisória: calibrar com os dados reais). Quintil = nota relativa entre os 21 pontos (Quintil 1 = 20% com menor valor). Preencha as colunas amarelas (N, O e P): Sim / Não / Parcial / Pendente. 'Fonte confirmada' = a base existe e é acessível; 'Dado existe na fonte' = a variável está lá, na escala do círculo de 300 m, e cobre os 21 pontos. Termos explicados na aba Glossário.</t>
         </is>
       </c>
     </row>
@@ -892,7 +892,7 @@
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>Frequência de alagamento</t>
+          <t>Frequência e recorrência histórica</t>
         </is>
       </c>
       <c r="D5" s="6" t="inlineStr">
@@ -957,7 +957,7 @@
       </c>
       <c r="P5" s="14" t="inlineStr">
         <is>
-          <t>Pedido ao COP via tutora/CGM. 156 só para conferir. Calibrar faixas com a distribuição real.</t>
+          <t>Pedido ao COP via tutora/CGM. 156 só para conferir. Calibrar faixas com a distribuição real. 'Recorrência histórica' (documento da equipe) fica aqui se for o mesmo que frequência (pendência 16).</t>
         </is>
       </c>
       <c r="Q5" s="6" t="inlineStr">
@@ -1327,7 +1327,7 @@
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>Baixio</t>
+          <t>Relevo (baixio)</t>
         </is>
       </c>
       <c r="D10" s="6" t="inlineStr">
@@ -1377,7 +1377,7 @@
       </c>
       <c r="M10" s="6" t="inlineStr">
         <is>
-          <t>ESIG (curvas de nível, a verificar); topografia da Prefeitura</t>
+          <t>Condepe/Fidem — Acervo Cartográfico (curvas de nível); ESIG (a verificar)</t>
         </is>
       </c>
       <c r="N10" s="13" t="inlineStr">
@@ -1392,12 +1392,12 @@
       </c>
       <c r="P10" s="14" t="inlineStr">
         <is>
-          <t>Medida mais objetiva de acúmulo de água.</t>
+          <t>Medida mais objetiva de acúmulo de água. 'Relevo' do documento da equipe.</t>
         </is>
       </c>
       <c r="Q10" s="6" t="inlineStr">
         <is>
-          <t>Não encontrado modelo de terreno público na busca.</t>
+          <t>Condepe/Fidem localizado na busca: curvas de 1 m na área urbana (não aberto).</t>
         </is>
       </c>
     </row>
@@ -1501,7 +1501,7 @@
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>Equipamentos sensíveis</t>
+          <t>Equipamentos públicos</t>
         </is>
       </c>
       <c r="D12" s="6" t="inlineStr">
@@ -1551,7 +1551,7 @@
       </c>
       <c r="M12" s="6" t="inlineStr">
         <is>
-          <t>IBGE — CNEFE 2022 (ensino e saúde); CNES/DATASUS</t>
+          <t>Portal de dados abertos (escolas municipais, UBS, hospitais, rede de saúde); IBGE — CNEFE 2022 (ensino e saúde); CNES/DATASUS</t>
         </is>
       </c>
       <c r="N12" s="13" t="inlineStr">
@@ -1566,12 +1566,12 @@
       </c>
       <c r="P12" s="14" t="inlineStr">
         <is>
-          <t>Calibrar com as contagens reais. Conferir se creches aparecem como 'ensino'.</t>
+          <t>Inclui 'hospitais/escolas atingidos' do documento da equipe (sem contar duas vezes no Impacto). Perguntar se 'equipamentos públicos' inclui outros (CRAS, abrigos). Calibrar com as contagens reais.</t>
         </is>
       </c>
       <c r="Q12" s="6" t="inlineStr">
         <is>
-          <t>CNEFE confirmado na busca (não baixado).</t>
+          <t>CNEFE confirmado na busca (não baixado). Bases do portal localizadas em 03/10 (não abertas).</t>
         </is>
       </c>
     </row>
@@ -1588,7 +1588,7 @@
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>Atividade econômica</t>
+          <t>Comércio e serviços</t>
         </is>
       </c>
       <c r="D13" s="6" t="inlineStr">
@@ -1638,7 +1638,7 @@
       </c>
       <c r="M13" s="6" t="inlineStr">
         <is>
-          <t>IBGE — CNEFE 2022 (outras finalidades)</t>
+          <t>IBGE — CNEFE 2022 (outras finalidades); IPTU (tipo de empreendimento)</t>
         </is>
       </c>
       <c r="N13" s="13" t="inlineStr">
@@ -1653,7 +1653,7 @@
       </c>
       <c r="P13" s="14" t="inlineStr">
         <is>
-          <t>'Outras finalidades' pode incluir templos e órgãos públicos.</t>
+          <t>'Outras finalidades' pode incluir templos e órgãos públicos. Inclui 'perdas econômicas' do documento da equipe, que não tem fonte própria.</t>
         </is>
       </c>
       <c r="Q13" s="6" t="inlineStr">
@@ -1675,7 +1675,7 @@
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>Grupos sensíveis</t>
+          <t>População vulnerável</t>
         </is>
       </c>
       <c r="D14" s="6" t="inlineStr">
@@ -1758,12 +1758,12 @@
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>Favelas e comunidades urbanas</t>
+          <t>ZEIS, favelas e comunidades</t>
         </is>
       </c>
       <c r="D15" s="6" t="inlineStr">
         <is>
-          <t>% da área do círculo em favelas e comunidades urbanas</t>
+          <t>% da área do círculo em favelas e comunidades urbanas (IBGE 2022) ou em ZEIS 1</t>
         </is>
       </c>
       <c r="E15" s="7" t="inlineStr">
@@ -1808,7 +1808,7 @@
       </c>
       <c r="M15" s="6" t="inlineStr">
         <is>
-          <t>IBGE — Favelas e Comunidades Urbanas 2022 (malha)</t>
+          <t>IBGE — Favelas e Comunidades Urbanas 2022 (malha); ZEIS do Plano Diretor e relação de favelas (portal)</t>
         </is>
       </c>
       <c r="N15" s="13" t="inlineStr">
@@ -1823,12 +1823,12 @@
       </c>
       <c r="P15" s="14" t="inlineStr">
         <is>
-          <t>Mais atual que o IVS (2010).</t>
+          <t>Mais atual que o IVS (2010). ZEIS 2 (terrenos vazios) não conta.</t>
         </is>
       </c>
       <c r="Q15" s="6" t="inlineStr">
         <is>
-          <t>Não verificado.</t>
+          <t>ZEIS e relação de favelas localizadas no portal (não abertas); malha IBGE não verificada.</t>
         </is>
       </c>
     </row>
@@ -1927,353 +1927,530 @@
       </c>
       <c r="B17" s="17" t="inlineStr">
         <is>
+          <t>V5</t>
+        </is>
+      </c>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>Dificuldade de evacuação</t>
+        </is>
+      </c>
+      <c r="D17" s="6" t="inlineStr">
+        <is>
+          <t>Definição pendente (pendência 15)</t>
+        </is>
+      </c>
+      <c r="E17" s="7" t="inlineStr"/>
+      <c r="F17" s="8" t="inlineStr"/>
+      <c r="G17" s="9" t="inlineStr"/>
+      <c r="H17" s="10" t="inlineStr"/>
+      <c r="I17" s="11" t="inlineStr"/>
+      <c r="J17" s="12" t="inlineStr"/>
+      <c r="K17" s="6" t="inlineStr">
+        <is>
+          <t>Documento da equipe (Hellis, 03/10/2026)</t>
+        </is>
+      </c>
+      <c r="L17" s="6" t="inlineStr">
+        <is>
+          <t>Nova — só entra com definição e fonte</t>
+        </is>
+      </c>
+      <c r="M17" s="6" t="inlineStr"/>
+      <c r="N17" s="13" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+      <c r="O17" s="13" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+      <c r="P17" s="14" t="inlineStr">
+        <is>
+          <t>Pedir a definição a Hellis antes de procurar dado.</t>
+        </is>
+      </c>
+      <c r="Q17" s="6" t="inlineStr">
+        <is>
+          <t>Não pesquisado.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="16" t="inlineStr">
+        <is>
+          <t>Vulnerabilidade</t>
+        </is>
+      </c>
+      <c r="B18" s="17" t="inlineStr">
+        <is>
+          <t>V6</t>
+        </is>
+      </c>
+      <c r="C18" s="6" t="inlineStr">
+        <is>
+          <t>Infraestrutura precária</t>
+        </is>
+      </c>
+      <c r="D18" s="6" t="inlineStr">
+        <is>
+          <t>Definição pendente (pendência 15)</t>
+        </is>
+      </c>
+      <c r="E18" s="7" t="inlineStr"/>
+      <c r="F18" s="8" t="inlineStr"/>
+      <c r="G18" s="9" t="inlineStr"/>
+      <c r="H18" s="10" t="inlineStr"/>
+      <c r="I18" s="11" t="inlineStr"/>
+      <c r="J18" s="12" t="inlineStr"/>
+      <c r="K18" s="6" t="inlineStr">
+        <is>
+          <t>Documento da equipe (Hellis, 03/10/2026)</t>
+        </is>
+      </c>
+      <c r="L18" s="6" t="inlineStr">
+        <is>
+          <t>Nova — só entra com definição e fonte</t>
+        </is>
+      </c>
+      <c r="M18" s="6" t="inlineStr"/>
+      <c r="N18" s="13" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+      <c r="O18" s="13" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+      <c r="P18" s="14" t="inlineStr">
+        <is>
+          <t>Pode absorver o V4 (tipo de moradia) e o I2 (esgoto). Pedir a definição a Hellis.</t>
+        </is>
+      </c>
+      <c r="Q18" s="6" t="inlineStr">
+        <is>
+          <t>Não pesquisado.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="16" t="inlineStr">
+        <is>
+          <t>Vulnerabilidade</t>
+        </is>
+      </c>
+      <c r="B19" s="17" t="inlineStr">
+        <is>
           <t>V1</t>
         </is>
       </c>
-      <c r="C17" s="6" t="inlineStr">
+      <c r="C19" s="6" t="inlineStr">
         <is>
           <t>Vulnerabilidade social (IVS)</t>
         </is>
       </c>
-      <c r="D17" s="6" t="inlineStr">
+      <c r="D19" s="6" t="inlineStr">
         <is>
           <t>Maior IVS entre as UDHs que tocam o círculo</t>
         </is>
       </c>
-      <c r="E17" s="7" t="inlineStr">
+      <c r="E19" s="7" t="inlineStr">
         <is>
           <t>Faixa fixa</t>
         </is>
       </c>
-      <c r="F17" s="8" t="inlineStr">
+      <c r="F19" s="8" t="inlineStr">
         <is>
           <t>Muito baixa (0–0,200)</t>
         </is>
       </c>
-      <c r="G17" s="9" t="inlineStr">
+      <c r="G19" s="9" t="inlineStr">
         <is>
           <t>Baixa (0,201–0,300)</t>
         </is>
       </c>
-      <c r="H17" s="10" t="inlineStr">
+      <c r="H19" s="10" t="inlineStr">
         <is>
           <t>Média (0,301–0,400)</t>
         </is>
       </c>
-      <c r="I17" s="11" t="inlineStr">
+      <c r="I19" s="11" t="inlineStr">
         <is>
           <t>Alta (0,401–0,500)</t>
         </is>
       </c>
-      <c r="J17" s="12" t="inlineStr">
+      <c r="J19" s="12" t="inlineStr">
         <is>
           <t>Muito alta (&gt; 0,500)</t>
         </is>
       </c>
-      <c r="K17" s="6" t="inlineStr">
+      <c r="K19" s="6" t="inlineStr">
         <is>
           <t>Faixas do Ipea (conferir no Atlas)</t>
         </is>
       </c>
-      <c r="L17" s="6" t="inlineStr">
+      <c r="L19" s="6" t="inlineStr">
         <is>
           <t>Plano B — só se o V3 não estiver disponível</t>
         </is>
       </c>
-      <c r="M17" s="6" t="inlineStr">
+      <c r="M19" s="6" t="inlineStr">
         <is>
           <t>Ipea — Atlas da Vulnerabilidade Social (UDH)</t>
         </is>
       </c>
-      <c r="N17" s="13" t="inlineStr">
+      <c r="N19" s="13" t="inlineStr">
         <is>
           <t>Pendente</t>
         </is>
       </c>
-      <c r="O17" s="13" t="inlineStr">
+      <c r="O19" s="13" t="inlineStr">
         <is>
           <t>Pendente</t>
         </is>
       </c>
-      <c r="P17" s="14" t="inlineStr">
+      <c r="P19" s="14" t="inlineStr">
         <is>
           <t>Base do Censo 2010.</t>
         </is>
       </c>
-      <c r="Q17" s="6" t="inlineStr">
+      <c r="Q19" s="6" t="inlineStr">
         <is>
           <t>Site confirmado na busca; faixas e ano-base a confirmar.</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="18" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="18" t="inlineStr">
         <is>
           <t>Impacto</t>
         </is>
       </c>
-      <c r="B18" s="19" t="inlineStr">
+      <c r="B20" s="19" t="inlineStr">
         <is>
           <t>I1</t>
         </is>
       </c>
-      <c r="C18" s="6" t="inlineStr">
-        <is>
-          <t>Mobilidade</t>
-        </is>
-      </c>
-      <c r="D18" s="6" t="inlineStr">
+      <c r="C20" s="6" t="inlineStr">
+        <is>
+          <t>Interrupção do trânsito</t>
+        </is>
+      </c>
+      <c r="D20" s="6" t="inlineStr">
         <is>
           <t>Classe da via mais importante afetada pelo alagamento; +1 se houver interdição registrada pela CTTU (máximo 5)</t>
         </is>
       </c>
-      <c r="E18" s="7" t="inlineStr">
+      <c r="E20" s="7" t="inlineStr">
         <is>
           <t>Classe</t>
         </is>
       </c>
-      <c r="F18" s="8" t="inlineStr">
+      <c r="F20" s="8" t="inlineStr">
         <is>
           <t>Via local ou de pedestres</t>
         </is>
       </c>
-      <c r="G18" s="9" t="inlineStr">
+      <c r="G20" s="9" t="inlineStr">
         <is>
           <t>Coletora</t>
         </is>
       </c>
-      <c r="H18" s="10" t="inlineStr">
+      <c r="H20" s="10" t="inlineStr">
         <is>
           <t>Arterial secundária</t>
         </is>
       </c>
-      <c r="I18" s="11" t="inlineStr">
+      <c r="I20" s="11" t="inlineStr">
         <is>
           <t>Arterial principal</t>
         </is>
       </c>
-      <c r="J18" s="12" t="inlineStr">
+      <c r="J20" s="12" t="inlineStr">
         <is>
           <t>Trânsito rápido ou corredor de ônibus</t>
         </is>
       </c>
-      <c r="K18" s="6" t="inlineStr">
+      <c r="K20" s="6" t="inlineStr">
         <is>
           <t>Proposta Claude, a partir da classificação viária usada na planilha original</t>
         </is>
       </c>
-      <c r="L18" s="6" t="inlineStr">
+      <c r="L20" s="6" t="inlineStr">
         <is>
           <t>Manter</t>
         </is>
       </c>
-      <c r="M18" s="6" t="inlineStr">
-        <is>
-          <t>Hierarquia viária (ESIG / CTTU); OSM; paradas (Grande Recife); interdições (CTTU)</t>
-        </is>
-      </c>
-      <c r="N18" s="13" t="inlineStr">
+      <c r="M20" s="6" t="inlineStr">
+        <is>
+          <t>Hierarquia viária (ESIG / CTTU); OSM; corredores de ônibus e fluxo de veículos (portal); paradas (Grande Recife); interdições (CTTU)</t>
+        </is>
+      </c>
+      <c r="N20" s="13" t="inlineStr">
         <is>
           <t>Pendente</t>
         </is>
       </c>
-      <c r="O18" s="13" t="inlineStr">
+      <c r="O20" s="13" t="inlineStr">
         <is>
           <t>Pendente</t>
         </is>
       </c>
-      <c r="P18" s="14" t="inlineStr">
-        <is>
-          <t>Pedir a Antônio (CTTU): hierarquia viária, linhas e registro de interdições.</t>
-        </is>
-      </c>
-      <c r="Q18" s="6" t="inlineStr">
+      <c r="P20" s="14" t="inlineStr">
+        <is>
+          <t>Junta 'vias principais' e 'interrupção do trânsito' do documento da equipe. Pedir a Antônio (CTTU): hierarquia viária, linhas e registro de interdições.</t>
+        </is>
+      </c>
+      <c r="Q20" s="6" t="inlineStr">
         <is>
           <t>Vias no ESIG confirmadas na busca; ônibus e interdições não verificados.</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="18" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="18" t="inlineStr">
         <is>
           <t>Impacto</t>
         </is>
       </c>
-      <c r="B19" s="19" t="inlineStr">
+      <c r="B21" s="19" t="inlineStr">
         <is>
           <t>I2</t>
         </is>
       </c>
-      <c r="C19" s="6" t="inlineStr">
+      <c r="C21" s="6" t="inlineStr">
         <is>
           <t>Risco sanitário</t>
         </is>
       </c>
-      <c r="D19" s="6" t="inlineStr">
+      <c r="D21" s="6" t="inlineStr">
         <is>
           <t>% de domicílios sem ligação à rede de esgoto nos setores do círculo</t>
         </is>
       </c>
-      <c r="E19" s="7" t="inlineStr">
+      <c r="E21" s="7" t="inlineStr">
         <is>
           <t>Quintil</t>
         </is>
       </c>
-      <c r="F19" s="8" t="inlineStr">
+      <c r="F21" s="8" t="inlineStr">
         <is>
           <t>Quintil 1 (20% menores)</t>
         </is>
       </c>
-      <c r="G19" s="9" t="inlineStr">
+      <c r="G21" s="9" t="inlineStr">
         <is>
           <t>Quintil 2</t>
         </is>
       </c>
-      <c r="H19" s="10" t="inlineStr">
+      <c r="H21" s="10" t="inlineStr">
         <is>
           <t>Quintil 3</t>
         </is>
       </c>
-      <c r="I19" s="11" t="inlineStr">
+      <c r="I21" s="11" t="inlineStr">
         <is>
           <t>Quintil 4</t>
         </is>
       </c>
-      <c r="J19" s="12" t="inlineStr">
+      <c r="J21" s="12" t="inlineStr">
         <is>
           <t>Quintil 5 (20% maiores)</t>
         </is>
       </c>
-      <c r="K19" s="6" t="inlineStr">
+      <c r="K21" s="6" t="inlineStr">
         <is>
           <t>Proposta Claude (quintis)</t>
         </is>
       </c>
-      <c r="L19" s="6" t="inlineStr">
+      <c r="L21" s="6" t="inlineStr">
         <is>
           <t>Manter</t>
         </is>
       </c>
-      <c r="M19" s="6" t="inlineStr">
+      <c r="M21" s="6" t="inlineStr">
         <is>
           <t>IBGE — Agregados por setor 2022 (esgotamento); Compesa</t>
         </is>
       </c>
-      <c r="N19" s="13" t="inlineStr">
+      <c r="N21" s="13" t="inlineStr">
         <is>
           <t>Pendente</t>
         </is>
       </c>
-      <c r="O19" s="13" t="inlineStr">
+      <c r="O21" s="13" t="inlineStr">
         <is>
           <t>Pendente</t>
         </is>
       </c>
-      <c r="P19" s="14" t="inlineStr">
-        <is>
-          <t>Quintis porque a cobertura de esgoto no Recife é baixa e faixas fixas podem saturar.</t>
-        </is>
-      </c>
-      <c r="Q19" s="6" t="inlineStr">
+      <c r="P21" s="14" t="inlineStr">
+        <is>
+          <t>Quintis porque a cobertura de esgoto no Recife é baixa e faixas fixas podem saturar. Pode passar para o V6 (infraestrutura precária).</t>
+        </is>
+      </c>
+      <c r="Q21" s="6" t="inlineStr">
         <is>
           <t>Esgotamento por setor confirmado na busca (não baixado).</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="20" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="18" t="inlineStr">
+        <is>
+          <t>Impacto</t>
+        </is>
+      </c>
+      <c r="B22" s="19" t="inlineStr">
+        <is>
+          <t>I3</t>
+        </is>
+      </c>
+      <c r="C22" s="6" t="inlineStr">
+        <is>
+          <t>Isolamento</t>
+        </is>
+      </c>
+      <c r="D22" s="6" t="inlineStr">
+        <is>
+          <t>Definição pendente (pendência 15)</t>
+        </is>
+      </c>
+      <c r="E22" s="7" t="inlineStr"/>
+      <c r="F22" s="8" t="inlineStr"/>
+      <c r="G22" s="9" t="inlineStr"/>
+      <c r="H22" s="10" t="inlineStr"/>
+      <c r="I22" s="11" t="inlineStr"/>
+      <c r="J22" s="12" t="inlineStr"/>
+      <c r="K22" s="6" t="inlineStr">
+        <is>
+          <t>Documento da equipe (Hellis, 03/10/2026)</t>
+        </is>
+      </c>
+      <c r="L22" s="6" t="inlineStr">
+        <is>
+          <t>Nova — só entra com definição e fonte</t>
+        </is>
+      </c>
+      <c r="M22" s="6" t="inlineStr"/>
+      <c r="N22" s="13" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+      <c r="O22" s="13" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+      <c r="P22" s="14" t="inlineStr">
+        <is>
+          <t>Leitura possível: comunidade sem rota alternativa quando o ponto alaga (malha viária). Confirmar com Hellis.</t>
+        </is>
+      </c>
+      <c r="Q22" s="6" t="inlineStr">
+        <is>
+          <t>Não pesquisado.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="20" t="inlineStr">
         <is>
           <t>Resumo</t>
         </is>
       </c>
-      <c r="N21" s="21" t="inlineStr">
+      <c r="N24" s="21" t="inlineStr">
         <is>
           <t>Fonte confirmada</t>
         </is>
       </c>
-      <c r="O21" s="21" t="inlineStr">
+      <c r="O24" s="21" t="inlineStr">
         <is>
           <t>Dado existe</t>
         </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="M22" s="22" t="inlineStr">
-        <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="N22" s="23">
-        <f>COUNTIF(N$5:N$19,$M22)</f>
-        <v/>
-      </c>
-      <c r="O22" s="23">
-        <f>COUNTIF(O$5:O$19,$M22)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="23">
-      <c r="M23" s="22" t="inlineStr">
-        <is>
-          <t>Parcial</t>
-        </is>
-      </c>
-      <c r="N23" s="23">
-        <f>COUNTIF(N$5:N$19,$M23)</f>
-        <v/>
-      </c>
-      <c r="O23" s="23">
-        <f>COUNTIF(O$5:O$19,$M23)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="24">
-      <c r="M24" s="22" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="N24" s="23">
-        <f>COUNTIF(N$5:N$19,$M24)</f>
-        <v/>
-      </c>
-      <c r="O24" s="23">
-        <f>COUNTIF(O$5:O$19,$M24)</f>
-        <v/>
       </c>
     </row>
     <row r="25">
       <c r="M25" s="22" t="inlineStr">
         <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="N25" s="23">
+        <f>COUNTIF(N$5:N$22,$M25)</f>
+        <v/>
+      </c>
+      <c r="O25" s="23">
+        <f>COUNTIF(O$5:O$22,$M25)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="M26" s="22" t="inlineStr">
+        <is>
+          <t>Parcial</t>
+        </is>
+      </c>
+      <c r="N26" s="23">
+        <f>COUNTIF(N$5:N$22,$M26)</f>
+        <v/>
+      </c>
+      <c r="O26" s="23">
+        <f>COUNTIF(O$5:O$22,$M26)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="M27" s="22" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="N27" s="23">
+        <f>COUNTIF(N$5:N$22,$M27)</f>
+        <v/>
+      </c>
+      <c r="O27" s="23">
+        <f>COUNTIF(O$5:O$22,$M27)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="M28" s="22" t="inlineStr">
+        <is>
           <t>Pendente</t>
         </is>
       </c>
-      <c r="N25" s="23">
-        <f>COUNTIF(N$5:N$19,$M25)</f>
-        <v/>
-      </c>
-      <c r="O25" s="23">
-        <f>COUNTIF(O$5:O$19,$M25)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="26">
-      <c r="M26" s="24" t="inlineStr">
+      <c r="N28" s="23">
+        <f>COUNTIF(N$5:N$22,$M28)</f>
+        <v/>
+      </c>
+      <c r="O28" s="23">
+        <f>COUNTIF(O$5:O$22,$M28)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="M29" s="24" t="inlineStr">
         <is>
           <t>Subcritérios com fonte e dado confirmados</t>
         </is>
       </c>
-      <c r="O26" s="25">
-        <f>COUNTIFS(N5:N19,"Sim",O5:O19,"Sim")&amp;" de "&amp;ROWS(N5:N19)</f>
+      <c r="O29" s="25">
+        <f>COUNTIFS(N5:N22,"Sim",O5:O22,"Sim")&amp;" de "&amp;ROWS(N5:N22)</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:Q19"/>
+  <autoFilter ref="A4:Q22"/>
   <mergeCells count="1">
     <mergeCell ref="A2:Q2"/>
   </mergeCells>
-  <conditionalFormatting sqref="N5:O19">
+  <conditionalFormatting sqref="N5:O22">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Sim"</formula>
     </cfRule>
@@ -2285,7 +2462,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="N5:O19" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="N5:O22" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Sim,Não,Parcial,Pendente"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2300,7 +2477,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AF34"/>
+  <dimension ref="A1:AI34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -2326,15 +2503,18 @@
     <col width="11" customWidth="1" min="21" max="21"/>
     <col width="11" customWidth="1" min="22" max="22"/>
     <col width="11" customWidth="1" min="23" max="23"/>
-    <col width="13" customWidth="1" min="24" max="24"/>
+    <col width="11" customWidth="1" min="24" max="24"/>
     <col width="11" customWidth="1" min="25" max="25"/>
-    <col width="11" customWidth="1" min="26" max="26"/>
-    <col width="13" customWidth="1" min="27" max="27"/>
-    <col width="13" customWidth="1" min="28" max="28"/>
-    <col width="13" customWidth="1" min="29" max="29"/>
+    <col width="13" customWidth="1" min="26" max="26"/>
+    <col width="11" customWidth="1" min="27" max="27"/>
+    <col width="11" customWidth="1" min="28" max="28"/>
+    <col width="11" customWidth="1" min="29" max="29"/>
     <col width="13" customWidth="1" min="30" max="30"/>
     <col width="13" customWidth="1" min="31" max="31"/>
     <col width="13" customWidth="1" min="32" max="32"/>
+    <col width="13" customWidth="1" min="33" max="33"/>
+    <col width="13" customWidth="1" min="34" max="34"/>
+    <col width="13" customWidth="1" min="35" max="35"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2347,7 +2527,7 @@
     <row r="2" ht="40" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Preencha as notas (1 a 5, 5 = mais crítico) nas células amarelas, conforme as escalas da aba 'Checklist subcritérios'. Linha 'Peso': vazia = todos os pesos iguais. Nota em branco fica fora da média (não vira zero). Sem nota de Probabilidade não há risco. P6 e V1 são condicionais: deixe em branco se não forem usados. Colunas cinza são calculadas: não edite. 'Grupo de sobreposição' (G1–G5) = pontos cujos círculos de 300 m se sobrepõem; vazio = ponto isolado. Coordenadas em graus decimais (WGS 84), ainda NÃO verificadas: 'Aproximado' e 'Interseção' foram localizadas automaticamente pelo OpenStreetMap.</t>
+          <t>Preencha as notas (1 a 5, 5 = mais crítico) nas células amarelas, conforme as escalas da aba 'Checklist subcritérios'. Linha 'Peso': vazia = todos os pesos iguais. Nota em branco fica fora da média (não vira zero). Sem nota de Probabilidade não há risco. P6 e V1 são condicionais e I3, V5 e V6 ainda não têm definição: deixe em branco se não forem usados. Colunas cinza são calculadas: não edite. 'Grupo de sobreposição' (G1–G5) = pontos cujos círculos de 300 m se sobrepõem; vazio = ponto isolado. Coordenadas em graus decimais (WGS 84), ainda NÃO verificadas: 'Aproximado' e 'Interseção' foram localizadas automaticamente pelo OpenStreetMap.</t>
         </is>
       </c>
     </row>
@@ -2367,12 +2547,12 @@
           <t>Vulnerabilidade</t>
         </is>
       </c>
-      <c r="Y4" s="29" t="inlineStr">
+      <c r="AA4" s="29" t="inlineStr">
         <is>
           <t>Impacto</t>
         </is>
       </c>
-      <c r="AB4" s="30" t="inlineStr">
+      <c r="AE4" s="30" t="inlineStr">
         <is>
           <t>Resultado</t>
         </is>
@@ -2403,10 +2583,13 @@
       <c r="U5" s="32" t="n"/>
       <c r="V5" s="32" t="n"/>
       <c r="W5" s="32" t="n"/>
-      <c r="X5" s="34" t="n"/>
+      <c r="X5" s="32" t="n"/>
       <c r="Y5" s="32" t="n"/>
-      <c r="Z5" s="32" t="n"/>
-      <c r="AA5" s="34" t="n"/>
+      <c r="Z5" s="34" t="n"/>
+      <c r="AA5" s="32" t="n"/>
+      <c r="AB5" s="32" t="n"/>
+      <c r="AC5" s="32" t="n"/>
+      <c r="AD5" s="34" t="n"/>
     </row>
     <row r="6" ht="54" customHeight="1">
       <c r="A6" s="35" t="inlineStr">
@@ -2454,7 +2637,7 @@
       <c r="I6" s="36" t="inlineStr">
         <is>
           <t>P1
-Frequência de alagamento</t>
+Frequência e recorrência histórica</t>
         </is>
       </c>
       <c r="J6" s="36" t="inlineStr">
@@ -2484,7 +2667,7 @@
       <c r="N6" s="36" t="inlineStr">
         <is>
           <t>P6
-Baixio</t>
+Relevo (baixio)</t>
         </is>
       </c>
       <c r="O6" s="37" t="inlineStr">
@@ -2502,13 +2685,13 @@
       <c r="Q6" s="38" t="inlineStr">
         <is>
           <t>E2
-Equipamentos sensíveis</t>
+Equipamentos públicos</t>
         </is>
       </c>
       <c r="R6" s="38" t="inlineStr">
         <is>
           <t>E3
-Atividade econômica</t>
+Comércio e serviços</t>
         </is>
       </c>
       <c r="S6" s="37" t="inlineStr">
@@ -2520,13 +2703,13 @@
       <c r="T6" s="39" t="inlineStr">
         <is>
           <t>V2
-Grupos sensíveis</t>
+População vulnerável</t>
         </is>
       </c>
       <c r="U6" s="39" t="inlineStr">
         <is>
           <t>V3
-Favelas e comunidades urbanas</t>
+ZEIS, favelas e comunidades</t>
         </is>
       </c>
       <c r="V6" s="39" t="inlineStr">
@@ -2537,58 +2720,76 @@
       </c>
       <c r="W6" s="39" t="inlineStr">
         <is>
+          <t>V5
+Dificuldade de evacuação</t>
+        </is>
+      </c>
+      <c r="X6" s="39" t="inlineStr">
+        <is>
+          <t>V6
+Infraestrutura precária</t>
+        </is>
+      </c>
+      <c r="Y6" s="39" t="inlineStr">
+        <is>
           <t>V1
 Vulnerabilidade social (IVS)</t>
         </is>
       </c>
-      <c r="X6" s="37" t="inlineStr">
+      <c r="Z6" s="37" t="inlineStr">
         <is>
           <t>Nota
 Vulnerabilidade</t>
         </is>
       </c>
-      <c r="Y6" s="40" t="inlineStr">
+      <c r="AA6" s="40" t="inlineStr">
         <is>
           <t>I1
-Mobilidade</t>
-        </is>
-      </c>
-      <c r="Z6" s="40" t="inlineStr">
+Interrupção do trânsito</t>
+        </is>
+      </c>
+      <c r="AB6" s="40" t="inlineStr">
         <is>
           <t>I2
 Risco sanitário</t>
         </is>
       </c>
-      <c r="AA6" s="37" t="inlineStr">
+      <c r="AC6" s="40" t="inlineStr">
+        <is>
+          <t>I3
+Isolamento</t>
+        </is>
+      </c>
+      <c r="AD6" s="37" t="inlineStr">
         <is>
           <t>Nota
 Impacto</t>
         </is>
       </c>
-      <c r="AB6" s="41" t="inlineStr">
+      <c r="AE6" s="41" t="inlineStr">
         <is>
           <t>Consequência
 (1–5)</t>
         </is>
       </c>
-      <c r="AC6" s="41" t="inlineStr">
+      <c r="AF6" s="41" t="inlineStr">
         <is>
           <t>Risco
 P × C (1–25)</t>
         </is>
       </c>
-      <c r="AD6" s="41" t="inlineStr">
+      <c r="AG6" s="41" t="inlineStr">
         <is>
           <t>Índice de risco
 (0–1)</t>
         </is>
       </c>
-      <c r="AE6" s="41" t="inlineStr">
+      <c r="AH6" s="41" t="inlineStr">
         <is>
           <t>Posição</t>
         </is>
       </c>
-      <c r="AF6" s="41" t="inlineStr">
+      <c r="AI6" s="41" t="inlineStr">
         <is>
           <t>Notas
 preenchidas</t>
@@ -2651,34 +2852,37 @@
       <c r="U7" s="45" t="n"/>
       <c r="V7" s="45" t="n"/>
       <c r="W7" s="45" t="n"/>
-      <c r="X7" s="46">
-        <f>IF(COUNT(T7:W7)=0,"",IFERROR(SUMPRODUCT(T7:W7,(T$5:W$5+(T$5:W$5="")))/SUMPRODUCT((T7:W7&lt;&gt;"")*(T$5:W$5+(T$5:W$5=""))),""))</f>
-        <v/>
-      </c>
+      <c r="X7" s="45" t="n"/>
       <c r="Y7" s="45" t="n"/>
-      <c r="Z7" s="45" t="n"/>
-      <c r="AA7" s="46">
-        <f>IF(COUNT(Y7:Z7)=0,"",IFERROR(SUMPRODUCT(Y7:Z7,(Y$5:Z$5+(Y$5:Z$5="")))/SUMPRODUCT((Y7:Z7&lt;&gt;"")*(Y$5:Z$5+(Y$5:Z$5=""))),""))</f>
-        <v/>
-      </c>
-      <c r="AB7" s="46">
-        <f>IFERROR(IF((ISNUMBER(S7)*(S$5+(S$5=""))+ISNUMBER(X7)*(X$5+(X$5=""))+ISNUMBER(AA7)*(AA$5+(AA$5="")))=0,"",(N(S7)*(S$5+(S$5=""))+N(X7)*(X$5+(X$5=""))+N(AA7)*(AA$5+(AA$5="")))/(ISNUMBER(S7)*(S$5+(S$5=""))+ISNUMBER(X7)*(X$5+(X$5=""))+ISNUMBER(AA7)*(AA$5+(AA$5="")))),"")</f>
-        <v/>
-      </c>
-      <c r="AC7" s="47">
-        <f>IF(AND(ISNUMBER(O7),ISNUMBER(AB7)),O7*AB7,"")</f>
-        <v/>
-      </c>
-      <c r="AD7" s="48">
-        <f>IF(ISNUMBER(AC7),(AC7-1)/24,"")</f>
-        <v/>
-      </c>
-      <c r="AE7" s="49">
-        <f>IF(ISNUMBER(AC7),COUNTIF(AC$7:AC$27,"&gt;"&amp;AC7)+1,"")</f>
-        <v/>
-      </c>
-      <c r="AF7" s="50">
-        <f>COUNT(I7,J7,K7,L7,M7,N7,P7,Q7,R7,T7,U7,V7,W7,Y7,Z7)</f>
+      <c r="Z7" s="46">
+        <f>IF(COUNT(T7:Y7)=0,"",IFERROR(SUMPRODUCT(T7:Y7,(T$5:Y$5+(T$5:Y$5="")))/SUMPRODUCT((T7:Y7&lt;&gt;"")*(T$5:Y$5+(T$5:Y$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="AA7" s="45" t="n"/>
+      <c r="AB7" s="45" t="n"/>
+      <c r="AC7" s="45" t="n"/>
+      <c r="AD7" s="46">
+        <f>IF(COUNT(AA7:AC7)=0,"",IFERROR(SUMPRODUCT(AA7:AC7,(AA$5:AC$5+(AA$5:AC$5="")))/SUMPRODUCT((AA7:AC7&lt;&gt;"")*(AA$5:AC$5+(AA$5:AC$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="AE7" s="46">
+        <f>IFERROR(IF((ISNUMBER(S7)*(S$5+(S$5=""))+ISNUMBER(Z7)*(Z$5+(Z$5=""))+ISNUMBER(AD7)*(AD$5+(AD$5="")))=0,"",(N(S7)*(S$5+(S$5=""))+N(Z7)*(Z$5+(Z$5=""))+N(AD7)*(AD$5+(AD$5="")))/(ISNUMBER(S7)*(S$5+(S$5=""))+ISNUMBER(Z7)*(Z$5+(Z$5=""))+ISNUMBER(AD7)*(AD$5+(AD$5="")))),"")</f>
+        <v/>
+      </c>
+      <c r="AF7" s="47">
+        <f>IF(AND(ISNUMBER(O7),ISNUMBER(AE7)),O7*AE7,"")</f>
+        <v/>
+      </c>
+      <c r="AG7" s="48">
+        <f>IF(ISNUMBER(AF7),(AF7-1)/24,"")</f>
+        <v/>
+      </c>
+      <c r="AH7" s="49">
+        <f>IF(ISNUMBER(AF7),COUNTIF(AF$7:AF$27,"&gt;"&amp;AF7)+1,"")</f>
+        <v/>
+      </c>
+      <c r="AI7" s="50">
+        <f>COUNT(I7,J7,K7,L7,M7,N7,P7,Q7,R7,T7,U7,V7,W7,X7,Y7,AA7,AB7,AC7)</f>
         <v/>
       </c>
     </row>
@@ -2738,34 +2942,37 @@
       <c r="U8" s="45" t="n"/>
       <c r="V8" s="45" t="n"/>
       <c r="W8" s="45" t="n"/>
-      <c r="X8" s="46">
-        <f>IF(COUNT(T8:W8)=0,"",IFERROR(SUMPRODUCT(T8:W8,(T$5:W$5+(T$5:W$5="")))/SUMPRODUCT((T8:W8&lt;&gt;"")*(T$5:W$5+(T$5:W$5=""))),""))</f>
-        <v/>
-      </c>
+      <c r="X8" s="45" t="n"/>
       <c r="Y8" s="45" t="n"/>
-      <c r="Z8" s="45" t="n"/>
-      <c r="AA8" s="46">
-        <f>IF(COUNT(Y8:Z8)=0,"",IFERROR(SUMPRODUCT(Y8:Z8,(Y$5:Z$5+(Y$5:Z$5="")))/SUMPRODUCT((Y8:Z8&lt;&gt;"")*(Y$5:Z$5+(Y$5:Z$5=""))),""))</f>
-        <v/>
-      </c>
-      <c r="AB8" s="46">
-        <f>IFERROR(IF((ISNUMBER(S8)*(S$5+(S$5=""))+ISNUMBER(X8)*(X$5+(X$5=""))+ISNUMBER(AA8)*(AA$5+(AA$5="")))=0,"",(N(S8)*(S$5+(S$5=""))+N(X8)*(X$5+(X$5=""))+N(AA8)*(AA$5+(AA$5="")))/(ISNUMBER(S8)*(S$5+(S$5=""))+ISNUMBER(X8)*(X$5+(X$5=""))+ISNUMBER(AA8)*(AA$5+(AA$5="")))),"")</f>
-        <v/>
-      </c>
-      <c r="AC8" s="47">
-        <f>IF(AND(ISNUMBER(O8),ISNUMBER(AB8)),O8*AB8,"")</f>
-        <v/>
-      </c>
-      <c r="AD8" s="48">
-        <f>IF(ISNUMBER(AC8),(AC8-1)/24,"")</f>
-        <v/>
-      </c>
-      <c r="AE8" s="49">
-        <f>IF(ISNUMBER(AC8),COUNTIF(AC$7:AC$27,"&gt;"&amp;AC8)+1,"")</f>
-        <v/>
-      </c>
-      <c r="AF8" s="50">
-        <f>COUNT(I8,J8,K8,L8,M8,N8,P8,Q8,R8,T8,U8,V8,W8,Y8,Z8)</f>
+      <c r="Z8" s="46">
+        <f>IF(COUNT(T8:Y8)=0,"",IFERROR(SUMPRODUCT(T8:Y8,(T$5:Y$5+(T$5:Y$5="")))/SUMPRODUCT((T8:Y8&lt;&gt;"")*(T$5:Y$5+(T$5:Y$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="AA8" s="45" t="n"/>
+      <c r="AB8" s="45" t="n"/>
+      <c r="AC8" s="45" t="n"/>
+      <c r="AD8" s="46">
+        <f>IF(COUNT(AA8:AC8)=0,"",IFERROR(SUMPRODUCT(AA8:AC8,(AA$5:AC$5+(AA$5:AC$5="")))/SUMPRODUCT((AA8:AC8&lt;&gt;"")*(AA$5:AC$5+(AA$5:AC$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="AE8" s="46">
+        <f>IFERROR(IF((ISNUMBER(S8)*(S$5+(S$5=""))+ISNUMBER(Z8)*(Z$5+(Z$5=""))+ISNUMBER(AD8)*(AD$5+(AD$5="")))=0,"",(N(S8)*(S$5+(S$5=""))+N(Z8)*(Z$5+(Z$5=""))+N(AD8)*(AD$5+(AD$5="")))/(ISNUMBER(S8)*(S$5+(S$5=""))+ISNUMBER(Z8)*(Z$5+(Z$5=""))+ISNUMBER(AD8)*(AD$5+(AD$5="")))),"")</f>
+        <v/>
+      </c>
+      <c r="AF8" s="47">
+        <f>IF(AND(ISNUMBER(O8),ISNUMBER(AE8)),O8*AE8,"")</f>
+        <v/>
+      </c>
+      <c r="AG8" s="48">
+        <f>IF(ISNUMBER(AF8),(AF8-1)/24,"")</f>
+        <v/>
+      </c>
+      <c r="AH8" s="49">
+        <f>IF(ISNUMBER(AF8),COUNTIF(AF$7:AF$27,"&gt;"&amp;AF8)+1,"")</f>
+        <v/>
+      </c>
+      <c r="AI8" s="50">
+        <f>COUNT(I8,J8,K8,L8,M8,N8,P8,Q8,R8,T8,U8,V8,W8,X8,Y8,AA8,AB8,AC8)</f>
         <v/>
       </c>
     </row>
@@ -2825,34 +3032,37 @@
       <c r="U9" s="45" t="n"/>
       <c r="V9" s="45" t="n"/>
       <c r="W9" s="45" t="n"/>
-      <c r="X9" s="46">
-        <f>IF(COUNT(T9:W9)=0,"",IFERROR(SUMPRODUCT(T9:W9,(T$5:W$5+(T$5:W$5="")))/SUMPRODUCT((T9:W9&lt;&gt;"")*(T$5:W$5+(T$5:W$5=""))),""))</f>
-        <v/>
-      </c>
+      <c r="X9" s="45" t="n"/>
       <c r="Y9" s="45" t="n"/>
-      <c r="Z9" s="45" t="n"/>
-      <c r="AA9" s="46">
-        <f>IF(COUNT(Y9:Z9)=0,"",IFERROR(SUMPRODUCT(Y9:Z9,(Y$5:Z$5+(Y$5:Z$5="")))/SUMPRODUCT((Y9:Z9&lt;&gt;"")*(Y$5:Z$5+(Y$5:Z$5=""))),""))</f>
-        <v/>
-      </c>
-      <c r="AB9" s="46">
-        <f>IFERROR(IF((ISNUMBER(S9)*(S$5+(S$5=""))+ISNUMBER(X9)*(X$5+(X$5=""))+ISNUMBER(AA9)*(AA$5+(AA$5="")))=0,"",(N(S9)*(S$5+(S$5=""))+N(X9)*(X$5+(X$5=""))+N(AA9)*(AA$5+(AA$5="")))/(ISNUMBER(S9)*(S$5+(S$5=""))+ISNUMBER(X9)*(X$5+(X$5=""))+ISNUMBER(AA9)*(AA$5+(AA$5="")))),"")</f>
-        <v/>
-      </c>
-      <c r="AC9" s="47">
-        <f>IF(AND(ISNUMBER(O9),ISNUMBER(AB9)),O9*AB9,"")</f>
-        <v/>
-      </c>
-      <c r="AD9" s="48">
-        <f>IF(ISNUMBER(AC9),(AC9-1)/24,"")</f>
-        <v/>
-      </c>
-      <c r="AE9" s="49">
-        <f>IF(ISNUMBER(AC9),COUNTIF(AC$7:AC$27,"&gt;"&amp;AC9)+1,"")</f>
-        <v/>
-      </c>
-      <c r="AF9" s="50">
-        <f>COUNT(I9,J9,K9,L9,M9,N9,P9,Q9,R9,T9,U9,V9,W9,Y9,Z9)</f>
+      <c r="Z9" s="46">
+        <f>IF(COUNT(T9:Y9)=0,"",IFERROR(SUMPRODUCT(T9:Y9,(T$5:Y$5+(T$5:Y$5="")))/SUMPRODUCT((T9:Y9&lt;&gt;"")*(T$5:Y$5+(T$5:Y$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="AA9" s="45" t="n"/>
+      <c r="AB9" s="45" t="n"/>
+      <c r="AC9" s="45" t="n"/>
+      <c r="AD9" s="46">
+        <f>IF(COUNT(AA9:AC9)=0,"",IFERROR(SUMPRODUCT(AA9:AC9,(AA$5:AC$5+(AA$5:AC$5="")))/SUMPRODUCT((AA9:AC9&lt;&gt;"")*(AA$5:AC$5+(AA$5:AC$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="AE9" s="46">
+        <f>IFERROR(IF((ISNUMBER(S9)*(S$5+(S$5=""))+ISNUMBER(Z9)*(Z$5+(Z$5=""))+ISNUMBER(AD9)*(AD$5+(AD$5="")))=0,"",(N(S9)*(S$5+(S$5=""))+N(Z9)*(Z$5+(Z$5=""))+N(AD9)*(AD$5+(AD$5="")))/(ISNUMBER(S9)*(S$5+(S$5=""))+ISNUMBER(Z9)*(Z$5+(Z$5=""))+ISNUMBER(AD9)*(AD$5+(AD$5="")))),"")</f>
+        <v/>
+      </c>
+      <c r="AF9" s="47">
+        <f>IF(AND(ISNUMBER(O9),ISNUMBER(AE9)),O9*AE9,"")</f>
+        <v/>
+      </c>
+      <c r="AG9" s="48">
+        <f>IF(ISNUMBER(AF9),(AF9-1)/24,"")</f>
+        <v/>
+      </c>
+      <c r="AH9" s="49">
+        <f>IF(ISNUMBER(AF9),COUNTIF(AF$7:AF$27,"&gt;"&amp;AF9)+1,"")</f>
+        <v/>
+      </c>
+      <c r="AI9" s="50">
+        <f>COUNT(I9,J9,K9,L9,M9,N9,P9,Q9,R9,T9,U9,V9,W9,X9,Y9,AA9,AB9,AC9)</f>
         <v/>
       </c>
     </row>
@@ -2912,34 +3122,37 @@
       <c r="U10" s="45" t="n"/>
       <c r="V10" s="45" t="n"/>
       <c r="W10" s="45" t="n"/>
-      <c r="X10" s="46">
-        <f>IF(COUNT(T10:W10)=0,"",IFERROR(SUMPRODUCT(T10:W10,(T$5:W$5+(T$5:W$5="")))/SUMPRODUCT((T10:W10&lt;&gt;"")*(T$5:W$5+(T$5:W$5=""))),""))</f>
-        <v/>
-      </c>
+      <c r="X10" s="45" t="n"/>
       <c r="Y10" s="45" t="n"/>
-      <c r="Z10" s="45" t="n"/>
-      <c r="AA10" s="46">
-        <f>IF(COUNT(Y10:Z10)=0,"",IFERROR(SUMPRODUCT(Y10:Z10,(Y$5:Z$5+(Y$5:Z$5="")))/SUMPRODUCT((Y10:Z10&lt;&gt;"")*(Y$5:Z$5+(Y$5:Z$5=""))),""))</f>
-        <v/>
-      </c>
-      <c r="AB10" s="46">
-        <f>IFERROR(IF((ISNUMBER(S10)*(S$5+(S$5=""))+ISNUMBER(X10)*(X$5+(X$5=""))+ISNUMBER(AA10)*(AA$5+(AA$5="")))=0,"",(N(S10)*(S$5+(S$5=""))+N(X10)*(X$5+(X$5=""))+N(AA10)*(AA$5+(AA$5="")))/(ISNUMBER(S10)*(S$5+(S$5=""))+ISNUMBER(X10)*(X$5+(X$5=""))+ISNUMBER(AA10)*(AA$5+(AA$5="")))),"")</f>
-        <v/>
-      </c>
-      <c r="AC10" s="47">
-        <f>IF(AND(ISNUMBER(O10),ISNUMBER(AB10)),O10*AB10,"")</f>
-        <v/>
-      </c>
-      <c r="AD10" s="48">
-        <f>IF(ISNUMBER(AC10),(AC10-1)/24,"")</f>
-        <v/>
-      </c>
-      <c r="AE10" s="49">
-        <f>IF(ISNUMBER(AC10),COUNTIF(AC$7:AC$27,"&gt;"&amp;AC10)+1,"")</f>
-        <v/>
-      </c>
-      <c r="AF10" s="50">
-        <f>COUNT(I10,J10,K10,L10,M10,N10,P10,Q10,R10,T10,U10,V10,W10,Y10,Z10)</f>
+      <c r="Z10" s="46">
+        <f>IF(COUNT(T10:Y10)=0,"",IFERROR(SUMPRODUCT(T10:Y10,(T$5:Y$5+(T$5:Y$5="")))/SUMPRODUCT((T10:Y10&lt;&gt;"")*(T$5:Y$5+(T$5:Y$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="AA10" s="45" t="n"/>
+      <c r="AB10" s="45" t="n"/>
+      <c r="AC10" s="45" t="n"/>
+      <c r="AD10" s="46">
+        <f>IF(COUNT(AA10:AC10)=0,"",IFERROR(SUMPRODUCT(AA10:AC10,(AA$5:AC$5+(AA$5:AC$5="")))/SUMPRODUCT((AA10:AC10&lt;&gt;"")*(AA$5:AC$5+(AA$5:AC$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="AE10" s="46">
+        <f>IFERROR(IF((ISNUMBER(S10)*(S$5+(S$5=""))+ISNUMBER(Z10)*(Z$5+(Z$5=""))+ISNUMBER(AD10)*(AD$5+(AD$5="")))=0,"",(N(S10)*(S$5+(S$5=""))+N(Z10)*(Z$5+(Z$5=""))+N(AD10)*(AD$5+(AD$5="")))/(ISNUMBER(S10)*(S$5+(S$5=""))+ISNUMBER(Z10)*(Z$5+(Z$5=""))+ISNUMBER(AD10)*(AD$5+(AD$5="")))),"")</f>
+        <v/>
+      </c>
+      <c r="AF10" s="47">
+        <f>IF(AND(ISNUMBER(O10),ISNUMBER(AE10)),O10*AE10,"")</f>
+        <v/>
+      </c>
+      <c r="AG10" s="48">
+        <f>IF(ISNUMBER(AF10),(AF10-1)/24,"")</f>
+        <v/>
+      </c>
+      <c r="AH10" s="49">
+        <f>IF(ISNUMBER(AF10),COUNTIF(AF$7:AF$27,"&gt;"&amp;AF10)+1,"")</f>
+        <v/>
+      </c>
+      <c r="AI10" s="50">
+        <f>COUNT(I10,J10,K10,L10,M10,N10,P10,Q10,R10,T10,U10,V10,W10,X10,Y10,AA10,AB10,AC10)</f>
         <v/>
       </c>
     </row>
@@ -2999,34 +3212,37 @@
       <c r="U11" s="45" t="n"/>
       <c r="V11" s="45" t="n"/>
       <c r="W11" s="45" t="n"/>
-      <c r="X11" s="46">
-        <f>IF(COUNT(T11:W11)=0,"",IFERROR(SUMPRODUCT(T11:W11,(T$5:W$5+(T$5:W$5="")))/SUMPRODUCT((T11:W11&lt;&gt;"")*(T$5:W$5+(T$5:W$5=""))),""))</f>
-        <v/>
-      </c>
+      <c r="X11" s="45" t="n"/>
       <c r="Y11" s="45" t="n"/>
-      <c r="Z11" s="45" t="n"/>
-      <c r="AA11" s="46">
-        <f>IF(COUNT(Y11:Z11)=0,"",IFERROR(SUMPRODUCT(Y11:Z11,(Y$5:Z$5+(Y$5:Z$5="")))/SUMPRODUCT((Y11:Z11&lt;&gt;"")*(Y$5:Z$5+(Y$5:Z$5=""))),""))</f>
-        <v/>
-      </c>
-      <c r="AB11" s="46">
-        <f>IFERROR(IF((ISNUMBER(S11)*(S$5+(S$5=""))+ISNUMBER(X11)*(X$5+(X$5=""))+ISNUMBER(AA11)*(AA$5+(AA$5="")))=0,"",(N(S11)*(S$5+(S$5=""))+N(X11)*(X$5+(X$5=""))+N(AA11)*(AA$5+(AA$5="")))/(ISNUMBER(S11)*(S$5+(S$5=""))+ISNUMBER(X11)*(X$5+(X$5=""))+ISNUMBER(AA11)*(AA$5+(AA$5="")))),"")</f>
-        <v/>
-      </c>
-      <c r="AC11" s="47">
-        <f>IF(AND(ISNUMBER(O11),ISNUMBER(AB11)),O11*AB11,"")</f>
-        <v/>
-      </c>
-      <c r="AD11" s="48">
-        <f>IF(ISNUMBER(AC11),(AC11-1)/24,"")</f>
-        <v/>
-      </c>
-      <c r="AE11" s="49">
-        <f>IF(ISNUMBER(AC11),COUNTIF(AC$7:AC$27,"&gt;"&amp;AC11)+1,"")</f>
-        <v/>
-      </c>
-      <c r="AF11" s="50">
-        <f>COUNT(I11,J11,K11,L11,M11,N11,P11,Q11,R11,T11,U11,V11,W11,Y11,Z11)</f>
+      <c r="Z11" s="46">
+        <f>IF(COUNT(T11:Y11)=0,"",IFERROR(SUMPRODUCT(T11:Y11,(T$5:Y$5+(T$5:Y$5="")))/SUMPRODUCT((T11:Y11&lt;&gt;"")*(T$5:Y$5+(T$5:Y$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="AA11" s="45" t="n"/>
+      <c r="AB11" s="45" t="n"/>
+      <c r="AC11" s="45" t="n"/>
+      <c r="AD11" s="46">
+        <f>IF(COUNT(AA11:AC11)=0,"",IFERROR(SUMPRODUCT(AA11:AC11,(AA$5:AC$5+(AA$5:AC$5="")))/SUMPRODUCT((AA11:AC11&lt;&gt;"")*(AA$5:AC$5+(AA$5:AC$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="AE11" s="46">
+        <f>IFERROR(IF((ISNUMBER(S11)*(S$5+(S$5=""))+ISNUMBER(Z11)*(Z$5+(Z$5=""))+ISNUMBER(AD11)*(AD$5+(AD$5="")))=0,"",(N(S11)*(S$5+(S$5=""))+N(Z11)*(Z$5+(Z$5=""))+N(AD11)*(AD$5+(AD$5="")))/(ISNUMBER(S11)*(S$5+(S$5=""))+ISNUMBER(Z11)*(Z$5+(Z$5=""))+ISNUMBER(AD11)*(AD$5+(AD$5="")))),"")</f>
+        <v/>
+      </c>
+      <c r="AF11" s="47">
+        <f>IF(AND(ISNUMBER(O11),ISNUMBER(AE11)),O11*AE11,"")</f>
+        <v/>
+      </c>
+      <c r="AG11" s="48">
+        <f>IF(ISNUMBER(AF11),(AF11-1)/24,"")</f>
+        <v/>
+      </c>
+      <c r="AH11" s="49">
+        <f>IF(ISNUMBER(AF11),COUNTIF(AF$7:AF$27,"&gt;"&amp;AF11)+1,"")</f>
+        <v/>
+      </c>
+      <c r="AI11" s="50">
+        <f>COUNT(I11,J11,K11,L11,M11,N11,P11,Q11,R11,T11,U11,V11,W11,X11,Y11,AA11,AB11,AC11)</f>
         <v/>
       </c>
     </row>
@@ -3086,34 +3302,37 @@
       <c r="U12" s="45" t="n"/>
       <c r="V12" s="45" t="n"/>
       <c r="W12" s="45" t="n"/>
-      <c r="X12" s="46">
-        <f>IF(COUNT(T12:W12)=0,"",IFERROR(SUMPRODUCT(T12:W12,(T$5:W$5+(T$5:W$5="")))/SUMPRODUCT((T12:W12&lt;&gt;"")*(T$5:W$5+(T$5:W$5=""))),""))</f>
-        <v/>
-      </c>
+      <c r="X12" s="45" t="n"/>
       <c r="Y12" s="45" t="n"/>
-      <c r="Z12" s="45" t="n"/>
-      <c r="AA12" s="46">
-        <f>IF(COUNT(Y12:Z12)=0,"",IFERROR(SUMPRODUCT(Y12:Z12,(Y$5:Z$5+(Y$5:Z$5="")))/SUMPRODUCT((Y12:Z12&lt;&gt;"")*(Y$5:Z$5+(Y$5:Z$5=""))),""))</f>
-        <v/>
-      </c>
-      <c r="AB12" s="46">
-        <f>IFERROR(IF((ISNUMBER(S12)*(S$5+(S$5=""))+ISNUMBER(X12)*(X$5+(X$5=""))+ISNUMBER(AA12)*(AA$5+(AA$5="")))=0,"",(N(S12)*(S$5+(S$5=""))+N(X12)*(X$5+(X$5=""))+N(AA12)*(AA$5+(AA$5="")))/(ISNUMBER(S12)*(S$5+(S$5=""))+ISNUMBER(X12)*(X$5+(X$5=""))+ISNUMBER(AA12)*(AA$5+(AA$5="")))),"")</f>
-        <v/>
-      </c>
-      <c r="AC12" s="47">
-        <f>IF(AND(ISNUMBER(O12),ISNUMBER(AB12)),O12*AB12,"")</f>
-        <v/>
-      </c>
-      <c r="AD12" s="48">
-        <f>IF(ISNUMBER(AC12),(AC12-1)/24,"")</f>
-        <v/>
-      </c>
-      <c r="AE12" s="49">
-        <f>IF(ISNUMBER(AC12),COUNTIF(AC$7:AC$27,"&gt;"&amp;AC12)+1,"")</f>
-        <v/>
-      </c>
-      <c r="AF12" s="50">
-        <f>COUNT(I12,J12,K12,L12,M12,N12,P12,Q12,R12,T12,U12,V12,W12,Y12,Z12)</f>
+      <c r="Z12" s="46">
+        <f>IF(COUNT(T12:Y12)=0,"",IFERROR(SUMPRODUCT(T12:Y12,(T$5:Y$5+(T$5:Y$5="")))/SUMPRODUCT((T12:Y12&lt;&gt;"")*(T$5:Y$5+(T$5:Y$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="AA12" s="45" t="n"/>
+      <c r="AB12" s="45" t="n"/>
+      <c r="AC12" s="45" t="n"/>
+      <c r="AD12" s="46">
+        <f>IF(COUNT(AA12:AC12)=0,"",IFERROR(SUMPRODUCT(AA12:AC12,(AA$5:AC$5+(AA$5:AC$5="")))/SUMPRODUCT((AA12:AC12&lt;&gt;"")*(AA$5:AC$5+(AA$5:AC$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="AE12" s="46">
+        <f>IFERROR(IF((ISNUMBER(S12)*(S$5+(S$5=""))+ISNUMBER(Z12)*(Z$5+(Z$5=""))+ISNUMBER(AD12)*(AD$5+(AD$5="")))=0,"",(N(S12)*(S$5+(S$5=""))+N(Z12)*(Z$5+(Z$5=""))+N(AD12)*(AD$5+(AD$5="")))/(ISNUMBER(S12)*(S$5+(S$5=""))+ISNUMBER(Z12)*(Z$5+(Z$5=""))+ISNUMBER(AD12)*(AD$5+(AD$5="")))),"")</f>
+        <v/>
+      </c>
+      <c r="AF12" s="47">
+        <f>IF(AND(ISNUMBER(O12),ISNUMBER(AE12)),O12*AE12,"")</f>
+        <v/>
+      </c>
+      <c r="AG12" s="48">
+        <f>IF(ISNUMBER(AF12),(AF12-1)/24,"")</f>
+        <v/>
+      </c>
+      <c r="AH12" s="49">
+        <f>IF(ISNUMBER(AF12),COUNTIF(AF$7:AF$27,"&gt;"&amp;AF12)+1,"")</f>
+        <v/>
+      </c>
+      <c r="AI12" s="50">
+        <f>COUNT(I12,J12,K12,L12,M12,N12,P12,Q12,R12,T12,U12,V12,W12,X12,Y12,AA12,AB12,AC12)</f>
         <v/>
       </c>
     </row>
@@ -3173,34 +3392,37 @@
       <c r="U13" s="45" t="n"/>
       <c r="V13" s="45" t="n"/>
       <c r="W13" s="45" t="n"/>
-      <c r="X13" s="46">
-        <f>IF(COUNT(T13:W13)=0,"",IFERROR(SUMPRODUCT(T13:W13,(T$5:W$5+(T$5:W$5="")))/SUMPRODUCT((T13:W13&lt;&gt;"")*(T$5:W$5+(T$5:W$5=""))),""))</f>
-        <v/>
-      </c>
+      <c r="X13" s="45" t="n"/>
       <c r="Y13" s="45" t="n"/>
-      <c r="Z13" s="45" t="n"/>
-      <c r="AA13" s="46">
-        <f>IF(COUNT(Y13:Z13)=0,"",IFERROR(SUMPRODUCT(Y13:Z13,(Y$5:Z$5+(Y$5:Z$5="")))/SUMPRODUCT((Y13:Z13&lt;&gt;"")*(Y$5:Z$5+(Y$5:Z$5=""))),""))</f>
-        <v/>
-      </c>
-      <c r="AB13" s="46">
-        <f>IFERROR(IF((ISNUMBER(S13)*(S$5+(S$5=""))+ISNUMBER(X13)*(X$5+(X$5=""))+ISNUMBER(AA13)*(AA$5+(AA$5="")))=0,"",(N(S13)*(S$5+(S$5=""))+N(X13)*(X$5+(X$5=""))+N(AA13)*(AA$5+(AA$5="")))/(ISNUMBER(S13)*(S$5+(S$5=""))+ISNUMBER(X13)*(X$5+(X$5=""))+ISNUMBER(AA13)*(AA$5+(AA$5="")))),"")</f>
-        <v/>
-      </c>
-      <c r="AC13" s="47">
-        <f>IF(AND(ISNUMBER(O13),ISNUMBER(AB13)),O13*AB13,"")</f>
-        <v/>
-      </c>
-      <c r="AD13" s="48">
-        <f>IF(ISNUMBER(AC13),(AC13-1)/24,"")</f>
-        <v/>
-      </c>
-      <c r="AE13" s="49">
-        <f>IF(ISNUMBER(AC13),COUNTIF(AC$7:AC$27,"&gt;"&amp;AC13)+1,"")</f>
-        <v/>
-      </c>
-      <c r="AF13" s="50">
-        <f>COUNT(I13,J13,K13,L13,M13,N13,P13,Q13,R13,T13,U13,V13,W13,Y13,Z13)</f>
+      <c r="Z13" s="46">
+        <f>IF(COUNT(T13:Y13)=0,"",IFERROR(SUMPRODUCT(T13:Y13,(T$5:Y$5+(T$5:Y$5="")))/SUMPRODUCT((T13:Y13&lt;&gt;"")*(T$5:Y$5+(T$5:Y$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="AA13" s="45" t="n"/>
+      <c r="AB13" s="45" t="n"/>
+      <c r="AC13" s="45" t="n"/>
+      <c r="AD13" s="46">
+        <f>IF(COUNT(AA13:AC13)=0,"",IFERROR(SUMPRODUCT(AA13:AC13,(AA$5:AC$5+(AA$5:AC$5="")))/SUMPRODUCT((AA13:AC13&lt;&gt;"")*(AA$5:AC$5+(AA$5:AC$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="AE13" s="46">
+        <f>IFERROR(IF((ISNUMBER(S13)*(S$5+(S$5=""))+ISNUMBER(Z13)*(Z$5+(Z$5=""))+ISNUMBER(AD13)*(AD$5+(AD$5="")))=0,"",(N(S13)*(S$5+(S$5=""))+N(Z13)*(Z$5+(Z$5=""))+N(AD13)*(AD$5+(AD$5="")))/(ISNUMBER(S13)*(S$5+(S$5=""))+ISNUMBER(Z13)*(Z$5+(Z$5=""))+ISNUMBER(AD13)*(AD$5+(AD$5="")))),"")</f>
+        <v/>
+      </c>
+      <c r="AF13" s="47">
+        <f>IF(AND(ISNUMBER(O13),ISNUMBER(AE13)),O13*AE13,"")</f>
+        <v/>
+      </c>
+      <c r="AG13" s="48">
+        <f>IF(ISNUMBER(AF13),(AF13-1)/24,"")</f>
+        <v/>
+      </c>
+      <c r="AH13" s="49">
+        <f>IF(ISNUMBER(AF13),COUNTIF(AF$7:AF$27,"&gt;"&amp;AF13)+1,"")</f>
+        <v/>
+      </c>
+      <c r="AI13" s="50">
+        <f>COUNT(I13,J13,K13,L13,M13,N13,P13,Q13,R13,T13,U13,V13,W13,X13,Y13,AA13,AB13,AC13)</f>
         <v/>
       </c>
     </row>
@@ -3256,34 +3478,37 @@
       <c r="U14" s="45" t="n"/>
       <c r="V14" s="45" t="n"/>
       <c r="W14" s="45" t="n"/>
-      <c r="X14" s="46">
-        <f>IF(COUNT(T14:W14)=0,"",IFERROR(SUMPRODUCT(T14:W14,(T$5:W$5+(T$5:W$5="")))/SUMPRODUCT((T14:W14&lt;&gt;"")*(T$5:W$5+(T$5:W$5=""))),""))</f>
-        <v/>
-      </c>
+      <c r="X14" s="45" t="n"/>
       <c r="Y14" s="45" t="n"/>
-      <c r="Z14" s="45" t="n"/>
-      <c r="AA14" s="46">
-        <f>IF(COUNT(Y14:Z14)=0,"",IFERROR(SUMPRODUCT(Y14:Z14,(Y$5:Z$5+(Y$5:Z$5="")))/SUMPRODUCT((Y14:Z14&lt;&gt;"")*(Y$5:Z$5+(Y$5:Z$5=""))),""))</f>
-        <v/>
-      </c>
-      <c r="AB14" s="46">
-        <f>IFERROR(IF((ISNUMBER(S14)*(S$5+(S$5=""))+ISNUMBER(X14)*(X$5+(X$5=""))+ISNUMBER(AA14)*(AA$5+(AA$5="")))=0,"",(N(S14)*(S$5+(S$5=""))+N(X14)*(X$5+(X$5=""))+N(AA14)*(AA$5+(AA$5="")))/(ISNUMBER(S14)*(S$5+(S$5=""))+ISNUMBER(X14)*(X$5+(X$5=""))+ISNUMBER(AA14)*(AA$5+(AA$5="")))),"")</f>
-        <v/>
-      </c>
-      <c r="AC14" s="47">
-        <f>IF(AND(ISNUMBER(O14),ISNUMBER(AB14)),O14*AB14,"")</f>
-        <v/>
-      </c>
-      <c r="AD14" s="48">
-        <f>IF(ISNUMBER(AC14),(AC14-1)/24,"")</f>
-        <v/>
-      </c>
-      <c r="AE14" s="49">
-        <f>IF(ISNUMBER(AC14),COUNTIF(AC$7:AC$27,"&gt;"&amp;AC14)+1,"")</f>
-        <v/>
-      </c>
-      <c r="AF14" s="50">
-        <f>COUNT(I14,J14,K14,L14,M14,N14,P14,Q14,R14,T14,U14,V14,W14,Y14,Z14)</f>
+      <c r="Z14" s="46">
+        <f>IF(COUNT(T14:Y14)=0,"",IFERROR(SUMPRODUCT(T14:Y14,(T$5:Y$5+(T$5:Y$5="")))/SUMPRODUCT((T14:Y14&lt;&gt;"")*(T$5:Y$5+(T$5:Y$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="AA14" s="45" t="n"/>
+      <c r="AB14" s="45" t="n"/>
+      <c r="AC14" s="45" t="n"/>
+      <c r="AD14" s="46">
+        <f>IF(COUNT(AA14:AC14)=0,"",IFERROR(SUMPRODUCT(AA14:AC14,(AA$5:AC$5+(AA$5:AC$5="")))/SUMPRODUCT((AA14:AC14&lt;&gt;"")*(AA$5:AC$5+(AA$5:AC$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="AE14" s="46">
+        <f>IFERROR(IF((ISNUMBER(S14)*(S$5+(S$5=""))+ISNUMBER(Z14)*(Z$5+(Z$5=""))+ISNUMBER(AD14)*(AD$5+(AD$5="")))=0,"",(N(S14)*(S$5+(S$5=""))+N(Z14)*(Z$5+(Z$5=""))+N(AD14)*(AD$5+(AD$5="")))/(ISNUMBER(S14)*(S$5+(S$5=""))+ISNUMBER(Z14)*(Z$5+(Z$5=""))+ISNUMBER(AD14)*(AD$5+(AD$5="")))),"")</f>
+        <v/>
+      </c>
+      <c r="AF14" s="47">
+        <f>IF(AND(ISNUMBER(O14),ISNUMBER(AE14)),O14*AE14,"")</f>
+        <v/>
+      </c>
+      <c r="AG14" s="48">
+        <f>IF(ISNUMBER(AF14),(AF14-1)/24,"")</f>
+        <v/>
+      </c>
+      <c r="AH14" s="49">
+        <f>IF(ISNUMBER(AF14),COUNTIF(AF$7:AF$27,"&gt;"&amp;AF14)+1,"")</f>
+        <v/>
+      </c>
+      <c r="AI14" s="50">
+        <f>COUNT(I14,J14,K14,L14,M14,N14,P14,Q14,R14,T14,U14,V14,W14,X14,Y14,AA14,AB14,AC14)</f>
         <v/>
       </c>
     </row>
@@ -3339,34 +3564,37 @@
       <c r="U15" s="45" t="n"/>
       <c r="V15" s="45" t="n"/>
       <c r="W15" s="45" t="n"/>
-      <c r="X15" s="46">
-        <f>IF(COUNT(T15:W15)=0,"",IFERROR(SUMPRODUCT(T15:W15,(T$5:W$5+(T$5:W$5="")))/SUMPRODUCT((T15:W15&lt;&gt;"")*(T$5:W$5+(T$5:W$5=""))),""))</f>
-        <v/>
-      </c>
+      <c r="X15" s="45" t="n"/>
       <c r="Y15" s="45" t="n"/>
-      <c r="Z15" s="45" t="n"/>
-      <c r="AA15" s="46">
-        <f>IF(COUNT(Y15:Z15)=0,"",IFERROR(SUMPRODUCT(Y15:Z15,(Y$5:Z$5+(Y$5:Z$5="")))/SUMPRODUCT((Y15:Z15&lt;&gt;"")*(Y$5:Z$5+(Y$5:Z$5=""))),""))</f>
-        <v/>
-      </c>
-      <c r="AB15" s="46">
-        <f>IFERROR(IF((ISNUMBER(S15)*(S$5+(S$5=""))+ISNUMBER(X15)*(X$5+(X$5=""))+ISNUMBER(AA15)*(AA$5+(AA$5="")))=0,"",(N(S15)*(S$5+(S$5=""))+N(X15)*(X$5+(X$5=""))+N(AA15)*(AA$5+(AA$5="")))/(ISNUMBER(S15)*(S$5+(S$5=""))+ISNUMBER(X15)*(X$5+(X$5=""))+ISNUMBER(AA15)*(AA$5+(AA$5="")))),"")</f>
-        <v/>
-      </c>
-      <c r="AC15" s="47">
-        <f>IF(AND(ISNUMBER(O15),ISNUMBER(AB15)),O15*AB15,"")</f>
-        <v/>
-      </c>
-      <c r="AD15" s="48">
-        <f>IF(ISNUMBER(AC15),(AC15-1)/24,"")</f>
-        <v/>
-      </c>
-      <c r="AE15" s="49">
-        <f>IF(ISNUMBER(AC15),COUNTIF(AC$7:AC$27,"&gt;"&amp;AC15)+1,"")</f>
-        <v/>
-      </c>
-      <c r="AF15" s="50">
-        <f>COUNT(I15,J15,K15,L15,M15,N15,P15,Q15,R15,T15,U15,V15,W15,Y15,Z15)</f>
+      <c r="Z15" s="46">
+        <f>IF(COUNT(T15:Y15)=0,"",IFERROR(SUMPRODUCT(T15:Y15,(T$5:Y$5+(T$5:Y$5="")))/SUMPRODUCT((T15:Y15&lt;&gt;"")*(T$5:Y$5+(T$5:Y$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="AA15" s="45" t="n"/>
+      <c r="AB15" s="45" t="n"/>
+      <c r="AC15" s="45" t="n"/>
+      <c r="AD15" s="46">
+        <f>IF(COUNT(AA15:AC15)=0,"",IFERROR(SUMPRODUCT(AA15:AC15,(AA$5:AC$5+(AA$5:AC$5="")))/SUMPRODUCT((AA15:AC15&lt;&gt;"")*(AA$5:AC$5+(AA$5:AC$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="AE15" s="46">
+        <f>IFERROR(IF((ISNUMBER(S15)*(S$5+(S$5=""))+ISNUMBER(Z15)*(Z$5+(Z$5=""))+ISNUMBER(AD15)*(AD$5+(AD$5="")))=0,"",(N(S15)*(S$5+(S$5=""))+N(Z15)*(Z$5+(Z$5=""))+N(AD15)*(AD$5+(AD$5="")))/(ISNUMBER(S15)*(S$5+(S$5=""))+ISNUMBER(Z15)*(Z$5+(Z$5=""))+ISNUMBER(AD15)*(AD$5+(AD$5="")))),"")</f>
+        <v/>
+      </c>
+      <c r="AF15" s="47">
+        <f>IF(AND(ISNUMBER(O15),ISNUMBER(AE15)),O15*AE15,"")</f>
+        <v/>
+      </c>
+      <c r="AG15" s="48">
+        <f>IF(ISNUMBER(AF15),(AF15-1)/24,"")</f>
+        <v/>
+      </c>
+      <c r="AH15" s="49">
+        <f>IF(ISNUMBER(AF15),COUNTIF(AF$7:AF$27,"&gt;"&amp;AF15)+1,"")</f>
+        <v/>
+      </c>
+      <c r="AI15" s="50">
+        <f>COUNT(I15,J15,K15,L15,M15,N15,P15,Q15,R15,T15,U15,V15,W15,X15,Y15,AA15,AB15,AC15)</f>
         <v/>
       </c>
     </row>
@@ -3422,34 +3650,37 @@
       <c r="U16" s="45" t="n"/>
       <c r="V16" s="45" t="n"/>
       <c r="W16" s="45" t="n"/>
-      <c r="X16" s="46">
-        <f>IF(COUNT(T16:W16)=0,"",IFERROR(SUMPRODUCT(T16:W16,(T$5:W$5+(T$5:W$5="")))/SUMPRODUCT((T16:W16&lt;&gt;"")*(T$5:W$5+(T$5:W$5=""))),""))</f>
-        <v/>
-      </c>
+      <c r="X16" s="45" t="n"/>
       <c r="Y16" s="45" t="n"/>
-      <c r="Z16" s="45" t="n"/>
-      <c r="AA16" s="46">
-        <f>IF(COUNT(Y16:Z16)=0,"",IFERROR(SUMPRODUCT(Y16:Z16,(Y$5:Z$5+(Y$5:Z$5="")))/SUMPRODUCT((Y16:Z16&lt;&gt;"")*(Y$5:Z$5+(Y$5:Z$5=""))),""))</f>
-        <v/>
-      </c>
-      <c r="AB16" s="46">
-        <f>IFERROR(IF((ISNUMBER(S16)*(S$5+(S$5=""))+ISNUMBER(X16)*(X$5+(X$5=""))+ISNUMBER(AA16)*(AA$5+(AA$5="")))=0,"",(N(S16)*(S$5+(S$5=""))+N(X16)*(X$5+(X$5=""))+N(AA16)*(AA$5+(AA$5="")))/(ISNUMBER(S16)*(S$5+(S$5=""))+ISNUMBER(X16)*(X$5+(X$5=""))+ISNUMBER(AA16)*(AA$5+(AA$5="")))),"")</f>
-        <v/>
-      </c>
-      <c r="AC16" s="47">
-        <f>IF(AND(ISNUMBER(O16),ISNUMBER(AB16)),O16*AB16,"")</f>
-        <v/>
-      </c>
-      <c r="AD16" s="48">
-        <f>IF(ISNUMBER(AC16),(AC16-1)/24,"")</f>
-        <v/>
-      </c>
-      <c r="AE16" s="49">
-        <f>IF(ISNUMBER(AC16),COUNTIF(AC$7:AC$27,"&gt;"&amp;AC16)+1,"")</f>
-        <v/>
-      </c>
-      <c r="AF16" s="50">
-        <f>COUNT(I16,J16,K16,L16,M16,N16,P16,Q16,R16,T16,U16,V16,W16,Y16,Z16)</f>
+      <c r="Z16" s="46">
+        <f>IF(COUNT(T16:Y16)=0,"",IFERROR(SUMPRODUCT(T16:Y16,(T$5:Y$5+(T$5:Y$5="")))/SUMPRODUCT((T16:Y16&lt;&gt;"")*(T$5:Y$5+(T$5:Y$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="AA16" s="45" t="n"/>
+      <c r="AB16" s="45" t="n"/>
+      <c r="AC16" s="45" t="n"/>
+      <c r="AD16" s="46">
+        <f>IF(COUNT(AA16:AC16)=0,"",IFERROR(SUMPRODUCT(AA16:AC16,(AA$5:AC$5+(AA$5:AC$5="")))/SUMPRODUCT((AA16:AC16&lt;&gt;"")*(AA$5:AC$5+(AA$5:AC$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="AE16" s="46">
+        <f>IFERROR(IF((ISNUMBER(S16)*(S$5+(S$5=""))+ISNUMBER(Z16)*(Z$5+(Z$5=""))+ISNUMBER(AD16)*(AD$5+(AD$5="")))=0,"",(N(S16)*(S$5+(S$5=""))+N(Z16)*(Z$5+(Z$5=""))+N(AD16)*(AD$5+(AD$5="")))/(ISNUMBER(S16)*(S$5+(S$5=""))+ISNUMBER(Z16)*(Z$5+(Z$5=""))+ISNUMBER(AD16)*(AD$5+(AD$5="")))),"")</f>
+        <v/>
+      </c>
+      <c r="AF16" s="47">
+        <f>IF(AND(ISNUMBER(O16),ISNUMBER(AE16)),O16*AE16,"")</f>
+        <v/>
+      </c>
+      <c r="AG16" s="48">
+        <f>IF(ISNUMBER(AF16),(AF16-1)/24,"")</f>
+        <v/>
+      </c>
+      <c r="AH16" s="49">
+        <f>IF(ISNUMBER(AF16),COUNTIF(AF$7:AF$27,"&gt;"&amp;AF16)+1,"")</f>
+        <v/>
+      </c>
+      <c r="AI16" s="50">
+        <f>COUNT(I16,J16,K16,L16,M16,N16,P16,Q16,R16,T16,U16,V16,W16,X16,Y16,AA16,AB16,AC16)</f>
         <v/>
       </c>
     </row>
@@ -3505,34 +3736,37 @@
       <c r="U17" s="45" t="n"/>
       <c r="V17" s="45" t="n"/>
       <c r="W17" s="45" t="n"/>
-      <c r="X17" s="46">
-        <f>IF(COUNT(T17:W17)=0,"",IFERROR(SUMPRODUCT(T17:W17,(T$5:W$5+(T$5:W$5="")))/SUMPRODUCT((T17:W17&lt;&gt;"")*(T$5:W$5+(T$5:W$5=""))),""))</f>
-        <v/>
-      </c>
+      <c r="X17" s="45" t="n"/>
       <c r="Y17" s="45" t="n"/>
-      <c r="Z17" s="45" t="n"/>
-      <c r="AA17" s="46">
-        <f>IF(COUNT(Y17:Z17)=0,"",IFERROR(SUMPRODUCT(Y17:Z17,(Y$5:Z$5+(Y$5:Z$5="")))/SUMPRODUCT((Y17:Z17&lt;&gt;"")*(Y$5:Z$5+(Y$5:Z$5=""))),""))</f>
-        <v/>
-      </c>
-      <c r="AB17" s="46">
-        <f>IFERROR(IF((ISNUMBER(S17)*(S$5+(S$5=""))+ISNUMBER(X17)*(X$5+(X$5=""))+ISNUMBER(AA17)*(AA$5+(AA$5="")))=0,"",(N(S17)*(S$5+(S$5=""))+N(X17)*(X$5+(X$5=""))+N(AA17)*(AA$5+(AA$5="")))/(ISNUMBER(S17)*(S$5+(S$5=""))+ISNUMBER(X17)*(X$5+(X$5=""))+ISNUMBER(AA17)*(AA$5+(AA$5="")))),"")</f>
-        <v/>
-      </c>
-      <c r="AC17" s="47">
-        <f>IF(AND(ISNUMBER(O17),ISNUMBER(AB17)),O17*AB17,"")</f>
-        <v/>
-      </c>
-      <c r="AD17" s="48">
-        <f>IF(ISNUMBER(AC17),(AC17-1)/24,"")</f>
-        <v/>
-      </c>
-      <c r="AE17" s="49">
-        <f>IF(ISNUMBER(AC17),COUNTIF(AC$7:AC$27,"&gt;"&amp;AC17)+1,"")</f>
-        <v/>
-      </c>
-      <c r="AF17" s="50">
-        <f>COUNT(I17,J17,K17,L17,M17,N17,P17,Q17,R17,T17,U17,V17,W17,Y17,Z17)</f>
+      <c r="Z17" s="46">
+        <f>IF(COUNT(T17:Y17)=0,"",IFERROR(SUMPRODUCT(T17:Y17,(T$5:Y$5+(T$5:Y$5="")))/SUMPRODUCT((T17:Y17&lt;&gt;"")*(T$5:Y$5+(T$5:Y$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="AA17" s="45" t="n"/>
+      <c r="AB17" s="45" t="n"/>
+      <c r="AC17" s="45" t="n"/>
+      <c r="AD17" s="46">
+        <f>IF(COUNT(AA17:AC17)=0,"",IFERROR(SUMPRODUCT(AA17:AC17,(AA$5:AC$5+(AA$5:AC$5="")))/SUMPRODUCT((AA17:AC17&lt;&gt;"")*(AA$5:AC$5+(AA$5:AC$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="AE17" s="46">
+        <f>IFERROR(IF((ISNUMBER(S17)*(S$5+(S$5=""))+ISNUMBER(Z17)*(Z$5+(Z$5=""))+ISNUMBER(AD17)*(AD$5+(AD$5="")))=0,"",(N(S17)*(S$5+(S$5=""))+N(Z17)*(Z$5+(Z$5=""))+N(AD17)*(AD$5+(AD$5="")))/(ISNUMBER(S17)*(S$5+(S$5=""))+ISNUMBER(Z17)*(Z$5+(Z$5=""))+ISNUMBER(AD17)*(AD$5+(AD$5="")))),"")</f>
+        <v/>
+      </c>
+      <c r="AF17" s="47">
+        <f>IF(AND(ISNUMBER(O17),ISNUMBER(AE17)),O17*AE17,"")</f>
+        <v/>
+      </c>
+      <c r="AG17" s="48">
+        <f>IF(ISNUMBER(AF17),(AF17-1)/24,"")</f>
+        <v/>
+      </c>
+      <c r="AH17" s="49">
+        <f>IF(ISNUMBER(AF17),COUNTIF(AF$7:AF$27,"&gt;"&amp;AF17)+1,"")</f>
+        <v/>
+      </c>
+      <c r="AI17" s="50">
+        <f>COUNT(I17,J17,K17,L17,M17,N17,P17,Q17,R17,T17,U17,V17,W17,X17,Y17,AA17,AB17,AC17)</f>
         <v/>
       </c>
     </row>
@@ -3588,34 +3822,37 @@
       <c r="U18" s="45" t="n"/>
       <c r="V18" s="45" t="n"/>
       <c r="W18" s="45" t="n"/>
-      <c r="X18" s="46">
-        <f>IF(COUNT(T18:W18)=0,"",IFERROR(SUMPRODUCT(T18:W18,(T$5:W$5+(T$5:W$5="")))/SUMPRODUCT((T18:W18&lt;&gt;"")*(T$5:W$5+(T$5:W$5=""))),""))</f>
-        <v/>
-      </c>
+      <c r="X18" s="45" t="n"/>
       <c r="Y18" s="45" t="n"/>
-      <c r="Z18" s="45" t="n"/>
-      <c r="AA18" s="46">
-        <f>IF(COUNT(Y18:Z18)=0,"",IFERROR(SUMPRODUCT(Y18:Z18,(Y$5:Z$5+(Y$5:Z$5="")))/SUMPRODUCT((Y18:Z18&lt;&gt;"")*(Y$5:Z$5+(Y$5:Z$5=""))),""))</f>
-        <v/>
-      </c>
-      <c r="AB18" s="46">
-        <f>IFERROR(IF((ISNUMBER(S18)*(S$5+(S$5=""))+ISNUMBER(X18)*(X$5+(X$5=""))+ISNUMBER(AA18)*(AA$5+(AA$5="")))=0,"",(N(S18)*(S$5+(S$5=""))+N(X18)*(X$5+(X$5=""))+N(AA18)*(AA$5+(AA$5="")))/(ISNUMBER(S18)*(S$5+(S$5=""))+ISNUMBER(X18)*(X$5+(X$5=""))+ISNUMBER(AA18)*(AA$5+(AA$5="")))),"")</f>
-        <v/>
-      </c>
-      <c r="AC18" s="47">
-        <f>IF(AND(ISNUMBER(O18),ISNUMBER(AB18)),O18*AB18,"")</f>
-        <v/>
-      </c>
-      <c r="AD18" s="48">
-        <f>IF(ISNUMBER(AC18),(AC18-1)/24,"")</f>
-        <v/>
-      </c>
-      <c r="AE18" s="49">
-        <f>IF(ISNUMBER(AC18),COUNTIF(AC$7:AC$27,"&gt;"&amp;AC18)+1,"")</f>
-        <v/>
-      </c>
-      <c r="AF18" s="50">
-        <f>COUNT(I18,J18,K18,L18,M18,N18,P18,Q18,R18,T18,U18,V18,W18,Y18,Z18)</f>
+      <c r="Z18" s="46">
+        <f>IF(COUNT(T18:Y18)=0,"",IFERROR(SUMPRODUCT(T18:Y18,(T$5:Y$5+(T$5:Y$5="")))/SUMPRODUCT((T18:Y18&lt;&gt;"")*(T$5:Y$5+(T$5:Y$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="AA18" s="45" t="n"/>
+      <c r="AB18" s="45" t="n"/>
+      <c r="AC18" s="45" t="n"/>
+      <c r="AD18" s="46">
+        <f>IF(COUNT(AA18:AC18)=0,"",IFERROR(SUMPRODUCT(AA18:AC18,(AA$5:AC$5+(AA$5:AC$5="")))/SUMPRODUCT((AA18:AC18&lt;&gt;"")*(AA$5:AC$5+(AA$5:AC$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="AE18" s="46">
+        <f>IFERROR(IF((ISNUMBER(S18)*(S$5+(S$5=""))+ISNUMBER(Z18)*(Z$5+(Z$5=""))+ISNUMBER(AD18)*(AD$5+(AD$5="")))=0,"",(N(S18)*(S$5+(S$5=""))+N(Z18)*(Z$5+(Z$5=""))+N(AD18)*(AD$5+(AD$5="")))/(ISNUMBER(S18)*(S$5+(S$5=""))+ISNUMBER(Z18)*(Z$5+(Z$5=""))+ISNUMBER(AD18)*(AD$5+(AD$5="")))),"")</f>
+        <v/>
+      </c>
+      <c r="AF18" s="47">
+        <f>IF(AND(ISNUMBER(O18),ISNUMBER(AE18)),O18*AE18,"")</f>
+        <v/>
+      </c>
+      <c r="AG18" s="48">
+        <f>IF(ISNUMBER(AF18),(AF18-1)/24,"")</f>
+        <v/>
+      </c>
+      <c r="AH18" s="49">
+        <f>IF(ISNUMBER(AF18),COUNTIF(AF$7:AF$27,"&gt;"&amp;AF18)+1,"")</f>
+        <v/>
+      </c>
+      <c r="AI18" s="50">
+        <f>COUNT(I18,J18,K18,L18,M18,N18,P18,Q18,R18,T18,U18,V18,W18,X18,Y18,AA18,AB18,AC18)</f>
         <v/>
       </c>
     </row>
@@ -3671,34 +3908,37 @@
       <c r="U19" s="45" t="n"/>
       <c r="V19" s="45" t="n"/>
       <c r="W19" s="45" t="n"/>
-      <c r="X19" s="46">
-        <f>IF(COUNT(T19:W19)=0,"",IFERROR(SUMPRODUCT(T19:W19,(T$5:W$5+(T$5:W$5="")))/SUMPRODUCT((T19:W19&lt;&gt;"")*(T$5:W$5+(T$5:W$5=""))),""))</f>
-        <v/>
-      </c>
+      <c r="X19" s="45" t="n"/>
       <c r="Y19" s="45" t="n"/>
-      <c r="Z19" s="45" t="n"/>
-      <c r="AA19" s="46">
-        <f>IF(COUNT(Y19:Z19)=0,"",IFERROR(SUMPRODUCT(Y19:Z19,(Y$5:Z$5+(Y$5:Z$5="")))/SUMPRODUCT((Y19:Z19&lt;&gt;"")*(Y$5:Z$5+(Y$5:Z$5=""))),""))</f>
-        <v/>
-      </c>
-      <c r="AB19" s="46">
-        <f>IFERROR(IF((ISNUMBER(S19)*(S$5+(S$5=""))+ISNUMBER(X19)*(X$5+(X$5=""))+ISNUMBER(AA19)*(AA$5+(AA$5="")))=0,"",(N(S19)*(S$5+(S$5=""))+N(X19)*(X$5+(X$5=""))+N(AA19)*(AA$5+(AA$5="")))/(ISNUMBER(S19)*(S$5+(S$5=""))+ISNUMBER(X19)*(X$5+(X$5=""))+ISNUMBER(AA19)*(AA$5+(AA$5="")))),"")</f>
-        <v/>
-      </c>
-      <c r="AC19" s="47">
-        <f>IF(AND(ISNUMBER(O19),ISNUMBER(AB19)),O19*AB19,"")</f>
-        <v/>
-      </c>
-      <c r="AD19" s="48">
-        <f>IF(ISNUMBER(AC19),(AC19-1)/24,"")</f>
-        <v/>
-      </c>
-      <c r="AE19" s="49">
-        <f>IF(ISNUMBER(AC19),COUNTIF(AC$7:AC$27,"&gt;"&amp;AC19)+1,"")</f>
-        <v/>
-      </c>
-      <c r="AF19" s="50">
-        <f>COUNT(I19,J19,K19,L19,M19,N19,P19,Q19,R19,T19,U19,V19,W19,Y19,Z19)</f>
+      <c r="Z19" s="46">
+        <f>IF(COUNT(T19:Y19)=0,"",IFERROR(SUMPRODUCT(T19:Y19,(T$5:Y$5+(T$5:Y$5="")))/SUMPRODUCT((T19:Y19&lt;&gt;"")*(T$5:Y$5+(T$5:Y$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="AA19" s="45" t="n"/>
+      <c r="AB19" s="45" t="n"/>
+      <c r="AC19" s="45" t="n"/>
+      <c r="AD19" s="46">
+        <f>IF(COUNT(AA19:AC19)=0,"",IFERROR(SUMPRODUCT(AA19:AC19,(AA$5:AC$5+(AA$5:AC$5="")))/SUMPRODUCT((AA19:AC19&lt;&gt;"")*(AA$5:AC$5+(AA$5:AC$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="AE19" s="46">
+        <f>IFERROR(IF((ISNUMBER(S19)*(S$5+(S$5=""))+ISNUMBER(Z19)*(Z$5+(Z$5=""))+ISNUMBER(AD19)*(AD$5+(AD$5="")))=0,"",(N(S19)*(S$5+(S$5=""))+N(Z19)*(Z$5+(Z$5=""))+N(AD19)*(AD$5+(AD$5="")))/(ISNUMBER(S19)*(S$5+(S$5=""))+ISNUMBER(Z19)*(Z$5+(Z$5=""))+ISNUMBER(AD19)*(AD$5+(AD$5="")))),"")</f>
+        <v/>
+      </c>
+      <c r="AF19" s="47">
+        <f>IF(AND(ISNUMBER(O19),ISNUMBER(AE19)),O19*AE19,"")</f>
+        <v/>
+      </c>
+      <c r="AG19" s="48">
+        <f>IF(ISNUMBER(AF19),(AF19-1)/24,"")</f>
+        <v/>
+      </c>
+      <c r="AH19" s="49">
+        <f>IF(ISNUMBER(AF19),COUNTIF(AF$7:AF$27,"&gt;"&amp;AF19)+1,"")</f>
+        <v/>
+      </c>
+      <c r="AI19" s="50">
+        <f>COUNT(I19,J19,K19,L19,M19,N19,P19,Q19,R19,T19,U19,V19,W19,X19,Y19,AA19,AB19,AC19)</f>
         <v/>
       </c>
     </row>
@@ -3758,34 +3998,37 @@
       <c r="U20" s="45" t="n"/>
       <c r="V20" s="45" t="n"/>
       <c r="W20" s="45" t="n"/>
-      <c r="X20" s="46">
-        <f>IF(COUNT(T20:W20)=0,"",IFERROR(SUMPRODUCT(T20:W20,(T$5:W$5+(T$5:W$5="")))/SUMPRODUCT((T20:W20&lt;&gt;"")*(T$5:W$5+(T$5:W$5=""))),""))</f>
-        <v/>
-      </c>
+      <c r="X20" s="45" t="n"/>
       <c r="Y20" s="45" t="n"/>
-      <c r="Z20" s="45" t="n"/>
-      <c r="AA20" s="46">
-        <f>IF(COUNT(Y20:Z20)=0,"",IFERROR(SUMPRODUCT(Y20:Z20,(Y$5:Z$5+(Y$5:Z$5="")))/SUMPRODUCT((Y20:Z20&lt;&gt;"")*(Y$5:Z$5+(Y$5:Z$5=""))),""))</f>
-        <v/>
-      </c>
-      <c r="AB20" s="46">
-        <f>IFERROR(IF((ISNUMBER(S20)*(S$5+(S$5=""))+ISNUMBER(X20)*(X$5+(X$5=""))+ISNUMBER(AA20)*(AA$5+(AA$5="")))=0,"",(N(S20)*(S$5+(S$5=""))+N(X20)*(X$5+(X$5=""))+N(AA20)*(AA$5+(AA$5="")))/(ISNUMBER(S20)*(S$5+(S$5=""))+ISNUMBER(X20)*(X$5+(X$5=""))+ISNUMBER(AA20)*(AA$5+(AA$5="")))),"")</f>
-        <v/>
-      </c>
-      <c r="AC20" s="47">
-        <f>IF(AND(ISNUMBER(O20),ISNUMBER(AB20)),O20*AB20,"")</f>
-        <v/>
-      </c>
-      <c r="AD20" s="48">
-        <f>IF(ISNUMBER(AC20),(AC20-1)/24,"")</f>
-        <v/>
-      </c>
-      <c r="AE20" s="49">
-        <f>IF(ISNUMBER(AC20),COUNTIF(AC$7:AC$27,"&gt;"&amp;AC20)+1,"")</f>
-        <v/>
-      </c>
-      <c r="AF20" s="50">
-        <f>COUNT(I20,J20,K20,L20,M20,N20,P20,Q20,R20,T20,U20,V20,W20,Y20,Z20)</f>
+      <c r="Z20" s="46">
+        <f>IF(COUNT(T20:Y20)=0,"",IFERROR(SUMPRODUCT(T20:Y20,(T$5:Y$5+(T$5:Y$5="")))/SUMPRODUCT((T20:Y20&lt;&gt;"")*(T$5:Y$5+(T$5:Y$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="AA20" s="45" t="n"/>
+      <c r="AB20" s="45" t="n"/>
+      <c r="AC20" s="45" t="n"/>
+      <c r="AD20" s="46">
+        <f>IF(COUNT(AA20:AC20)=0,"",IFERROR(SUMPRODUCT(AA20:AC20,(AA$5:AC$5+(AA$5:AC$5="")))/SUMPRODUCT((AA20:AC20&lt;&gt;"")*(AA$5:AC$5+(AA$5:AC$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="AE20" s="46">
+        <f>IFERROR(IF((ISNUMBER(S20)*(S$5+(S$5=""))+ISNUMBER(Z20)*(Z$5+(Z$5=""))+ISNUMBER(AD20)*(AD$5+(AD$5="")))=0,"",(N(S20)*(S$5+(S$5=""))+N(Z20)*(Z$5+(Z$5=""))+N(AD20)*(AD$5+(AD$5="")))/(ISNUMBER(S20)*(S$5+(S$5=""))+ISNUMBER(Z20)*(Z$5+(Z$5=""))+ISNUMBER(AD20)*(AD$5+(AD$5="")))),"")</f>
+        <v/>
+      </c>
+      <c r="AF20" s="47">
+        <f>IF(AND(ISNUMBER(O20),ISNUMBER(AE20)),O20*AE20,"")</f>
+        <v/>
+      </c>
+      <c r="AG20" s="48">
+        <f>IF(ISNUMBER(AF20),(AF20-1)/24,"")</f>
+        <v/>
+      </c>
+      <c r="AH20" s="49">
+        <f>IF(ISNUMBER(AF20),COUNTIF(AF$7:AF$27,"&gt;"&amp;AF20)+1,"")</f>
+        <v/>
+      </c>
+      <c r="AI20" s="50">
+        <f>COUNT(I20,J20,K20,L20,M20,N20,P20,Q20,R20,T20,U20,V20,W20,X20,Y20,AA20,AB20,AC20)</f>
         <v/>
       </c>
     </row>
@@ -3845,34 +4088,37 @@
       <c r="U21" s="45" t="n"/>
       <c r="V21" s="45" t="n"/>
       <c r="W21" s="45" t="n"/>
-      <c r="X21" s="46">
-        <f>IF(COUNT(T21:W21)=0,"",IFERROR(SUMPRODUCT(T21:W21,(T$5:W$5+(T$5:W$5="")))/SUMPRODUCT((T21:W21&lt;&gt;"")*(T$5:W$5+(T$5:W$5=""))),""))</f>
-        <v/>
-      </c>
+      <c r="X21" s="45" t="n"/>
       <c r="Y21" s="45" t="n"/>
-      <c r="Z21" s="45" t="n"/>
-      <c r="AA21" s="46">
-        <f>IF(COUNT(Y21:Z21)=0,"",IFERROR(SUMPRODUCT(Y21:Z21,(Y$5:Z$5+(Y$5:Z$5="")))/SUMPRODUCT((Y21:Z21&lt;&gt;"")*(Y$5:Z$5+(Y$5:Z$5=""))),""))</f>
-        <v/>
-      </c>
-      <c r="AB21" s="46">
-        <f>IFERROR(IF((ISNUMBER(S21)*(S$5+(S$5=""))+ISNUMBER(X21)*(X$5+(X$5=""))+ISNUMBER(AA21)*(AA$5+(AA$5="")))=0,"",(N(S21)*(S$5+(S$5=""))+N(X21)*(X$5+(X$5=""))+N(AA21)*(AA$5+(AA$5="")))/(ISNUMBER(S21)*(S$5+(S$5=""))+ISNUMBER(X21)*(X$5+(X$5=""))+ISNUMBER(AA21)*(AA$5+(AA$5="")))),"")</f>
-        <v/>
-      </c>
-      <c r="AC21" s="47">
-        <f>IF(AND(ISNUMBER(O21),ISNUMBER(AB21)),O21*AB21,"")</f>
-        <v/>
-      </c>
-      <c r="AD21" s="48">
-        <f>IF(ISNUMBER(AC21),(AC21-1)/24,"")</f>
-        <v/>
-      </c>
-      <c r="AE21" s="49">
-        <f>IF(ISNUMBER(AC21),COUNTIF(AC$7:AC$27,"&gt;"&amp;AC21)+1,"")</f>
-        <v/>
-      </c>
-      <c r="AF21" s="50">
-        <f>COUNT(I21,J21,K21,L21,M21,N21,P21,Q21,R21,T21,U21,V21,W21,Y21,Z21)</f>
+      <c r="Z21" s="46">
+        <f>IF(COUNT(T21:Y21)=0,"",IFERROR(SUMPRODUCT(T21:Y21,(T$5:Y$5+(T$5:Y$5="")))/SUMPRODUCT((T21:Y21&lt;&gt;"")*(T$5:Y$5+(T$5:Y$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="AA21" s="45" t="n"/>
+      <c r="AB21" s="45" t="n"/>
+      <c r="AC21" s="45" t="n"/>
+      <c r="AD21" s="46">
+        <f>IF(COUNT(AA21:AC21)=0,"",IFERROR(SUMPRODUCT(AA21:AC21,(AA$5:AC$5+(AA$5:AC$5="")))/SUMPRODUCT((AA21:AC21&lt;&gt;"")*(AA$5:AC$5+(AA$5:AC$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="AE21" s="46">
+        <f>IFERROR(IF((ISNUMBER(S21)*(S$5+(S$5=""))+ISNUMBER(Z21)*(Z$5+(Z$5=""))+ISNUMBER(AD21)*(AD$5+(AD$5="")))=0,"",(N(S21)*(S$5+(S$5=""))+N(Z21)*(Z$5+(Z$5=""))+N(AD21)*(AD$5+(AD$5="")))/(ISNUMBER(S21)*(S$5+(S$5=""))+ISNUMBER(Z21)*(Z$5+(Z$5=""))+ISNUMBER(AD21)*(AD$5+(AD$5="")))),"")</f>
+        <v/>
+      </c>
+      <c r="AF21" s="47">
+        <f>IF(AND(ISNUMBER(O21),ISNUMBER(AE21)),O21*AE21,"")</f>
+        <v/>
+      </c>
+      <c r="AG21" s="48">
+        <f>IF(ISNUMBER(AF21),(AF21-1)/24,"")</f>
+        <v/>
+      </c>
+      <c r="AH21" s="49">
+        <f>IF(ISNUMBER(AF21),COUNTIF(AF$7:AF$27,"&gt;"&amp;AF21)+1,"")</f>
+        <v/>
+      </c>
+      <c r="AI21" s="50">
+        <f>COUNT(I21,J21,K21,L21,M21,N21,P21,Q21,R21,T21,U21,V21,W21,X21,Y21,AA21,AB21,AC21)</f>
         <v/>
       </c>
     </row>
@@ -3932,34 +4178,37 @@
       <c r="U22" s="45" t="n"/>
       <c r="V22" s="45" t="n"/>
       <c r="W22" s="45" t="n"/>
-      <c r="X22" s="46">
-        <f>IF(COUNT(T22:W22)=0,"",IFERROR(SUMPRODUCT(T22:W22,(T$5:W$5+(T$5:W$5="")))/SUMPRODUCT((T22:W22&lt;&gt;"")*(T$5:W$5+(T$5:W$5=""))),""))</f>
-        <v/>
-      </c>
+      <c r="X22" s="45" t="n"/>
       <c r="Y22" s="45" t="n"/>
-      <c r="Z22" s="45" t="n"/>
-      <c r="AA22" s="46">
-        <f>IF(COUNT(Y22:Z22)=0,"",IFERROR(SUMPRODUCT(Y22:Z22,(Y$5:Z$5+(Y$5:Z$5="")))/SUMPRODUCT((Y22:Z22&lt;&gt;"")*(Y$5:Z$5+(Y$5:Z$5=""))),""))</f>
-        <v/>
-      </c>
-      <c r="AB22" s="46">
-        <f>IFERROR(IF((ISNUMBER(S22)*(S$5+(S$5=""))+ISNUMBER(X22)*(X$5+(X$5=""))+ISNUMBER(AA22)*(AA$5+(AA$5="")))=0,"",(N(S22)*(S$5+(S$5=""))+N(X22)*(X$5+(X$5=""))+N(AA22)*(AA$5+(AA$5="")))/(ISNUMBER(S22)*(S$5+(S$5=""))+ISNUMBER(X22)*(X$5+(X$5=""))+ISNUMBER(AA22)*(AA$5+(AA$5="")))),"")</f>
-        <v/>
-      </c>
-      <c r="AC22" s="47">
-        <f>IF(AND(ISNUMBER(O22),ISNUMBER(AB22)),O22*AB22,"")</f>
-        <v/>
-      </c>
-      <c r="AD22" s="48">
-        <f>IF(ISNUMBER(AC22),(AC22-1)/24,"")</f>
-        <v/>
-      </c>
-      <c r="AE22" s="49">
-        <f>IF(ISNUMBER(AC22),COUNTIF(AC$7:AC$27,"&gt;"&amp;AC22)+1,"")</f>
-        <v/>
-      </c>
-      <c r="AF22" s="50">
-        <f>COUNT(I22,J22,K22,L22,M22,N22,P22,Q22,R22,T22,U22,V22,W22,Y22,Z22)</f>
+      <c r="Z22" s="46">
+        <f>IF(COUNT(T22:Y22)=0,"",IFERROR(SUMPRODUCT(T22:Y22,(T$5:Y$5+(T$5:Y$5="")))/SUMPRODUCT((T22:Y22&lt;&gt;"")*(T$5:Y$5+(T$5:Y$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="AA22" s="45" t="n"/>
+      <c r="AB22" s="45" t="n"/>
+      <c r="AC22" s="45" t="n"/>
+      <c r="AD22" s="46">
+        <f>IF(COUNT(AA22:AC22)=0,"",IFERROR(SUMPRODUCT(AA22:AC22,(AA$5:AC$5+(AA$5:AC$5="")))/SUMPRODUCT((AA22:AC22&lt;&gt;"")*(AA$5:AC$5+(AA$5:AC$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="AE22" s="46">
+        <f>IFERROR(IF((ISNUMBER(S22)*(S$5+(S$5=""))+ISNUMBER(Z22)*(Z$5+(Z$5=""))+ISNUMBER(AD22)*(AD$5+(AD$5="")))=0,"",(N(S22)*(S$5+(S$5=""))+N(Z22)*(Z$5+(Z$5=""))+N(AD22)*(AD$5+(AD$5="")))/(ISNUMBER(S22)*(S$5+(S$5=""))+ISNUMBER(Z22)*(Z$5+(Z$5=""))+ISNUMBER(AD22)*(AD$5+(AD$5="")))),"")</f>
+        <v/>
+      </c>
+      <c r="AF22" s="47">
+        <f>IF(AND(ISNUMBER(O22),ISNUMBER(AE22)),O22*AE22,"")</f>
+        <v/>
+      </c>
+      <c r="AG22" s="48">
+        <f>IF(ISNUMBER(AF22),(AF22-1)/24,"")</f>
+        <v/>
+      </c>
+      <c r="AH22" s="49">
+        <f>IF(ISNUMBER(AF22),COUNTIF(AF$7:AF$27,"&gt;"&amp;AF22)+1,"")</f>
+        <v/>
+      </c>
+      <c r="AI22" s="50">
+        <f>COUNT(I22,J22,K22,L22,M22,N22,P22,Q22,R22,T22,U22,V22,W22,X22,Y22,AA22,AB22,AC22)</f>
         <v/>
       </c>
     </row>
@@ -4019,34 +4268,37 @@
       <c r="U23" s="45" t="n"/>
       <c r="V23" s="45" t="n"/>
       <c r="W23" s="45" t="n"/>
-      <c r="X23" s="46">
-        <f>IF(COUNT(T23:W23)=0,"",IFERROR(SUMPRODUCT(T23:W23,(T$5:W$5+(T$5:W$5="")))/SUMPRODUCT((T23:W23&lt;&gt;"")*(T$5:W$5+(T$5:W$5=""))),""))</f>
-        <v/>
-      </c>
+      <c r="X23" s="45" t="n"/>
       <c r="Y23" s="45" t="n"/>
-      <c r="Z23" s="45" t="n"/>
-      <c r="AA23" s="46">
-        <f>IF(COUNT(Y23:Z23)=0,"",IFERROR(SUMPRODUCT(Y23:Z23,(Y$5:Z$5+(Y$5:Z$5="")))/SUMPRODUCT((Y23:Z23&lt;&gt;"")*(Y$5:Z$5+(Y$5:Z$5=""))),""))</f>
-        <v/>
-      </c>
-      <c r="AB23" s="46">
-        <f>IFERROR(IF((ISNUMBER(S23)*(S$5+(S$5=""))+ISNUMBER(X23)*(X$5+(X$5=""))+ISNUMBER(AA23)*(AA$5+(AA$5="")))=0,"",(N(S23)*(S$5+(S$5=""))+N(X23)*(X$5+(X$5=""))+N(AA23)*(AA$5+(AA$5="")))/(ISNUMBER(S23)*(S$5+(S$5=""))+ISNUMBER(X23)*(X$5+(X$5=""))+ISNUMBER(AA23)*(AA$5+(AA$5="")))),"")</f>
-        <v/>
-      </c>
-      <c r="AC23" s="47">
-        <f>IF(AND(ISNUMBER(O23),ISNUMBER(AB23)),O23*AB23,"")</f>
-        <v/>
-      </c>
-      <c r="AD23" s="48">
-        <f>IF(ISNUMBER(AC23),(AC23-1)/24,"")</f>
-        <v/>
-      </c>
-      <c r="AE23" s="49">
-        <f>IF(ISNUMBER(AC23),COUNTIF(AC$7:AC$27,"&gt;"&amp;AC23)+1,"")</f>
-        <v/>
-      </c>
-      <c r="AF23" s="50">
-        <f>COUNT(I23,J23,K23,L23,M23,N23,P23,Q23,R23,T23,U23,V23,W23,Y23,Z23)</f>
+      <c r="Z23" s="46">
+        <f>IF(COUNT(T23:Y23)=0,"",IFERROR(SUMPRODUCT(T23:Y23,(T$5:Y$5+(T$5:Y$5="")))/SUMPRODUCT((T23:Y23&lt;&gt;"")*(T$5:Y$5+(T$5:Y$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="AA23" s="45" t="n"/>
+      <c r="AB23" s="45" t="n"/>
+      <c r="AC23" s="45" t="n"/>
+      <c r="AD23" s="46">
+        <f>IF(COUNT(AA23:AC23)=0,"",IFERROR(SUMPRODUCT(AA23:AC23,(AA$5:AC$5+(AA$5:AC$5="")))/SUMPRODUCT((AA23:AC23&lt;&gt;"")*(AA$5:AC$5+(AA$5:AC$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="AE23" s="46">
+        <f>IFERROR(IF((ISNUMBER(S23)*(S$5+(S$5=""))+ISNUMBER(Z23)*(Z$5+(Z$5=""))+ISNUMBER(AD23)*(AD$5+(AD$5="")))=0,"",(N(S23)*(S$5+(S$5=""))+N(Z23)*(Z$5+(Z$5=""))+N(AD23)*(AD$5+(AD$5="")))/(ISNUMBER(S23)*(S$5+(S$5=""))+ISNUMBER(Z23)*(Z$5+(Z$5=""))+ISNUMBER(AD23)*(AD$5+(AD$5="")))),"")</f>
+        <v/>
+      </c>
+      <c r="AF23" s="47">
+        <f>IF(AND(ISNUMBER(O23),ISNUMBER(AE23)),O23*AE23,"")</f>
+        <v/>
+      </c>
+      <c r="AG23" s="48">
+        <f>IF(ISNUMBER(AF23),(AF23-1)/24,"")</f>
+        <v/>
+      </c>
+      <c r="AH23" s="49">
+        <f>IF(ISNUMBER(AF23),COUNTIF(AF$7:AF$27,"&gt;"&amp;AF23)+1,"")</f>
+        <v/>
+      </c>
+      <c r="AI23" s="50">
+        <f>COUNT(I23,J23,K23,L23,M23,N23,P23,Q23,R23,T23,U23,V23,W23,X23,Y23,AA23,AB23,AC23)</f>
         <v/>
       </c>
     </row>
@@ -4106,34 +4358,37 @@
       <c r="U24" s="45" t="n"/>
       <c r="V24" s="45" t="n"/>
       <c r="W24" s="45" t="n"/>
-      <c r="X24" s="46">
-        <f>IF(COUNT(T24:W24)=0,"",IFERROR(SUMPRODUCT(T24:W24,(T$5:W$5+(T$5:W$5="")))/SUMPRODUCT((T24:W24&lt;&gt;"")*(T$5:W$5+(T$5:W$5=""))),""))</f>
-        <v/>
-      </c>
+      <c r="X24" s="45" t="n"/>
       <c r="Y24" s="45" t="n"/>
-      <c r="Z24" s="45" t="n"/>
-      <c r="AA24" s="46">
-        <f>IF(COUNT(Y24:Z24)=0,"",IFERROR(SUMPRODUCT(Y24:Z24,(Y$5:Z$5+(Y$5:Z$5="")))/SUMPRODUCT((Y24:Z24&lt;&gt;"")*(Y$5:Z$5+(Y$5:Z$5=""))),""))</f>
-        <v/>
-      </c>
-      <c r="AB24" s="46">
-        <f>IFERROR(IF((ISNUMBER(S24)*(S$5+(S$5=""))+ISNUMBER(X24)*(X$5+(X$5=""))+ISNUMBER(AA24)*(AA$5+(AA$5="")))=0,"",(N(S24)*(S$5+(S$5=""))+N(X24)*(X$5+(X$5=""))+N(AA24)*(AA$5+(AA$5="")))/(ISNUMBER(S24)*(S$5+(S$5=""))+ISNUMBER(X24)*(X$5+(X$5=""))+ISNUMBER(AA24)*(AA$5+(AA$5="")))),"")</f>
-        <v/>
-      </c>
-      <c r="AC24" s="47">
-        <f>IF(AND(ISNUMBER(O24),ISNUMBER(AB24)),O24*AB24,"")</f>
-        <v/>
-      </c>
-      <c r="AD24" s="48">
-        <f>IF(ISNUMBER(AC24),(AC24-1)/24,"")</f>
-        <v/>
-      </c>
-      <c r="AE24" s="49">
-        <f>IF(ISNUMBER(AC24),COUNTIF(AC$7:AC$27,"&gt;"&amp;AC24)+1,"")</f>
-        <v/>
-      </c>
-      <c r="AF24" s="50">
-        <f>COUNT(I24,J24,K24,L24,M24,N24,P24,Q24,R24,T24,U24,V24,W24,Y24,Z24)</f>
+      <c r="Z24" s="46">
+        <f>IF(COUNT(T24:Y24)=0,"",IFERROR(SUMPRODUCT(T24:Y24,(T$5:Y$5+(T$5:Y$5="")))/SUMPRODUCT((T24:Y24&lt;&gt;"")*(T$5:Y$5+(T$5:Y$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="AA24" s="45" t="n"/>
+      <c r="AB24" s="45" t="n"/>
+      <c r="AC24" s="45" t="n"/>
+      <c r="AD24" s="46">
+        <f>IF(COUNT(AA24:AC24)=0,"",IFERROR(SUMPRODUCT(AA24:AC24,(AA$5:AC$5+(AA$5:AC$5="")))/SUMPRODUCT((AA24:AC24&lt;&gt;"")*(AA$5:AC$5+(AA$5:AC$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="AE24" s="46">
+        <f>IFERROR(IF((ISNUMBER(S24)*(S$5+(S$5=""))+ISNUMBER(Z24)*(Z$5+(Z$5=""))+ISNUMBER(AD24)*(AD$5+(AD$5="")))=0,"",(N(S24)*(S$5+(S$5=""))+N(Z24)*(Z$5+(Z$5=""))+N(AD24)*(AD$5+(AD$5="")))/(ISNUMBER(S24)*(S$5+(S$5=""))+ISNUMBER(Z24)*(Z$5+(Z$5=""))+ISNUMBER(AD24)*(AD$5+(AD$5="")))),"")</f>
+        <v/>
+      </c>
+      <c r="AF24" s="47">
+        <f>IF(AND(ISNUMBER(O24),ISNUMBER(AE24)),O24*AE24,"")</f>
+        <v/>
+      </c>
+      <c r="AG24" s="48">
+        <f>IF(ISNUMBER(AF24),(AF24-1)/24,"")</f>
+        <v/>
+      </c>
+      <c r="AH24" s="49">
+        <f>IF(ISNUMBER(AF24),COUNTIF(AF$7:AF$27,"&gt;"&amp;AF24)+1,"")</f>
+        <v/>
+      </c>
+      <c r="AI24" s="50">
+        <f>COUNT(I24,J24,K24,L24,M24,N24,P24,Q24,R24,T24,U24,V24,W24,X24,Y24,AA24,AB24,AC24)</f>
         <v/>
       </c>
     </row>
@@ -4193,34 +4448,37 @@
       <c r="U25" s="45" t="n"/>
       <c r="V25" s="45" t="n"/>
       <c r="W25" s="45" t="n"/>
-      <c r="X25" s="46">
-        <f>IF(COUNT(T25:W25)=0,"",IFERROR(SUMPRODUCT(T25:W25,(T$5:W$5+(T$5:W$5="")))/SUMPRODUCT((T25:W25&lt;&gt;"")*(T$5:W$5+(T$5:W$5=""))),""))</f>
-        <v/>
-      </c>
+      <c r="X25" s="45" t="n"/>
       <c r="Y25" s="45" t="n"/>
-      <c r="Z25" s="45" t="n"/>
-      <c r="AA25" s="46">
-        <f>IF(COUNT(Y25:Z25)=0,"",IFERROR(SUMPRODUCT(Y25:Z25,(Y$5:Z$5+(Y$5:Z$5="")))/SUMPRODUCT((Y25:Z25&lt;&gt;"")*(Y$5:Z$5+(Y$5:Z$5=""))),""))</f>
-        <v/>
-      </c>
-      <c r="AB25" s="46">
-        <f>IFERROR(IF((ISNUMBER(S25)*(S$5+(S$5=""))+ISNUMBER(X25)*(X$5+(X$5=""))+ISNUMBER(AA25)*(AA$5+(AA$5="")))=0,"",(N(S25)*(S$5+(S$5=""))+N(X25)*(X$5+(X$5=""))+N(AA25)*(AA$5+(AA$5="")))/(ISNUMBER(S25)*(S$5+(S$5=""))+ISNUMBER(X25)*(X$5+(X$5=""))+ISNUMBER(AA25)*(AA$5+(AA$5="")))),"")</f>
-        <v/>
-      </c>
-      <c r="AC25" s="47">
-        <f>IF(AND(ISNUMBER(O25),ISNUMBER(AB25)),O25*AB25,"")</f>
-        <v/>
-      </c>
-      <c r="AD25" s="48">
-        <f>IF(ISNUMBER(AC25),(AC25-1)/24,"")</f>
-        <v/>
-      </c>
-      <c r="AE25" s="49">
-        <f>IF(ISNUMBER(AC25),COUNTIF(AC$7:AC$27,"&gt;"&amp;AC25)+1,"")</f>
-        <v/>
-      </c>
-      <c r="AF25" s="50">
-        <f>COUNT(I25,J25,K25,L25,M25,N25,P25,Q25,R25,T25,U25,V25,W25,Y25,Z25)</f>
+      <c r="Z25" s="46">
+        <f>IF(COUNT(T25:Y25)=0,"",IFERROR(SUMPRODUCT(T25:Y25,(T$5:Y$5+(T$5:Y$5="")))/SUMPRODUCT((T25:Y25&lt;&gt;"")*(T$5:Y$5+(T$5:Y$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="AA25" s="45" t="n"/>
+      <c r="AB25" s="45" t="n"/>
+      <c r="AC25" s="45" t="n"/>
+      <c r="AD25" s="46">
+        <f>IF(COUNT(AA25:AC25)=0,"",IFERROR(SUMPRODUCT(AA25:AC25,(AA$5:AC$5+(AA$5:AC$5="")))/SUMPRODUCT((AA25:AC25&lt;&gt;"")*(AA$5:AC$5+(AA$5:AC$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="AE25" s="46">
+        <f>IFERROR(IF((ISNUMBER(S25)*(S$5+(S$5=""))+ISNUMBER(Z25)*(Z$5+(Z$5=""))+ISNUMBER(AD25)*(AD$5+(AD$5="")))=0,"",(N(S25)*(S$5+(S$5=""))+N(Z25)*(Z$5+(Z$5=""))+N(AD25)*(AD$5+(AD$5="")))/(ISNUMBER(S25)*(S$5+(S$5=""))+ISNUMBER(Z25)*(Z$5+(Z$5=""))+ISNUMBER(AD25)*(AD$5+(AD$5="")))),"")</f>
+        <v/>
+      </c>
+      <c r="AF25" s="47">
+        <f>IF(AND(ISNUMBER(O25),ISNUMBER(AE25)),O25*AE25,"")</f>
+        <v/>
+      </c>
+      <c r="AG25" s="48">
+        <f>IF(ISNUMBER(AF25),(AF25-1)/24,"")</f>
+        <v/>
+      </c>
+      <c r="AH25" s="49">
+        <f>IF(ISNUMBER(AF25),COUNTIF(AF$7:AF$27,"&gt;"&amp;AF25)+1,"")</f>
+        <v/>
+      </c>
+      <c r="AI25" s="50">
+        <f>COUNT(I25,J25,K25,L25,M25,N25,P25,Q25,R25,T25,U25,V25,W25,X25,Y25,AA25,AB25,AC25)</f>
         <v/>
       </c>
     </row>
@@ -4276,34 +4534,37 @@
       <c r="U26" s="45" t="n"/>
       <c r="V26" s="45" t="n"/>
       <c r="W26" s="45" t="n"/>
-      <c r="X26" s="46">
-        <f>IF(COUNT(T26:W26)=0,"",IFERROR(SUMPRODUCT(T26:W26,(T$5:W$5+(T$5:W$5="")))/SUMPRODUCT((T26:W26&lt;&gt;"")*(T$5:W$5+(T$5:W$5=""))),""))</f>
-        <v/>
-      </c>
+      <c r="X26" s="45" t="n"/>
       <c r="Y26" s="45" t="n"/>
-      <c r="Z26" s="45" t="n"/>
-      <c r="AA26" s="46">
-        <f>IF(COUNT(Y26:Z26)=0,"",IFERROR(SUMPRODUCT(Y26:Z26,(Y$5:Z$5+(Y$5:Z$5="")))/SUMPRODUCT((Y26:Z26&lt;&gt;"")*(Y$5:Z$5+(Y$5:Z$5=""))),""))</f>
-        <v/>
-      </c>
-      <c r="AB26" s="46">
-        <f>IFERROR(IF((ISNUMBER(S26)*(S$5+(S$5=""))+ISNUMBER(X26)*(X$5+(X$5=""))+ISNUMBER(AA26)*(AA$5+(AA$5="")))=0,"",(N(S26)*(S$5+(S$5=""))+N(X26)*(X$5+(X$5=""))+N(AA26)*(AA$5+(AA$5="")))/(ISNUMBER(S26)*(S$5+(S$5=""))+ISNUMBER(X26)*(X$5+(X$5=""))+ISNUMBER(AA26)*(AA$5+(AA$5="")))),"")</f>
-        <v/>
-      </c>
-      <c r="AC26" s="47">
-        <f>IF(AND(ISNUMBER(O26),ISNUMBER(AB26)),O26*AB26,"")</f>
-        <v/>
-      </c>
-      <c r="AD26" s="48">
-        <f>IF(ISNUMBER(AC26),(AC26-1)/24,"")</f>
-        <v/>
-      </c>
-      <c r="AE26" s="49">
-        <f>IF(ISNUMBER(AC26),COUNTIF(AC$7:AC$27,"&gt;"&amp;AC26)+1,"")</f>
-        <v/>
-      </c>
-      <c r="AF26" s="50">
-        <f>COUNT(I26,J26,K26,L26,M26,N26,P26,Q26,R26,T26,U26,V26,W26,Y26,Z26)</f>
+      <c r="Z26" s="46">
+        <f>IF(COUNT(T26:Y26)=0,"",IFERROR(SUMPRODUCT(T26:Y26,(T$5:Y$5+(T$5:Y$5="")))/SUMPRODUCT((T26:Y26&lt;&gt;"")*(T$5:Y$5+(T$5:Y$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="AA26" s="45" t="n"/>
+      <c r="AB26" s="45" t="n"/>
+      <c r="AC26" s="45" t="n"/>
+      <c r="AD26" s="46">
+        <f>IF(COUNT(AA26:AC26)=0,"",IFERROR(SUMPRODUCT(AA26:AC26,(AA$5:AC$5+(AA$5:AC$5="")))/SUMPRODUCT((AA26:AC26&lt;&gt;"")*(AA$5:AC$5+(AA$5:AC$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="AE26" s="46">
+        <f>IFERROR(IF((ISNUMBER(S26)*(S$5+(S$5=""))+ISNUMBER(Z26)*(Z$5+(Z$5=""))+ISNUMBER(AD26)*(AD$5+(AD$5="")))=0,"",(N(S26)*(S$5+(S$5=""))+N(Z26)*(Z$5+(Z$5=""))+N(AD26)*(AD$5+(AD$5="")))/(ISNUMBER(S26)*(S$5+(S$5=""))+ISNUMBER(Z26)*(Z$5+(Z$5=""))+ISNUMBER(AD26)*(AD$5+(AD$5="")))),"")</f>
+        <v/>
+      </c>
+      <c r="AF26" s="47">
+        <f>IF(AND(ISNUMBER(O26),ISNUMBER(AE26)),O26*AE26,"")</f>
+        <v/>
+      </c>
+      <c r="AG26" s="48">
+        <f>IF(ISNUMBER(AF26),(AF26-1)/24,"")</f>
+        <v/>
+      </c>
+      <c r="AH26" s="49">
+        <f>IF(ISNUMBER(AF26),COUNTIF(AF$7:AF$27,"&gt;"&amp;AF26)+1,"")</f>
+        <v/>
+      </c>
+      <c r="AI26" s="50">
+        <f>COUNT(I26,J26,K26,L26,M26,N26,P26,Q26,R26,T26,U26,V26,W26,X26,Y26,AA26,AB26,AC26)</f>
         <v/>
       </c>
     </row>
@@ -4363,34 +4624,37 @@
       <c r="U27" s="45" t="n"/>
       <c r="V27" s="45" t="n"/>
       <c r="W27" s="45" t="n"/>
-      <c r="X27" s="46">
-        <f>IF(COUNT(T27:W27)=0,"",IFERROR(SUMPRODUCT(T27:W27,(T$5:W$5+(T$5:W$5="")))/SUMPRODUCT((T27:W27&lt;&gt;"")*(T$5:W$5+(T$5:W$5=""))),""))</f>
-        <v/>
-      </c>
+      <c r="X27" s="45" t="n"/>
       <c r="Y27" s="45" t="n"/>
-      <c r="Z27" s="45" t="n"/>
-      <c r="AA27" s="46">
-        <f>IF(COUNT(Y27:Z27)=0,"",IFERROR(SUMPRODUCT(Y27:Z27,(Y$5:Z$5+(Y$5:Z$5="")))/SUMPRODUCT((Y27:Z27&lt;&gt;"")*(Y$5:Z$5+(Y$5:Z$5=""))),""))</f>
-        <v/>
-      </c>
-      <c r="AB27" s="46">
-        <f>IFERROR(IF((ISNUMBER(S27)*(S$5+(S$5=""))+ISNUMBER(X27)*(X$5+(X$5=""))+ISNUMBER(AA27)*(AA$5+(AA$5="")))=0,"",(N(S27)*(S$5+(S$5=""))+N(X27)*(X$5+(X$5=""))+N(AA27)*(AA$5+(AA$5="")))/(ISNUMBER(S27)*(S$5+(S$5=""))+ISNUMBER(X27)*(X$5+(X$5=""))+ISNUMBER(AA27)*(AA$5+(AA$5="")))),"")</f>
-        <v/>
-      </c>
-      <c r="AC27" s="47">
-        <f>IF(AND(ISNUMBER(O27),ISNUMBER(AB27)),O27*AB27,"")</f>
-        <v/>
-      </c>
-      <c r="AD27" s="48">
-        <f>IF(ISNUMBER(AC27),(AC27-1)/24,"")</f>
-        <v/>
-      </c>
-      <c r="AE27" s="49">
-        <f>IF(ISNUMBER(AC27),COUNTIF(AC$7:AC$27,"&gt;"&amp;AC27)+1,"")</f>
-        <v/>
-      </c>
-      <c r="AF27" s="50">
-        <f>COUNT(I27,J27,K27,L27,M27,N27,P27,Q27,R27,T27,U27,V27,W27,Y27,Z27)</f>
+      <c r="Z27" s="46">
+        <f>IF(COUNT(T27:Y27)=0,"",IFERROR(SUMPRODUCT(T27:Y27,(T$5:Y$5+(T$5:Y$5="")))/SUMPRODUCT((T27:Y27&lt;&gt;"")*(T$5:Y$5+(T$5:Y$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="AA27" s="45" t="n"/>
+      <c r="AB27" s="45" t="n"/>
+      <c r="AC27" s="45" t="n"/>
+      <c r="AD27" s="46">
+        <f>IF(COUNT(AA27:AC27)=0,"",IFERROR(SUMPRODUCT(AA27:AC27,(AA$5:AC$5+(AA$5:AC$5="")))/SUMPRODUCT((AA27:AC27&lt;&gt;"")*(AA$5:AC$5+(AA$5:AC$5=""))),""))</f>
+        <v/>
+      </c>
+      <c r="AE27" s="46">
+        <f>IFERROR(IF((ISNUMBER(S27)*(S$5+(S$5=""))+ISNUMBER(Z27)*(Z$5+(Z$5=""))+ISNUMBER(AD27)*(AD$5+(AD$5="")))=0,"",(N(S27)*(S$5+(S$5=""))+N(Z27)*(Z$5+(Z$5=""))+N(AD27)*(AD$5+(AD$5="")))/(ISNUMBER(S27)*(S$5+(S$5=""))+ISNUMBER(Z27)*(Z$5+(Z$5=""))+ISNUMBER(AD27)*(AD$5+(AD$5="")))),"")</f>
+        <v/>
+      </c>
+      <c r="AF27" s="47">
+        <f>IF(AND(ISNUMBER(O27),ISNUMBER(AE27)),O27*AE27,"")</f>
+        <v/>
+      </c>
+      <c r="AG27" s="48">
+        <f>IF(ISNUMBER(AF27),(AF27-1)/24,"")</f>
+        <v/>
+      </c>
+      <c r="AH27" s="49">
+        <f>IF(ISNUMBER(AF27),COUNTIF(AF$7:AF$27,"&gt;"&amp;AF27)+1,"")</f>
+        <v/>
+      </c>
+      <c r="AI27" s="50">
+        <f>COUNT(I27,J27,K27,L27,M27,N27,P27,Q27,R27,T27,U27,V27,W27,X27,Y27,AA27,AB27,AC27)</f>
         <v/>
       </c>
     </row>
@@ -4438,13 +4702,13 @@
     </row>
   </sheetData>
   <mergeCells count="5">
-    <mergeCell ref="AB4:AF4"/>
+    <mergeCell ref="AE4:AI4"/>
+    <mergeCell ref="AA4:AD4"/>
+    <mergeCell ref="T4:Z4"/>
     <mergeCell ref="I4:O4"/>
     <mergeCell ref="P4:S4"/>
-    <mergeCell ref="Y4:AA4"/>
-    <mergeCell ref="T4:X4"/>
   </mergeCells>
-  <conditionalFormatting sqref="AD7:AD27">
+  <conditionalFormatting sqref="AG7:AG27">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="num" val="0"/>
@@ -4457,11 +4721,11 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="I7:I27 J7:J27 K7:K27 L7:L27 M7:M27 N7:N27 P7:P27 Q7:Q27 R7:R27 T7:T27 U7:U27 V7:V27 W7:W27 Y7:Y27 Z7:Z27" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Nota inválida" error="Use um número inteiro de 1 a 5 (5 = mais crítico)." type="whole" operator="between">
+    <dataValidation sqref="I7:I27 J7:J27 K7:K27 L7:L27 M7:M27 N7:N27 P7:P27 Q7:Q27 R7:R27 T7:T27 U7:U27 V7:V27 W7:W27 X7:X27 Y7:Y27 AA7:AA27 AB7:AB27 AC7:AC27" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Nota inválida" error="Use um número inteiro de 1 a 5 (5 = mais crítico)." type="whole" operator="between">
       <formula1>1</formula1>
       <formula2>5</formula2>
     </dataValidation>
-    <dataValidation sqref="I5 J5 K5 L5 M5 N5 P5 Q5 R5 S5 T5 U5 V5 W5 X5 Y5 Z5 AA5" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Peso deve ser um número maior ou igual a zero." type="decimal" operator="greaterThanOrEqual">
+    <dataValidation sqref="I5 J5 K5 L5 M5 N5 P5 Q5 R5 S5 T5 U5 V5 W5 X5 Y5 Z5 AA5 AB5 AC5 AD5" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Peso deve ser um número maior ou igual a zero." type="decimal" operator="greaterThanOrEqual">
       <formula1>0</formula1>
     </dataValidation>
   </dataValidations>
@@ -4476,7 +4740,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D67"/>
+  <dimension ref="A1:D68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -4622,12 +4886,12 @@
       </c>
       <c r="C9" s="43" t="inlineStr">
         <is>
-          <t>Quem e o que está no caminho da água dentro do círculo de 300 m: moradores, escolas, unidades de saúde, comércio.</t>
+          <t>Quem e o que está no caminho da água dentro do círculo de 300 m: moradores, equipamentos públicos, comércio. O que está no círculo conta só aqui, não no Impacto.</t>
         </is>
       </c>
       <c r="D9" s="43" t="inlineStr">
         <is>
-          <t>Um ponto com muitas escolas por perto tem Equipamentos sensíveis (E2) alto.</t>
+          <t>Um ponto com muitas escolas por perto tem Equipamentos públicos (E2) alto.</t>
         </is>
       </c>
     </row>
@@ -4644,7 +4908,7 @@
       </c>
       <c r="C10" s="43" t="inlineStr">
         <is>
-          <t>Quanto quem está ali tem dificuldade de lidar com o alagamento: idosos e crianças, favelas e comunidades, moradia térrea.</t>
+          <t>Quanto quem está ali tem dificuldade de lidar com o alagamento: idosos e crianças, ZEIS, favelas e comunidades, moradia térrea.</t>
         </is>
       </c>
       <c r="D10" s="43" t="inlineStr">
@@ -4666,12 +4930,12 @@
       </c>
       <c r="C11" s="43" t="inlineStr">
         <is>
-          <t>Consequência que vai além do local: mobilidade da cidade e saúde pública (esgoto).</t>
+          <t>Consequência que vai além do local: trânsito nas vias principais, saúde pública (esgoto) e isolamento.</t>
         </is>
       </c>
       <c r="D11" s="43" t="inlineStr">
         <is>
-          <t>Alagamento numa avenida arterial com ônibus tem Mobilidade (I1) alta.</t>
+          <t>Alagamento numa avenida arterial com ônibus tem Interrupção do trânsito (I1) alta.</t>
         </is>
       </c>
     </row>
@@ -4815,17 +5079,17 @@
       </c>
       <c r="B18" s="55" t="inlineStr">
         <is>
-          <t>Tratabilidade</t>
+          <t>Contexto no painel</t>
         </is>
       </c>
       <c r="C18" s="43" t="inlineStr">
         <is>
-          <t>Se é fácil agir no ponto (governança, natureza da causa, obra ou orçamento em andamento). Fica FORA do risco. 5 = mais fácil.</t>
+          <t>Informação mostrada no painel sem entrar na nota, porque varia pouco entre os 21 pontos ou não tem dado por ponto.</t>
         </is>
       </c>
       <c r="D18" s="43" t="inlineStr">
         <is>
-          <t>Ponto com dono definido e causa de manutenção tem tratabilidade alta.</t>
+          <t>Intensidade das chuvas (documento da equipe).</t>
         </is>
       </c>
     </row>
@@ -4837,17 +5101,17 @@
       </c>
       <c r="B19" s="55" t="inlineStr">
         <is>
-          <t>Matriz risco × tratabilidade</t>
+          <t>Tratabilidade</t>
         </is>
       </c>
       <c r="C19" s="43" t="inlineStr">
         <is>
-          <t>Cruza o risco (corte em 9) com a tratabilidade (corte em 3) e coloca cada ponto num de 4 quadrantes.</t>
+          <t>Se é fácil agir no ponto (governança, natureza da causa, obra ou orçamento em andamento). Fica FORA do risco. 5 = mais fácil.</t>
         </is>
       </c>
       <c r="D19" s="43" t="inlineStr">
         <is>
-          <t>Risco 12 e tratabilidade 4 = quadrante Agir já.</t>
+          <t>Ponto com dono definido e causa de manutenção tem tratabilidade alta.</t>
         </is>
       </c>
     </row>
@@ -4859,15 +5123,19 @@
       </c>
       <c r="B20" s="55" t="inlineStr">
         <is>
-          <t>Agir já / Estruturar / Oportunidade / Monitorar</t>
+          <t>Matriz risco × tratabilidade</t>
         </is>
       </c>
       <c r="C20" s="43" t="inlineStr">
         <is>
-          <t>Quadrantes da matriz. Agir já: risco alto, fácil de agir. Estruturar: risco alto, difícil (exige articulação). Oportunidade: risco baixo, fácil. Monitorar: risco baixo, difícil.</t>
-        </is>
-      </c>
-      <c r="D20" s="43" t="inlineStr"/>
+          <t>Cruza o risco (corte em 9) com a tratabilidade (corte em 3) e coloca cada ponto num de 4 quadrantes.</t>
+        </is>
+      </c>
+      <c r="D20" s="43" t="inlineStr">
+        <is>
+          <t>Risco 12 e tratabilidade 4 = quadrante Agir já.</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="54" t="inlineStr">
@@ -4877,19 +5145,15 @@
       </c>
       <c r="B21" s="55" t="inlineStr">
         <is>
-          <t>Diagnóstico de causa</t>
+          <t>Agir já / Estruturar / Oportunidade / Monitorar</t>
         </is>
       </c>
       <c r="C21" s="43" t="inlineStr">
         <is>
-          <t>Por que o ponto alaga (drenagem obstruída, subdimensionada, maré, esgoto). Fica fora do risco e indica qual órgão age.</t>
-        </is>
-      </c>
-      <c r="D21" s="43" t="inlineStr">
-        <is>
-          <t>Galeria assoreada → EMLURB (manutenção).</t>
-        </is>
-      </c>
+          <t>Quadrantes da matriz. Agir já: risco alto, fácil de agir. Estruturar: risco alto, difícil (exige articulação). Oportunidade: risco baixo, fácil. Monitorar: risco baixo, difícil.</t>
+        </is>
+      </c>
+      <c r="D21" s="43" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="54" t="inlineStr">
@@ -4899,39 +5163,39 @@
       </c>
       <c r="B22" s="55" t="inlineStr">
         <is>
+          <t>Diagnóstico de causa</t>
+        </is>
+      </c>
+      <c r="C22" s="43" t="inlineStr">
+        <is>
+          <t>Por que o ponto alaga (drenagem obstruída, subdimensionada, maré, esgoto). Fica fora do risco e indica qual órgão age.</t>
+        </is>
+      </c>
+      <c r="D22" s="43" t="inlineStr">
+        <is>
+          <t>Galeria assoreada → EMLURB (manutenção).</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="54" t="inlineStr">
+        <is>
+          <t>Modelo de risco</t>
+        </is>
+      </c>
+      <c r="B23" s="55" t="inlineStr">
+        <is>
           <t>Análise de sensibilidade</t>
         </is>
       </c>
-      <c r="C22" s="43" t="inlineStr">
+      <c r="C23" s="43" t="inlineStr">
         <is>
           <t>Recalcular o ranking com outros pesos (ex.: pesos iguais) para ver se o resultado depende demais dos pesos escolhidos.</t>
         </is>
       </c>
-      <c r="D22" s="43" t="inlineStr">
+      <c r="D23" s="43" t="inlineStr">
         <is>
           <t>Se o top 5 muda muito, avisar a alta gestão.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="56" t="inlineStr">
-        <is>
-          <t>Tipo de nota</t>
-        </is>
-      </c>
-      <c r="B23" s="55" t="inlineStr">
-        <is>
-          <t>Faixa fixa</t>
-        </is>
-      </c>
-      <c r="C23" s="43" t="inlineStr">
-        <is>
-          <t>O valor medido cai numa faixa definida antes da coleta. A nota não depende dos outros pontos.</t>
-        </is>
-      </c>
-      <c r="D23" s="43" t="inlineStr">
-        <is>
-          <t>P1: 5 alagamentos/ano cai em '5–6' = nota 4.</t>
         </is>
       </c>
     </row>
@@ -4943,17 +5207,17 @@
       </c>
       <c r="B24" s="55" t="inlineStr">
         <is>
-          <t>Classe</t>
+          <t>Faixa fixa</t>
         </is>
       </c>
       <c r="C24" s="43" t="inlineStr">
         <is>
-          <t>O ponto é encaixado numa categoria descritiva, não num número.</t>
+          <t>O valor medido cai numa faixa definida antes da coleta. A nota não depende dos outros pontos.</t>
         </is>
       </c>
       <c r="D24" s="43" t="inlineStr">
         <is>
-          <t>P3: 'agrava ocasionalmente' = nota 3.</t>
+          <t>P1: 5 alagamentos/ano cai em '5–6' = nota 4.</t>
         </is>
       </c>
     </row>
@@ -4965,17 +5229,17 @@
       </c>
       <c r="B25" s="55" t="inlineStr">
         <is>
-          <t>Quintil</t>
+          <t>Classe</t>
         </is>
       </c>
       <c r="C25" s="43" t="inlineStr">
         <is>
-          <t>Nota relativa entre os 21 pontos: os valores são ordenados e divididos em 5 grupos de ~4 pontos. Os 20% menores recebem 1; os 20% maiores, 5.</t>
+          <t>O ponto é encaixado numa categoria descritiva, não num número.</t>
         </is>
       </c>
       <c r="D25" s="43" t="inlineStr">
         <is>
-          <t>E1: os ~4 pontos com mais moradores recebem nota 5.</t>
+          <t>P3: 'agrava ocasionalmente' = nota 3.</t>
         </is>
       </c>
     </row>
@@ -4987,17 +5251,17 @@
       </c>
       <c r="B26" s="55" t="inlineStr">
         <is>
-          <t>Quintil invertido</t>
+          <t>Quintil</t>
         </is>
       </c>
       <c r="C26" s="43" t="inlineStr">
         <is>
-          <t>Igual ao quintil, mas o MENOR valor recebe a nota mais alta.</t>
+          <t>Nota relativa entre os 21 pontos: os valores são ordenados e divididos em 5 grupos de ~4 pontos. Os 20% menores recebem 1; os 20% maiores, 5.</t>
         </is>
       </c>
       <c r="D26" s="43" t="inlineStr">
         <is>
-          <t>P4: o ponto mais perto do rio recebe nota 5.</t>
+          <t>E1: os ~4 pontos com mais moradores recebem nota 5.</t>
         </is>
       </c>
     </row>
@@ -5009,17 +5273,17 @@
       </c>
       <c r="B27" s="55" t="inlineStr">
         <is>
-          <t>Faixa provisória</t>
+          <t>Quintil invertido</t>
         </is>
       </c>
       <c r="C27" s="43" t="inlineStr">
         <is>
-          <t>Faixa proposta antes de ver os dados reais. Deve ser calibrada quando os dados chegarem.</t>
+          <t>Igual ao quintil, mas o MENOR valor recebe a nota mais alta.</t>
         </is>
       </c>
       <c r="D27" s="43" t="inlineStr">
         <is>
-          <t>Se todos os pontos caírem na mesma faixa, ela precisa ser ajustada.</t>
+          <t>P4: o ponto mais perto do rio recebe nota 5.</t>
         </is>
       </c>
     </row>
@@ -5031,37 +5295,37 @@
       </c>
       <c r="B28" s="55" t="inlineStr">
         <is>
+          <t>Faixa provisória</t>
+        </is>
+      </c>
+      <c r="C28" s="43" t="inlineStr">
+        <is>
+          <t>Faixa proposta antes de ver os dados reais. Deve ser calibrada quando os dados chegarem.</t>
+        </is>
+      </c>
+      <c r="D28" s="43" t="inlineStr">
+        <is>
+          <t>Se todos os pontos caírem na mesma faixa, ela precisa ser ajustada.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="56" t="inlineStr">
+        <is>
+          <t>Tipo de nota</t>
+        </is>
+      </c>
+      <c r="B29" s="55" t="inlineStr">
+        <is>
           <t>Origem da faixa</t>
         </is>
       </c>
-      <c r="C28" s="43" t="inlineStr">
+      <c r="C29" s="43" t="inlineStr">
         <is>
           <t>De onde veio a escala: planilha original da equipe, referência oficial (ex.: Ipea) ou proposta do Claude (a revisar pelo grupo).</t>
         </is>
       </c>
-      <c r="D28" s="43" t="inlineStr"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="57" t="inlineStr">
-        <is>
-          <t>Território e SIG</t>
-        </is>
-      </c>
-      <c r="B29" s="55" t="inlineStr">
-        <is>
-          <t>Ponto crítico</t>
-        </is>
-      </c>
-      <c r="C29" s="43" t="inlineStr">
-        <is>
-          <t>Local da lista da EMLURB onde há alagamento recorrente. Pode ser um ponto, um trecho de rua ou vários trechos.</t>
-        </is>
-      </c>
-      <c r="D29" s="43" t="inlineStr">
-        <is>
-          <t>Ponto 24 — Ipsep, Rua Blumenau (até a maré).</t>
-        </is>
-      </c>
+      <c r="D29" s="43" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="57" t="inlineStr">
@@ -5071,17 +5335,17 @@
       </c>
       <c r="B30" s="55" t="inlineStr">
         <is>
-          <t>Trecho (Linha / Vários)</t>
+          <t>Ponto crítico</t>
         </is>
       </c>
       <c r="C30" s="43" t="inlineStr">
         <is>
-          <t>Ponto crítico que é uma extensão de rua, não um local único. 12 dos 21 pontos são trechos.</t>
+          <t>Local da lista da EMLURB onde há alagamento recorrente. Pode ser um ponto, um trecho de rua ou vários trechos.</t>
         </is>
       </c>
       <c r="D30" s="43" t="inlineStr">
         <is>
-          <t>Ponto 11 — Rua Professor José Brandão (toda a extensão).</t>
+          <t>Ponto 24 — Ipsep, Rua Blumenau (até a maré).</t>
         </is>
       </c>
     </row>
@@ -5093,15 +5357,19 @@
       </c>
       <c r="B31" s="55" t="inlineStr">
         <is>
-          <t>RPA 6</t>
+          <t>Trecho (Linha / Vários)</t>
         </is>
       </c>
       <c r="C31" s="43" t="inlineStr">
         <is>
-          <t>Região Político-Administrativa 6 do Recife (Boa Viagem, Pina, Imbiribeira, Ipsep, Ibura, Jordão, entre outros bairros). Escopo do piloto.</t>
-        </is>
-      </c>
-      <c r="D31" s="43" t="inlineStr"/>
+          <t>Ponto crítico que é uma extensão de rua, não um local único. 12 dos 21 pontos são trechos.</t>
+        </is>
+      </c>
+      <c r="D31" s="43" t="inlineStr">
+        <is>
+          <t>Ponto 11 — Rua Professor José Brandão (toda a extensão).</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="57" t="inlineStr">
@@ -5111,12 +5379,12 @@
       </c>
       <c r="B32" s="55" t="inlineStr">
         <is>
-          <t>SIG</t>
+          <t>RPA 6</t>
         </is>
       </c>
       <c r="C32" s="43" t="inlineStr">
         <is>
-          <t>Sistema de Informação Geográfica: programa para mapas e cálculos espaciais. Usamos o ArcGIS Pro.</t>
+          <t>Região Político-Administrativa 6 do Recife (Boa Viagem, Pina, Imbiribeira, Ipsep, Ibura, Jordão, entre outros bairros). Escopo do piloto.</t>
         </is>
       </c>
       <c r="D32" s="43" t="inlineStr"/>
@@ -5129,19 +5397,15 @@
       </c>
       <c r="B33" s="55" t="inlineStr">
         <is>
-          <t>Círculo de 300 m (buffer)</t>
+          <t>SIG</t>
         </is>
       </c>
       <c r="C33" s="43" t="inlineStr">
         <is>
-          <t>Área de 300 m em volta do ponto (ou da linha do trecho) onde se medem os subcritérios do SIG. Usado no cálculo do risco.</t>
-        </is>
-      </c>
-      <c r="D33" s="43" t="inlineStr">
-        <is>
-          <t>Moradores dentro do círculo = População (E1).</t>
-        </is>
-      </c>
+          <t>Sistema de Informação Geográfica: programa para mapas e cálculos espaciais. Usamos o ArcGIS Pro.</t>
+        </is>
+      </c>
+      <c r="D33" s="43" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="57" t="inlineStr">
@@ -5151,15 +5415,19 @@
       </c>
       <c r="B34" s="55" t="inlineStr">
         <is>
-          <t>Área de influência de 1 km</t>
+          <t>Círculo de 300 m (buffer)</t>
         </is>
       </c>
       <c r="C34" s="43" t="inlineStr">
         <is>
-          <t>Círculo de 1 km mostrado no painel só como informação. Não entra no cálculo, porque com 1 km quase todos os pontos se sobrepõem.</t>
-        </is>
-      </c>
-      <c r="D34" s="43" t="inlineStr"/>
+          <t>Área de 300 m em volta do ponto (ou da linha do trecho) onde se medem os subcritérios do SIG. Usado no cálculo do risco.</t>
+        </is>
+      </c>
+      <c r="D34" s="43" t="inlineStr">
+        <is>
+          <t>Moradores dentro do círculo = População (E1).</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="57" t="inlineStr">
@@ -5169,19 +5437,15 @@
       </c>
       <c r="B35" s="55" t="inlineStr">
         <is>
-          <t>Grupo de sobreposição (G1–G5)</t>
+          <t>Área de influência de 1 km</t>
         </is>
       </c>
       <c r="C35" s="43" t="inlineStr">
         <is>
-          <t>Pontos cujos círculos de 300 m se sobrepõem. Nesses grupos os subcritérios do SIG tendem a dar notas parecidas.</t>
-        </is>
-      </c>
-      <c r="D35" s="43" t="inlineStr">
-        <is>
-          <t>G1 = pontos 5, 6, 7, 11 e 12 (Conselheiro Aguiar).</t>
-        </is>
-      </c>
+          <t>Círculo de 1 km mostrado no painel só como informação. Não entra no cálculo, porque com 1 km quase todos os pontos se sobrepõem.</t>
+        </is>
+      </c>
+      <c r="D35" s="43" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="57" t="inlineStr">
@@ -5191,17 +5455,17 @@
       </c>
       <c r="B36" s="55" t="inlineStr">
         <is>
-          <t>Ponderação por área</t>
+          <t>Grupo de sobreposição (G1–G5)</t>
         </is>
       </c>
       <c r="C36" s="43" t="inlineStr">
         <is>
-          <t>Quando uma área de dados (setor, célula) corta o círculo, conta só a parte que fica dentro dele.</t>
+          <t>Pontos cujos círculos de 300 m se sobrepõem. Nesses grupos os subcritérios do SIG tendem a dar notas parecidas.</t>
         </is>
       </c>
       <c r="D36" s="43" t="inlineStr">
         <is>
-          <t>Setor com 40% da área no círculo contribui com 40% da população.</t>
+          <t>G1 = pontos 5, 6, 7, 11 e 12 (Conselheiro Aguiar).</t>
         </is>
       </c>
     </row>
@@ -5213,15 +5477,19 @@
       </c>
       <c r="B37" s="55" t="inlineStr">
         <is>
-          <t>EPSG:31985 (SIRGAS 2000 / UTM 25S)</t>
+          <t>Ponderação por área</t>
         </is>
       </c>
       <c r="C37" s="43" t="inlineStr">
         <is>
-          <t>Sistema de coordenadas usado no projeto. Todas as camadas precisam estar nele antes dos cálculos.</t>
-        </is>
-      </c>
-      <c r="D37" s="43" t="inlineStr"/>
+          <t>Quando uma área de dados (setor, célula) corta o círculo, conta só a parte que fica dentro dele.</t>
+        </is>
+      </c>
+      <c r="D37" s="43" t="inlineStr">
+        <is>
+          <t>Setor com 40% da área no círculo contribui com 40% da população.</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="57" t="inlineStr">
@@ -5231,19 +5499,15 @@
       </c>
       <c r="B38" s="55" t="inlineStr">
         <is>
-          <t>Coordenada aproximada / verificada</t>
+          <t>EPSG:31985 (SIRGAS 2000 / UTM 25S)</t>
         </is>
       </c>
       <c r="C38" s="43" t="inlineStr">
         <is>
-          <t>Aproximada = localizada automaticamente e ainda não conferida. Verificada = conferida com a EMLURB ou por imagem de satélite.</t>
-        </is>
-      </c>
-      <c r="D38" s="43" t="inlineStr">
-        <is>
-          <t>Hoje nenhuma das 21 coordenadas está verificada.</t>
-        </is>
-      </c>
+          <t>Sistema de coordenadas usado no projeto. Todas as camadas precisam estar nele antes dos cálculos.</t>
+        </is>
+      </c>
+      <c r="D38" s="43" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="57" t="inlineStr">
@@ -5253,17 +5517,17 @@
       </c>
       <c r="B39" s="55" t="inlineStr">
         <is>
-          <t>Bacia / sub-bacia</t>
+          <t>Coordenada aproximada / verificada</t>
         </is>
       </c>
       <c r="C39" s="43" t="inlineStr">
         <is>
-          <t>Área que drena para um mesmo rio ou canal. Hierarquia do Plano de Drenagem: Bacia → Sub-bacia → Ponto crítico → Obra.</t>
+          <t>Aproximada = localizada automaticamente e ainda não conferida. Verificada = conferida com a EMLURB ou por imagem de satélite.</t>
         </is>
       </c>
       <c r="D39" s="43" t="inlineStr">
         <is>
-          <t>Usada para ligar obras aos pontos.</t>
+          <t>Hoje nenhuma das 21 coordenadas está verificada.</t>
         </is>
       </c>
     </row>
@@ -5275,37 +5539,41 @@
       </c>
       <c r="B40" s="55" t="inlineStr">
         <is>
+          <t>Bacia / sub-bacia</t>
+        </is>
+      </c>
+      <c r="C40" s="43" t="inlineStr">
+        <is>
+          <t>Área que drena para um mesmo rio ou canal. Hierarquia do Plano de Drenagem: Bacia → Sub-bacia → Ponto crítico → Obra.</t>
+        </is>
+      </c>
+      <c r="D40" s="43" t="inlineStr">
+        <is>
+          <t>Usada para ligar obras aos pontos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="57" t="inlineStr">
+        <is>
+          <t>Território e SIG</t>
+        </is>
+      </c>
+      <c r="B41" s="55" t="inlineStr">
+        <is>
           <t>Shapefile / GeoJSON</t>
         </is>
       </c>
-      <c r="C40" s="43" t="inlineStr">
+      <c r="C41" s="43" t="inlineStr">
         <is>
           <t>Formatos de arquivo de mapa que o ArcGIS abre.</t>
         </is>
       </c>
-      <c r="D40" s="43" t="inlineStr">
+      <c r="D41" s="43" t="inlineStr">
         <is>
           <t>dados/processados/pontos_rpa6.geojson tem os 21 pontos.</t>
         </is>
       </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="58" t="inlineStr">
-        <is>
-          <t>Fontes de dados</t>
-        </is>
-      </c>
-      <c r="B41" s="55" t="inlineStr">
-        <is>
-          <t>Censo 2022 (IBGE)</t>
-        </is>
-      </c>
-      <c r="C41" s="43" t="inlineStr">
-        <is>
-          <t>Recenseamento de 2022. Fonte de população, idade, tipo de domicílio e esgotamento.</t>
-        </is>
-      </c>
-      <c r="D41" s="43" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="58" t="inlineStr">
@@ -5315,12 +5583,12 @@
       </c>
       <c r="B42" s="55" t="inlineStr">
         <is>
-          <t>Setor censitário</t>
+          <t>Censo 2022 (IBGE)</t>
         </is>
       </c>
       <c r="C42" s="43" t="inlineStr">
         <is>
-          <t>Menor área de divulgação do Censo (no Recife adensado, poucos quarteirões).</t>
+          <t>Recenseamento de 2022. Fonte de população, idade, tipo de domicílio e esgotamento.</t>
         </is>
       </c>
       <c r="D42" s="43" t="inlineStr"/>
@@ -5333,19 +5601,15 @@
       </c>
       <c r="B43" s="55" t="inlineStr">
         <is>
-          <t>Grade Estatística (IBGE)</t>
+          <t>Setor censitário</t>
         </is>
       </c>
       <c r="C43" s="43" t="inlineStr">
         <is>
-          <t>Malha de quadrados de 200 × 200 m (área urbana) com a população do Censo 2022.</t>
-        </is>
-      </c>
-      <c r="D43" s="43" t="inlineStr">
-        <is>
-          <t>Fonte do E1.</t>
-        </is>
-      </c>
+          <t>Menor área de divulgação do Censo (no Recife adensado, poucos quarteirões).</t>
+        </is>
+      </c>
+      <c r="D43" s="43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="58" t="inlineStr">
@@ -5355,17 +5619,17 @@
       </c>
       <c r="B44" s="55" t="inlineStr">
         <is>
-          <t>CNEFE (IBGE)</t>
+          <t>Grade Estatística (IBGE)</t>
         </is>
       </c>
       <c r="C44" s="43" t="inlineStr">
         <is>
-          <t>Cadastro de endereços do Censo 2022, com coordenada e tipo de uso (domicílio, ensino, saúde, outras finalidades).</t>
+          <t>Malha de quadrados de 200 × 200 m (área urbana) com a população do Censo 2022.</t>
         </is>
       </c>
       <c r="D44" s="43" t="inlineStr">
         <is>
-          <t>Fonte do E2 e do E3.</t>
+          <t>Fonte do E1.</t>
         </is>
       </c>
     </row>
@@ -5377,17 +5641,17 @@
       </c>
       <c r="B45" s="55" t="inlineStr">
         <is>
-          <t>Favelas e Comunidades Urbanas (IBGE)</t>
+          <t>CNEFE (IBGE)</t>
         </is>
       </c>
       <c r="C45" s="43" t="inlineStr">
         <is>
-          <t>Mapeamento do IBGE das favelas e comunidades urbanas no Censo 2022. Publicação da malha ainda não confirmada.</t>
+          <t>Cadastro de endereços do Censo 2022, com coordenada e tipo de uso (domicílio, ensino, saúde, outras finalidades).</t>
         </is>
       </c>
       <c r="D45" s="43" t="inlineStr">
         <is>
-          <t>Fonte do V3.</t>
+          <t>Fonte do E2 e do E3.</t>
         </is>
       </c>
     </row>
@@ -5399,17 +5663,17 @@
       </c>
       <c r="B46" s="55" t="inlineStr">
         <is>
-          <t>IVS (Ipea)</t>
+          <t>Favelas e Comunidades Urbanas (IBGE)</t>
         </is>
       </c>
       <c r="C46" s="43" t="inlineStr">
         <is>
-          <t>Índice de Vulnerabilidade Social do Ipea, de 0 a 1 (quanto maior, mais vulnerável). Base do Censo 2010.</t>
+          <t>Mapeamento do IBGE das favelas e comunidades urbanas no Censo 2022. Publicação da malha ainda não confirmada.</t>
         </is>
       </c>
       <c r="D46" s="43" t="inlineStr">
         <is>
-          <t>Plano B do V3.</t>
+          <t>Fonte do V3.</t>
         </is>
       </c>
     </row>
@@ -5421,15 +5685,19 @@
       </c>
       <c r="B47" s="55" t="inlineStr">
         <is>
-          <t>UDH</t>
+          <t>IVS (Ipea)</t>
         </is>
       </c>
       <c r="C47" s="43" t="inlineStr">
         <is>
-          <t>Unidade de Desenvolvimento Humano: área usada pelo Ipea, maior que o setor censitário.</t>
-        </is>
-      </c>
-      <c r="D47" s="43" t="inlineStr"/>
+          <t>Índice de Vulnerabilidade Social do Ipea, de 0 a 1 (quanto maior, mais vulnerável). Base do Censo 2010.</t>
+        </is>
+      </c>
+      <c r="D47" s="43" t="inlineStr">
+        <is>
+          <t>Plano B do V3.</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="58" t="inlineStr">
@@ -5439,19 +5707,15 @@
       </c>
       <c r="B48" s="55" t="inlineStr">
         <is>
-          <t>MapBiomas</t>
+          <t>UDH</t>
         </is>
       </c>
       <c r="C48" s="43" t="inlineStr">
         <is>
-          <t>Mapa de cobertura do solo (vegetação, área construída etc.) com pixels de 30 m. Não verificado.</t>
-        </is>
-      </c>
-      <c r="D48" s="43" t="inlineStr">
-        <is>
-          <t>Fonte do P5.</t>
-        </is>
-      </c>
+          <t>Unidade de Desenvolvimento Humano: área usada pelo Ipea, maior que o setor censitário.</t>
+        </is>
+      </c>
+      <c r="D48" s="43" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="58" t="inlineStr">
@@ -5461,15 +5725,19 @@
       </c>
       <c r="B49" s="55" t="inlineStr">
         <is>
-          <t>ESIG</t>
+          <t>MapBiomas</t>
         </is>
       </c>
       <c r="C49" s="43" t="inlineStr">
         <is>
-          <t>Sistema de informações geográficas da Prefeitura do Recife (vias, lotes, edificações, recursos hídricos).</t>
-        </is>
-      </c>
-      <c r="D49" s="43" t="inlineStr"/>
+          <t>Mapa de cobertura do solo (vegetação, área construída etc.) com pixels de 30 m. Não verificado.</t>
+        </is>
+      </c>
+      <c r="D49" s="43" t="inlineStr">
+        <is>
+          <t>Fonte do P5.</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="58" t="inlineStr">
@@ -5479,19 +5747,15 @@
       </c>
       <c r="B50" s="55" t="inlineStr">
         <is>
-          <t>CNES / DATASUS</t>
+          <t>ESIG</t>
         </is>
       </c>
       <c r="C50" s="43" t="inlineStr">
         <is>
-          <t>Cadastro Nacional de Estabelecimentos de Saúde.</t>
-        </is>
-      </c>
-      <c r="D50" s="43" t="inlineStr">
-        <is>
-          <t>Complementa o E2.</t>
-        </is>
-      </c>
+          <t>Sistema de informações geográficas da Prefeitura do Recife (vias, lotes, edificações, recursos hídricos).</t>
+        </is>
+      </c>
+      <c r="D50" s="43" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="58" t="inlineStr">
@@ -5501,15 +5765,19 @@
       </c>
       <c r="B51" s="55" t="inlineStr">
         <is>
-          <t>APAC / Cemaden</t>
+          <t>CNES / DATASUS</t>
         </is>
       </c>
       <c r="C51" s="43" t="inlineStr">
         <is>
-          <t>Agência Pernambucana de Águas e Clima / Centro Nacional de Monitoramento de Desastres: dados de chuva e marés.</t>
-        </is>
-      </c>
-      <c r="D51" s="43" t="inlineStr"/>
+          <t>Cadastro Nacional de Estabelecimentos de Saúde.</t>
+        </is>
+      </c>
+      <c r="D51" s="43" t="inlineStr">
+        <is>
+          <t>Complementa o E2.</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="58" t="inlineStr">
@@ -5519,12 +5787,12 @@
       </c>
       <c r="B52" s="55" t="inlineStr">
         <is>
-          <t>PMDR</t>
+          <t>APAC / Cemaden</t>
         </is>
       </c>
       <c r="C52" s="43" t="inlineStr">
         <is>
-          <t>Plano Municipal de Drenagem do Recife. Define bacias e sub-bacias.</t>
+          <t>Agência Pernambucana de Águas e Clima / Centro Nacional de Monitoramento de Desastres: dados de chuva e marés.</t>
         </is>
       </c>
       <c r="D52" s="43" t="inlineStr"/>
@@ -5537,37 +5805,37 @@
       </c>
       <c r="B53" s="55" t="inlineStr">
         <is>
+          <t>PMDR</t>
+        </is>
+      </c>
+      <c r="C53" s="43" t="inlineStr">
+        <is>
+          <t>Plano Municipal de Drenagem do Recife. Define bacias e sub-bacias.</t>
+        </is>
+      </c>
+      <c r="D53" s="43" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="58" t="inlineStr">
+        <is>
+          <t>Fontes de dados</t>
+        </is>
+      </c>
+      <c r="B54" s="55" t="inlineStr">
+        <is>
           <t>Ficha EMLURB</t>
         </is>
       </c>
-      <c r="C53" s="43" t="inlineStr">
+      <c r="C54" s="43" t="inlineStr">
         <is>
           <t>Formulário a ser preenchido com a EMLURB, com uma linha por ponto: localização, frequência, severidade, maré e obras ligadas.</t>
         </is>
       </c>
-      <c r="D53" s="43" t="inlineStr">
+      <c r="D54" s="43" t="inlineStr">
         <is>
           <t>Fonte provisória de P1, P2 e P3.</t>
         </is>
       </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="59" t="inlineStr">
-        <is>
-          <t>Checklist</t>
-        </is>
-      </c>
-      <c r="B54" s="55" t="inlineStr">
-        <is>
-          <t>Recomendação</t>
-        </is>
-      </c>
-      <c r="C54" s="43" t="inlineStr">
-        <is>
-          <t>Manter = entra no modelo. Condicional = só entra se o dado existir. Plano B = usado só se outro subcritério falhar. Peso alto / menor = sugestão para a definição dos pesos.</t>
-        </is>
-      </c>
-      <c r="D54" s="43" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" s="59" t="inlineStr">
@@ -5577,12 +5845,12 @@
       </c>
       <c r="B55" s="55" t="inlineStr">
         <is>
-          <t>Fonte confirmada?</t>
+          <t>Recomendação</t>
         </is>
       </c>
       <c r="C55" s="43" t="inlineStr">
         <is>
-          <t>A base de dados existe e a equipe consegue acessá-la (download ou pedido atendido).</t>
+          <t>Manter = entra no modelo. Condicional = só entra se o dado existir. Plano B = usado só se outro subcritério falhar. Peso alto / menor = sugestão para a definição dos pesos.</t>
         </is>
       </c>
       <c r="D55" s="43" t="inlineStr"/>
@@ -5595,19 +5863,15 @@
       </c>
       <c r="B56" s="55" t="inlineStr">
         <is>
-          <t>Dado existe na fonte?</t>
+          <t>Fonte confirmada?</t>
         </is>
       </c>
       <c r="C56" s="43" t="inlineStr">
         <is>
-          <t>A variável necessária está na base, na escala do círculo de 300 m, e cobre os 21 pontos.</t>
-        </is>
-      </c>
-      <c r="D56" s="43" t="inlineStr">
-        <is>
-          <t>O IBGE existe (fonte confirmada), mas falta checar se o tipo de domicílio vem por setor.</t>
-        </is>
-      </c>
+          <t>A base de dados existe e a equipe consegue acessá-la (download ou pedido atendido).</t>
+        </is>
+      </c>
+      <c r="D56" s="43" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" s="59" t="inlineStr">
@@ -5617,15 +5881,19 @@
       </c>
       <c r="B57" s="55" t="inlineStr">
         <is>
-          <t>Sim / Parcial / Não / Pendente</t>
+          <t>Dado existe na fonte?</t>
         </is>
       </c>
       <c r="C57" s="43" t="inlineStr">
         <is>
-          <t>Sim = confirmado. Parcial = existe, mas com limitação (escala, cobertura, data). Não = não existe ou não é acessível. Pendente = ainda não checado.</t>
-        </is>
-      </c>
-      <c r="D57" s="43" t="inlineStr"/>
+          <t>A variável necessária está na base, na escala do círculo de 300 m, e cobre os 21 pontos.</t>
+        </is>
+      </c>
+      <c r="D57" s="43" t="inlineStr">
+        <is>
+          <t>O IBGE existe (fonte confirmada), mas falta checar se o tipo de domicílio vem por setor.</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="59" t="inlineStr">
@@ -5635,30 +5903,30 @@
       </c>
       <c r="B58" s="55" t="inlineStr">
         <is>
+          <t>Sim / Parcial / Não / Pendente</t>
+        </is>
+      </c>
+      <c r="C58" s="43" t="inlineStr">
+        <is>
+          <t>Sim = confirmado. Parcial = existe, mas com limitação (escala, cobertura, data). Não = não existe ou não é acessível. Pendente = ainda não checado.</t>
+        </is>
+      </c>
+      <c r="D58" s="43" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="59" t="inlineStr">
+        <is>
+          <t>Checklist</t>
+        </is>
+      </c>
+      <c r="B59" s="55" t="inlineStr">
+        <is>
           <t>Busca prévia (Claude)</t>
         </is>
       </c>
-      <c r="C58" s="43" t="inlineStr">
+      <c r="C59" s="43" t="inlineStr">
         <is>
           <t>O que foi encontrado em busca na internet. 'Confirmado na busca' = a base aparece como publicada, mas o arquivo não foi aberto.</t>
-        </is>
-      </c>
-      <c r="D58" s="43" t="inlineStr"/>
-    </row>
-    <row r="59">
-      <c r="A59" s="60" t="inlineStr">
-        <is>
-          <t>Órgãos</t>
-        </is>
-      </c>
-      <c r="B59" s="55" t="inlineStr">
-        <is>
-          <t>COP</t>
-        </is>
-      </c>
-      <c r="C59" s="43" t="inlineStr">
-        <is>
-          <t>Centro de Operações do Recife: monitoramento e resposta aos eventos.</t>
         </is>
       </c>
       <c r="D59" s="43" t="inlineStr"/>
@@ -5671,12 +5939,12 @@
       </c>
       <c r="B60" s="55" t="inlineStr">
         <is>
-          <t>EMLURB</t>
+          <t>COP</t>
         </is>
       </c>
       <c r="C60" s="43" t="inlineStr">
         <is>
-          <t>Empresa de Manutenção e Limpeza Urbana: manutenção da drenagem e lista de pontos críticos.</t>
+          <t>Centro de Operações do Recife: monitoramento e resposta aos eventos.</t>
         </is>
       </c>
       <c r="D60" s="43" t="inlineStr"/>
@@ -5689,12 +5957,12 @@
       </c>
       <c r="B61" s="55" t="inlineStr">
         <is>
-          <t>Defesa Civil (Sedec)</t>
+          <t>EMLURB</t>
         </is>
       </c>
       <c r="C61" s="43" t="inlineStr">
         <is>
-          <t>Áreas de risco, alertas e vistorias.</t>
+          <t>Empresa de Manutenção e Limpeza Urbana: manutenção da drenagem e lista de pontos críticos.</t>
         </is>
       </c>
       <c r="D61" s="43" t="inlineStr"/>
@@ -5707,12 +5975,12 @@
       </c>
       <c r="B62" s="55" t="inlineStr">
         <is>
-          <t>URB</t>
+          <t>Defesa Civil (Sedec)</t>
         </is>
       </c>
       <c r="C62" s="43" t="inlineStr">
         <is>
-          <t>Autarquia de Urbanização do Recife: obras urbanas e de drenagem.</t>
+          <t>Áreas de risco, alertas e vistorias.</t>
         </is>
       </c>
       <c r="D62" s="43" t="inlineStr"/>
@@ -5725,12 +5993,12 @@
       </c>
       <c r="B63" s="55" t="inlineStr">
         <is>
-          <t>CTTU</t>
+          <t>URB</t>
         </is>
       </c>
       <c r="C63" s="43" t="inlineStr">
         <is>
-          <t>Autarquia de Trânsito e Transporte Urbano: trânsito, vias e interdições.</t>
+          <t>Autarquia de Urbanização do Recife: obras urbanas e de drenagem.</t>
         </is>
       </c>
       <c r="D63" s="43" t="inlineStr"/>
@@ -5743,12 +6011,12 @@
       </c>
       <c r="B64" s="55" t="inlineStr">
         <is>
-          <t>Compesa</t>
+          <t>CTTU</t>
         </is>
       </c>
       <c r="C64" s="43" t="inlineStr">
         <is>
-          <t>Companhia Pernambucana de Saneamento: água e esgoto.</t>
+          <t>Autarquia de Trânsito e Transporte Urbano: trânsito, vias e interdições.</t>
         </is>
       </c>
       <c r="D64" s="43" t="inlineStr"/>
@@ -5761,12 +6029,12 @@
       </c>
       <c r="B65" s="55" t="inlineStr">
         <is>
-          <t>ProMorar</t>
+          <t>Compesa</t>
         </is>
       </c>
       <c r="C65" s="43" t="inlineStr">
         <is>
-          <t>Programa de urbanização de comunidades.</t>
+          <t>Companhia Pernambucana de Saneamento: água e esgoto.</t>
         </is>
       </c>
       <c r="D65" s="43" t="inlineStr"/>
@@ -5779,12 +6047,12 @@
       </c>
       <c r="B66" s="55" t="inlineStr">
         <is>
-          <t>SEPLAG / SEPLAN</t>
+          <t>ProMorar</t>
         </is>
       </c>
       <c r="C66" s="43" t="inlineStr">
         <is>
-          <t>Planejamento e gestão. A SEPLAN não é a SEPLAG; o papel dela no projeto ainda será definido.</t>
+          <t>Programa de urbanização de comunidades.</t>
         </is>
       </c>
       <c r="D66" s="43" t="inlineStr"/>
@@ -5797,18 +6065,36 @@
       </c>
       <c r="B67" s="55" t="inlineStr">
         <is>
+          <t>SEPLAG / SEPLAN</t>
+        </is>
+      </c>
+      <c r="C67" s="43" t="inlineStr">
+        <is>
+          <t>Planejamento e gestão. A SEPLAN não é a SEPLAG; o papel dela no projeto ainda será definido.</t>
+        </is>
+      </c>
+      <c r="D67" s="43" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="60" t="inlineStr">
+        <is>
+          <t>Órgãos</t>
+        </is>
+      </c>
+      <c r="B68" s="55" t="inlineStr">
+        <is>
           <t>Grande Recife Consórcio</t>
         </is>
       </c>
-      <c r="C67" s="43" t="inlineStr">
+      <c r="C68" s="43" t="inlineStr">
         <is>
           <t>Consórcio de transporte metropolitano: linhas e paradas de ônibus.</t>
         </is>
       </c>
-      <c r="D67" s="43" t="inlineStr"/>
+      <c r="D68" s="43" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A4:D67"/>
+  <autoFilter ref="A4:D68"/>
   <mergeCells count="1">
     <mergeCell ref="A2:D2"/>
   </mergeCells>

</xml_diff>

<commit_message>
I1 Tipo de via: escala de 1 a 5 por classe de corredor (Pedro); pendência 17
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R5swnHARNHJ12oc84LP2b9
</commit_message>
<xml_diff>
--- a/dados/Recife_Resiliente_Checklist_Subcriterios.xlsx
+++ b/dados/Recife_Resiliente_Checklist_Subcriterios.xlsx
@@ -2137,12 +2137,12 @@
       </c>
       <c r="C20" s="6" t="inlineStr">
         <is>
-          <t>Interrupção do trânsito</t>
+          <t>Tipo de via</t>
         </is>
       </c>
       <c r="D20" s="6" t="inlineStr">
         <is>
-          <t>Classe da via mais importante afetada pelo alagamento; +1 se houver interdição registrada pela CTTU (máximo 5)</t>
+          <t>Classe da via mais importante afetada pelo alagamento (no trecho: a própria via)</t>
         </is>
       </c>
       <c r="E20" s="7" t="inlineStr">
@@ -2152,32 +2152,32 @@
       </c>
       <c r="F20" s="8" t="inlineStr">
         <is>
-          <t>Via local ou de pedestres</t>
+          <t>Ruas</t>
         </is>
       </c>
       <c r="G20" s="9" t="inlineStr">
         <is>
-          <t>Coletora</t>
+          <t>Demais avenidas</t>
         </is>
       </c>
       <c r="H20" s="10" t="inlineStr">
         <is>
-          <t>Arterial secundária</t>
+          <t>Corredor de transporte urbano secundário</t>
         </is>
       </c>
       <c r="I20" s="11" t="inlineStr">
         <is>
-          <t>Arterial principal</t>
+          <t>Corredor de transporte urbano principal</t>
         </is>
       </c>
       <c r="J20" s="12" t="inlineStr">
         <is>
-          <t>Trânsito rápido ou corredor de ônibus</t>
+          <t>Corredor de transporte metropolitano</t>
         </is>
       </c>
       <c r="K20" s="6" t="inlineStr">
         <is>
-          <t>Proposta Claude, a partir da classificação viária usada na planilha original</t>
+          <t>Pedro (03/10/2026)</t>
         </is>
       </c>
       <c r="L20" s="6" t="inlineStr">
@@ -2187,7 +2187,7 @@
       </c>
       <c r="M20" s="6" t="inlineStr">
         <is>
-          <t>Hierarquia viária (ESIG / CTTU); OSM; corredores de ônibus e fluxo de veículos (portal); paradas (Grande Recife); interdições (CTTU)</t>
+          <t>Corredores de ônibus (portal de dados abertos); hierarquia viária e corredores (CTTU / Grande Recife)</t>
         </is>
       </c>
       <c r="N20" s="13" t="inlineStr">
@@ -2202,12 +2202,12 @@
       </c>
       <c r="P20" s="14" t="inlineStr">
         <is>
-          <t>Junta 'vias principais' e 'interrupção do trânsito' do documento da equipe. Pedir a Antônio (CTTU): hierarquia viária, linhas e registro de interdições.</t>
+          <t>Interdição registrada pela CTTU serve só para conferir a nota (não soma). Junta 'vias principais' e 'interrupção do trânsito' do documento da equipe. Confirmar qual base classifica os corredores em metropolitano / urbano principal / urbano secundário (pendência 17).</t>
         </is>
       </c>
       <c r="Q20" s="6" t="inlineStr">
         <is>
-          <t>Vias no ESIG confirmadas na busca; ônibus e interdições não verificados.</t>
+          <t>Corredores de ônibus localizados no portal (não abertos); classificação dos corredores não verificada.</t>
         </is>
       </c>
     </row>
@@ -2745,7 +2745,7 @@
       <c r="AA6" s="40" t="inlineStr">
         <is>
           <t>I1
-Interrupção do trânsito</t>
+Tipo de via</t>
         </is>
       </c>
       <c r="AB6" s="40" t="inlineStr">
@@ -4935,7 +4935,7 @@
       </c>
       <c r="D11" s="43" t="inlineStr">
         <is>
-          <t>Alagamento numa avenida arterial com ônibus tem Interrupção do trânsito (I1) alta.</t>
+          <t>Alagamento num corredor de transporte metropolitano tem Tipo de via (I1) = 5.</t>
         </is>
       </c>
     </row>

</xml_diff>